<commit_message>
wireframes updated, slide nos. added to user stories following wireframes ppt
</commit_message>
<xml_diff>
--- a/Soubhanik/checkupp_product_backlog_final.xlsx
+++ b/Soubhanik/checkupp_product_backlog_final.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Anodiam\2026\CheckUpp_Parent\CheckUpp\Soubhanik\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="11_D94C620D5273205F6B5D70B55D9C46FE70986E68" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{277A931B-5C20-4135-8FCF-678BD972299A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="296" uniqueCount="222">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="285" uniqueCount="224">
   <si>
     <t>Epic #</t>
   </si>
@@ -275,9 +275,6 @@
 2. Uploaded document must be visible in wallet</t>
   </si>
   <si>
-    <t>Slide 12</t>
-  </si>
-  <si>
     <t>Discussion #10 – NATHAN</t>
   </si>
   <si>
@@ -320,9 +317,6 @@
     <t>1. 'Save as link' action must be available on the eScript screen
 2. Short link must be generated (checkupp.app/s/…)
 3. Link must be copyable</t>
-  </si>
-  <si>
-    <t>Slide 13</t>
   </si>
   <si>
     <t>Discussion #11 – NATHAN; per wireframe user story</t>
@@ -340,9 +334,6 @@
 4. Copyable short link must be shown below QR</t>
   </si>
   <si>
-    <t>Slides 13–14</t>
-  </si>
-  <si>
     <t>view the details of my e-Script before sharing</t>
   </si>
   <si>
@@ -364,9 +355,6 @@
   <si>
     <t>1. Health check list screen must be accessible from home
 2. All available checks must be displayed</t>
-  </si>
-  <si>
-    <t>Slide 16</t>
   </si>
   <si>
     <t>user who has completed a health check</t>
@@ -604,9 +592,6 @@
     <t>1. App must display the current week, trimester, and EDD.</t>
   </si>
   <si>
-    <t>Slide 11</t>
-  </si>
-  <si>
     <t>view recommended prenatal tests and doctor visits</t>
   </si>
   <si>
@@ -658,9 +643,6 @@
     <t>1. User must be able to select and save symptoms.</t>
   </si>
   <si>
-    <t>Slide 9, 11</t>
-  </si>
-  <si>
     <t>Post-menopausal user</t>
   </si>
   <si>
@@ -752,13 +734,37 @@
   </si>
   <si>
     <t>1. User must be able to attach documents to the custom health check.</t>
+  </si>
+  <si>
+    <t>Slide 5</t>
+  </si>
+  <si>
+    <t>Slide 1</t>
+  </si>
+  <si>
+    <t>Slide 2,3,4</t>
+  </si>
+  <si>
+    <t>Slide 8-11</t>
+  </si>
+  <si>
+    <t>Slide 14</t>
+  </si>
+  <si>
+    <t>Slide 15</t>
+  </si>
+  <si>
+    <t>Slides 15</t>
+  </si>
+  <si>
+    <t>Slide 24</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -797,8 +803,14 @@
       <sz val="10"/>
       <name val="Calibri"/>
     </font>
+    <font>
+      <sz val="8"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="18">
+  <fills count="19">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -886,6 +898,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFF0000"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1007,7 +1025,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="73">
+  <cellXfs count="76">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1168,51 +1186,64 @@
     <xf numFmtId="0" fontId="5" fillId="16" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="11" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="17" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="10" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="9" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="13" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="14" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="16" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="12" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="8" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="15" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="11" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="17" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="10" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="14" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="9" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="13" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="16" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="15" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="18" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1506,41 +1537,41 @@
     <col min="5" max="5" width="65" style="2" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="41" style="3" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="49.77734375" style="3" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="10.77734375" style="2" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="11.6640625" style="2" customWidth="1"/>
     <col min="9" max="9" width="10.33203125" style="3" bestFit="1" customWidth="1"/>
     <col min="10" max="12" width="8.88671875" style="5" customWidth="1"/>
     <col min="13" max="16384" width="8.88671875" style="5"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="39.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="72" t="s">
+      <c r="A1" s="70" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="59" t="s">
+      <c r="B1" s="60" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="59" t="s">
+      <c r="C1" s="60" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="59" t="s">
+      <c r="D1" s="60" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="70"/>
-      <c r="F1" s="71"/>
-      <c r="G1" s="59" t="s">
+      <c r="E1" s="71"/>
+      <c r="F1" s="72"/>
+      <c r="G1" s="73" t="s">
         <v>4</v>
       </c>
-      <c r="H1" s="59" t="s">
+      <c r="H1" s="60" t="s">
         <v>5</v>
       </c>
-      <c r="I1" s="59" t="s">
+      <c r="I1" s="60" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A2" s="56"/>
-      <c r="B2" s="60"/>
-      <c r="C2" s="60"/>
+      <c r="A2" s="55"/>
+      <c r="B2" s="61"/>
+      <c r="C2" s="61"/>
       <c r="D2" s="1" t="s">
         <v>7</v>
       </c>
@@ -1550,9 +1581,9 @@
       <c r="F2" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="G2" s="60"/>
-      <c r="H2" s="60"/>
-      <c r="I2" s="60"/>
+      <c r="G2" s="74"/>
+      <c r="H2" s="61"/>
+      <c r="I2" s="61"/>
     </row>
     <row r="3" spans="1:9" s="8" customFormat="1" ht="55.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="36">
@@ -1577,17 +1608,17 @@
         <v>14</v>
       </c>
       <c r="H3" s="9" t="s">
-        <v>15</v>
+        <v>158</v>
       </c>
       <c r="I3" s="10" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="4" spans="1:9" s="8" customFormat="1" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="62">
+      <c r="A4" s="69">
         <v>3</v>
       </c>
-      <c r="B4" s="62" t="s">
+      <c r="B4" s="69" t="s">
         <v>17</v>
       </c>
       <c r="C4" s="11">
@@ -1606,15 +1637,15 @@
         <v>20</v>
       </c>
       <c r="H4" s="11" t="s">
-        <v>21</v>
+        <v>217</v>
       </c>
       <c r="I4" s="12" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="5" spans="1:9" s="8" customFormat="1" ht="55.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="55"/>
-      <c r="B5" s="55"/>
+      <c r="A5" s="57"/>
+      <c r="B5" s="57"/>
       <c r="C5" s="11">
         <v>3.2</v>
       </c>
@@ -1630,14 +1661,16 @@
       <c r="G5" s="42" t="s">
         <v>25</v>
       </c>
-      <c r="H5" s="11"/>
+      <c r="H5" s="11" t="s">
+        <v>218</v>
+      </c>
       <c r="I5" s="12" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="6" spans="1:9" s="8" customFormat="1" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="56"/>
-      <c r="B6" s="56"/>
+      <c r="A6" s="55"/>
+      <c r="B6" s="55"/>
       <c r="C6" s="11">
         <v>3.3</v>
       </c>
@@ -1654,17 +1687,17 @@
         <v>28</v>
       </c>
       <c r="H6" s="11" t="s">
-        <v>21</v>
+        <v>217</v>
       </c>
       <c r="I6" s="12" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="7" spans="1:9" s="8" customFormat="1" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="57">
+      <c r="A7" s="56">
         <v>4</v>
       </c>
-      <c r="B7" s="57" t="s">
+      <c r="B7" s="56" t="s">
         <v>29</v>
       </c>
       <c r="C7" s="13">
@@ -1683,15 +1716,15 @@
         <v>33</v>
       </c>
       <c r="H7" s="13" t="s">
-        <v>34</v>
+        <v>216</v>
       </c>
       <c r="I7" s="14" t="s">
         <v>35</v>
       </c>
     </row>
     <row r="8" spans="1:9" s="8" customFormat="1" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="55"/>
-      <c r="B8" s="55"/>
+      <c r="A8" s="57"/>
+      <c r="B8" s="57"/>
       <c r="C8" s="13">
         <v>4.2</v>
       </c>
@@ -1708,13 +1741,13 @@
         <v>38</v>
       </c>
       <c r="H8" s="13" t="s">
-        <v>34</v>
+        <v>216</v>
       </c>
       <c r="I8" s="14"/>
     </row>
     <row r="9" spans="1:9" s="8" customFormat="1" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="55"/>
-      <c r="B9" s="55"/>
+      <c r="A9" s="57"/>
+      <c r="B9" s="57"/>
       <c r="C9" s="13">
         <v>4.3</v>
       </c>
@@ -1731,15 +1764,15 @@
         <v>42</v>
       </c>
       <c r="H9" s="13" t="s">
-        <v>43</v>
+        <v>21</v>
       </c>
       <c r="I9" s="14" t="s">
         <v>44</v>
       </c>
     </row>
     <row r="10" spans="1:9" s="8" customFormat="1" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="55"/>
-      <c r="B10" s="55"/>
+      <c r="A10" s="57"/>
+      <c r="B10" s="57"/>
       <c r="C10" s="13">
         <v>4.4000000000000004</v>
       </c>
@@ -1756,16 +1789,16 @@
         <v>48</v>
       </c>
       <c r="H10" s="13" t="s">
-        <v>43</v>
+        <v>34</v>
       </c>
       <c r="I10" s="14" t="s">
         <v>49</v>
       </c>
     </row>
     <row r="11" spans="1:9" s="8" customFormat="1" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="55"/>
-      <c r="B11" s="55"/>
-      <c r="C11" s="13">
+      <c r="A11" s="57"/>
+      <c r="B11" s="57"/>
+      <c r="C11" s="75">
         <v>4.5</v>
       </c>
       <c r="D11" s="14" t="s">
@@ -1786,9 +1819,9 @@
       <c r="I11" s="14"/>
     </row>
     <row r="12" spans="1:9" s="8" customFormat="1" ht="55.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="56"/>
-      <c r="B12" s="56"/>
-      <c r="C12" s="13">
+      <c r="A12" s="55"/>
+      <c r="B12" s="55"/>
+      <c r="C12" s="75">
         <v>4.5999999999999996</v>
       </c>
       <c r="D12" s="14" t="s">
@@ -1809,10 +1842,10 @@
       <c r="I12" s="14"/>
     </row>
     <row r="13" spans="1:9" s="8" customFormat="1" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="61">
+      <c r="A13" s="59">
         <v>5</v>
       </c>
-      <c r="B13" s="61" t="s">
+      <c r="B13" s="59" t="s">
         <v>58</v>
       </c>
       <c r="C13" s="15">
@@ -1838,8 +1871,8 @@
       </c>
     </row>
     <row r="14" spans="1:9" s="8" customFormat="1" ht="96.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="55"/>
-      <c r="B14" s="55"/>
+      <c r="A14" s="57"/>
+      <c r="B14" s="57"/>
       <c r="C14" s="15">
         <v>5.2</v>
       </c>
@@ -1856,15 +1889,15 @@
         <v>66</v>
       </c>
       <c r="H14" s="17" t="s">
-        <v>62</v>
+        <v>219</v>
       </c>
       <c r="I14" s="16" t="s">
         <v>67</v>
       </c>
     </row>
     <row r="15" spans="1:9" s="8" customFormat="1" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="56"/>
-      <c r="B15" s="56"/>
+      <c r="A15" s="55"/>
+      <c r="B15" s="55"/>
       <c r="C15" s="15">
         <v>5.3</v>
       </c>
@@ -1881,15 +1914,15 @@
         <v>70</v>
       </c>
       <c r="H15" s="17" t="s">
-        <v>62</v>
+        <v>219</v>
       </c>
       <c r="I15" s="16"/>
     </row>
     <row r="16" spans="1:9" s="8" customFormat="1" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="66">
+      <c r="A16" s="62">
         <v>6</v>
       </c>
-      <c r="B16" s="66" t="s">
+      <c r="B16" s="62" t="s">
         <v>71</v>
       </c>
       <c r="C16" s="18">
@@ -1908,15 +1941,15 @@
         <v>74</v>
       </c>
       <c r="H16" s="20" t="s">
+        <v>220</v>
+      </c>
+      <c r="I16" s="19" t="s">
         <v>75</v>
       </c>
-      <c r="I16" s="19" t="s">
-        <v>76</v>
-      </c>
     </row>
     <row r="17" spans="1:9" s="8" customFormat="1" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="55"/>
-      <c r="B17" s="55"/>
+      <c r="A17" s="57"/>
+      <c r="B17" s="57"/>
       <c r="C17" s="18">
         <v>6.2</v>
       </c>
@@ -1924,24 +1957,24 @@
         <v>30</v>
       </c>
       <c r="E17" s="19" t="s">
+        <v>76</v>
+      </c>
+      <c r="F17" s="19" t="s">
         <v>77</v>
       </c>
-      <c r="F17" s="19" t="s">
+      <c r="G17" s="45" t="s">
         <v>78</v>
       </c>
-      <c r="G17" s="45" t="s">
+      <c r="H17" s="18" t="s">
+        <v>220</v>
+      </c>
+      <c r="I17" s="19" t="s">
         <v>79</v>
       </c>
-      <c r="H17" s="18" t="s">
-        <v>75</v>
-      </c>
-      <c r="I17" s="19" t="s">
-        <v>80</v>
-      </c>
     </row>
     <row r="18" spans="1:9" s="8" customFormat="1" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="56"/>
-      <c r="B18" s="56"/>
+      <c r="A18" s="55"/>
+      <c r="B18" s="55"/>
       <c r="C18" s="18">
         <v>6.3</v>
       </c>
@@ -1949,102 +1982,102 @@
         <v>30</v>
       </c>
       <c r="E18" s="19" t="s">
+        <v>80</v>
+      </c>
+      <c r="F18" s="19" t="s">
         <v>81</v>
       </c>
-      <c r="F18" s="19" t="s">
+      <c r="G18" s="45" t="s">
         <v>82</v>
       </c>
-      <c r="G18" s="45" t="s">
+      <c r="H18" s="18" t="s">
+        <v>220</v>
+      </c>
+      <c r="I18" s="19"/>
+    </row>
+    <row r="19" spans="1:9" s="8" customFormat="1" ht="82.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A19" s="58">
+        <v>7</v>
+      </c>
+      <c r="B19" s="58" t="s">
         <v>83</v>
-      </c>
-      <c r="H18" s="18" t="s">
-        <v>75</v>
-      </c>
-      <c r="I18" s="19"/>
-    </row>
-    <row r="19" spans="1:9" s="8" customFormat="1" ht="82.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="64">
-        <v>7</v>
-      </c>
-      <c r="B19" s="64" t="s">
-        <v>84</v>
       </c>
       <c r="C19" s="21">
         <v>7.1</v>
       </c>
       <c r="D19" s="22" t="s">
+        <v>84</v>
+      </c>
+      <c r="E19" s="22" t="s">
         <v>85</v>
       </c>
-      <c r="E19" s="22" t="s">
+      <c r="F19" s="22" t="s">
         <v>86</v>
       </c>
-      <c r="F19" s="22" t="s">
+      <c r="G19" s="46" t="s">
         <v>87</v>
       </c>
-      <c r="G19" s="46" t="s">
+      <c r="H19" s="23" t="s">
+        <v>221</v>
+      </c>
+      <c r="I19" s="22" t="s">
         <v>88</v>
       </c>
-      <c r="H19" s="23" t="s">
-        <v>89</v>
-      </c>
-      <c r="I19" s="22" t="s">
-        <v>90</v>
-      </c>
     </row>
     <row r="20" spans="1:9" s="8" customFormat="1" ht="82.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="55"/>
-      <c r="B20" s="55"/>
+      <c r="A20" s="57"/>
+      <c r="B20" s="57"/>
       <c r="C20" s="21">
         <v>7.2</v>
       </c>
       <c r="D20" s="22" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="E20" s="22" t="s">
+        <v>89</v>
+      </c>
+      <c r="F20" s="22" t="s">
+        <v>90</v>
+      </c>
+      <c r="G20" s="46" t="s">
         <v>91</v>
       </c>
-      <c r="F20" s="22" t="s">
-        <v>92</v>
-      </c>
-      <c r="G20" s="46" t="s">
-        <v>93</v>
-      </c>
       <c r="H20" s="21" t="s">
-        <v>94</v>
+        <v>222</v>
       </c>
       <c r="I20" s="22" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
     </row>
     <row r="21" spans="1:9" s="8" customFormat="1" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A21" s="56"/>
-      <c r="B21" s="56"/>
+      <c r="A21" s="55"/>
+      <c r="B21" s="55"/>
       <c r="C21" s="21">
         <v>7.3</v>
       </c>
       <c r="D21" s="22" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="E21" s="22" t="s">
+        <v>92</v>
+      </c>
+      <c r="F21" s="22" t="s">
+        <v>93</v>
+      </c>
+      <c r="G21" s="46" t="s">
+        <v>94</v>
+      </c>
+      <c r="H21" s="21" t="s">
+        <v>221</v>
+      </c>
+      <c r="I21" s="22"/>
+    </row>
+    <row r="22" spans="1:9" s="8" customFormat="1" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A22" s="68">
+        <v>9</v>
+      </c>
+      <c r="B22" s="68" t="s">
         <v>95</v>
-      </c>
-      <c r="F21" s="22" t="s">
-        <v>96</v>
-      </c>
-      <c r="G21" s="46" t="s">
-        <v>97</v>
-      </c>
-      <c r="H21" s="21" t="s">
-        <v>89</v>
-      </c>
-      <c r="I21" s="22"/>
-    </row>
-    <row r="22" spans="1:9" s="8" customFormat="1" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A22" s="54">
-        <v>9</v>
-      </c>
-      <c r="B22" s="54" t="s">
-        <v>98</v>
       </c>
       <c r="C22" s="24">
         <v>9.1</v>
@@ -2053,70 +2086,64 @@
         <v>30</v>
       </c>
       <c r="E22" s="25" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="F22" s="25" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="G22" s="47" t="s">
-        <v>101</v>
-      </c>
-      <c r="H22" s="24" t="s">
-        <v>102</v>
-      </c>
+        <v>98</v>
+      </c>
+      <c r="H22" s="24"/>
       <c r="I22" s="25"/>
     </row>
     <row r="23" spans="1:9" s="8" customFormat="1" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A23" s="55"/>
-      <c r="B23" s="55"/>
+      <c r="A23" s="57"/>
+      <c r="B23" s="57"/>
       <c r="C23" s="24">
         <v>9.1999999999999993</v>
       </c>
       <c r="D23" s="25" t="s">
-        <v>103</v>
+        <v>99</v>
       </c>
       <c r="E23" s="25" t="s">
-        <v>104</v>
+        <v>100</v>
       </c>
       <c r="F23" s="25" t="s">
-        <v>105</v>
+        <v>101</v>
       </c>
       <c r="G23" s="47" t="s">
-        <v>106</v>
-      </c>
-      <c r="H23" s="24" t="s">
         <v>102</v>
       </c>
+      <c r="H23" s="24"/>
       <c r="I23" s="25"/>
     </row>
     <row r="24" spans="1:9" s="8" customFormat="1" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A24" s="55"/>
-      <c r="B24" s="55"/>
+      <c r="A24" s="57"/>
+      <c r="B24" s="57"/>
       <c r="C24" s="24">
         <v>9.3000000000000007</v>
       </c>
       <c r="D24" s="25" t="s">
+        <v>103</v>
+      </c>
+      <c r="E24" s="25" t="s">
+        <v>104</v>
+      </c>
+      <c r="F24" s="25" t="s">
+        <v>105</v>
+      </c>
+      <c r="G24" s="47" t="s">
+        <v>106</v>
+      </c>
+      <c r="H24" s="24"/>
+      <c r="I24" s="25" t="s">
         <v>107</v>
       </c>
-      <c r="E24" s="25" t="s">
-        <v>108</v>
-      </c>
-      <c r="F24" s="25" t="s">
-        <v>109</v>
-      </c>
-      <c r="G24" s="47" t="s">
-        <v>110</v>
-      </c>
-      <c r="H24" s="24" t="s">
-        <v>102</v>
-      </c>
-      <c r="I24" s="25" t="s">
-        <v>111</v>
-      </c>
     </row>
     <row r="25" spans="1:9" s="8" customFormat="1" ht="55.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A25" s="56"/>
-      <c r="B25" s="56"/>
+      <c r="A25" s="55"/>
+      <c r="B25" s="55"/>
       <c r="C25" s="24">
         <v>9.4</v>
       </c>
@@ -2124,27 +2151,25 @@
         <v>30</v>
       </c>
       <c r="E25" s="25" t="s">
-        <v>112</v>
+        <v>108</v>
       </c>
       <c r="F25" s="25" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="G25" s="47" t="s">
-        <v>114</v>
-      </c>
-      <c r="H25" s="24" t="s">
-        <v>102</v>
-      </c>
+        <v>110</v>
+      </c>
+      <c r="H25" s="24"/>
       <c r="I25" s="25" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="26" spans="1:9" s="39" customFormat="1" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A26" s="54">
+        <v>10</v>
+      </c>
+      <c r="B26" s="54" t="s">
         <v>111</v>
-      </c>
-    </row>
-    <row r="26" spans="1:9" s="39" customFormat="1" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A26" s="63">
-        <v>10</v>
-      </c>
-      <c r="B26" s="63" t="s">
-        <v>115</v>
       </c>
       <c r="C26" s="37">
         <v>10.1</v>
@@ -2153,22 +2178,22 @@
         <v>30</v>
       </c>
       <c r="E26" s="38" t="s">
-        <v>116</v>
+        <v>112</v>
       </c>
       <c r="F26" s="38" t="s">
-        <v>117</v>
+        <v>113</v>
       </c>
       <c r="G26" s="48" t="s">
-        <v>118</v>
+        <v>114</v>
       </c>
       <c r="H26" s="37" t="s">
-        <v>119</v>
+        <v>115</v>
       </c>
       <c r="I26" s="38"/>
     </row>
     <row r="27" spans="1:9" s="39" customFormat="1" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A27" s="56"/>
-      <c r="B27" s="56"/>
+      <c r="A27" s="55"/>
+      <c r="B27" s="55"/>
       <c r="C27" s="37">
         <v>10.199999999999999</v>
       </c>
@@ -2176,25 +2201,25 @@
         <v>30</v>
       </c>
       <c r="E27" s="38" t="s">
-        <v>120</v>
+        <v>116</v>
       </c>
       <c r="F27" s="38" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="G27" s="48" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="H27" s="37" t="s">
+        <v>115</v>
+      </c>
+      <c r="I27" s="38"/>
+    </row>
+    <row r="28" spans="1:9" s="39" customFormat="1" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A28" s="54">
+        <v>11</v>
+      </c>
+      <c r="B28" s="54" t="s">
         <v>119</v>
-      </c>
-      <c r="I27" s="38"/>
-    </row>
-    <row r="28" spans="1:9" s="39" customFormat="1" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A28" s="63">
-        <v>11</v>
-      </c>
-      <c r="B28" s="63" t="s">
-        <v>123</v>
       </c>
       <c r="C28" s="37">
         <v>11.1</v>
@@ -2203,22 +2228,22 @@
         <v>30</v>
       </c>
       <c r="E28" s="38" t="s">
-        <v>124</v>
+        <v>120</v>
       </c>
       <c r="F28" s="38" t="s">
-        <v>125</v>
+        <v>121</v>
       </c>
       <c r="G28" s="48" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="H28" s="37" t="s">
-        <v>127</v>
+        <v>123</v>
       </c>
       <c r="I28" s="38"/>
     </row>
     <row r="29" spans="1:9" s="39" customFormat="1" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A29" s="56"/>
-      <c r="B29" s="56"/>
+      <c r="A29" s="55"/>
+      <c r="B29" s="55"/>
       <c r="C29" s="37">
         <v>11.2</v>
       </c>
@@ -2226,25 +2251,25 @@
         <v>30</v>
       </c>
       <c r="E29" s="38" t="s">
-        <v>128</v>
+        <v>124</v>
       </c>
       <c r="F29" s="38" t="s">
-        <v>129</v>
+        <v>125</v>
       </c>
       <c r="G29" s="48" t="s">
-        <v>130</v>
+        <v>126</v>
       </c>
       <c r="H29" s="37" t="s">
+        <v>123</v>
+      </c>
+      <c r="I29" s="38"/>
+    </row>
+    <row r="30" spans="1:9" s="8" customFormat="1" ht="55.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A30" s="66">
+        <v>12</v>
+      </c>
+      <c r="B30" s="66" t="s">
         <v>127</v>
-      </c>
-      <c r="I29" s="38"/>
-    </row>
-    <row r="30" spans="1:9" s="8" customFormat="1" ht="55.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A30" s="58">
-        <v>12</v>
-      </c>
-      <c r="B30" s="58" t="s">
-        <v>131</v>
       </c>
       <c r="C30" s="26">
         <v>12.1</v>
@@ -2253,24 +2278,24 @@
         <v>30</v>
       </c>
       <c r="E30" s="27" t="s">
+        <v>128</v>
+      </c>
+      <c r="F30" s="27" t="s">
+        <v>129</v>
+      </c>
+      <c r="G30" s="49" t="s">
+        <v>130</v>
+      </c>
+      <c r="H30" s="26" t="s">
+        <v>131</v>
+      </c>
+      <c r="I30" s="27" t="s">
         <v>132</v>
       </c>
-      <c r="F30" s="27" t="s">
-        <v>133</v>
-      </c>
-      <c r="G30" s="49" t="s">
-        <v>134</v>
-      </c>
-      <c r="H30" s="26" t="s">
-        <v>135</v>
-      </c>
-      <c r="I30" s="27" t="s">
-        <v>136</v>
-      </c>
     </row>
     <row r="31" spans="1:9" s="8" customFormat="1" ht="55.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A31" s="55"/>
-      <c r="B31" s="55"/>
+      <c r="A31" s="57"/>
+      <c r="B31" s="57"/>
       <c r="C31" s="26">
         <v>12.2</v>
       </c>
@@ -2278,24 +2303,24 @@
         <v>30</v>
       </c>
       <c r="E31" s="27" t="s">
-        <v>137</v>
+        <v>133</v>
       </c>
       <c r="F31" s="27" t="s">
-        <v>138</v>
+        <v>134</v>
       </c>
       <c r="G31" s="49" t="s">
-        <v>139</v>
+        <v>135</v>
       </c>
       <c r="H31" s="26" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="I31" s="27" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
     </row>
     <row r="32" spans="1:9" s="8" customFormat="1" ht="55.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A32" s="56"/>
-      <c r="B32" s="56"/>
+      <c r="A32" s="55"/>
+      <c r="B32" s="55"/>
       <c r="C32" s="26">
         <v>12.3</v>
       </c>
@@ -2303,25 +2328,25 @@
         <v>30</v>
       </c>
       <c r="E32" s="27" t="s">
-        <v>140</v>
+        <v>136</v>
       </c>
       <c r="F32" s="27" t="s">
-        <v>141</v>
+        <v>137</v>
       </c>
       <c r="G32" s="49" t="s">
-        <v>142</v>
+        <v>138</v>
       </c>
       <c r="H32" s="26" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="I32" s="27"/>
     </row>
     <row r="33" spans="1:9" s="8" customFormat="1" ht="55.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A33" s="67">
+      <c r="A33" s="63">
         <v>13</v>
       </c>
-      <c r="B33" s="67" t="s">
-        <v>143</v>
+      <c r="B33" s="63" t="s">
+        <v>139</v>
       </c>
       <c r="C33" s="28">
         <v>13.1</v>
@@ -2330,24 +2355,24 @@
         <v>30</v>
       </c>
       <c r="E33" s="29" t="s">
+        <v>140</v>
+      </c>
+      <c r="F33" s="29" t="s">
+        <v>141</v>
+      </c>
+      <c r="G33" s="50" t="s">
+        <v>142</v>
+      </c>
+      <c r="H33" s="28" t="s">
+        <v>143</v>
+      </c>
+      <c r="I33" s="29" t="s">
         <v>144</v>
       </c>
-      <c r="F33" s="29" t="s">
-        <v>145</v>
-      </c>
-      <c r="G33" s="50" t="s">
-        <v>146</v>
-      </c>
-      <c r="H33" s="28" t="s">
-        <v>147</v>
-      </c>
-      <c r="I33" s="29" t="s">
-        <v>148</v>
-      </c>
     </row>
     <row r="34" spans="1:9" s="8" customFormat="1" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A34" s="55"/>
-      <c r="B34" s="55"/>
+      <c r="A34" s="57"/>
+      <c r="B34" s="57"/>
       <c r="C34" s="28">
         <v>13.2</v>
       </c>
@@ -2355,29 +2380,29 @@
         <v>30</v>
       </c>
       <c r="E34" s="29" t="s">
-        <v>149</v>
+        <v>145</v>
       </c>
       <c r="F34" s="29" t="s">
-        <v>150</v>
+        <v>146</v>
       </c>
       <c r="G34" s="50" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="H34" s="28" t="s">
-        <v>147</v>
+        <v>143</v>
       </c>
       <c r="I34" s="29" t="s">
-        <v>148</v>
+        <v>144</v>
       </c>
     </row>
     <row r="35" spans="1:9" s="8" customFormat="1" ht="55.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A35" s="55"/>
-      <c r="B35" s="55"/>
+      <c r="A35" s="57"/>
+      <c r="B35" s="57"/>
       <c r="C35" s="28">
         <v>13.3</v>
       </c>
       <c r="D35" s="29" t="s">
-        <v>152</v>
+        <v>148</v>
       </c>
       <c r="E35" s="29" t="s">
         <v>12</v>
@@ -2389,15 +2414,15 @@
         <v>14</v>
       </c>
       <c r="H35" s="28" t="s">
-        <v>15</v>
+        <v>158</v>
       </c>
       <c r="I35" s="29" t="s">
-        <v>153</v>
-      </c>
-    </row>
-    <row r="36" spans="1:9" s="8" customFormat="1" ht="82.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A36" s="56"/>
-      <c r="B36" s="56"/>
+        <v>149</v>
+      </c>
+    </row>
+    <row r="36" spans="1:9" s="8" customFormat="1" ht="60.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A36" s="55"/>
+      <c r="B36" s="55"/>
       <c r="C36" s="28">
         <v>13.4</v>
       </c>
@@ -2405,27 +2430,27 @@
         <v>30</v>
       </c>
       <c r="E36" s="29" t="s">
+        <v>150</v>
+      </c>
+      <c r="F36" s="29" t="s">
+        <v>151</v>
+      </c>
+      <c r="G36" s="50" t="s">
+        <v>152</v>
+      </c>
+      <c r="H36" s="28" t="s">
+        <v>15</v>
+      </c>
+      <c r="I36" s="29" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="37" spans="1:9" s="8" customFormat="1" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A37" s="64">
+        <v>14</v>
+      </c>
+      <c r="B37" s="64" t="s">
         <v>154</v>
-      </c>
-      <c r="F36" s="29" t="s">
-        <v>155</v>
-      </c>
-      <c r="G36" s="50" t="s">
-        <v>156</v>
-      </c>
-      <c r="H36" s="28" t="s">
-        <v>147</v>
-      </c>
-      <c r="I36" s="29" t="s">
-        <v>157</v>
-      </c>
-    </row>
-    <row r="37" spans="1:9" s="8" customFormat="1" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A37" s="65">
-        <v>14</v>
-      </c>
-      <c r="B37" s="65" t="s">
-        <v>158</v>
       </c>
       <c r="C37" s="30">
         <v>14.1</v>
@@ -2434,24 +2459,24 @@
         <v>30</v>
       </c>
       <c r="E37" s="31" t="s">
+        <v>155</v>
+      </c>
+      <c r="F37" s="31" t="s">
+        <v>156</v>
+      </c>
+      <c r="G37" s="51" t="s">
+        <v>157</v>
+      </c>
+      <c r="H37" s="30" t="s">
+        <v>223</v>
+      </c>
+      <c r="I37" s="31" t="s">
         <v>159</v>
       </c>
-      <c r="F37" s="31" t="s">
-        <v>160</v>
-      </c>
-      <c r="G37" s="51" t="s">
-        <v>161</v>
-      </c>
-      <c r="H37" s="30" t="s">
-        <v>162</v>
-      </c>
-      <c r="I37" s="31" t="s">
-        <v>163</v>
-      </c>
     </row>
     <row r="38" spans="1:9" s="8" customFormat="1" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A38" s="56"/>
-      <c r="B38" s="56"/>
+      <c r="A38" s="55"/>
+      <c r="B38" s="55"/>
       <c r="C38" s="30">
         <v>14.2</v>
       </c>
@@ -2459,362 +2484,346 @@
         <v>30</v>
       </c>
       <c r="E38" s="31" t="s">
-        <v>164</v>
+        <v>160</v>
       </c>
       <c r="F38" s="31" t="s">
-        <v>165</v>
+        <v>161</v>
       </c>
       <c r="G38" s="51" t="s">
-        <v>166</v>
+        <v>162</v>
       </c>
       <c r="H38" s="30" t="s">
-        <v>162</v>
+        <v>223</v>
       </c>
       <c r="I38" s="31" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="39" spans="1:9" s="8" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A39" s="67">
+        <v>15</v>
+      </c>
+      <c r="B39" s="67" t="s">
         <v>163</v>
-      </c>
-    </row>
-    <row r="39" spans="1:9" s="8" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A39" s="69">
-        <v>15</v>
-      </c>
-      <c r="B39" s="69" t="s">
-        <v>167</v>
       </c>
       <c r="C39" s="32">
         <v>15.1</v>
       </c>
       <c r="D39" s="33" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
       <c r="E39" s="33" t="s">
-        <v>169</v>
+        <v>165</v>
       </c>
       <c r="F39" s="33" t="s">
-        <v>170</v>
+        <v>166</v>
       </c>
       <c r="G39" s="52" t="s">
-        <v>171</v>
-      </c>
-      <c r="H39" s="32" t="s">
-        <v>172</v>
-      </c>
+        <v>167</v>
+      </c>
+      <c r="H39" s="32"/>
       <c r="I39" s="33"/>
     </row>
     <row r="40" spans="1:9" s="8" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A40" s="55"/>
-      <c r="B40" s="55"/>
+      <c r="A40" s="57"/>
+      <c r="B40" s="57"/>
       <c r="C40" s="32">
         <v>15.2</v>
       </c>
       <c r="D40" s="33" t="s">
+        <v>164</v>
+      </c>
+      <c r="E40" s="33" t="s">
         <v>168</v>
       </c>
-      <c r="E40" s="33" t="s">
-        <v>173</v>
-      </c>
       <c r="F40" s="33" t="s">
-        <v>174</v>
+        <v>169</v>
       </c>
       <c r="G40" s="52" t="s">
-        <v>175</v>
-      </c>
-      <c r="H40" s="32" t="s">
-        <v>172</v>
-      </c>
+        <v>170</v>
+      </c>
+      <c r="H40" s="32"/>
       <c r="I40" s="33"/>
     </row>
     <row r="41" spans="1:9" s="8" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A41" s="55"/>
-      <c r="B41" s="55"/>
+      <c r="A41" s="57"/>
+      <c r="B41" s="57"/>
       <c r="C41" s="32">
         <v>15.3</v>
       </c>
       <c r="D41" s="33" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
       <c r="E41" s="33" t="s">
-        <v>176</v>
+        <v>171</v>
       </c>
       <c r="F41" s="33" t="s">
-        <v>177</v>
+        <v>172</v>
       </c>
       <c r="G41" s="52" t="s">
-        <v>178</v>
-      </c>
-      <c r="H41" s="32" t="s">
-        <v>172</v>
-      </c>
+        <v>173</v>
+      </c>
+      <c r="H41" s="32"/>
       <c r="I41" s="33"/>
     </row>
     <row r="42" spans="1:9" s="8" customFormat="1" ht="27.6" x14ac:dyDescent="0.3">
-      <c r="A42" s="55"/>
-      <c r="B42" s="55"/>
+      <c r="A42" s="57"/>
+      <c r="B42" s="57"/>
       <c r="C42" s="32">
         <v>15.4</v>
       </c>
       <c r="D42" s="33" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
       <c r="E42" s="33" t="s">
-        <v>179</v>
+        <v>174</v>
       </c>
       <c r="F42" s="33" t="s">
-        <v>180</v>
+        <v>175</v>
       </c>
       <c r="G42" s="52" t="s">
-        <v>181</v>
-      </c>
-      <c r="H42" s="32" t="s">
-        <v>172</v>
-      </c>
+        <v>176</v>
+      </c>
+      <c r="H42" s="32"/>
       <c r="I42" s="33"/>
     </row>
     <row r="43" spans="1:9" s="8" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A43" s="56"/>
-      <c r="B43" s="56"/>
+      <c r="A43" s="55"/>
+      <c r="B43" s="55"/>
       <c r="C43" s="32">
         <v>15.5</v>
       </c>
       <c r="D43" s="33" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
       <c r="E43" s="33" t="s">
-        <v>182</v>
+        <v>177</v>
       </c>
       <c r="F43" s="33" t="s">
-        <v>183</v>
+        <v>178</v>
       </c>
       <c r="G43" s="52" t="s">
-        <v>184</v>
-      </c>
-      <c r="H43" s="32" t="s">
-        <v>172</v>
-      </c>
+        <v>179</v>
+      </c>
+      <c r="H43" s="32"/>
       <c r="I43" s="33"/>
     </row>
     <row r="44" spans="1:9" s="8" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A44" s="68">
+      <c r="A44" s="65">
         <v>16</v>
       </c>
-      <c r="B44" s="68" t="s">
-        <v>185</v>
+      <c r="B44" s="65" t="s">
+        <v>180</v>
       </c>
       <c r="C44" s="34">
         <v>16.100000000000001</v>
       </c>
       <c r="D44" s="35" t="s">
-        <v>186</v>
+        <v>181</v>
       </c>
       <c r="E44" s="35" t="s">
-        <v>187</v>
+        <v>182</v>
       </c>
       <c r="F44" s="35" t="s">
-        <v>188</v>
+        <v>183</v>
       </c>
       <c r="G44" s="53" t="s">
-        <v>189</v>
-      </c>
-      <c r="H44" s="34" t="s">
-        <v>190</v>
-      </c>
+        <v>184</v>
+      </c>
+      <c r="H44" s="34"/>
       <c r="I44" s="35"/>
     </row>
     <row r="45" spans="1:9" s="8" customFormat="1" ht="27.6" x14ac:dyDescent="0.3">
-      <c r="A45" s="56"/>
-      <c r="B45" s="56"/>
+      <c r="A45" s="55"/>
+      <c r="B45" s="55"/>
       <c r="C45" s="34">
         <v>16.2</v>
       </c>
       <c r="D45" s="35" t="s">
-        <v>191</v>
+        <v>185</v>
       </c>
       <c r="E45" s="35" t="s">
-        <v>192</v>
+        <v>186</v>
       </c>
       <c r="F45" s="35" t="s">
-        <v>193</v>
+        <v>187</v>
       </c>
       <c r="G45" s="53" t="s">
-        <v>194</v>
-      </c>
-      <c r="H45" s="34" t="s">
-        <v>190</v>
-      </c>
+        <v>188</v>
+      </c>
+      <c r="H45" s="34"/>
       <c r="I45" s="35"/>
     </row>
     <row r="46" spans="1:9" s="8" customFormat="1" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A46" s="61">
+      <c r="A46" s="59">
         <v>17</v>
       </c>
-      <c r="B46" s="61" t="s">
-        <v>195</v>
+      <c r="B46" s="59" t="s">
+        <v>189</v>
       </c>
       <c r="C46" s="15">
         <v>17.100000000000001</v>
       </c>
       <c r="D46" s="16" t="s">
-        <v>196</v>
+        <v>190</v>
       </c>
       <c r="E46" s="16" t="s">
-        <v>197</v>
+        <v>191</v>
       </c>
       <c r="F46" s="16" t="s">
-        <v>198</v>
+        <v>192</v>
       </c>
       <c r="G46" s="44" t="s">
-        <v>199</v>
-      </c>
-      <c r="H46" s="15" t="s">
-        <v>102</v>
-      </c>
+        <v>193</v>
+      </c>
+      <c r="H46" s="15"/>
       <c r="I46" s="16" t="s">
-        <v>200</v>
+        <v>194</v>
       </c>
     </row>
     <row r="47" spans="1:9" s="8" customFormat="1" ht="27.6" x14ac:dyDescent="0.3">
-      <c r="A47" s="55"/>
-      <c r="B47" s="55"/>
+      <c r="A47" s="57"/>
+      <c r="B47" s="57"/>
       <c r="C47" s="15">
         <v>17.2</v>
       </c>
       <c r="D47" s="16" t="s">
+        <v>190</v>
+      </c>
+      <c r="E47" s="16" t="s">
+        <v>195</v>
+      </c>
+      <c r="F47" s="16" t="s">
         <v>196</v>
       </c>
-      <c r="E47" s="16" t="s">
-        <v>201</v>
-      </c>
-      <c r="F47" s="16" t="s">
-        <v>202</v>
-      </c>
       <c r="G47" s="44" t="s">
-        <v>203</v>
+        <v>197</v>
       </c>
       <c r="H47" s="15"/>
       <c r="I47" s="16"/>
     </row>
     <row r="48" spans="1:9" s="8" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A48" s="55"/>
-      <c r="B48" s="55"/>
+      <c r="A48" s="57"/>
+      <c r="B48" s="57"/>
       <c r="C48" s="15">
         <v>17.3</v>
       </c>
       <c r="D48" s="16" t="s">
-        <v>196</v>
+        <v>190</v>
       </c>
       <c r="E48" s="16" t="s">
-        <v>204</v>
+        <v>198</v>
       </c>
       <c r="F48" s="16" t="s">
-        <v>205</v>
+        <v>199</v>
       </c>
       <c r="G48" s="44" t="s">
-        <v>206</v>
+        <v>200</v>
       </c>
       <c r="H48" s="15"/>
       <c r="I48" s="16"/>
     </row>
     <row r="49" spans="1:9" s="8" customFormat="1" ht="27.6" x14ac:dyDescent="0.3">
-      <c r="A49" s="55"/>
-      <c r="B49" s="55"/>
+      <c r="A49" s="57"/>
+      <c r="B49" s="57"/>
       <c r="C49" s="15">
         <v>17.399999999999999</v>
       </c>
       <c r="D49" s="16" t="s">
-        <v>196</v>
+        <v>190</v>
       </c>
       <c r="E49" s="16" t="s">
-        <v>207</v>
+        <v>201</v>
       </c>
       <c r="F49" s="16" t="s">
-        <v>208</v>
+        <v>202</v>
       </c>
       <c r="G49" s="44" t="s">
-        <v>209</v>
+        <v>203</v>
       </c>
       <c r="H49" s="15"/>
       <c r="I49" s="16"/>
     </row>
     <row r="50" spans="1:9" s="8" customFormat="1" ht="27.6" x14ac:dyDescent="0.3">
-      <c r="A50" s="55"/>
-      <c r="B50" s="55"/>
+      <c r="A50" s="57"/>
+      <c r="B50" s="57"/>
       <c r="C50" s="15">
         <v>17.5</v>
       </c>
       <c r="D50" s="16" t="s">
-        <v>196</v>
+        <v>190</v>
       </c>
       <c r="E50" s="16" t="s">
-        <v>210</v>
+        <v>204</v>
       </c>
       <c r="F50" s="16" t="s">
-        <v>211</v>
+        <v>205</v>
       </c>
       <c r="G50" s="44" t="s">
-        <v>212</v>
+        <v>206</v>
       </c>
       <c r="H50" s="15"/>
       <c r="I50" s="16"/>
     </row>
     <row r="51" spans="1:9" s="8" customFormat="1" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A51" s="55"/>
-      <c r="B51" s="55"/>
+      <c r="A51" s="57"/>
+      <c r="B51" s="57"/>
       <c r="C51" s="15">
         <v>17.600000000000001</v>
       </c>
       <c r="D51" s="16" t="s">
-        <v>196</v>
+        <v>190</v>
       </c>
       <c r="E51" s="16" t="s">
-        <v>213</v>
+        <v>207</v>
       </c>
       <c r="F51" s="16" t="s">
-        <v>214</v>
+        <v>208</v>
       </c>
       <c r="G51" s="44" t="s">
-        <v>215</v>
+        <v>209</v>
       </c>
       <c r="H51" s="15"/>
       <c r="I51" s="16"/>
     </row>
     <row r="52" spans="1:9" s="8" customFormat="1" ht="27.6" x14ac:dyDescent="0.3">
-      <c r="A52" s="55"/>
-      <c r="B52" s="55"/>
+      <c r="A52" s="57"/>
+      <c r="B52" s="57"/>
       <c r="C52" s="15">
         <v>17.7</v>
       </c>
       <c r="D52" s="16" t="s">
-        <v>196</v>
+        <v>190</v>
       </c>
       <c r="E52" s="16" t="s">
-        <v>216</v>
+        <v>210</v>
       </c>
       <c r="F52" s="16" t="s">
-        <v>217</v>
+        <v>211</v>
       </c>
       <c r="G52" s="44" t="s">
-        <v>218</v>
+        <v>212</v>
       </c>
       <c r="H52" s="15"/>
       <c r="I52" s="16"/>
     </row>
     <row r="53" spans="1:9" s="8" customFormat="1" ht="27.6" x14ac:dyDescent="0.3">
-      <c r="A53" s="56"/>
-      <c r="B53" s="56"/>
+      <c r="A53" s="55"/>
+      <c r="B53" s="55"/>
       <c r="C53" s="15">
         <v>17.8</v>
       </c>
       <c r="D53" s="16" t="s">
-        <v>196</v>
+        <v>190</v>
       </c>
       <c r="E53" s="16" t="s">
-        <v>219</v>
+        <v>213</v>
       </c>
       <c r="F53" s="16" t="s">
-        <v>220</v>
+        <v>214</v>
       </c>
       <c r="G53" s="44" t="s">
-        <v>221</v>
+        <v>215</v>
       </c>
       <c r="H53" s="15"/>
       <c r="I53" s="16"/>
@@ -2856,8 +2865,6 @@
   </sheetData>
   <autoFilter ref="I1:I33" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
   <mergeCells count="35">
-    <mergeCell ref="G1:G2"/>
-    <mergeCell ref="B33:B36"/>
     <mergeCell ref="I1:I2"/>
     <mergeCell ref="D1:F1"/>
     <mergeCell ref="A44:A45"/>
@@ -2871,6 +2878,15 @@
     <mergeCell ref="B39:B43"/>
     <mergeCell ref="A1:A2"/>
     <mergeCell ref="A37:A38"/>
+    <mergeCell ref="C1:C2"/>
+    <mergeCell ref="A13:A15"/>
+    <mergeCell ref="A4:A6"/>
+    <mergeCell ref="B4:B6"/>
+    <mergeCell ref="G1:G2"/>
+    <mergeCell ref="B33:B36"/>
+    <mergeCell ref="A26:A27"/>
+    <mergeCell ref="A7:A12"/>
+    <mergeCell ref="A19:A21"/>
     <mergeCell ref="B46:B53"/>
     <mergeCell ref="B1:B2"/>
     <mergeCell ref="B16:B18"/>
@@ -2884,14 +2900,8 @@
     <mergeCell ref="B22:B25"/>
     <mergeCell ref="B7:B12"/>
     <mergeCell ref="B30:B32"/>
-    <mergeCell ref="C1:C2"/>
-    <mergeCell ref="A13:A15"/>
-    <mergeCell ref="A4:A6"/>
-    <mergeCell ref="B4:B6"/>
-    <mergeCell ref="A26:A27"/>
-    <mergeCell ref="A7:A12"/>
-    <mergeCell ref="A19:A21"/>
   </mergeCells>
+  <phoneticPr fontId="6" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait"/>
 </worksheet>

</xml_diff>

<commit_message>
Updated wireframes and user stories for syncing ailment to calender
</commit_message>
<xml_diff>
--- a/Soubhanik/checkupp_product_backlog_final.xlsx
+++ b/Soubhanik/checkupp_product_backlog_final.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30026"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Anodiam\2026\CheckUpp_Parent\CheckUpp\Soubhanik\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Checkupp\CheckUpp\Soubhanik\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F47E8F26-9D1B-4D6F-8625-8AAB133B5B06}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B421AD34-2558-489C-B84F-60DF859C85DF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -130,7 +130,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="191" uniqueCount="151">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="266" uniqueCount="183">
   <si>
     <t>Epic #</t>
   </si>
@@ -340,31 +340,9 @@
     <t>Screenings Schedule</t>
   </si>
   <si>
-    <t>view my upcoming and overdue screenings in a schedule view</t>
-  </si>
-  <si>
-    <t>I know exactly what health checks I need and when</t>
-  </si>
-  <si>
-    <t>1. Screenings schedule screen must show upcoming and due tests
-2. Overdue tests must be highlighted
-3. Dates must be clearly shown</t>
-  </si>
-  <si>
     <t>Discussion #9 – TANVI</t>
   </si>
   <si>
-    <t>sync health check appointments to my device calendar</t>
-  </si>
-  <si>
-    <t>I receive reminders and don't miss health checks</t>
-  </si>
-  <si>
-    <t>1. Calendar sync must be available per appointment
-2. App must sync to Google Calendar / iCal
-3. Appointment details must be included in the calendar entry</t>
-  </si>
-  <si>
     <t>Pregnancy Tracking</t>
   </si>
   <si>
@@ -447,9 +425,6 @@
   </si>
   <si>
     <t>Logged-in User</t>
-  </si>
-  <si>
-    <t>access an "Other Ailments" option from Health Checks</t>
   </si>
   <si>
     <t>I can document conditions not listed in the app</t>
@@ -518,10 +493,6 @@
     <t>1. Tapping must open the detailed view of the selected appointment
 2. Detail view must clearly display Appointment date and time, medical facility, facility address, and doctor's name
 3. Tapping on the back button must take the user back to the Your Appointments screen</t>
-  </si>
-  <si>
-    <t>1. "Other Ailments" tab must appear in the Health Checks list.
-2. The tab must be tappable.</t>
   </si>
   <si>
     <t>select a condition from a dropdown or enter a custom condition</t>
@@ -624,6 +595,148 @@
   </si>
   <si>
     <t xml:space="preserve"> </t>
+  </si>
+  <si>
+    <t>Slide 25</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Slide 13 </t>
+  </si>
+  <si>
+    <t>Discussion #8 – TANVI</t>
+  </si>
+  <si>
+    <t>Slide 13</t>
+  </si>
+  <si>
+    <t>add appointment details when creating a custom health check</t>
+  </si>
+  <si>
+    <t>I can schedule future health appointments</t>
+  </si>
+  <si>
+    <t>receive an option to add my appointment to my device calendar after saving a health check</t>
+  </si>
+  <si>
+    <t>I can easily sync important appointments</t>
+  </si>
+  <si>
+    <t>first-time user</t>
+  </si>
+  <si>
+    <t>grant calendar access</t>
+  </si>
+  <si>
+    <t>the app can add appointments to my device calendar</t>
+  </si>
+  <si>
+    <t>choose which calendar to sync my appointments with</t>
+  </si>
+  <si>
+    <t>appointments are added to my preferred calendar</t>
+  </si>
+  <si>
+    <t>preview appointment details before syncing</t>
+  </si>
+  <si>
+    <t>I can verify the information is correct</t>
+  </si>
+  <si>
+    <t>receive confirmation when my appointment has been added to my calendar</t>
+  </si>
+  <si>
+    <t>I know the sync was successful</t>
+  </si>
+  <si>
+    <t>view all synced health appointments in one place</t>
+  </si>
+  <si>
+    <t>I can manage my upcoming appointments</t>
+  </si>
+  <si>
+    <t>access Calendar &amp; Sync Settings from the calendar icon in the Screenings tab</t>
+  </si>
+  <si>
+    <t>I can manage my calendar preferences</t>
+  </si>
+  <si>
+    <t>enable or disable calendar syncing</t>
+  </si>
+  <si>
+    <t>I can control whether appointments are synced</t>
+  </si>
+  <si>
+    <t>choose which health modules sync appointments</t>
+  </si>
+  <si>
+    <t>only relevant appointments appear in my calendar</t>
+  </si>
+  <si>
+    <t>configure reminder preferences for synced appointments</t>
+  </si>
+  <si>
+    <t>I receive reminders at my preferred time</t>
+  </si>
+  <si>
+    <t>access an Other Ailments option from Health Checks</t>
+  </si>
+  <si>
+    <t>1. Other Ailments tab must appear in the Health Checks list.
+2. The tab must be tappable.</t>
+  </si>
+  <si>
+    <t>1. User must be able to enter appointment date, time and location 2. Appointment details must be linked to the health check
+3. Appointment information must be saved successfully</t>
+  </si>
+  <si>
+    <t>1. App must display an 'Add to Calendar' prompt after saving
+2. User must be able to add or dismiss the prompt
+3. Appointment details must be retained regardless of the user's choice</t>
+  </si>
+  <si>
+    <t>1. App must request calendar permission before the first sync
+2. User must be able to allow or deny access
+3. Permission request should not appear again once a choice has been made</t>
+  </si>
+  <si>
+    <t>1. User must be able to choose Google Calendar, Apple Calendar/iCal or Outlook (where supported)
+2. Selected calendar must be remembered for future syncs
+3. User must be able to change the selected calendar later</t>
+  </si>
+  <si>
+    <t>1. Event preview must display title, date, time, location and reminder
+2. User must be able to edit or cancel before syncing
+3. Calendar event must match the displayed details</t>
+  </si>
+  <si>
+    <t>1. Upcoming Appointments screen must display all synced appointments
+2. Appointments must be grouped by date
+3. User must be able to open the device calendar from this screen</t>
+  </si>
+  <si>
+    <t>1. Tapping the calendar icon must open Calendar &amp; Sync Settings
+2. Settings must display current sync status
+3. User must be able to access settings at any time</t>
+  </si>
+  <si>
+    <t>1. User must be able to turn Calendar Sync on or off
+2. Preference must be saved across sessions
+3. Existing calendar events must remain unaffected when sync is disabled</t>
+  </si>
+  <si>
+    <t>1. User must be able to enable or disable sync for individual modules
+2. Modules include Screenings, Pregnancy, Midlife Health, Menopause and Other Ailments
+3. Only enabled modules should sync appointments</t>
+  </si>
+  <si>
+    <t>1. User must be able to choose reminder intervals
+2. Reminder settings must apply to newly synced appointments
+3. Default reminder must be configurable</t>
+  </si>
+  <si>
+    <t>1. App must display a success message after syncing
+2. User must be able to view the calendar event
+3. Appointment must exist in the selected calendar</t>
   </si>
 </sst>
 </file>
@@ -733,7 +846,7 @@
       <charset val="1"/>
     </font>
   </fonts>
-  <fills count="16">
+  <fills count="17">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -811,6 +924,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.79998168889431442"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -932,7 +1051,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="74">
+  <cellXfs count="79">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1000,12 +1119,6 @@
     <xf numFmtId="0" fontId="5" fillId="11" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="12" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="12" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="13" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1096,56 +1209,77 @@
     <xf numFmtId="0" fontId="11" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="10" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="13" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="9" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="12" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="14" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="8" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="15" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="15" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="14" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="9" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="13" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="12" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="15" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="15" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="10" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="16" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="16" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="16" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="12" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="12" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1163,10 +1297,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1432,51 +1562,51 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:I41"/>
-  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:L59"/>
+  <sheetFormatPr defaultColWidth="8.90625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="5.88671875" style="2" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="32.88671875" style="2" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="11.109375" style="2" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="20.88671875" style="3" customWidth="1"/>
+    <col min="1" max="1" width="5.90625" style="2" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="32.90625" style="2" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="11.08984375" style="2" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="20.90625" style="3" customWidth="1"/>
     <col min="5" max="5" width="65" style="2" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="41" style="3" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="52" style="3" customWidth="1"/>
-    <col min="8" max="8" width="11.6640625" style="2" customWidth="1"/>
-    <col min="9" max="9" width="15.33203125" style="3" customWidth="1"/>
-    <col min="10" max="12" width="8.88671875" style="5" customWidth="1"/>
-    <col min="13" max="16384" width="8.88671875" style="5"/>
+    <col min="8" max="8" width="11.6328125" style="2" customWidth="1"/>
+    <col min="9" max="9" width="15.36328125" style="3" customWidth="1"/>
+    <col min="10" max="12" width="8.90625" style="5" customWidth="1"/>
+    <col min="13" max="16384" width="8.90625" style="5"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="39.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="71" t="s">
+    <row r="1" spans="1:9" ht="39.65" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A1" s="64" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="61" t="s">
+      <c r="B1" s="53" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="61" t="s">
+      <c r="C1" s="53" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="61" t="s">
+      <c r="D1" s="53" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="69"/>
-      <c r="F1" s="70"/>
-      <c r="G1" s="72" t="s">
+      <c r="E1" s="55"/>
+      <c r="F1" s="56"/>
+      <c r="G1" s="66" t="s">
         <v>4</v>
       </c>
-      <c r="H1" s="61" t="s">
+      <c r="H1" s="53" t="s">
         <v>5</v>
       </c>
-      <c r="I1" s="61" t="s">
+      <c r="I1" s="53" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A2" s="57"/>
-      <c r="B2" s="62"/>
-      <c r="C2" s="62"/>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A2" s="58"/>
+      <c r="B2" s="54"/>
+      <c r="C2" s="54"/>
       <c r="D2" s="1" t="s">
         <v>7</v>
       </c>
@@ -1486,188 +1616,188 @@
       <c r="F2" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="G2" s="73"/>
-      <c r="H2" s="62"/>
-      <c r="I2" s="62"/>
-    </row>
-    <row r="3" spans="1:9" s="8" customFormat="1" ht="82.8" x14ac:dyDescent="0.3">
-      <c r="A3" s="39" t="s">
-        <v>150</v>
-      </c>
-      <c r="B3" s="39" t="s">
-        <v>134</v>
+      <c r="G2" s="67"/>
+      <c r="H2" s="54"/>
+      <c r="I2" s="54"/>
+    </row>
+    <row r="3" spans="1:9" s="8" customFormat="1" ht="78" x14ac:dyDescent="0.35">
+      <c r="A3" s="37" t="s">
+        <v>142</v>
+      </c>
+      <c r="B3" s="37" t="s">
+        <v>126</v>
       </c>
       <c r="C3" s="22">
         <v>13.2</v>
       </c>
-      <c r="D3" s="40" t="s">
-        <v>135</v>
-      </c>
-      <c r="E3" s="40" t="s">
-        <v>136</v>
-      </c>
-      <c r="F3" s="40" t="s">
-        <v>137</v>
-      </c>
-      <c r="G3" s="41" t="s">
-        <v>140</v>
+      <c r="D3" s="38" t="s">
+        <v>127</v>
+      </c>
+      <c r="E3" s="38" t="s">
+        <v>128</v>
+      </c>
+      <c r="F3" s="38" t="s">
+        <v>129</v>
+      </c>
+      <c r="G3" s="39" t="s">
+        <v>132</v>
       </c>
       <c r="H3" s="22" t="s">
         <v>61</v>
       </c>
-      <c r="I3" s="40" t="s">
-        <v>141</v>
-      </c>
-    </row>
-    <row r="4" spans="1:9" s="8" customFormat="1" ht="55.2" x14ac:dyDescent="0.3">
-      <c r="A4" s="49">
+      <c r="I3" s="38" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" s="8" customFormat="1" ht="52" x14ac:dyDescent="0.35">
+      <c r="A4" s="47">
         <v>1</v>
       </c>
-      <c r="B4" s="49" t="s">
+      <c r="B4" s="47" t="s">
         <v>10</v>
       </c>
-      <c r="C4" s="50">
+      <c r="C4" s="48">
         <v>1.1000000000000001</v>
       </c>
-      <c r="D4" s="51" t="s">
+      <c r="D4" s="49" t="s">
         <v>11</v>
       </c>
-      <c r="E4" s="51" t="s">
+      <c r="E4" s="49" t="s">
+        <v>104</v>
+      </c>
+      <c r="F4" s="49" t="s">
+        <v>105</v>
+      </c>
+      <c r="G4" s="50" t="s">
+        <v>106</v>
+      </c>
+      <c r="H4" s="48" t="s">
+        <v>12</v>
+      </c>
+      <c r="I4" s="49" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" s="36" customFormat="1" ht="78" x14ac:dyDescent="0.35">
+      <c r="A5" s="68">
+        <v>3</v>
+      </c>
+      <c r="B5" s="68" t="s">
+        <v>13</v>
+      </c>
+      <c r="C5" s="35">
+        <v>3.1</v>
+      </c>
+      <c r="D5" s="40" t="s">
+        <v>11</v>
+      </c>
+      <c r="E5" s="41" t="s">
+        <v>107</v>
+      </c>
+      <c r="F5" s="41" t="s">
+        <v>108</v>
+      </c>
+      <c r="G5" s="42" t="s">
         <v>111</v>
       </c>
-      <c r="F4" s="51" t="s">
+      <c r="H5" s="43" t="s">
+        <v>98</v>
+      </c>
+      <c r="I5" s="40" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" s="8" customFormat="1" ht="78" x14ac:dyDescent="0.35">
+      <c r="A6" s="69"/>
+      <c r="B6" s="69"/>
+      <c r="C6" s="35">
+        <v>3.2</v>
+      </c>
+      <c r="D6" s="40" t="s">
+        <v>11</v>
+      </c>
+      <c r="E6" s="41" t="s">
+        <v>109</v>
+      </c>
+      <c r="F6" s="41" t="s">
+        <v>110</v>
+      </c>
+      <c r="G6" s="42" t="s">
         <v>112</v>
       </c>
-      <c r="G4" s="52" t="s">
-        <v>113</v>
-      </c>
-      <c r="H4" s="50" t="s">
-        <v>12</v>
-      </c>
-      <c r="I4" s="51" t="s">
-        <v>138</v>
-      </c>
-    </row>
-    <row r="5" spans="1:9" s="38" customFormat="1" ht="82.8" x14ac:dyDescent="0.3">
-      <c r="A5" s="67">
-        <v>3</v>
-      </c>
-      <c r="B5" s="67" t="s">
-        <v>13</v>
-      </c>
-      <c r="C5" s="37">
-        <v>3.1</v>
-      </c>
-      <c r="D5" s="42" t="s">
-        <v>11</v>
-      </c>
-      <c r="E5" s="43" t="s">
-        <v>114</v>
-      </c>
-      <c r="F5" s="43" t="s">
-        <v>115</v>
-      </c>
-      <c r="G5" s="44" t="s">
-        <v>118</v>
-      </c>
-      <c r="H5" s="45" t="s">
-        <v>105</v>
-      </c>
-      <c r="I5" s="42" t="s">
+      <c r="H6" s="35" t="s">
+        <v>98</v>
+      </c>
+      <c r="I6" s="40" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="6" spans="1:9" s="8" customFormat="1" ht="82.8" x14ac:dyDescent="0.3">
-      <c r="A6" s="68"/>
-      <c r="B6" s="68"/>
-      <c r="C6" s="37">
-        <v>3.2</v>
-      </c>
-      <c r="D6" s="42" t="s">
-        <v>11</v>
-      </c>
-      <c r="E6" s="43" t="s">
-        <v>116</v>
-      </c>
-      <c r="F6" s="43" t="s">
-        <v>117</v>
-      </c>
-      <c r="G6" s="44" t="s">
-        <v>119</v>
-      </c>
-      <c r="H6" s="37" t="s">
-        <v>105</v>
-      </c>
-      <c r="I6" s="42" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="7" spans="1:9" s="8" customFormat="1" ht="124.2" x14ac:dyDescent="0.3">
-      <c r="A7" s="48">
+    <row r="7" spans="1:9" s="8" customFormat="1" ht="117" x14ac:dyDescent="0.35">
+      <c r="A7" s="46">
         <v>5</v>
       </c>
-      <c r="B7" s="48" t="s">
+      <c r="B7" s="46" t="s">
         <v>16</v>
       </c>
       <c r="C7" s="9">
         <v>5.2</v>
       </c>
       <c r="D7" s="10" t="s">
-        <v>142</v>
+        <v>134</v>
       </c>
       <c r="E7" s="10" t="s">
-        <v>144</v>
+        <v>136</v>
       </c>
       <c r="F7" s="10" t="s">
-        <v>143</v>
-      </c>
-      <c r="G7" s="29" t="s">
-        <v>145</v>
+        <v>135</v>
+      </c>
+      <c r="G7" s="27" t="s">
+        <v>137</v>
       </c>
       <c r="H7" s="11" t="s">
-        <v>106</v>
+        <v>99</v>
       </c>
       <c r="I7" s="10" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="8" spans="1:9" s="8" customFormat="1" ht="27.6" x14ac:dyDescent="0.3">
-      <c r="A8" s="63">
+    <row r="8" spans="1:9" s="8" customFormat="1" ht="26" x14ac:dyDescent="0.35">
+      <c r="A8" s="61">
         <v>6</v>
       </c>
-      <c r="B8" s="63" t="s">
+      <c r="B8" s="61" t="s">
         <v>18</v>
       </c>
       <c r="C8" s="12">
         <v>6.1</v>
       </c>
       <c r="D8" s="13" t="s">
-        <v>135</v>
-      </c>
-      <c r="E8" s="53" t="s">
-        <v>146</v>
-      </c>
-      <c r="F8" s="53" t="s">
-        <v>147</v>
-      </c>
-      <c r="G8" s="54" t="s">
-        <v>148</v>
+        <v>127</v>
+      </c>
+      <c r="E8" s="51" t="s">
+        <v>138</v>
+      </c>
+      <c r="F8" s="51" t="s">
+        <v>139</v>
+      </c>
+      <c r="G8" s="52" t="s">
+        <v>140</v>
       </c>
       <c r="H8" s="14" t="s">
-        <v>107</v>
+        <v>100</v>
       </c>
       <c r="I8" s="13" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="9" spans="1:9" s="8" customFormat="1" ht="55.2" x14ac:dyDescent="0.3">
-      <c r="A9" s="57"/>
-      <c r="B9" s="57"/>
+    <row r="9" spans="1:9" s="8" customFormat="1" ht="52" x14ac:dyDescent="0.35">
+      <c r="A9" s="58"/>
+      <c r="B9" s="58"/>
       <c r="C9" s="12">
         <v>6.3</v>
       </c>
       <c r="D9" s="13" t="s">
-        <v>135</v>
+        <v>127</v>
       </c>
       <c r="E9" s="13" t="s">
         <v>20</v>
@@ -1675,26 +1805,26 @@
       <c r="F9" s="13" t="s">
         <v>21</v>
       </c>
-      <c r="G9" s="30" t="s">
-        <v>149</v>
+      <c r="G9" s="28" t="s">
+        <v>141</v>
       </c>
       <c r="H9" s="12" t="s">
-        <v>107</v>
+        <v>100</v>
       </c>
       <c r="I9" s="13"/>
     </row>
-    <row r="10" spans="1:9" s="8" customFormat="1" ht="55.2" x14ac:dyDescent="0.3">
-      <c r="A10" s="66">
+    <row r="10" spans="1:9" s="8" customFormat="1" ht="52" x14ac:dyDescent="0.35">
+      <c r="A10" s="62">
         <v>7</v>
       </c>
-      <c r="B10" s="66" t="s">
+      <c r="B10" s="62" t="s">
         <v>22</v>
       </c>
       <c r="C10" s="15">
         <v>7.1</v>
       </c>
       <c r="D10" s="16" t="s">
-        <v>135</v>
+        <v>127</v>
       </c>
       <c r="E10" s="16" t="s">
         <v>23</v>
@@ -1702,24 +1832,24 @@
       <c r="F10" s="16" t="s">
         <v>24</v>
       </c>
-      <c r="G10" s="31" t="s">
+      <c r="G10" s="29" t="s">
         <v>25</v>
       </c>
       <c r="H10" s="17" t="s">
-        <v>108</v>
+        <v>101</v>
       </c>
       <c r="I10" s="16" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="11" spans="1:9" s="8" customFormat="1" ht="55.2" x14ac:dyDescent="0.3">
-      <c r="A11" s="56"/>
-      <c r="B11" s="56"/>
+    <row r="11" spans="1:9" s="8" customFormat="1" ht="52" x14ac:dyDescent="0.35">
+      <c r="A11" s="60"/>
+      <c r="B11" s="60"/>
       <c r="C11" s="15">
         <v>7.2</v>
       </c>
       <c r="D11" s="16" t="s">
-        <v>135</v>
+        <v>127</v>
       </c>
       <c r="E11" s="16" t="s">
         <v>27</v>
@@ -1727,24 +1857,24 @@
       <c r="F11" s="16" t="s">
         <v>28</v>
       </c>
-      <c r="G11" s="31" t="s">
+      <c r="G11" s="29" t="s">
         <v>29</v>
       </c>
       <c r="H11" s="15" t="s">
-        <v>109</v>
+        <v>102</v>
       </c>
       <c r="I11" s="16" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="12" spans="1:9" s="8" customFormat="1" ht="41.4" x14ac:dyDescent="0.3">
-      <c r="A12" s="57"/>
-      <c r="B12" s="57"/>
+    <row r="12" spans="1:9" s="8" customFormat="1" ht="39" x14ac:dyDescent="0.35">
+      <c r="A12" s="58"/>
+      <c r="B12" s="58"/>
       <c r="C12" s="15">
         <v>7.3</v>
       </c>
       <c r="D12" s="16" t="s">
-        <v>135</v>
+        <v>127</v>
       </c>
       <c r="E12" s="16" t="s">
         <v>30</v>
@@ -1752,19 +1882,19 @@
       <c r="F12" s="16" t="s">
         <v>31</v>
       </c>
-      <c r="G12" s="31" t="s">
+      <c r="G12" s="29" t="s">
         <v>32</v>
       </c>
       <c r="H12" s="15" t="s">
-        <v>108</v>
+        <v>101</v>
       </c>
       <c r="I12" s="16"/>
     </row>
-    <row r="13" spans="1:9" s="8" customFormat="1" ht="82.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="60">
+    <row r="13" spans="1:9" s="8" customFormat="1" ht="82.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A13" s="59">
         <v>9</v>
       </c>
-      <c r="B13" s="60" t="s">
+      <c r="B13" s="59" t="s">
         <v>33</v>
       </c>
       <c r="C13" s="18">
@@ -1779,15 +1909,15 @@
       <c r="F13" s="19" t="s">
         <v>35</v>
       </c>
-      <c r="G13" s="32" t="s">
+      <c r="G13" s="30" t="s">
         <v>36</v>
       </c>
       <c r="H13" s="18"/>
       <c r="I13" s="19"/>
     </row>
-    <row r="14" spans="1:9" s="8" customFormat="1" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="56"/>
-      <c r="B14" s="56"/>
+    <row r="14" spans="1:9" s="8" customFormat="1" ht="41.4" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A14" s="60"/>
+      <c r="B14" s="60"/>
       <c r="C14" s="18">
         <v>9.1999999999999993</v>
       </c>
@@ -1800,15 +1930,15 @@
       <c r="F14" s="19" t="s">
         <v>39</v>
       </c>
-      <c r="G14" s="32" t="s">
+      <c r="G14" s="30" t="s">
         <v>40</v>
       </c>
       <c r="H14" s="18"/>
       <c r="I14" s="19"/>
     </row>
-    <row r="15" spans="1:9" s="8" customFormat="1" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="56"/>
-      <c r="B15" s="56"/>
+    <row r="15" spans="1:9" s="8" customFormat="1" ht="27.65" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A15" s="60"/>
+      <c r="B15" s="60"/>
       <c r="C15" s="18">
         <v>9.3000000000000007</v>
       </c>
@@ -1821,7 +1951,7 @@
       <c r="F15" s="19" t="s">
         <v>43</v>
       </c>
-      <c r="G15" s="32" t="s">
+      <c r="G15" s="30" t="s">
         <v>44</v>
       </c>
       <c r="H15" s="18"/>
@@ -1829,9 +1959,9 @@
         <v>45</v>
       </c>
     </row>
-    <row r="16" spans="1:9" s="8" customFormat="1" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="57"/>
-      <c r="B16" s="57"/>
+    <row r="16" spans="1:9" s="8" customFormat="1" ht="41.4" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A16" s="58"/>
+      <c r="B16" s="58"/>
       <c r="C16" s="18">
         <v>9.4</v>
       </c>
@@ -1844,7 +1974,7 @@
       <c r="F16" s="19" t="s">
         <v>47</v>
       </c>
-      <c r="G16" s="32" t="s">
+      <c r="G16" s="30" t="s">
         <v>48</v>
       </c>
       <c r="H16" s="18"/>
@@ -1852,11 +1982,11 @@
         <v>45</v>
       </c>
     </row>
-    <row r="17" spans="1:9" s="8" customFormat="1" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="55">
+    <row r="17" spans="1:9" s="8" customFormat="1" ht="41.4" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A17" s="70">
         <v>12</v>
       </c>
-      <c r="B17" s="55" t="s">
+      <c r="B17" s="70" t="s">
         <v>49</v>
       </c>
       <c r="C17" s="20">
@@ -1871,7 +2001,7 @@
       <c r="F17" s="21" t="s">
         <v>51</v>
       </c>
-      <c r="G17" s="33" t="s">
+      <c r="G17" s="31" t="s">
         <v>52</v>
       </c>
       <c r="H17" s="20" t="s">
@@ -1881,9 +2011,9 @@
         <v>54</v>
       </c>
     </row>
-    <row r="18" spans="1:9" s="8" customFormat="1" ht="55.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="56"/>
-      <c r="B18" s="56"/>
+    <row r="18" spans="1:9" s="8" customFormat="1" ht="55.25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A18" s="60"/>
+      <c r="B18" s="60"/>
       <c r="C18" s="20">
         <v>12.2</v>
       </c>
@@ -1896,7 +2026,7 @@
       <c r="F18" s="21" t="s">
         <v>56</v>
       </c>
-      <c r="G18" s="33" t="s">
+      <c r="G18" s="31" t="s">
         <v>57</v>
       </c>
       <c r="H18" s="20" t="s">
@@ -1906,9 +2036,9 @@
         <v>54</v>
       </c>
     </row>
-    <row r="19" spans="1:9" s="8" customFormat="1" ht="55.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="57"/>
-      <c r="B19" s="57"/>
+    <row r="19" spans="1:9" s="8" customFormat="1" ht="55.25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A19" s="58"/>
+      <c r="B19" s="58"/>
       <c r="C19" s="20">
         <v>12.3</v>
       </c>
@@ -1921,7 +2051,7 @@
       <c r="F19" s="21" t="s">
         <v>59</v>
       </c>
-      <c r="G19" s="33" t="s">
+      <c r="G19" s="31" t="s">
         <v>60</v>
       </c>
       <c r="H19" s="20" t="s">
@@ -1929,458 +2059,801 @@
       </c>
       <c r="I19" s="21"/>
     </row>
-    <row r="20" spans="1:9" s="8" customFormat="1" ht="55.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="64">
+    <row r="20" spans="1:9" s="8" customFormat="1" ht="55" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A20" s="65">
         <v>14</v>
       </c>
-      <c r="B20" s="64" t="s">
+      <c r="B20" s="65" t="s">
         <v>62</v>
       </c>
-      <c r="C20" s="23">
+      <c r="C20" s="76">
         <v>14.1</v>
       </c>
-      <c r="D20" s="24" t="s">
+      <c r="D20" s="32" t="s">
         <v>15</v>
       </c>
-      <c r="E20" s="24" t="s">
+      <c r="E20" s="32" t="s">
+        <v>147</v>
+      </c>
+      <c r="F20" s="32" t="s">
+        <v>148</v>
+      </c>
+      <c r="G20" s="32" t="s">
+        <v>172</v>
+      </c>
+      <c r="H20" s="76" t="s">
+        <v>103</v>
+      </c>
+      <c r="I20" s="32" t="s">
         <v>63</v>
       </c>
-      <c r="F20" s="24" t="s">
+    </row>
+    <row r="21" spans="1:9" s="8" customFormat="1" ht="55" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A21" s="75"/>
+      <c r="B21" s="75"/>
+      <c r="C21" s="76">
+        <v>14.2</v>
+      </c>
+      <c r="D21" s="32" t="s">
+        <v>15</v>
+      </c>
+      <c r="E21" s="32" t="s">
+        <v>149</v>
+      </c>
+      <c r="F21" s="32" t="s">
+        <v>150</v>
+      </c>
+      <c r="G21" s="32" t="s">
+        <v>173</v>
+      </c>
+      <c r="H21" s="76" t="s">
+        <v>103</v>
+      </c>
+      <c r="I21" s="32" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="22" spans="1:9" s="8" customFormat="1" ht="55" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A22" s="75"/>
+      <c r="B22" s="75"/>
+      <c r="C22" s="76">
+        <v>14.3</v>
+      </c>
+      <c r="D22" s="32" t="s">
+        <v>151</v>
+      </c>
+      <c r="E22" s="32" t="s">
+        <v>152</v>
+      </c>
+      <c r="F22" s="32" t="s">
+        <v>153</v>
+      </c>
+      <c r="G22" s="32" t="s">
+        <v>174</v>
+      </c>
+      <c r="H22" s="76" t="s">
+        <v>103</v>
+      </c>
+      <c r="I22" s="32" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="23" spans="1:9" s="8" customFormat="1" ht="55" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A23" s="75"/>
+      <c r="B23" s="75"/>
+      <c r="C23" s="76">
+        <v>14.4</v>
+      </c>
+      <c r="D23" s="32" t="s">
+        <v>15</v>
+      </c>
+      <c r="E23" s="32" t="s">
+        <v>154</v>
+      </c>
+      <c r="F23" s="32" t="s">
+        <v>155</v>
+      </c>
+      <c r="G23" s="32" t="s">
+        <v>175</v>
+      </c>
+      <c r="H23" s="76" t="s">
+        <v>103</v>
+      </c>
+      <c r="I23" s="32" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="24" spans="1:9" s="8" customFormat="1" ht="55" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A24" s="75"/>
+      <c r="B24" s="75"/>
+      <c r="C24" s="76">
+        <v>14.5</v>
+      </c>
+      <c r="D24" s="32" t="s">
+        <v>15</v>
+      </c>
+      <c r="E24" s="32" t="s">
+        <v>156</v>
+      </c>
+      <c r="F24" s="32" t="s">
+        <v>157</v>
+      </c>
+      <c r="G24" s="32" t="s">
+        <v>176</v>
+      </c>
+      <c r="H24" s="76" t="s">
+        <v>103</v>
+      </c>
+      <c r="I24" s="32" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="25" spans="1:9" s="8" customFormat="1" ht="55" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A25" s="75"/>
+      <c r="B25" s="75"/>
+      <c r="C25" s="76">
+        <v>14.6</v>
+      </c>
+      <c r="D25" s="32" t="s">
+        <v>15</v>
+      </c>
+      <c r="E25" s="32" t="s">
+        <v>158</v>
+      </c>
+      <c r="F25" s="32" t="s">
+        <v>159</v>
+      </c>
+      <c r="G25" s="32" t="s">
+        <v>182</v>
+      </c>
+      <c r="H25" s="76" t="s">
+        <v>103</v>
+      </c>
+      <c r="I25" s="32" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="26" spans="1:9" s="8" customFormat="1" ht="55" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A26" s="75"/>
+      <c r="B26" s="75"/>
+      <c r="C26" s="76">
+        <v>14.7</v>
+      </c>
+      <c r="D26" s="32" t="s">
+        <v>15</v>
+      </c>
+      <c r="E26" s="32" t="s">
+        <v>160</v>
+      </c>
+      <c r="F26" s="32" t="s">
+        <v>161</v>
+      </c>
+      <c r="G26" s="32" t="s">
+        <v>177</v>
+      </c>
+      <c r="H26" s="76" t="s">
+        <v>103</v>
+      </c>
+      <c r="I26" s="32" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="27" spans="1:9" s="8" customFormat="1" ht="55" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A27" s="75"/>
+      <c r="B27" s="75"/>
+      <c r="C27" s="76">
+        <v>14.8</v>
+      </c>
+      <c r="D27" s="32" t="s">
+        <v>15</v>
+      </c>
+      <c r="E27" s="32" t="s">
+        <v>162</v>
+      </c>
+      <c r="F27" s="32" t="s">
+        <v>163</v>
+      </c>
+      <c r="G27" s="32" t="s">
+        <v>178</v>
+      </c>
+      <c r="H27" s="76" t="s">
+        <v>143</v>
+      </c>
+      <c r="I27" s="32" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="28" spans="1:9" s="8" customFormat="1" ht="55" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A28" s="75"/>
+      <c r="B28" s="75"/>
+      <c r="C28" s="76">
+        <v>14.9</v>
+      </c>
+      <c r="D28" s="32" t="s">
+        <v>15</v>
+      </c>
+      <c r="E28" s="32" t="s">
+        <v>164</v>
+      </c>
+      <c r="F28" s="32" t="s">
+        <v>165</v>
+      </c>
+      <c r="G28" s="32" t="s">
+        <v>179</v>
+      </c>
+      <c r="H28" s="76" t="s">
+        <v>143</v>
+      </c>
+      <c r="I28" s="32" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="29" spans="1:9" s="8" customFormat="1" ht="55" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A29" s="75"/>
+      <c r="B29" s="75"/>
+      <c r="C29" s="76">
+        <v>14.1</v>
+      </c>
+      <c r="D29" s="32" t="s">
+        <v>15</v>
+      </c>
+      <c r="E29" s="32" t="s">
+        <v>166</v>
+      </c>
+      <c r="F29" s="32" t="s">
+        <v>167</v>
+      </c>
+      <c r="G29" s="32" t="s">
+        <v>180</v>
+      </c>
+      <c r="H29" s="76" t="s">
+        <v>143</v>
+      </c>
+      <c r="I29" s="32" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="30" spans="1:9" s="8" customFormat="1" ht="55" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A30" s="75"/>
+      <c r="B30" s="75"/>
+      <c r="C30" s="76">
+        <v>14.11</v>
+      </c>
+      <c r="D30" s="32" t="s">
+        <v>15</v>
+      </c>
+      <c r="E30" s="32" t="s">
+        <v>168</v>
+      </c>
+      <c r="F30" s="32" t="s">
+        <v>169</v>
+      </c>
+      <c r="G30" s="32" t="s">
+        <v>181</v>
+      </c>
+      <c r="H30" s="76" t="s">
+        <v>143</v>
+      </c>
+      <c r="I30" s="32" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="31" spans="1:9" s="8" customFormat="1" ht="26" x14ac:dyDescent="0.35">
+      <c r="A31" s="63">
+        <v>15</v>
+      </c>
+      <c r="B31" s="63" t="s">
         <v>64</v>
       </c>
-      <c r="G20" s="34" t="s">
+      <c r="C31" s="23">
+        <v>15.1</v>
+      </c>
+      <c r="D31" s="24" t="s">
         <v>65</v>
       </c>
-      <c r="H20" s="23" t="s">
-        <v>110</v>
-      </c>
-      <c r="I20" s="24" t="s">
+      <c r="E31" s="24" t="s">
         <v>66</v>
       </c>
-    </row>
-    <row r="21" spans="1:9" s="8" customFormat="1" ht="55.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A21" s="57"/>
-      <c r="B21" s="57"/>
-      <c r="C21" s="23">
-        <v>14.2</v>
-      </c>
-      <c r="D21" s="24" t="s">
-        <v>15</v>
-      </c>
-      <c r="E21" s="24" t="s">
+      <c r="F31" s="24" t="s">
         <v>67</v>
       </c>
-      <c r="F21" s="24" t="s">
+      <c r="G31" s="33" t="s">
         <v>68</v>
       </c>
-      <c r="G21" s="34" t="s">
+      <c r="H31" s="23" t="s">
+        <v>144</v>
+      </c>
+      <c r="I31" s="24" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="32" spans="1:9" s="8" customFormat="1" ht="26" x14ac:dyDescent="0.35">
+      <c r="A32" s="60"/>
+      <c r="B32" s="60"/>
+      <c r="C32" s="23">
+        <v>15.2</v>
+      </c>
+      <c r="D32" s="24" t="s">
+        <v>65</v>
+      </c>
+      <c r="E32" s="24" t="s">
         <v>69</v>
       </c>
-      <c r="H21" s="23" t="s">
-        <v>110</v>
-      </c>
-      <c r="I21" s="24" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="22" spans="1:9" s="8" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A22" s="58">
-        <v>15</v>
-      </c>
-      <c r="B22" s="58" t="s">
+      <c r="F32" s="24" t="s">
         <v>70</v>
       </c>
-      <c r="C22" s="25">
-        <v>15.1</v>
-      </c>
-      <c r="D22" s="26" t="s">
+      <c r="G32" s="33" t="s">
         <v>71</v>
       </c>
-      <c r="E22" s="26" t="s">
+      <c r="H32" s="23" t="s">
+        <v>144</v>
+      </c>
+      <c r="I32" s="24" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="33" spans="1:12" s="8" customFormat="1" ht="26" x14ac:dyDescent="0.35">
+      <c r="A33" s="60"/>
+      <c r="B33" s="60"/>
+      <c r="C33" s="23">
+        <v>15.3</v>
+      </c>
+      <c r="D33" s="24" t="s">
+        <v>65</v>
+      </c>
+      <c r="E33" s="24" t="s">
         <v>72</v>
       </c>
-      <c r="F22" s="26" t="s">
+      <c r="F33" s="24" t="s">
         <v>73</v>
       </c>
-      <c r="G22" s="35" t="s">
+      <c r="G33" s="33" t="s">
         <v>74</v>
       </c>
-      <c r="H22" s="25"/>
-      <c r="I22" s="26"/>
-    </row>
-    <row r="23" spans="1:9" s="8" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A23" s="56"/>
-      <c r="B23" s="56"/>
-      <c r="C23" s="25">
-        <v>15.2</v>
-      </c>
-      <c r="D23" s="26" t="s">
-        <v>71</v>
-      </c>
-      <c r="E23" s="26" t="s">
+      <c r="H33" s="23" t="s">
+        <v>144</v>
+      </c>
+      <c r="I33" s="24" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="34" spans="1:12" s="8" customFormat="1" ht="26" x14ac:dyDescent="0.35">
+      <c r="A34" s="60"/>
+      <c r="B34" s="60"/>
+      <c r="C34" s="23">
+        <v>15.4</v>
+      </c>
+      <c r="D34" s="24" t="s">
+        <v>65</v>
+      </c>
+      <c r="E34" s="24" t="s">
         <v>75</v>
       </c>
-      <c r="F23" s="26" t="s">
+      <c r="F34" s="24" t="s">
         <v>76</v>
       </c>
-      <c r="G23" s="35" t="s">
+      <c r="G34" s="33" t="s">
         <v>77</v>
       </c>
-      <c r="H23" s="25"/>
-      <c r="I23" s="26"/>
-    </row>
-    <row r="24" spans="1:9" s="8" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A24" s="56"/>
-      <c r="B24" s="56"/>
-      <c r="C24" s="25">
-        <v>15.3</v>
-      </c>
-      <c r="D24" s="26" t="s">
-        <v>71</v>
-      </c>
-      <c r="E24" s="26" t="s">
+      <c r="H34" s="23" t="s">
+        <v>146</v>
+      </c>
+      <c r="I34" s="24" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="35" spans="1:12" s="8" customFormat="1" ht="26" x14ac:dyDescent="0.35">
+      <c r="A35" s="58"/>
+      <c r="B35" s="58"/>
+      <c r="C35" s="23">
+        <v>15.5</v>
+      </c>
+      <c r="D35" s="24" t="s">
+        <v>65</v>
+      </c>
+      <c r="E35" s="24" t="s">
         <v>78</v>
       </c>
-      <c r="F24" s="26" t="s">
+      <c r="F35" s="24" t="s">
         <v>79</v>
       </c>
-      <c r="G24" s="35" t="s">
+      <c r="G35" s="33" t="s">
         <v>80</v>
       </c>
-      <c r="H24" s="25"/>
-      <c r="I24" s="26"/>
-    </row>
-    <row r="25" spans="1:9" s="8" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A25" s="56"/>
-      <c r="B25" s="56"/>
-      <c r="C25" s="25">
-        <v>15.4</v>
-      </c>
-      <c r="D25" s="26" t="s">
-        <v>71</v>
-      </c>
-      <c r="E25" s="26" t="s">
+      <c r="H35" s="23" t="s">
+        <v>146</v>
+      </c>
+      <c r="I35" s="24" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="36" spans="1:12" s="8" customFormat="1" ht="26" x14ac:dyDescent="0.35">
+      <c r="A36" s="57">
+        <v>16</v>
+      </c>
+      <c r="B36" s="57" t="s">
         <v>81</v>
       </c>
-      <c r="F25" s="26" t="s">
+      <c r="C36" s="25">
+        <v>16.100000000000001</v>
+      </c>
+      <c r="D36" s="26" t="s">
         <v>82</v>
       </c>
-      <c r="G25" s="35" t="s">
+      <c r="E36" s="26" t="s">
         <v>83</v>
       </c>
-      <c r="H25" s="25"/>
-      <c r="I25" s="26"/>
-    </row>
-    <row r="26" spans="1:9" s="8" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A26" s="57"/>
-      <c r="B26" s="57"/>
-      <c r="C26" s="25">
-        <v>15.5</v>
-      </c>
-      <c r="D26" s="26" t="s">
-        <v>71</v>
-      </c>
-      <c r="E26" s="26" t="s">
+      <c r="F36" s="26" t="s">
         <v>84</v>
       </c>
-      <c r="F26" s="26" t="s">
+      <c r="G36" s="72" t="s">
         <v>85</v>
       </c>
-      <c r="G26" s="35" t="s">
+      <c r="H36" s="73" t="s">
+        <v>146</v>
+      </c>
+      <c r="I36" s="74" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="37" spans="1:12" s="8" customFormat="1" ht="26" x14ac:dyDescent="0.35">
+      <c r="A37" s="58"/>
+      <c r="B37" s="58"/>
+      <c r="C37" s="25">
+        <v>16.2</v>
+      </c>
+      <c r="D37" s="26" t="s">
         <v>86</v>
       </c>
-      <c r="H26" s="25"/>
-      <c r="I26" s="26"/>
-    </row>
-    <row r="27" spans="1:9" s="8" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A27" s="65">
-        <v>16</v>
-      </c>
-      <c r="B27" s="65" t="s">
+      <c r="E37" s="26" t="s">
         <v>87</v>
       </c>
-      <c r="C27" s="27">
-        <v>16.100000000000001</v>
-      </c>
-      <c r="D27" s="28" t="s">
+      <c r="F37" s="26" t="s">
         <v>88</v>
       </c>
-      <c r="E27" s="28" t="s">
+      <c r="G37" s="34" t="s">
         <v>89</v>
       </c>
-      <c r="F27" s="28" t="s">
+      <c r="H37" s="73" t="s">
+        <v>146</v>
+      </c>
+      <c r="I37" s="74" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="38" spans="1:12" s="8" customFormat="1" ht="26" x14ac:dyDescent="0.35">
+      <c r="A38" s="71">
+        <v>17</v>
+      </c>
+      <c r="B38" s="71" t="s">
         <v>90</v>
       </c>
-      <c r="G27" s="36" t="s">
+      <c r="C38" s="9">
+        <v>17.100000000000001</v>
+      </c>
+      <c r="D38" s="10" t="s">
         <v>91</v>
       </c>
-      <c r="H27" s="27"/>
-      <c r="I27" s="28"/>
-    </row>
-    <row r="28" spans="1:9" s="8" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A28" s="57"/>
-      <c r="B28" s="57"/>
-      <c r="C28" s="27">
-        <v>16.2</v>
-      </c>
-      <c r="D28" s="28" t="s">
+      <c r="E38" s="44" t="s">
+        <v>170</v>
+      </c>
+      <c r="F38" s="10" t="s">
         <v>92</v>
       </c>
-      <c r="E28" s="28" t="s">
+      <c r="G38" s="45" t="s">
+        <v>171</v>
+      </c>
+      <c r="H38" s="9" t="s">
+        <v>103</v>
+      </c>
+      <c r="I38" s="44" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="39" spans="1:12" s="8" customFormat="1" ht="26" x14ac:dyDescent="0.35">
+      <c r="A39" s="60"/>
+      <c r="B39" s="60"/>
+      <c r="C39" s="9">
+        <v>17.2</v>
+      </c>
+      <c r="D39" s="10" t="s">
+        <v>91</v>
+      </c>
+      <c r="E39" s="44" t="s">
+        <v>113</v>
+      </c>
+      <c r="F39" s="10" t="s">
         <v>93</v>
       </c>
-      <c r="F28" s="28" t="s">
+      <c r="G39" s="45" t="s">
         <v>94</v>
       </c>
-      <c r="G28" s="36" t="s">
+      <c r="H39" s="9" t="s">
+        <v>103</v>
+      </c>
+      <c r="I39" s="44" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="40" spans="1:12" s="8" customFormat="1" ht="39" x14ac:dyDescent="0.35">
+      <c r="A40" s="60"/>
+      <c r="B40" s="60"/>
+      <c r="C40" s="9">
+        <v>17.3</v>
+      </c>
+      <c r="D40" s="10" t="s">
+        <v>91</v>
+      </c>
+      <c r="E40" s="10" t="s">
         <v>95</v>
       </c>
-      <c r="H28" s="27"/>
-      <c r="I28" s="28"/>
-    </row>
-    <row r="29" spans="1:9" s="8" customFormat="1" ht="27.6" x14ac:dyDescent="0.3">
-      <c r="A29" s="59">
-        <v>17</v>
-      </c>
-      <c r="B29" s="59" t="s">
+      <c r="F40" s="44" t="s">
+        <v>114</v>
+      </c>
+      <c r="G40" s="45" t="s">
+        <v>117</v>
+      </c>
+      <c r="H40" s="9" t="s">
+        <v>103</v>
+      </c>
+      <c r="I40" s="44" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="41" spans="1:12" s="8" customFormat="1" ht="26" x14ac:dyDescent="0.35">
+      <c r="A41" s="60"/>
+      <c r="B41" s="60"/>
+      <c r="C41" s="9">
+        <v>17.399999999999999</v>
+      </c>
+      <c r="D41" s="10" t="s">
+        <v>91</v>
+      </c>
+      <c r="E41" s="44" t="s">
+        <v>116</v>
+      </c>
+      <c r="F41" s="44" t="s">
+        <v>115</v>
+      </c>
+      <c r="G41" s="45" t="s">
+        <v>121</v>
+      </c>
+      <c r="H41" s="9" t="s">
+        <v>103</v>
+      </c>
+      <c r="I41" s="44" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="42" spans="1:12" s="8" customFormat="1" ht="26" x14ac:dyDescent="0.35">
+      <c r="A42" s="60"/>
+      <c r="B42" s="60"/>
+      <c r="C42" s="9">
+        <v>17.5</v>
+      </c>
+      <c r="D42" s="10" t="s">
+        <v>91</v>
+      </c>
+      <c r="E42" s="44" t="s">
+        <v>118</v>
+      </c>
+      <c r="F42" s="44" t="s">
+        <v>119</v>
+      </c>
+      <c r="G42" s="45" t="s">
+        <v>120</v>
+      </c>
+      <c r="H42" s="9" t="s">
+        <v>103</v>
+      </c>
+      <c r="I42" s="44" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="43" spans="1:12" s="8" customFormat="1" ht="26" x14ac:dyDescent="0.35">
+      <c r="A43" s="60"/>
+      <c r="B43" s="60"/>
+      <c r="C43" s="9">
+        <v>17.600000000000001</v>
+      </c>
+      <c r="D43" s="10" t="s">
+        <v>91</v>
+      </c>
+      <c r="E43" s="10" t="s">
         <v>96</v>
       </c>
-      <c r="C29" s="9">
-        <v>17.100000000000001</v>
-      </c>
-      <c r="D29" s="10" t="s">
+      <c r="F43" s="44" t="s">
+        <v>122</v>
+      </c>
+      <c r="G43" s="45" t="s">
+        <v>123</v>
+      </c>
+      <c r="H43" s="9" t="s">
+        <v>103</v>
+      </c>
+      <c r="I43" s="44" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="44" spans="1:12" s="8" customFormat="1" ht="26" x14ac:dyDescent="0.35">
+      <c r="A44" s="60"/>
+      <c r="B44" s="60"/>
+      <c r="C44" s="9">
+        <v>17.7</v>
+      </c>
+      <c r="D44" s="10" t="s">
+        <v>91</v>
+      </c>
+      <c r="E44" s="10" t="s">
         <v>97</v>
       </c>
-      <c r="E29" s="46" t="s">
-        <v>98</v>
-      </c>
-      <c r="F29" s="10" t="s">
-        <v>99</v>
-      </c>
-      <c r="G29" s="47" t="s">
-        <v>120</v>
-      </c>
-      <c r="H29" s="9"/>
-      <c r="I29" s="46" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="30" spans="1:9" s="8" customFormat="1" ht="27.6" x14ac:dyDescent="0.3">
-      <c r="A30" s="56"/>
-      <c r="B30" s="56"/>
-      <c r="C30" s="9">
-        <v>17.2</v>
-      </c>
-      <c r="D30" s="10" t="s">
-        <v>97</v>
-      </c>
-      <c r="E30" s="46" t="s">
-        <v>121</v>
-      </c>
-      <c r="F30" s="10" t="s">
-        <v>100</v>
-      </c>
-      <c r="G30" s="47" t="s">
-        <v>101</v>
-      </c>
-      <c r="H30" s="9"/>
-      <c r="I30" s="46" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="31" spans="1:9" s="8" customFormat="1" ht="27.6" x14ac:dyDescent="0.3">
-      <c r="A31" s="56"/>
-      <c r="B31" s="56"/>
-      <c r="C31" s="9">
-        <v>17.3</v>
-      </c>
-      <c r="D31" s="10" t="s">
-        <v>97</v>
-      </c>
-      <c r="E31" s="10" t="s">
-        <v>102</v>
-      </c>
-      <c r="F31" s="46" t="s">
-        <v>122</v>
-      </c>
-      <c r="G31" s="47" t="s">
+      <c r="F44" s="44" t="s">
+        <v>124</v>
+      </c>
+      <c r="G44" s="45" t="s">
+        <v>131</v>
+      </c>
+      <c r="H44" s="9" t="s">
+        <v>103</v>
+      </c>
+      <c r="I44" s="44" t="s">
         <v>125</v>
       </c>
-      <c r="H31" s="9"/>
-      <c r="I31" s="46" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="32" spans="1:9" s="8" customFormat="1" ht="27.6" x14ac:dyDescent="0.3">
-      <c r="A32" s="56"/>
-      <c r="B32" s="56"/>
-      <c r="C32" s="9">
-        <v>17.399999999999999</v>
-      </c>
-      <c r="D32" s="10" t="s">
-        <v>97</v>
-      </c>
-      <c r="E32" s="46" t="s">
-        <v>124</v>
-      </c>
-      <c r="F32" s="46" t="s">
-        <v>123</v>
-      </c>
-      <c r="G32" s="47" t="s">
-        <v>129</v>
-      </c>
-      <c r="H32" s="9"/>
-      <c r="I32" s="46" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="33" spans="1:9" s="8" customFormat="1" ht="27.6" x14ac:dyDescent="0.3">
-      <c r="A33" s="56"/>
-      <c r="B33" s="56"/>
-      <c r="C33" s="9">
-        <v>17.5</v>
-      </c>
-      <c r="D33" s="10" t="s">
-        <v>97</v>
-      </c>
-      <c r="E33" s="46" t="s">
-        <v>126</v>
-      </c>
-      <c r="F33" s="46" t="s">
-        <v>127</v>
-      </c>
-      <c r="G33" s="47" t="s">
-        <v>128</v>
-      </c>
-      <c r="H33" s="9"/>
-      <c r="I33" s="46" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="34" spans="1:9" s="8" customFormat="1" ht="27.6" x14ac:dyDescent="0.3">
-      <c r="A34" s="56"/>
-      <c r="B34" s="56"/>
-      <c r="C34" s="9">
-        <v>17.600000000000001</v>
-      </c>
-      <c r="D34" s="10" t="s">
-        <v>97</v>
-      </c>
-      <c r="E34" s="10" t="s">
-        <v>103</v>
-      </c>
-      <c r="F34" s="46" t="s">
-        <v>130</v>
-      </c>
-      <c r="G34" s="47" t="s">
-        <v>131</v>
-      </c>
-      <c r="H34" s="9"/>
-      <c r="I34" s="46" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="35" spans="1:9" s="8" customFormat="1" ht="27.6" x14ac:dyDescent="0.3">
-      <c r="A35" s="56"/>
-      <c r="B35" s="56"/>
-      <c r="C35" s="9">
-        <v>17.7</v>
-      </c>
-      <c r="D35" s="10" t="s">
-        <v>97</v>
-      </c>
-      <c r="E35" s="10" t="s">
-        <v>104</v>
-      </c>
-      <c r="F35" s="46" t="s">
-        <v>132</v>
-      </c>
-      <c r="G35" s="47" t="s">
-        <v>139</v>
-      </c>
-      <c r="H35" s="9"/>
-      <c r="I35" s="46" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="36" spans="1:9" s="8" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A36" s="2"/>
-      <c r="B36" s="3"/>
-      <c r="C36" s="3"/>
-      <c r="D36" s="3"/>
-      <c r="E36" s="3"/>
-      <c r="F36" s="3"/>
-      <c r="G36" s="4"/>
-      <c r="H36" s="6"/>
-      <c r="I36" s="3"/>
-    </row>
-    <row r="37" spans="1:9" s="8" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A37" s="7"/>
-      <c r="B37" s="2"/>
-      <c r="C37" s="2"/>
-      <c r="D37" s="3"/>
-      <c r="E37" s="2"/>
-      <c r="F37" s="3"/>
-      <c r="G37" s="4"/>
-      <c r="H37" s="2"/>
-      <c r="I37" s="3"/>
-    </row>
-    <row r="38" spans="1:9" s="8" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A38" s="7"/>
-      <c r="B38" s="2"/>
-      <c r="C38" s="2"/>
-      <c r="D38" s="3"/>
-      <c r="E38" s="2"/>
-      <c r="F38" s="3"/>
-      <c r="G38" s="3"/>
-      <c r="H38" s="2"/>
-      <c r="I38" s="3"/>
-    </row>
-    <row r="39" spans="1:9" s="8" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A39" s="7"/>
-      <c r="B39" s="2"/>
-      <c r="C39" s="2"/>
-      <c r="D39" s="3"/>
-      <c r="E39" s="2"/>
-      <c r="F39" s="3"/>
-      <c r="G39" s="3"/>
-      <c r="H39" s="2"/>
-      <c r="I39" s="3"/>
-    </row>
-    <row r="40" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A40" s="7"/>
-    </row>
-    <row r="41" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A41" s="7"/>
+    </row>
+    <row r="45" spans="1:12" s="8" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A45" s="2"/>
+      <c r="B45" s="3"/>
+      <c r="C45" s="3"/>
+      <c r="D45" s="3"/>
+      <c r="E45" s="3"/>
+      <c r="F45" s="3"/>
+      <c r="G45" s="4"/>
+      <c r="H45" s="6"/>
+      <c r="I45" s="3"/>
+    </row>
+    <row r="46" spans="1:12" s="8" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A46" s="7"/>
+      <c r="B46" s="2"/>
+      <c r="C46" s="2"/>
+      <c r="D46" s="3"/>
+      <c r="E46" s="2"/>
+      <c r="F46" s="3"/>
+      <c r="G46" s="4"/>
+      <c r="H46" s="2"/>
+      <c r="I46" s="3"/>
+    </row>
+    <row r="47" spans="1:12" s="8" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A47" s="7"/>
+      <c r="B47" s="2"/>
+      <c r="C47" s="2"/>
+      <c r="D47" s="3"/>
+      <c r="E47" s="2"/>
+      <c r="F47" s="3"/>
+      <c r="G47" s="3"/>
+      <c r="H47" s="2"/>
+      <c r="I47" s="3"/>
+    </row>
+    <row r="48" spans="1:12" s="8" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A48" s="7"/>
+      <c r="B48" s="77"/>
+      <c r="C48" s="78"/>
+      <c r="D48" s="78"/>
+      <c r="E48" s="78"/>
+      <c r="F48" s="78"/>
+      <c r="G48" s="78"/>
+      <c r="H48" s="78"/>
+      <c r="I48" s="78"/>
+      <c r="J48" s="5"/>
+      <c r="K48" s="5"/>
+      <c r="L48" s="5"/>
+    </row>
+    <row r="49" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A49" s="3"/>
+      <c r="B49" s="3"/>
+      <c r="C49" s="3"/>
+      <c r="E49" s="3"/>
+      <c r="H49" s="3"/>
+    </row>
+    <row r="50" spans="1:9" ht="17" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="D50" s="2"/>
+      <c r="F50" s="2"/>
+      <c r="G50" s="2"/>
+      <c r="I50" s="2"/>
+    </row>
+    <row r="51" spans="1:9" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="D51" s="2"/>
+      <c r="F51" s="2"/>
+      <c r="G51" s="2"/>
+      <c r="I51" s="2"/>
+    </row>
+    <row r="52" spans="1:9" ht="36.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A52" s="77"/>
+      <c r="B52" s="77"/>
+      <c r="C52" s="77"/>
+      <c r="D52" s="77"/>
+      <c r="E52" s="77"/>
+      <c r="F52" s="77"/>
+      <c r="G52" s="77"/>
+      <c r="H52" s="77"/>
+      <c r="I52" s="77"/>
+    </row>
+    <row r="53" spans="1:9" ht="36" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A53" s="3"/>
+      <c r="B53" s="3"/>
+      <c r="C53" s="3"/>
+      <c r="E53" s="3"/>
+      <c r="H53" s="3"/>
+    </row>
+    <row r="54" spans="1:9" ht="31" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="D54" s="2"/>
+      <c r="F54" s="2"/>
+      <c r="G54" s="2"/>
+      <c r="I54" s="2"/>
+    </row>
+    <row r="55" spans="1:9" ht="35" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="D55" s="2"/>
+      <c r="F55" s="2"/>
+      <c r="G55" s="2"/>
+      <c r="I55" s="2"/>
+    </row>
+    <row r="56" spans="1:9" ht="32" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A56" s="77"/>
+      <c r="B56" s="77"/>
+      <c r="C56" s="77"/>
+      <c r="D56" s="77"/>
+      <c r="E56" s="77"/>
+      <c r="F56" s="77"/>
+      <c r="G56" s="77"/>
+      <c r="H56" s="77"/>
+      <c r="I56" s="77"/>
+    </row>
+    <row r="57" spans="1:9" ht="33.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A57" s="3"/>
+      <c r="B57" s="3"/>
+      <c r="C57" s="3"/>
+      <c r="E57" s="3"/>
+      <c r="H57" s="3"/>
+    </row>
+    <row r="58" spans="1:9" ht="31.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="D58" s="2"/>
+      <c r="F58" s="2"/>
+      <c r="G58" s="2"/>
+      <c r="I58" s="2"/>
+    </row>
+    <row r="59" spans="1:9" ht="27.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B59" s="3"/>
+      <c r="F59" s="2"/>
+      <c r="G59" s="2"/>
+      <c r="I59" s="2"/>
     </row>
   </sheetData>
   <autoFilter ref="I1:I19" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
   <mergeCells count="25">
+    <mergeCell ref="A38:A44"/>
+    <mergeCell ref="B13:B16"/>
+    <mergeCell ref="B17:B19"/>
+    <mergeCell ref="B38:B44"/>
+    <mergeCell ref="A10:A12"/>
+    <mergeCell ref="B5:B6"/>
+    <mergeCell ref="A5:A6"/>
+    <mergeCell ref="A17:A19"/>
+    <mergeCell ref="A31:A35"/>
     <mergeCell ref="I1:I2"/>
     <mergeCell ref="D1:F1"/>
-    <mergeCell ref="A27:A28"/>
+    <mergeCell ref="A36:A37"/>
     <mergeCell ref="A13:A16"/>
     <mergeCell ref="A8:A9"/>
     <mergeCell ref="B10:B12"/>
     <mergeCell ref="H1:H2"/>
-    <mergeCell ref="B22:B26"/>
+    <mergeCell ref="B31:B35"/>
     <mergeCell ref="A1:A2"/>
-    <mergeCell ref="A20:A21"/>
+    <mergeCell ref="A20:A30"/>
     <mergeCell ref="C1:C2"/>
     <mergeCell ref="G1:G2"/>
     <mergeCell ref="B1:B2"/>
     <mergeCell ref="B8:B9"/>
-    <mergeCell ref="B20:B21"/>
-    <mergeCell ref="B27:B28"/>
-    <mergeCell ref="A10:A12"/>
-    <mergeCell ref="B5:B6"/>
-    <mergeCell ref="A5:A6"/>
-    <mergeCell ref="A17:A19"/>
-    <mergeCell ref="A22:A26"/>
-    <mergeCell ref="A29:A35"/>
-    <mergeCell ref="B13:B16"/>
-    <mergeCell ref="B17:B19"/>
-    <mergeCell ref="B29:B35"/>
+    <mergeCell ref="B20:B30"/>
+    <mergeCell ref="B36:B37"/>
   </mergeCells>
   <phoneticPr fontId="6" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
partial save for user stories WIP
</commit_message>
<xml_diff>
--- a/Soubhanik/checkupp_product_backlog_final.xlsx
+++ b/Soubhanik/checkupp_product_backlog_final.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30131"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Checkupp\CheckUpp\Soubhanik\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Anodiam\2026\CheckUpp_Parent\CheckUpp\Soubhanik\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B421AD34-2558-489C-B84F-60DF859C85DF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E3EDB0C3-02C7-43A0-8C41-F3EFE5342C94}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -125,12 +125,36 @@
         </r>
       </text>
     </comment>
+    <comment ref="E20" authorId="0" shapeId="0" xr:uid="{3CA1A3BC-210A-4820-BB92-615ED01D6D27}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Anirban:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+Invalid User Story: This is not an action by the user.</t>
+        </r>
+      </text>
+    </comment>
   </commentList>
 </comments>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="266" uniqueCount="183">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="271" uniqueCount="188">
   <si>
     <t>Epic #</t>
   </si>
@@ -289,9 +313,6 @@
     <t>1. Book Appointment screen must be accessible after selecting 'No' on a health check
 2. Integration with HotDocs API via Railway must be in place
 3. Booking confirmation must be displayed on success</t>
-  </si>
-  <si>
-    <t>Mental Health Check</t>
   </si>
   <si>
     <t>complete the K-10 and DASS-21 mental health assessments</t>
@@ -737,6 +758,28 @@
     <t>1. App must display a success message after syncing
 2. User must be able to view the calendar event
 3. Appointment must exist in the selected calendar</t>
+  </si>
+  <si>
+    <t>logged in user navigating the Mental Health Assessment screen</t>
+  </si>
+  <si>
+    <t>Mental Health Assessment</t>
+  </si>
+  <si>
+    <t>have the data I enter in the available fields(K-10 score, DASS-21 Depression, DASS-21 Anxiety, etc) or used the toggle switches (difficulty falling asleep and frequent night waking) autosaved in the system if I tap the 'Back' button or close/remove the app from the background</t>
+  </si>
+  <si>
+    <t>I don't have to re-enter the data in the fields(K-10 score, DASS-21 Depression, DASS-21 Anxiety, etc.) or re-toggle the switches (difficulty falling asleep and frequent night waking) again</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. All entered assessment field values (e.g., K-10 score, DASS-21 Depression, DASS-21 Anxiety) must be automatically saved whenever the user enters or updates them.
+2. All toggle switch states (e.g., Difficulty Falling Asleep, Frequent Night Waking) must be automatically saved whenever they are changed.
+3. All autosaved assessment data must be restored when the user returns to the Mental Health Assessment screen after tapping the Back button.
+4. All autosaved assessment data must be restored when the user reopens the app after it has been closed or removed from the background.
+</t>
+  </si>
+  <si>
+    <t>5. The most recent changes made to all assessment fields and toggle switches must be displayed when the assessment is resumed, without requiring the user to re-enter the information.</t>
   </si>
 </sst>
 </file>
@@ -1051,7 +1094,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="79">
+  <cellXfs count="82">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1146,9 +1189,6 @@
     <xf numFmtId="0" fontId="5" fillId="10" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="12" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="13" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
@@ -1208,6 +1248,41 @@
     </xf>
     <xf numFmtId="0" fontId="11" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="16" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="16" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="16" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="9" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="15" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="15" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="13" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1222,64 +1297,41 @@
     <xf numFmtId="0" fontId="4" fillId="14" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="9" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="8" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="13" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="12" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="12" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="15" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="15" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="10" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="16" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="16" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="16" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="12" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="12" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="12" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="12" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="4" fillId="10" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="10" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="10" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="10" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1562,51 +1614,51 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:L59"/>
-  <sheetFormatPr defaultColWidth="8.90625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:L61"/>
+  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="5.90625" style="2" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="32.90625" style="2" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="11.08984375" style="2" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="20.90625" style="3" customWidth="1"/>
+    <col min="1" max="1" width="5.88671875" style="2" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="32.88671875" style="2" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="11.109375" style="2" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="20.88671875" style="3" customWidth="1"/>
     <col min="5" max="5" width="65" style="2" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="41" style="3" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="52" style="3" customWidth="1"/>
-    <col min="8" max="8" width="11.6328125" style="2" customWidth="1"/>
-    <col min="9" max="9" width="15.36328125" style="3" customWidth="1"/>
-    <col min="10" max="12" width="8.90625" style="5" customWidth="1"/>
-    <col min="13" max="16384" width="8.90625" style="5"/>
+    <col min="7" max="7" width="61.44140625" style="3" customWidth="1"/>
+    <col min="8" max="8" width="11.6640625" style="2" customWidth="1"/>
+    <col min="9" max="9" width="15.33203125" style="3" customWidth="1"/>
+    <col min="10" max="12" width="8.88671875" style="5" customWidth="1"/>
+    <col min="13" max="16384" width="8.88671875" style="5"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="39.65" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="64" t="s">
+    <row r="1" spans="1:9" ht="39.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="71" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="53" t="s">
+      <c r="B1" s="65" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="53" t="s">
+      <c r="C1" s="65" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="53" t="s">
+      <c r="D1" s="65" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="55"/>
-      <c r="F1" s="56"/>
-      <c r="G1" s="66" t="s">
+      <c r="E1" s="67"/>
+      <c r="F1" s="68"/>
+      <c r="G1" s="74" t="s">
         <v>4</v>
       </c>
-      <c r="H1" s="53" t="s">
+      <c r="H1" s="65" t="s">
         <v>5</v>
       </c>
-      <c r="I1" s="53" t="s">
+      <c r="I1" s="65" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A2" s="58"/>
-      <c r="B2" s="54"/>
-      <c r="C2" s="54"/>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A2" s="60"/>
+      <c r="B2" s="66"/>
+      <c r="C2" s="66"/>
       <c r="D2" s="1" t="s">
         <v>7</v>
       </c>
@@ -1616,188 +1668,188 @@
       <c r="F2" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="G2" s="67"/>
-      <c r="H2" s="54"/>
-      <c r="I2" s="54"/>
-    </row>
-    <row r="3" spans="1:9" s="8" customFormat="1" ht="78" x14ac:dyDescent="0.35">
-      <c r="A3" s="37" t="s">
-        <v>142</v>
-      </c>
-      <c r="B3" s="37" t="s">
-        <v>126</v>
+      <c r="G2" s="75"/>
+      <c r="H2" s="66"/>
+      <c r="I2" s="66"/>
+    </row>
+    <row r="3" spans="1:9" s="8" customFormat="1" ht="82.8" x14ac:dyDescent="0.3">
+      <c r="A3" s="36" t="s">
+        <v>141</v>
+      </c>
+      <c r="B3" s="36" t="s">
+        <v>125</v>
       </c>
       <c r="C3" s="22">
         <v>13.2</v>
       </c>
-      <c r="D3" s="38" t="s">
+      <c r="D3" s="37" t="s">
+        <v>126</v>
+      </c>
+      <c r="E3" s="37" t="s">
         <v>127</v>
       </c>
-      <c r="E3" s="38" t="s">
+      <c r="F3" s="37" t="s">
         <v>128</v>
       </c>
-      <c r="F3" s="38" t="s">
+      <c r="G3" s="38" t="s">
+        <v>131</v>
+      </c>
+      <c r="H3" s="22" t="s">
+        <v>60</v>
+      </c>
+      <c r="I3" s="37" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" s="8" customFormat="1" ht="55.2" x14ac:dyDescent="0.3">
+      <c r="A4" s="46">
+        <v>1</v>
+      </c>
+      <c r="B4" s="46" t="s">
+        <v>10</v>
+      </c>
+      <c r="C4" s="47">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="D4" s="48" t="s">
+        <v>11</v>
+      </c>
+      <c r="E4" s="48" t="s">
+        <v>103</v>
+      </c>
+      <c r="F4" s="48" t="s">
+        <v>104</v>
+      </c>
+      <c r="G4" s="49" t="s">
+        <v>105</v>
+      </c>
+      <c r="H4" s="47" t="s">
+        <v>12</v>
+      </c>
+      <c r="I4" s="48" t="s">
         <v>129</v>
       </c>
-      <c r="G3" s="39" t="s">
-        <v>132</v>
-      </c>
-      <c r="H3" s="22" t="s">
-        <v>61</v>
-      </c>
-      <c r="I3" s="38" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="4" spans="1:9" s="8" customFormat="1" ht="52" x14ac:dyDescent="0.35">
-      <c r="A4" s="47">
-        <v>1</v>
-      </c>
-      <c r="B4" s="47" t="s">
-        <v>10</v>
-      </c>
-      <c r="C4" s="48">
-        <v>1.1000000000000001</v>
-      </c>
-      <c r="D4" s="49" t="s">
+    </row>
+    <row r="5" spans="1:9" s="35" customFormat="1" ht="82.8" x14ac:dyDescent="0.3">
+      <c r="A5" s="62">
+        <v>3</v>
+      </c>
+      <c r="B5" s="62" t="s">
+        <v>13</v>
+      </c>
+      <c r="C5" s="34">
+        <v>3.1</v>
+      </c>
+      <c r="D5" s="39" t="s">
         <v>11</v>
       </c>
-      <c r="E4" s="49" t="s">
-        <v>104</v>
-      </c>
-      <c r="F4" s="49" t="s">
-        <v>105</v>
-      </c>
-      <c r="G4" s="50" t="s">
+      <c r="E5" s="40" t="s">
         <v>106</v>
       </c>
-      <c r="H4" s="48" t="s">
-        <v>12</v>
-      </c>
-      <c r="I4" s="49" t="s">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="5" spans="1:9" s="36" customFormat="1" ht="78" x14ac:dyDescent="0.35">
-      <c r="A5" s="68">
-        <v>3</v>
-      </c>
-      <c r="B5" s="68" t="s">
-        <v>13</v>
-      </c>
-      <c r="C5" s="35">
-        <v>3.1</v>
-      </c>
-      <c r="D5" s="40" t="s">
+      <c r="F5" s="40" t="s">
+        <v>107</v>
+      </c>
+      <c r="G5" s="41" t="s">
+        <v>110</v>
+      </c>
+      <c r="H5" s="42" t="s">
+        <v>97</v>
+      </c>
+      <c r="I5" s="39" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" s="8" customFormat="1" ht="82.8" x14ac:dyDescent="0.3">
+      <c r="A6" s="63"/>
+      <c r="B6" s="63"/>
+      <c r="C6" s="34">
+        <v>3.2</v>
+      </c>
+      <c r="D6" s="39" t="s">
         <v>11</v>
       </c>
-      <c r="E5" s="41" t="s">
-        <v>107</v>
-      </c>
-      <c r="F5" s="41" t="s">
+      <c r="E6" s="40" t="s">
         <v>108</v>
       </c>
-      <c r="G5" s="42" t="s">
+      <c r="F6" s="40" t="s">
+        <v>109</v>
+      </c>
+      <c r="G6" s="41" t="s">
         <v>111</v>
       </c>
-      <c r="H5" s="43" t="s">
-        <v>98</v>
-      </c>
-      <c r="I5" s="40" t="s">
+      <c r="H6" s="34" t="s">
+        <v>97</v>
+      </c>
+      <c r="I6" s="39" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="6" spans="1:9" s="8" customFormat="1" ht="78" x14ac:dyDescent="0.35">
-      <c r="A6" s="69"/>
-      <c r="B6" s="69"/>
-      <c r="C6" s="35">
-        <v>3.2</v>
-      </c>
-      <c r="D6" s="40" t="s">
-        <v>11</v>
-      </c>
-      <c r="E6" s="41" t="s">
-        <v>109</v>
-      </c>
-      <c r="F6" s="41" t="s">
-        <v>110</v>
-      </c>
-      <c r="G6" s="42" t="s">
-        <v>112</v>
-      </c>
-      <c r="H6" s="35" t="s">
-        <v>98</v>
-      </c>
-      <c r="I6" s="40" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="7" spans="1:9" s="8" customFormat="1" ht="117" x14ac:dyDescent="0.35">
-      <c r="A7" s="46">
+    <row r="7" spans="1:9" s="8" customFormat="1" ht="138" x14ac:dyDescent="0.3">
+      <c r="A7" s="45">
         <v>5</v>
       </c>
-      <c r="B7" s="46" t="s">
+      <c r="B7" s="45" t="s">
         <v>16</v>
       </c>
       <c r="C7" s="9">
         <v>5.2</v>
       </c>
       <c r="D7" s="10" t="s">
+        <v>133</v>
+      </c>
+      <c r="E7" s="10" t="s">
+        <v>135</v>
+      </c>
+      <c r="F7" s="10" t="s">
         <v>134</v>
       </c>
-      <c r="E7" s="10" t="s">
+      <c r="G7" s="27" t="s">
         <v>136</v>
       </c>
-      <c r="F7" s="10" t="s">
-        <v>135</v>
-      </c>
-      <c r="G7" s="27" t="s">
-        <v>137</v>
-      </c>
       <c r="H7" s="11" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="I7" s="10" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="8" spans="1:9" s="8" customFormat="1" ht="26" x14ac:dyDescent="0.35">
-      <c r="A8" s="61">
+    <row r="8" spans="1:9" s="8" customFormat="1" ht="27.6" x14ac:dyDescent="0.3">
+      <c r="A8" s="70">
         <v>6</v>
       </c>
-      <c r="B8" s="61" t="s">
+      <c r="B8" s="70" t="s">
         <v>18</v>
       </c>
       <c r="C8" s="12">
         <v>6.1</v>
       </c>
       <c r="D8" s="13" t="s">
-        <v>127</v>
-      </c>
-      <c r="E8" s="51" t="s">
+        <v>126</v>
+      </c>
+      <c r="E8" s="50" t="s">
+        <v>137</v>
+      </c>
+      <c r="F8" s="50" t="s">
         <v>138</v>
       </c>
-      <c r="F8" s="51" t="s">
+      <c r="G8" s="51" t="s">
         <v>139</v>
       </c>
-      <c r="G8" s="52" t="s">
-        <v>140</v>
-      </c>
       <c r="H8" s="14" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="I8" s="13" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="9" spans="1:9" s="8" customFormat="1" ht="52" x14ac:dyDescent="0.35">
-      <c r="A9" s="58"/>
-      <c r="B9" s="58"/>
+    <row r="9" spans="1:9" s="8" customFormat="1" ht="55.2" x14ac:dyDescent="0.3">
+      <c r="A9" s="60"/>
+      <c r="B9" s="60"/>
       <c r="C9" s="12">
         <v>6.3</v>
       </c>
       <c r="D9" s="13" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="E9" s="13" t="s">
         <v>20</v>
@@ -1806,25 +1858,25 @@
         <v>21</v>
       </c>
       <c r="G9" s="28" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="H9" s="12" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="I9" s="13"/>
     </row>
-    <row r="10" spans="1:9" s="8" customFormat="1" ht="52" x14ac:dyDescent="0.35">
-      <c r="A10" s="62">
+    <row r="10" spans="1:9" s="8" customFormat="1" ht="55.2" x14ac:dyDescent="0.3">
+      <c r="A10" s="61">
         <v>7</v>
       </c>
-      <c r="B10" s="62" t="s">
+      <c r="B10" s="61" t="s">
         <v>22</v>
       </c>
       <c r="C10" s="15">
         <v>7.1</v>
       </c>
       <c r="D10" s="16" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="E10" s="16" t="s">
         <v>23</v>
@@ -1836,20 +1888,20 @@
         <v>25</v>
       </c>
       <c r="H10" s="17" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="I10" s="16" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="11" spans="1:9" s="8" customFormat="1" ht="52" x14ac:dyDescent="0.35">
-      <c r="A11" s="60"/>
-      <c r="B11" s="60"/>
+    <row r="11" spans="1:9" s="8" customFormat="1" ht="55.2" x14ac:dyDescent="0.3">
+      <c r="A11" s="58"/>
+      <c r="B11" s="58"/>
       <c r="C11" s="15">
         <v>7.2</v>
       </c>
       <c r="D11" s="16" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="E11" s="16" t="s">
         <v>27</v>
@@ -1861,20 +1913,20 @@
         <v>29</v>
       </c>
       <c r="H11" s="15" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="I11" s="16" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="12" spans="1:9" s="8" customFormat="1" ht="39" x14ac:dyDescent="0.35">
-      <c r="A12" s="58"/>
-      <c r="B12" s="58"/>
+    <row r="12" spans="1:9" s="8" customFormat="1" ht="41.4" x14ac:dyDescent="0.3">
+      <c r="A12" s="60"/>
+      <c r="B12" s="60"/>
       <c r="C12" s="15">
         <v>7.3</v>
       </c>
       <c r="D12" s="16" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="E12" s="16" t="s">
         <v>30</v>
@@ -1886,11 +1938,11 @@
         <v>32</v>
       </c>
       <c r="H12" s="15" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="I12" s="16"/>
     </row>
-    <row r="13" spans="1:9" s="8" customFormat="1" ht="82.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:9" s="8" customFormat="1" ht="27.6" x14ac:dyDescent="0.3">
       <c r="A13" s="59">
         <v>9</v>
       </c>
@@ -1915,9 +1967,9 @@
       <c r="H13" s="18"/>
       <c r="I13" s="19"/>
     </row>
-    <row r="14" spans="1:9" s="8" customFormat="1" ht="41.4" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A14" s="60"/>
-      <c r="B14" s="60"/>
+    <row r="14" spans="1:9" s="8" customFormat="1" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A14" s="58"/>
+      <c r="B14" s="58"/>
       <c r="C14" s="18">
         <v>9.1999999999999993</v>
       </c>
@@ -1936,9 +1988,9 @@
       <c r="H14" s="18"/>
       <c r="I14" s="19"/>
     </row>
-    <row r="15" spans="1:9" s="8" customFormat="1" ht="27.65" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A15" s="60"/>
-      <c r="B15" s="60"/>
+    <row r="15" spans="1:9" s="8" customFormat="1" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A15" s="58"/>
+      <c r="B15" s="58"/>
       <c r="C15" s="18">
         <v>9.3000000000000007</v>
       </c>
@@ -1959,9 +2011,9 @@
         <v>45</v>
       </c>
     </row>
-    <row r="16" spans="1:9" s="8" customFormat="1" ht="41.4" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A16" s="58"/>
-      <c r="B16" s="58"/>
+    <row r="16" spans="1:9" s="8" customFormat="1" ht="55.2" x14ac:dyDescent="0.3">
+      <c r="A16" s="60"/>
+      <c r="B16" s="60"/>
       <c r="C16" s="18">
         <v>9.4</v>
       </c>
@@ -1982,878 +2034,912 @@
         <v>45</v>
       </c>
     </row>
-    <row r="17" spans="1:9" s="8" customFormat="1" ht="41.4" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A17" s="70">
+    <row r="17" spans="1:9" s="8" customFormat="1" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A17" s="78">
         <v>12</v>
       </c>
-      <c r="B17" s="70" t="s">
-        <v>49</v>
+      <c r="B17" s="78" t="s">
+        <v>183</v>
       </c>
       <c r="C17" s="20">
         <v>12.1</v>
       </c>
       <c r="D17" s="21" t="s">
-        <v>15</v>
+        <v>126</v>
       </c>
       <c r="E17" s="21" t="s">
+        <v>49</v>
+      </c>
+      <c r="F17" s="21" t="s">
         <v>50</v>
       </c>
-      <c r="F17" s="21" t="s">
+      <c r="G17" s="31" t="s">
         <v>51</v>
       </c>
-      <c r="G17" s="31" t="s">
+      <c r="H17" s="20" t="s">
         <v>52</v>
       </c>
-      <c r="H17" s="20" t="s">
+      <c r="I17" s="21" t="s">
         <v>53</v>
       </c>
-      <c r="I17" s="21" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="18" spans="1:9" s="8" customFormat="1" ht="55.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A18" s="60"/>
-      <c r="B18" s="60"/>
+    </row>
+    <row r="18" spans="1:9" s="8" customFormat="1" ht="55.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A18" s="79"/>
+      <c r="B18" s="79"/>
       <c r="C18" s="20">
         <v>12.2</v>
       </c>
       <c r="D18" s="21" t="s">
-        <v>15</v>
+        <v>126</v>
       </c>
       <c r="E18" s="21" t="s">
+        <v>54</v>
+      </c>
+      <c r="F18" s="21" t="s">
         <v>55</v>
       </c>
-      <c r="F18" s="21" t="s">
+      <c r="G18" s="31" t="s">
         <v>56</v>
       </c>
-      <c r="G18" s="31" t="s">
-        <v>57</v>
-      </c>
       <c r="H18" s="20" t="s">
+        <v>52</v>
+      </c>
+      <c r="I18" s="21" t="s">
         <v>53</v>
       </c>
-      <c r="I18" s="21" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="19" spans="1:9" s="8" customFormat="1" ht="55.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A19" s="58"/>
-      <c r="B19" s="58"/>
+    </row>
+    <row r="19" spans="1:9" s="8" customFormat="1" ht="55.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A19" s="79"/>
+      <c r="B19" s="79"/>
       <c r="C19" s="20">
         <v>12.3</v>
       </c>
       <c r="D19" s="21" t="s">
+        <v>126</v>
+      </c>
+      <c r="E19" s="21" t="s">
+        <v>57</v>
+      </c>
+      <c r="F19" s="21" t="s">
+        <v>58</v>
+      </c>
+      <c r="G19" s="31" t="s">
+        <v>59</v>
+      </c>
+      <c r="H19" s="20" t="s">
+        <v>52</v>
+      </c>
+      <c r="I19" s="21"/>
+    </row>
+    <row r="20" spans="1:9" s="8" customFormat="1" ht="138" x14ac:dyDescent="0.3">
+      <c r="A20" s="80"/>
+      <c r="B20" s="80"/>
+      <c r="C20" s="20">
+        <v>12.4</v>
+      </c>
+      <c r="D20" s="21" t="s">
+        <v>182</v>
+      </c>
+      <c r="E20" s="21" t="s">
+        <v>184</v>
+      </c>
+      <c r="F20" s="21" t="s">
+        <v>185</v>
+      </c>
+      <c r="G20" s="21" t="s">
+        <v>186</v>
+      </c>
+      <c r="H20" s="20"/>
+      <c r="I20" s="21"/>
+    </row>
+    <row r="21" spans="1:9" s="8" customFormat="1" ht="41.4" x14ac:dyDescent="0.3">
+      <c r="A21" s="81"/>
+      <c r="B21" s="81"/>
+      <c r="C21" s="20"/>
+      <c r="D21" s="21"/>
+      <c r="E21" s="21"/>
+      <c r="F21" s="21"/>
+      <c r="G21" s="31" t="s">
+        <v>187</v>
+      </c>
+      <c r="H21" s="20"/>
+      <c r="I21" s="21"/>
+    </row>
+    <row r="22" spans="1:9" s="8" customFormat="1" ht="41.4" x14ac:dyDescent="0.3">
+      <c r="A22" s="72">
+        <v>14</v>
+      </c>
+      <c r="B22" s="72" t="s">
+        <v>61</v>
+      </c>
+      <c r="C22" s="76">
+        <v>14.1</v>
+      </c>
+      <c r="D22" s="77" t="s">
         <v>15</v>
       </c>
-      <c r="E19" s="21" t="s">
-        <v>58</v>
-      </c>
-      <c r="F19" s="21" t="s">
-        <v>59</v>
-      </c>
-      <c r="G19" s="31" t="s">
-        <v>60</v>
-      </c>
-      <c r="H19" s="20" t="s">
-        <v>53</v>
-      </c>
-      <c r="I19" s="21"/>
-    </row>
-    <row r="20" spans="1:9" s="8" customFormat="1" ht="55" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A20" s="65">
-        <v>14</v>
-      </c>
-      <c r="B20" s="65" t="s">
+      <c r="E22" s="77" t="s">
+        <v>146</v>
+      </c>
+      <c r="F22" s="77" t="s">
+        <v>147</v>
+      </c>
+      <c r="G22" s="77" t="s">
+        <v>171</v>
+      </c>
+      <c r="H22" s="76" t="s">
+        <v>102</v>
+      </c>
+      <c r="I22" s="77" t="s">
         <v>62</v>
       </c>
-      <c r="C20" s="76">
+    </row>
+    <row r="23" spans="1:9" s="8" customFormat="1" ht="55.2" x14ac:dyDescent="0.3">
+      <c r="A23" s="73"/>
+      <c r="B23" s="73"/>
+      <c r="C23" s="76">
+        <v>14.2</v>
+      </c>
+      <c r="D23" s="77" t="s">
+        <v>15</v>
+      </c>
+      <c r="E23" s="77" t="s">
+        <v>148</v>
+      </c>
+      <c r="F23" s="77" t="s">
+        <v>149</v>
+      </c>
+      <c r="G23" s="77" t="s">
+        <v>172</v>
+      </c>
+      <c r="H23" s="76" t="s">
+        <v>102</v>
+      </c>
+      <c r="I23" s="77" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="24" spans="1:9" s="8" customFormat="1" ht="55.2" x14ac:dyDescent="0.3">
+      <c r="A24" s="73"/>
+      <c r="B24" s="73"/>
+      <c r="C24" s="76">
+        <v>14.3</v>
+      </c>
+      <c r="D24" s="77" t="s">
+        <v>150</v>
+      </c>
+      <c r="E24" s="77" t="s">
+        <v>151</v>
+      </c>
+      <c r="F24" s="77" t="s">
+        <v>152</v>
+      </c>
+      <c r="G24" s="77" t="s">
+        <v>173</v>
+      </c>
+      <c r="H24" s="76" t="s">
+        <v>102</v>
+      </c>
+      <c r="I24" s="77" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="25" spans="1:9" s="8" customFormat="1" ht="55.2" x14ac:dyDescent="0.3">
+      <c r="A25" s="73"/>
+      <c r="B25" s="73"/>
+      <c r="C25" s="76">
+        <v>14.4</v>
+      </c>
+      <c r="D25" s="77" t="s">
+        <v>15</v>
+      </c>
+      <c r="E25" s="77" t="s">
+        <v>153</v>
+      </c>
+      <c r="F25" s="77" t="s">
+        <v>154</v>
+      </c>
+      <c r="G25" s="77" t="s">
+        <v>174</v>
+      </c>
+      <c r="H25" s="76" t="s">
+        <v>102</v>
+      </c>
+      <c r="I25" s="77" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="26" spans="1:9" s="8" customFormat="1" ht="55.2" x14ac:dyDescent="0.3">
+      <c r="A26" s="73"/>
+      <c r="B26" s="73"/>
+      <c r="C26" s="76">
+        <v>14.5</v>
+      </c>
+      <c r="D26" s="77" t="s">
+        <v>15</v>
+      </c>
+      <c r="E26" s="77" t="s">
+        <v>155</v>
+      </c>
+      <c r="F26" s="77" t="s">
+        <v>156</v>
+      </c>
+      <c r="G26" s="77" t="s">
+        <v>175</v>
+      </c>
+      <c r="H26" s="76" t="s">
+        <v>102</v>
+      </c>
+      <c r="I26" s="77" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="27" spans="1:9" s="8" customFormat="1" ht="41.4" x14ac:dyDescent="0.3">
+      <c r="A27" s="73"/>
+      <c r="B27" s="73"/>
+      <c r="C27" s="76">
+        <v>14.6</v>
+      </c>
+      <c r="D27" s="77" t="s">
+        <v>15</v>
+      </c>
+      <c r="E27" s="77" t="s">
+        <v>157</v>
+      </c>
+      <c r="F27" s="77" t="s">
+        <v>158</v>
+      </c>
+      <c r="G27" s="77" t="s">
+        <v>181</v>
+      </c>
+      <c r="H27" s="76" t="s">
+        <v>102</v>
+      </c>
+      <c r="I27" s="77" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="28" spans="1:9" s="8" customFormat="1" ht="69" x14ac:dyDescent="0.3">
+      <c r="A28" s="73"/>
+      <c r="B28" s="73"/>
+      <c r="C28" s="76">
+        <v>14.7</v>
+      </c>
+      <c r="D28" s="77" t="s">
+        <v>15</v>
+      </c>
+      <c r="E28" s="77" t="s">
+        <v>159</v>
+      </c>
+      <c r="F28" s="77" t="s">
+        <v>160</v>
+      </c>
+      <c r="G28" s="77" t="s">
+        <v>176</v>
+      </c>
+      <c r="H28" s="76" t="s">
+        <v>102</v>
+      </c>
+      <c r="I28" s="77" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="29" spans="1:9" s="8" customFormat="1" ht="55.2" x14ac:dyDescent="0.3">
+      <c r="A29" s="73"/>
+      <c r="B29" s="73"/>
+      <c r="C29" s="76">
+        <v>14.8</v>
+      </c>
+      <c r="D29" s="77" t="s">
+        <v>15</v>
+      </c>
+      <c r="E29" s="77" t="s">
+        <v>161</v>
+      </c>
+      <c r="F29" s="77" t="s">
+        <v>162</v>
+      </c>
+      <c r="G29" s="77" t="s">
+        <v>177</v>
+      </c>
+      <c r="H29" s="76" t="s">
+        <v>142</v>
+      </c>
+      <c r="I29" s="77" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="30" spans="1:9" s="8" customFormat="1" ht="55.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A30" s="73"/>
+      <c r="B30" s="73"/>
+      <c r="C30" s="76">
+        <v>14.9</v>
+      </c>
+      <c r="D30" s="77" t="s">
+        <v>15</v>
+      </c>
+      <c r="E30" s="77" t="s">
+        <v>163</v>
+      </c>
+      <c r="F30" s="77" t="s">
+        <v>164</v>
+      </c>
+      <c r="G30" s="77" t="s">
+        <v>178</v>
+      </c>
+      <c r="H30" s="76" t="s">
+        <v>142</v>
+      </c>
+      <c r="I30" s="77" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="31" spans="1:9" s="8" customFormat="1" ht="69" x14ac:dyDescent="0.3">
+      <c r="A31" s="73"/>
+      <c r="B31" s="73"/>
+      <c r="C31" s="76">
         <v>14.1</v>
       </c>
-      <c r="D20" s="32" t="s">
+      <c r="D31" s="77" t="s">
         <v>15</v>
       </c>
-      <c r="E20" s="32" t="s">
-        <v>147</v>
-      </c>
-      <c r="F20" s="32" t="s">
-        <v>148</v>
-      </c>
-      <c r="G20" s="32" t="s">
-        <v>172</v>
-      </c>
-      <c r="H20" s="76" t="s">
-        <v>103</v>
-      </c>
-      <c r="I20" s="32" t="s">
+      <c r="E31" s="77" t="s">
+        <v>165</v>
+      </c>
+      <c r="F31" s="77" t="s">
+        <v>166</v>
+      </c>
+      <c r="G31" s="77" t="s">
+        <v>179</v>
+      </c>
+      <c r="H31" s="76" t="s">
+        <v>142</v>
+      </c>
+      <c r="I31" s="77" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="32" spans="1:9" s="8" customFormat="1" ht="41.4" x14ac:dyDescent="0.3">
+      <c r="A32" s="73"/>
+      <c r="B32" s="73"/>
+      <c r="C32" s="76">
+        <v>14.11</v>
+      </c>
+      <c r="D32" s="77" t="s">
+        <v>15</v>
+      </c>
+      <c r="E32" s="77" t="s">
+        <v>167</v>
+      </c>
+      <c r="F32" s="77" t="s">
+        <v>168</v>
+      </c>
+      <c r="G32" s="77" t="s">
+        <v>180</v>
+      </c>
+      <c r="H32" s="76" t="s">
+        <v>142</v>
+      </c>
+      <c r="I32" s="77" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="33" spans="1:9" s="8" customFormat="1" ht="27.6" x14ac:dyDescent="0.3">
+      <c r="A33" s="64">
+        <v>15</v>
+      </c>
+      <c r="B33" s="64" t="s">
         <v>63</v>
       </c>
-    </row>
-    <row r="21" spans="1:9" s="8" customFormat="1" ht="55" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A21" s="75"/>
-      <c r="B21" s="75"/>
-      <c r="C21" s="76">
-        <v>14.2</v>
-      </c>
-      <c r="D21" s="32" t="s">
-        <v>15</v>
-      </c>
-      <c r="E21" s="32" t="s">
-        <v>149</v>
-      </c>
-      <c r="F21" s="32" t="s">
-        <v>150</v>
-      </c>
-      <c r="G21" s="32" t="s">
-        <v>173</v>
-      </c>
-      <c r="H21" s="76" t="s">
-        <v>103</v>
-      </c>
-      <c r="I21" s="32" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="22" spans="1:9" s="8" customFormat="1" ht="55" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A22" s="75"/>
-      <c r="B22" s="75"/>
-      <c r="C22" s="76">
-        <v>14.3</v>
-      </c>
-      <c r="D22" s="32" t="s">
-        <v>151</v>
-      </c>
-      <c r="E22" s="32" t="s">
-        <v>152</v>
-      </c>
-      <c r="F22" s="32" t="s">
-        <v>153</v>
-      </c>
-      <c r="G22" s="32" t="s">
-        <v>174</v>
-      </c>
-      <c r="H22" s="76" t="s">
-        <v>103</v>
-      </c>
-      <c r="I22" s="32" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="23" spans="1:9" s="8" customFormat="1" ht="55" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A23" s="75"/>
-      <c r="B23" s="75"/>
-      <c r="C23" s="76">
-        <v>14.4</v>
-      </c>
-      <c r="D23" s="32" t="s">
-        <v>15</v>
-      </c>
-      <c r="E23" s="32" t="s">
-        <v>154</v>
-      </c>
-      <c r="F23" s="32" t="s">
-        <v>155</v>
-      </c>
-      <c r="G23" s="32" t="s">
-        <v>175</v>
-      </c>
-      <c r="H23" s="76" t="s">
-        <v>103</v>
-      </c>
-      <c r="I23" s="32" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="24" spans="1:9" s="8" customFormat="1" ht="55" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A24" s="75"/>
-      <c r="B24" s="75"/>
-      <c r="C24" s="76">
-        <v>14.5</v>
-      </c>
-      <c r="D24" s="32" t="s">
-        <v>15</v>
-      </c>
-      <c r="E24" s="32" t="s">
-        <v>156</v>
-      </c>
-      <c r="F24" s="32" t="s">
-        <v>157</v>
-      </c>
-      <c r="G24" s="32" t="s">
-        <v>176</v>
-      </c>
-      <c r="H24" s="76" t="s">
-        <v>103</v>
-      </c>
-      <c r="I24" s="32" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="25" spans="1:9" s="8" customFormat="1" ht="55" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A25" s="75"/>
-      <c r="B25" s="75"/>
-      <c r="C25" s="76">
-        <v>14.6</v>
-      </c>
-      <c r="D25" s="32" t="s">
-        <v>15</v>
-      </c>
-      <c r="E25" s="32" t="s">
-        <v>158</v>
-      </c>
-      <c r="F25" s="32" t="s">
-        <v>159</v>
-      </c>
-      <c r="G25" s="32" t="s">
-        <v>182</v>
-      </c>
-      <c r="H25" s="76" t="s">
-        <v>103</v>
-      </c>
-      <c r="I25" s="32" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="26" spans="1:9" s="8" customFormat="1" ht="55" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A26" s="75"/>
-      <c r="B26" s="75"/>
-      <c r="C26" s="76">
-        <v>14.7</v>
-      </c>
-      <c r="D26" s="32" t="s">
-        <v>15</v>
-      </c>
-      <c r="E26" s="32" t="s">
-        <v>160</v>
-      </c>
-      <c r="F26" s="32" t="s">
-        <v>161</v>
-      </c>
-      <c r="G26" s="32" t="s">
-        <v>177</v>
-      </c>
-      <c r="H26" s="76" t="s">
-        <v>103</v>
-      </c>
-      <c r="I26" s="32" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="27" spans="1:9" s="8" customFormat="1" ht="55" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A27" s="75"/>
-      <c r="B27" s="75"/>
-      <c r="C27" s="76">
-        <v>14.8</v>
-      </c>
-      <c r="D27" s="32" t="s">
-        <v>15</v>
-      </c>
-      <c r="E27" s="32" t="s">
-        <v>162</v>
-      </c>
-      <c r="F27" s="32" t="s">
-        <v>163</v>
-      </c>
-      <c r="G27" s="32" t="s">
-        <v>178</v>
-      </c>
-      <c r="H27" s="76" t="s">
+      <c r="C33" s="23">
+        <v>15.1</v>
+      </c>
+      <c r="D33" s="24" t="s">
+        <v>64</v>
+      </c>
+      <c r="E33" s="24" t="s">
+        <v>65</v>
+      </c>
+      <c r="F33" s="24" t="s">
+        <v>66</v>
+      </c>
+      <c r="G33" s="32" t="s">
+        <v>67</v>
+      </c>
+      <c r="H33" s="23" t="s">
         <v>143</v>
       </c>
-      <c r="I27" s="32" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="28" spans="1:9" s="8" customFormat="1" ht="55" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A28" s="75"/>
-      <c r="B28" s="75"/>
-      <c r="C28" s="76">
-        <v>14.9</v>
-      </c>
-      <c r="D28" s="32" t="s">
-        <v>15</v>
-      </c>
-      <c r="E28" s="32" t="s">
-        <v>164</v>
-      </c>
-      <c r="F28" s="32" t="s">
-        <v>165</v>
-      </c>
-      <c r="G28" s="32" t="s">
-        <v>179</v>
-      </c>
-      <c r="H28" s="76" t="s">
+      <c r="I33" s="24" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="34" spans="1:9" s="8" customFormat="1" ht="27.6" x14ac:dyDescent="0.3">
+      <c r="A34" s="58"/>
+      <c r="B34" s="58"/>
+      <c r="C34" s="23">
+        <v>15.2</v>
+      </c>
+      <c r="D34" s="24" t="s">
+        <v>64</v>
+      </c>
+      <c r="E34" s="24" t="s">
+        <v>68</v>
+      </c>
+      <c r="F34" s="24" t="s">
+        <v>69</v>
+      </c>
+      <c r="G34" s="32" t="s">
+        <v>70</v>
+      </c>
+      <c r="H34" s="23" t="s">
         <v>143</v>
       </c>
-      <c r="I28" s="32" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="29" spans="1:9" s="8" customFormat="1" ht="55" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A29" s="75"/>
-      <c r="B29" s="75"/>
-      <c r="C29" s="76">
-        <v>14.1</v>
-      </c>
-      <c r="D29" s="32" t="s">
-        <v>15</v>
-      </c>
-      <c r="E29" s="32" t="s">
-        <v>166</v>
-      </c>
-      <c r="F29" s="32" t="s">
-        <v>167</v>
-      </c>
-      <c r="G29" s="32" t="s">
-        <v>180</v>
-      </c>
-      <c r="H29" s="76" t="s">
-        <v>143</v>
-      </c>
-      <c r="I29" s="32" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="30" spans="1:9" s="8" customFormat="1" ht="55" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A30" s="75"/>
-      <c r="B30" s="75"/>
-      <c r="C30" s="76">
-        <v>14.11</v>
-      </c>
-      <c r="D30" s="32" t="s">
-        <v>15</v>
-      </c>
-      <c r="E30" s="32" t="s">
-        <v>168</v>
-      </c>
-      <c r="F30" s="32" t="s">
-        <v>169</v>
-      </c>
-      <c r="G30" s="32" t="s">
-        <v>181</v>
-      </c>
-      <c r="H30" s="76" t="s">
-        <v>143</v>
-      </c>
-      <c r="I30" s="32" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="31" spans="1:9" s="8" customFormat="1" ht="26" x14ac:dyDescent="0.35">
-      <c r="A31" s="63">
-        <v>15</v>
-      </c>
-      <c r="B31" s="63" t="s">
-        <v>64</v>
-      </c>
-      <c r="C31" s="23">
-        <v>15.1</v>
-      </c>
-      <c r="D31" s="24" t="s">
-        <v>65</v>
-      </c>
-      <c r="E31" s="24" t="s">
-        <v>66</v>
-      </c>
-      <c r="F31" s="24" t="s">
-        <v>67</v>
-      </c>
-      <c r="G31" s="33" t="s">
-        <v>68</v>
-      </c>
-      <c r="H31" s="23" t="s">
+      <c r="I34" s="24" t="s">
         <v>144</v>
       </c>
-      <c r="I31" s="24" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="32" spans="1:9" s="8" customFormat="1" ht="26" x14ac:dyDescent="0.35">
-      <c r="A32" s="60"/>
-      <c r="B32" s="60"/>
-      <c r="C32" s="23">
-        <v>15.2</v>
-      </c>
-      <c r="D32" s="24" t="s">
-        <v>65</v>
-      </c>
-      <c r="E32" s="24" t="s">
-        <v>69</v>
-      </c>
-      <c r="F32" s="24" t="s">
-        <v>70</v>
-      </c>
-      <c r="G32" s="33" t="s">
-        <v>71</v>
-      </c>
-      <c r="H32" s="23" t="s">
-        <v>144</v>
-      </c>
-      <c r="I32" s="24" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="33" spans="1:12" s="8" customFormat="1" ht="26" x14ac:dyDescent="0.35">
-      <c r="A33" s="60"/>
-      <c r="B33" s="60"/>
-      <c r="C33" s="23">
-        <v>15.3</v>
-      </c>
-      <c r="D33" s="24" t="s">
-        <v>65</v>
-      </c>
-      <c r="E33" s="24" t="s">
-        <v>72</v>
-      </c>
-      <c r="F33" s="24" t="s">
-        <v>73</v>
-      </c>
-      <c r="G33" s="33" t="s">
-        <v>74</v>
-      </c>
-      <c r="H33" s="23" t="s">
-        <v>144</v>
-      </c>
-      <c r="I33" s="24" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="34" spans="1:12" s="8" customFormat="1" ht="26" x14ac:dyDescent="0.35">
-      <c r="A34" s="60"/>
-      <c r="B34" s="60"/>
-      <c r="C34" s="23">
-        <v>15.4</v>
-      </c>
-      <c r="D34" s="24" t="s">
-        <v>65</v>
-      </c>
-      <c r="E34" s="24" t="s">
-        <v>75</v>
-      </c>
-      <c r="F34" s="24" t="s">
-        <v>76</v>
-      </c>
-      <c r="G34" s="33" t="s">
-        <v>77</v>
-      </c>
-      <c r="H34" s="23" t="s">
-        <v>146</v>
-      </c>
-      <c r="I34" s="24" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="35" spans="1:12" s="8" customFormat="1" ht="26" x14ac:dyDescent="0.35">
+    </row>
+    <row r="35" spans="1:9" s="8" customFormat="1" ht="27.6" x14ac:dyDescent="0.3">
       <c r="A35" s="58"/>
       <c r="B35" s="58"/>
       <c r="C35" s="23">
+        <v>15.3</v>
+      </c>
+      <c r="D35" s="24" t="s">
+        <v>64</v>
+      </c>
+      <c r="E35" s="24" t="s">
+        <v>71</v>
+      </c>
+      <c r="F35" s="24" t="s">
+        <v>72</v>
+      </c>
+      <c r="G35" s="32" t="s">
+        <v>73</v>
+      </c>
+      <c r="H35" s="23" t="s">
+        <v>143</v>
+      </c>
+      <c r="I35" s="24" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="36" spans="1:9" s="8" customFormat="1" ht="27.6" x14ac:dyDescent="0.3">
+      <c r="A36" s="58"/>
+      <c r="B36" s="58"/>
+      <c r="C36" s="23">
+        <v>15.4</v>
+      </c>
+      <c r="D36" s="24" t="s">
+        <v>64</v>
+      </c>
+      <c r="E36" s="24" t="s">
+        <v>74</v>
+      </c>
+      <c r="F36" s="24" t="s">
+        <v>75</v>
+      </c>
+      <c r="G36" s="32" t="s">
+        <v>76</v>
+      </c>
+      <c r="H36" s="23" t="s">
+        <v>145</v>
+      </c>
+      <c r="I36" s="24" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="37" spans="1:9" s="8" customFormat="1" ht="27.6" x14ac:dyDescent="0.3">
+      <c r="A37" s="60"/>
+      <c r="B37" s="60"/>
+      <c r="C37" s="23">
         <v>15.5</v>
       </c>
-      <c r="D35" s="24" t="s">
-        <v>65</v>
-      </c>
-      <c r="E35" s="24" t="s">
+      <c r="D37" s="24" t="s">
+        <v>64</v>
+      </c>
+      <c r="E37" s="24" t="s">
+        <v>77</v>
+      </c>
+      <c r="F37" s="24" t="s">
         <v>78</v>
       </c>
-      <c r="F35" s="24" t="s">
+      <c r="G37" s="32" t="s">
         <v>79</v>
       </c>
-      <c r="G35" s="33" t="s">
+      <c r="H37" s="23" t="s">
+        <v>145</v>
+      </c>
+      <c r="I37" s="24" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="38" spans="1:9" s="8" customFormat="1" ht="27.6" x14ac:dyDescent="0.3">
+      <c r="A38" s="69">
+        <v>16</v>
+      </c>
+      <c r="B38" s="69" t="s">
         <v>80</v>
       </c>
-      <c r="H35" s="23" t="s">
-        <v>146</v>
-      </c>
-      <c r="I35" s="24" t="s">
+      <c r="C38" s="25">
+        <v>16.100000000000001</v>
+      </c>
+      <c r="D38" s="26" t="s">
+        <v>81</v>
+      </c>
+      <c r="E38" s="26" t="s">
+        <v>82</v>
+      </c>
+      <c r="F38" s="26" t="s">
+        <v>83</v>
+      </c>
+      <c r="G38" s="52" t="s">
+        <v>84</v>
+      </c>
+      <c r="H38" s="53" t="s">
         <v>145</v>
       </c>
-    </row>
-    <row r="36" spans="1:12" s="8" customFormat="1" ht="26" x14ac:dyDescent="0.35">
-      <c r="A36" s="57">
-        <v>16</v>
-      </c>
-      <c r="B36" s="57" t="s">
-        <v>81</v>
-      </c>
-      <c r="C36" s="25">
-        <v>16.100000000000001</v>
-      </c>
-      <c r="D36" s="26" t="s">
-        <v>82</v>
-      </c>
-      <c r="E36" s="26" t="s">
-        <v>83</v>
-      </c>
-      <c r="F36" s="26" t="s">
-        <v>84</v>
-      </c>
-      <c r="G36" s="72" t="s">
-        <v>85</v>
-      </c>
-      <c r="H36" s="73" t="s">
-        <v>146</v>
-      </c>
-      <c r="I36" s="74" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="37" spans="1:12" s="8" customFormat="1" ht="26" x14ac:dyDescent="0.35">
-      <c r="A37" s="58"/>
-      <c r="B37" s="58"/>
-      <c r="C37" s="25">
-        <v>16.2</v>
-      </c>
-      <c r="D37" s="26" t="s">
-        <v>86</v>
-      </c>
-      <c r="E37" s="26" t="s">
-        <v>87</v>
-      </c>
-      <c r="F37" s="26" t="s">
-        <v>88</v>
-      </c>
-      <c r="G37" s="34" t="s">
-        <v>89</v>
-      </c>
-      <c r="H37" s="73" t="s">
-        <v>146</v>
-      </c>
-      <c r="I37" s="74" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="38" spans="1:12" s="8" customFormat="1" ht="26" x14ac:dyDescent="0.35">
-      <c r="A38" s="71">
-        <v>17</v>
-      </c>
-      <c r="B38" s="71" t="s">
-        <v>90</v>
-      </c>
-      <c r="C38" s="9">
-        <v>17.100000000000001</v>
-      </c>
-      <c r="D38" s="10" t="s">
-        <v>91</v>
-      </c>
-      <c r="E38" s="44" t="s">
-        <v>170</v>
-      </c>
-      <c r="F38" s="10" t="s">
-        <v>92</v>
-      </c>
-      <c r="G38" s="45" t="s">
-        <v>171</v>
-      </c>
-      <c r="H38" s="9" t="s">
-        <v>103</v>
-      </c>
-      <c r="I38" s="44" t="s">
-        <v>125</v>
-      </c>
-    </row>
-    <row r="39" spans="1:12" s="8" customFormat="1" ht="26" x14ac:dyDescent="0.35">
+      <c r="I38" s="54" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="39" spans="1:9" s="8" customFormat="1" ht="27.6" x14ac:dyDescent="0.3">
       <c r="A39" s="60"/>
       <c r="B39" s="60"/>
-      <c r="C39" s="9">
+      <c r="C39" s="25">
+        <v>16.2</v>
+      </c>
+      <c r="D39" s="26" t="s">
+        <v>85</v>
+      </c>
+      <c r="E39" s="26" t="s">
+        <v>86</v>
+      </c>
+      <c r="F39" s="26" t="s">
+        <v>87</v>
+      </c>
+      <c r="G39" s="33" t="s">
+        <v>88</v>
+      </c>
+      <c r="H39" s="53" t="s">
+        <v>145</v>
+      </c>
+      <c r="I39" s="54" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="40" spans="1:9" s="8" customFormat="1" ht="27.6" x14ac:dyDescent="0.3">
+      <c r="A40" s="57">
+        <v>17</v>
+      </c>
+      <c r="B40" s="57" t="s">
+        <v>89</v>
+      </c>
+      <c r="C40" s="9">
+        <v>17.100000000000001</v>
+      </c>
+      <c r="D40" s="10" t="s">
+        <v>90</v>
+      </c>
+      <c r="E40" s="43" t="s">
+        <v>169</v>
+      </c>
+      <c r="F40" s="10" t="s">
+        <v>91</v>
+      </c>
+      <c r="G40" s="44" t="s">
+        <v>170</v>
+      </c>
+      <c r="H40" s="9" t="s">
+        <v>102</v>
+      </c>
+      <c r="I40" s="43" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="41" spans="1:9" s="8" customFormat="1" ht="27.6" x14ac:dyDescent="0.3">
+      <c r="A41" s="58"/>
+      <c r="B41" s="58"/>
+      <c r="C41" s="9">
         <v>17.2</v>
       </c>
-      <c r="D39" s="10" t="s">
-        <v>91</v>
-      </c>
-      <c r="E39" s="44" t="s">
+      <c r="D41" s="10" t="s">
+        <v>90</v>
+      </c>
+      <c r="E41" s="43" t="s">
+        <v>112</v>
+      </c>
+      <c r="F41" s="10" t="s">
+        <v>92</v>
+      </c>
+      <c r="G41" s="44" t="s">
+        <v>93</v>
+      </c>
+      <c r="H41" s="9" t="s">
+        <v>102</v>
+      </c>
+      <c r="I41" s="43" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="42" spans="1:9" s="8" customFormat="1" ht="41.4" x14ac:dyDescent="0.3">
+      <c r="A42" s="58"/>
+      <c r="B42" s="58"/>
+      <c r="C42" s="9">
+        <v>17.3</v>
+      </c>
+      <c r="D42" s="10" t="s">
+        <v>90</v>
+      </c>
+      <c r="E42" s="10" t="s">
+        <v>94</v>
+      </c>
+      <c r="F42" s="43" t="s">
         <v>113</v>
       </c>
-      <c r="F39" s="10" t="s">
-        <v>93</v>
-      </c>
-      <c r="G39" s="45" t="s">
-        <v>94</v>
-      </c>
-      <c r="H39" s="9" t="s">
-        <v>103</v>
-      </c>
-      <c r="I39" s="44" t="s">
-        <v>125</v>
-      </c>
-    </row>
-    <row r="40" spans="1:12" s="8" customFormat="1" ht="39" x14ac:dyDescent="0.35">
-      <c r="A40" s="60"/>
-      <c r="B40" s="60"/>
-      <c r="C40" s="9">
-        <v>17.3</v>
-      </c>
-      <c r="D40" s="10" t="s">
-        <v>91</v>
-      </c>
-      <c r="E40" s="10" t="s">
+      <c r="G42" s="44" t="s">
+        <v>116</v>
+      </c>
+      <c r="H42" s="9" t="s">
+        <v>102</v>
+      </c>
+      <c r="I42" s="43" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="43" spans="1:9" s="8" customFormat="1" ht="27.6" x14ac:dyDescent="0.3">
+      <c r="A43" s="58"/>
+      <c r="B43" s="58"/>
+      <c r="C43" s="9">
+        <v>17.399999999999999</v>
+      </c>
+      <c r="D43" s="10" t="s">
+        <v>90</v>
+      </c>
+      <c r="E43" s="43" t="s">
+        <v>115</v>
+      </c>
+      <c r="F43" s="43" t="s">
+        <v>114</v>
+      </c>
+      <c r="G43" s="44" t="s">
+        <v>120</v>
+      </c>
+      <c r="H43" s="9" t="s">
+        <v>102</v>
+      </c>
+      <c r="I43" s="43" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="44" spans="1:9" s="8" customFormat="1" ht="27.6" x14ac:dyDescent="0.3">
+      <c r="A44" s="58"/>
+      <c r="B44" s="58"/>
+      <c r="C44" s="9">
+        <v>17.5</v>
+      </c>
+      <c r="D44" s="10" t="s">
+        <v>90</v>
+      </c>
+      <c r="E44" s="43" t="s">
+        <v>117</v>
+      </c>
+      <c r="F44" s="43" t="s">
+        <v>118</v>
+      </c>
+      <c r="G44" s="44" t="s">
+        <v>119</v>
+      </c>
+      <c r="H44" s="9" t="s">
+        <v>102</v>
+      </c>
+      <c r="I44" s="43" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="45" spans="1:9" s="8" customFormat="1" ht="27.6" x14ac:dyDescent="0.3">
+      <c r="A45" s="58"/>
+      <c r="B45" s="58"/>
+      <c r="C45" s="9">
+        <v>17.600000000000001</v>
+      </c>
+      <c r="D45" s="10" t="s">
+        <v>90</v>
+      </c>
+      <c r="E45" s="10" t="s">
         <v>95</v>
       </c>
-      <c r="F40" s="44" t="s">
-        <v>114</v>
-      </c>
-      <c r="G40" s="45" t="s">
-        <v>117</v>
-      </c>
-      <c r="H40" s="9" t="s">
-        <v>103</v>
-      </c>
-      <c r="I40" s="44" t="s">
-        <v>125</v>
-      </c>
-    </row>
-    <row r="41" spans="1:12" s="8" customFormat="1" ht="26" x14ac:dyDescent="0.35">
-      <c r="A41" s="60"/>
-      <c r="B41" s="60"/>
-      <c r="C41" s="9">
-        <v>17.399999999999999</v>
-      </c>
-      <c r="D41" s="10" t="s">
-        <v>91</v>
-      </c>
-      <c r="E41" s="44" t="s">
-        <v>116</v>
-      </c>
-      <c r="F41" s="44" t="s">
-        <v>115</v>
-      </c>
-      <c r="G41" s="45" t="s">
+      <c r="F45" s="43" t="s">
         <v>121</v>
       </c>
-      <c r="H41" s="9" t="s">
-        <v>103</v>
-      </c>
-      <c r="I41" s="44" t="s">
-        <v>125</v>
-      </c>
-    </row>
-    <row r="42" spans="1:12" s="8" customFormat="1" ht="26" x14ac:dyDescent="0.35">
-      <c r="A42" s="60"/>
-      <c r="B42" s="60"/>
-      <c r="C42" s="9">
-        <v>17.5</v>
-      </c>
-      <c r="D42" s="10" t="s">
-        <v>91</v>
-      </c>
-      <c r="E42" s="44" t="s">
-        <v>118</v>
-      </c>
-      <c r="F42" s="44" t="s">
-        <v>119</v>
-      </c>
-      <c r="G42" s="45" t="s">
-        <v>120</v>
-      </c>
-      <c r="H42" s="9" t="s">
-        <v>103</v>
-      </c>
-      <c r="I42" s="44" t="s">
-        <v>125</v>
-      </c>
-    </row>
-    <row r="43" spans="1:12" s="8" customFormat="1" ht="26" x14ac:dyDescent="0.35">
-      <c r="A43" s="60"/>
-      <c r="B43" s="60"/>
-      <c r="C43" s="9">
-        <v>17.600000000000001</v>
-      </c>
-      <c r="D43" s="10" t="s">
-        <v>91</v>
-      </c>
-      <c r="E43" s="10" t="s">
+      <c r="G45" s="44" t="s">
+        <v>122</v>
+      </c>
+      <c r="H45" s="9" t="s">
+        <v>102</v>
+      </c>
+      <c r="I45" s="43" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="46" spans="1:9" s="8" customFormat="1" ht="27.6" x14ac:dyDescent="0.3">
+      <c r="A46" s="58"/>
+      <c r="B46" s="58"/>
+      <c r="C46" s="9">
+        <v>17.7</v>
+      </c>
+      <c r="D46" s="10" t="s">
+        <v>90</v>
+      </c>
+      <c r="E46" s="10" t="s">
         <v>96</v>
       </c>
-      <c r="F43" s="44" t="s">
-        <v>122</v>
-      </c>
-      <c r="G43" s="45" t="s">
+      <c r="F46" s="43" t="s">
         <v>123</v>
       </c>
-      <c r="H43" s="9" t="s">
-        <v>103</v>
-      </c>
-      <c r="I43" s="44" t="s">
-        <v>125</v>
-      </c>
-    </row>
-    <row r="44" spans="1:12" s="8" customFormat="1" ht="26" x14ac:dyDescent="0.35">
-      <c r="A44" s="60"/>
-      <c r="B44" s="60"/>
-      <c r="C44" s="9">
-        <v>17.7</v>
-      </c>
-      <c r="D44" s="10" t="s">
-        <v>91</v>
-      </c>
-      <c r="E44" s="10" t="s">
-        <v>97</v>
-      </c>
-      <c r="F44" s="44" t="s">
+      <c r="G46" s="44" t="s">
+        <v>130</v>
+      </c>
+      <c r="H46" s="9" t="s">
+        <v>102</v>
+      </c>
+      <c r="I46" s="43" t="s">
         <v>124</v>
       </c>
-      <c r="G44" s="45" t="s">
-        <v>131</v>
-      </c>
-      <c r="H44" s="9" t="s">
-        <v>103</v>
-      </c>
-      <c r="I44" s="44" t="s">
-        <v>125</v>
-      </c>
-    </row>
-    <row r="45" spans="1:12" s="8" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A45" s="2"/>
-      <c r="B45" s="3"/>
-      <c r="C45" s="3"/>
-      <c r="D45" s="3"/>
-      <c r="E45" s="3"/>
-      <c r="F45" s="3"/>
-      <c r="G45" s="4"/>
-      <c r="H45" s="6"/>
-      <c r="I45" s="3"/>
-    </row>
-    <row r="46" spans="1:12" s="8" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A46" s="7"/>
-      <c r="B46" s="2"/>
-      <c r="C46" s="2"/>
-      <c r="D46" s="3"/>
-      <c r="E46" s="2"/>
-      <c r="F46" s="3"/>
-      <c r="G46" s="4"/>
-      <c r="H46" s="2"/>
-      <c r="I46" s="3"/>
-    </row>
-    <row r="47" spans="1:12" s="8" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A47" s="7"/>
-      <c r="B47" s="2"/>
-      <c r="C47" s="2"/>
+    </row>
+    <row r="47" spans="1:9" s="8" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A47" s="2"/>
+      <c r="B47" s="3"/>
+      <c r="C47" s="3"/>
       <c r="D47" s="3"/>
-      <c r="E47" s="2"/>
+      <c r="E47" s="3"/>
       <c r="F47" s="3"/>
-      <c r="G47" s="3"/>
-      <c r="H47" s="2"/>
+      <c r="G47" s="4"/>
+      <c r="H47" s="6"/>
       <c r="I47" s="3"/>
     </row>
-    <row r="48" spans="1:12" s="8" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:9" s="8" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A48" s="7"/>
-      <c r="B48" s="77"/>
-      <c r="C48" s="78"/>
-      <c r="D48" s="78"/>
-      <c r="E48" s="78"/>
-      <c r="F48" s="78"/>
-      <c r="G48" s="78"/>
-      <c r="H48" s="78"/>
-      <c r="I48" s="78"/>
-      <c r="J48" s="5"/>
-      <c r="K48" s="5"/>
-      <c r="L48" s="5"/>
-    </row>
-    <row r="49" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A49" s="3"/>
-      <c r="B49" s="3"/>
-      <c r="C49" s="3"/>
-      <c r="E49" s="3"/>
-      <c r="H49" s="3"/>
-    </row>
-    <row r="50" spans="1:9" ht="17" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="D50" s="2"/>
-      <c r="F50" s="2"/>
-      <c r="G50" s="2"/>
-      <c r="I50" s="2"/>
-    </row>
-    <row r="51" spans="1:9" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="D51" s="2"/>
-      <c r="F51" s="2"/>
-      <c r="G51" s="2"/>
-      <c r="I51" s="2"/>
-    </row>
-    <row r="52" spans="1:9" ht="36.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A52" s="77"/>
-      <c r="B52" s="77"/>
-      <c r="C52" s="77"/>
-      <c r="D52" s="77"/>
-      <c r="E52" s="77"/>
-      <c r="F52" s="77"/>
-      <c r="G52" s="77"/>
-      <c r="H52" s="77"/>
-      <c r="I52" s="77"/>
-    </row>
-    <row r="53" spans="1:9" ht="36" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A53" s="3"/>
-      <c r="B53" s="3"/>
-      <c r="C53" s="3"/>
-      <c r="E53" s="3"/>
-      <c r="H53" s="3"/>
-    </row>
-    <row r="54" spans="1:9" ht="31" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="D54" s="2"/>
-      <c r="F54" s="2"/>
-      <c r="G54" s="2"/>
-      <c r="I54" s="2"/>
-    </row>
-    <row r="55" spans="1:9" ht="35" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="D55" s="2"/>
-      <c r="F55" s="2"/>
-      <c r="G55" s="2"/>
-      <c r="I55" s="2"/>
-    </row>
-    <row r="56" spans="1:9" ht="32" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A56" s="77"/>
-      <c r="B56" s="77"/>
-      <c r="C56" s="77"/>
-      <c r="D56" s="77"/>
-      <c r="E56" s="77"/>
-      <c r="F56" s="77"/>
-      <c r="G56" s="77"/>
-      <c r="H56" s="77"/>
-      <c r="I56" s="77"/>
-    </row>
-    <row r="57" spans="1:9" ht="33.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A57" s="3"/>
-      <c r="B57" s="3"/>
-      <c r="C57" s="3"/>
-      <c r="E57" s="3"/>
-      <c r="H57" s="3"/>
-    </row>
-    <row r="58" spans="1:9" ht="31.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="D58" s="2"/>
-      <c r="F58" s="2"/>
-      <c r="G58" s="2"/>
-      <c r="I58" s="2"/>
-    </row>
-    <row r="59" spans="1:9" ht="27.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B48" s="2"/>
+      <c r="C48" s="2"/>
+      <c r="D48" s="3"/>
+      <c r="E48" s="2"/>
+      <c r="F48" s="3"/>
+      <c r="G48" s="4"/>
+      <c r="H48" s="2"/>
+      <c r="I48" s="3"/>
+    </row>
+    <row r="49" spans="1:12" s="8" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A49" s="7"/>
+      <c r="B49" s="2"/>
+      <c r="C49" s="2"/>
+      <c r="D49" s="3"/>
+      <c r="E49" s="2"/>
+      <c r="F49" s="3"/>
+      <c r="G49" s="3"/>
+      <c r="H49" s="2"/>
+      <c r="I49" s="3"/>
+    </row>
+    <row r="50" spans="1:12" s="8" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A50" s="7"/>
+      <c r="B50" s="55"/>
+      <c r="C50" s="56"/>
+      <c r="D50" s="56"/>
+      <c r="E50" s="56"/>
+      <c r="F50" s="56"/>
+      <c r="G50" s="56"/>
+      <c r="H50" s="56"/>
+      <c r="I50" s="56"/>
+      <c r="J50" s="5"/>
+      <c r="K50" s="5"/>
+      <c r="L50" s="5"/>
+    </row>
+    <row r="51" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A51" s="3"/>
+      <c r="B51" s="3"/>
+      <c r="C51" s="3"/>
+      <c r="E51" s="3"/>
+      <c r="H51" s="3"/>
+    </row>
+    <row r="52" spans="1:12" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="D52" s="2"/>
+      <c r="F52" s="2"/>
+      <c r="G52" s="2"/>
+      <c r="I52" s="2"/>
+    </row>
+    <row r="53" spans="1:12" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="D53" s="2"/>
+      <c r="F53" s="2"/>
+      <c r="G53" s="2"/>
+      <c r="I53" s="2"/>
+    </row>
+    <row r="54" spans="1:12" ht="36.450000000000003" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A54" s="55"/>
+      <c r="B54" s="55"/>
+      <c r="C54" s="55"/>
+      <c r="D54" s="55"/>
+      <c r="E54" s="55"/>
+      <c r="F54" s="55"/>
+      <c r="G54" s="55"/>
+      <c r="H54" s="55"/>
+      <c r="I54" s="55"/>
+    </row>
+    <row r="55" spans="1:12" ht="36" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A55" s="3"/>
+      <c r="B55" s="3"/>
+      <c r="C55" s="3"/>
+      <c r="E55" s="3"/>
+      <c r="H55" s="3"/>
+    </row>
+    <row r="56" spans="1:12" ht="31.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="D56" s="2"/>
+      <c r="F56" s="2"/>
+      <c r="G56" s="2"/>
+      <c r="I56" s="2"/>
+    </row>
+    <row r="57" spans="1:12" ht="34.950000000000003" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="D57" s="2"/>
+      <c r="F57" s="2"/>
+      <c r="G57" s="2"/>
+      <c r="I57" s="2"/>
+    </row>
+    <row r="58" spans="1:12" ht="31.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A58" s="55"/>
+      <c r="B58" s="55"/>
+      <c r="C58" s="55"/>
+      <c r="D58" s="55"/>
+      <c r="E58" s="55"/>
+      <c r="F58" s="55"/>
+      <c r="G58" s="55"/>
+      <c r="H58" s="55"/>
+      <c r="I58" s="55"/>
+    </row>
+    <row r="59" spans="1:12" ht="33.450000000000003" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A59" s="3"/>
       <c r="B59" s="3"/>
-      <c r="F59" s="2"/>
-      <c r="G59" s="2"/>
-      <c r="I59" s="2"/>
+      <c r="C59" s="3"/>
+      <c r="E59" s="3"/>
+      <c r="H59" s="3"/>
+    </row>
+    <row r="60" spans="1:12" ht="31.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="D60" s="2"/>
+      <c r="F60" s="2"/>
+      <c r="G60" s="2"/>
+      <c r="I60" s="2"/>
+    </row>
+    <row r="61" spans="1:12" ht="27.45" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B61" s="3"/>
+      <c r="F61" s="2"/>
+      <c r="G61" s="2"/>
+      <c r="I61" s="2"/>
     </row>
   </sheetData>
   <autoFilter ref="I1:I19" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
   <mergeCells count="25">
-    <mergeCell ref="A38:A44"/>
-    <mergeCell ref="B13:B16"/>
-    <mergeCell ref="B17:B19"/>
-    <mergeCell ref="B38:B44"/>
-    <mergeCell ref="A10:A12"/>
+    <mergeCell ref="B8:B9"/>
+    <mergeCell ref="B22:B32"/>
+    <mergeCell ref="B38:B39"/>
+    <mergeCell ref="B17:B20"/>
+    <mergeCell ref="A17:A20"/>
     <mergeCell ref="B5:B6"/>
     <mergeCell ref="A5:A6"/>
-    <mergeCell ref="A17:A19"/>
-    <mergeCell ref="A31:A35"/>
+    <mergeCell ref="A33:A37"/>
     <mergeCell ref="I1:I2"/>
     <mergeCell ref="D1:F1"/>
-    <mergeCell ref="A36:A37"/>
     <mergeCell ref="A13:A16"/>
     <mergeCell ref="A8:A9"/>
     <mergeCell ref="B10:B12"/>
     <mergeCell ref="H1:H2"/>
-    <mergeCell ref="B31:B35"/>
+    <mergeCell ref="B33:B37"/>
     <mergeCell ref="A1:A2"/>
-    <mergeCell ref="A20:A30"/>
+    <mergeCell ref="A22:A32"/>
     <mergeCell ref="C1:C2"/>
     <mergeCell ref="G1:G2"/>
     <mergeCell ref="B1:B2"/>
-    <mergeCell ref="B8:B9"/>
-    <mergeCell ref="B20:B30"/>
-    <mergeCell ref="B36:B37"/>
+    <mergeCell ref="A40:A46"/>
+    <mergeCell ref="B13:B16"/>
+    <mergeCell ref="B40:B46"/>
+    <mergeCell ref="A10:A12"/>
+    <mergeCell ref="A38:A39"/>
   </mergeCells>
   <phoneticPr fontId="6" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
pending user stories for partial/autosave and toast message added
</commit_message>
<xml_diff>
--- a/Soubhanik/checkupp_product_backlog_final.xlsx
+++ b/Soubhanik/checkupp_product_backlog_final.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Anodiam\2026\CheckUpp_Parent\CheckUpp\Soubhanik\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E3EDB0C3-02C7-43A0-8C41-F3EFE5342C94}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6480953D-E16A-4C70-83B6-EA3AE4CB5417}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -125,36 +125,12 @@
         </r>
       </text>
     </comment>
-    <comment ref="E20" authorId="0" shapeId="0" xr:uid="{3CA1A3BC-210A-4820-BB92-615ED01D6D27}">
-      <text>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>Anirban:</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">
-Invalid User Story: This is not an action by the user.</t>
-        </r>
-      </text>
-    </comment>
   </commentList>
 </comments>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="271" uniqueCount="188">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="310" uniqueCount="223">
   <si>
     <t>Epic #</t>
   </si>
@@ -779,7 +755,138 @@
 </t>
   </si>
   <si>
-    <t>5. The most recent changes made to all assessment fields and toggle switches must be displayed when the assessment is resumed, without requiring the user to re-enter the information.</t>
+    <t>logged in user revisiting the mental health assessment</t>
+  </si>
+  <si>
+    <t>I am informed that my autosaved data was restored.</t>
+  </si>
+  <si>
+    <t>see my previously entered data in available fields(K-10 score, DASS-21 Depression, DASS-21 Anxiety, etc) or the status of the toggle switches (difficulty falling asleep and frequent night waking) restored along with an affirming notification(toast)</t>
+  </si>
+  <si>
+    <t>1. Previously autosaved assessment data must be restored automatically when the logged-in user revisits the Mental Health Assessment screen.
+2. An affirming notification (toast) saying 'Data restored', indicating that the autosaved data has been restored must be displayed after the assessment data is successfully loaded and must not appear if no saved data exists.
+3. The restored values for all available fields and toggle switches must be identical to the most recently autosaved data. 
+4. The restored data and affirming notification must be visible without requiring any additional action from the user.</t>
+  </si>
+  <si>
+    <t>Cardiovascular Reading</t>
+  </si>
+  <si>
+    <t>logged in user navigating the Cardiovascular Reading screen</t>
+  </si>
+  <si>
+    <t>have the data I enter in the available fields(systolic, diastolic, heart rate, etc.)  autosaved in the system if I tap the 'Back' button or close/remove the app from the background</t>
+  </si>
+  <si>
+    <t>I don't have to re-enter the data in the fields(systolic, diastolic, heart rate, etc.) again</t>
+  </si>
+  <si>
+    <t>logged in user revisiting the Cardiovascular Reading</t>
+  </si>
+  <si>
+    <t>see my previously entered data in available fields(systolic, diastolic, heart rate, etc.) restored along with an affirming notification(toast)</t>
+  </si>
+  <si>
+    <t>1. Previously autosaved available data must be restored automatically when the logged-in user revisits the Cardiovascular Reading screen.
+2. An affirming notification (toast) saying 'Data restored', indicating that the autosaved data has been restored must be displayed after the assessment data is successfully loaded and must not appear if no saved data exists.
+3. The restored values for all available fields must be identical to the most recently autosaved data. 
+4. The restored data and affirming notification must be visible without requiring any additional action from the user.</t>
+  </si>
+  <si>
+    <t>1. All entered assessment field fields(systolic, diastolic, heart rate, etc.) must be automatically saved whenever the user enters or updates them.
+2. All autosaved assessment data must be restored when the user returns to the Cardiovascular Reading screen after tapping the Back button.
+3. All autosaved assessment data must be restored when the user reopens the app after it has been closed or removed from the background.</t>
+  </si>
+  <si>
+    <t>Diabetes Test</t>
+  </si>
+  <si>
+    <t>logged in user navigating the Diabetes Test screen</t>
+  </si>
+  <si>
+    <t>logged in user revisiting the Diabetes Test</t>
+  </si>
+  <si>
+    <t>have the data I enter in the available fields(fasting glucose, random glucose, etc.)  autosaved in the system if I tap the 'Back' button or close/remove the app from the background</t>
+  </si>
+  <si>
+    <t>see my previously entered data in available fields(fasting glucose, random glucose, etc.) restored along with an affirming notification(toast)</t>
+  </si>
+  <si>
+    <t>I don't have to re-enter the data in the fields(fasting glucose, random glucose, etc.) again</t>
+  </si>
+  <si>
+    <t>1. All entered assessment fields(fasting glucose, random glucose, etc.) must be automatically saved whenever the user enters or updates them.
+2. All autosaved assessment data must be restored when the user returns to the Diabetes Test screen after tapping the Back button.
+3. All autosaved assessment data must be restored when the user reopens the app after it has been closed or removed from the background.</t>
+  </si>
+  <si>
+    <t>1. Previously autosaved available data must be restored automatically when the logged-in user revisits the Diabetes Test screen.
+2. An affirming notification (toast) saying 'Data restored', indicating that the autosaved data has been restored must be displayed after the assessment data is successfully loaded and must not appear if no saved data exists.
+3. The restored values for all available fields must be identical to the most recently autosaved data. 
+4. The restored data and affirming notification must be visible without requiring any additional action from the user.</t>
+  </si>
+  <si>
+    <t>Vision Test</t>
+  </si>
+  <si>
+    <t>logged in user navigating the Vision Test screen</t>
+  </si>
+  <si>
+    <t>logged in user revisiting the Vision Test</t>
+  </si>
+  <si>
+    <t>1. Previously autosaved available data must be restored automatically when the logged-in user revisits the Vision Test screen.
+2. An affirming notification (toast) saying 'Data restored', indicating that the autosaved data has been restored must be displayed after the assessment data is successfully loaded and must not appear if no saved data exists.
+3. The restored values for all available fields must be identical to the most recently autosaved data. 
+4. The restored data and affirming notification must be visible without requiring any additional action from the user.</t>
+  </si>
+  <si>
+    <t>see my previously entered data in available fields(Right Eye, Left Eye, etc.) restored along with an affirming notification(toast)</t>
+  </si>
+  <si>
+    <t>I don't have to re-enter the data in the fields(Right Eye, Left Eye, etc.) again</t>
+  </si>
+  <si>
+    <t>have the data I enter in the available fields(Right Eye, Left Eye, etc.)  autosaved in the system if I tap the 'Back' button or close/remove the app from the background</t>
+  </si>
+  <si>
+    <t>1. All entered assessment fields(Right Eye, Left Eye, etc.) must be automatically saved whenever the user enters or updates them.
+2. All autosaved assessment data must be restored when the user returns to the Vision Test screen after tapping the Back button.
+3. All autosaved assessment data must be restored when the user reopens the app after it has been closed or removed from the background.</t>
+  </si>
+  <si>
+    <t>Dental Health Check</t>
+  </si>
+  <si>
+    <t>logged in user navigating the Dental Health Check screen</t>
+  </si>
+  <si>
+    <t>logged in user revisiting the Dental Health Check</t>
+  </si>
+  <si>
+    <t>1. Previously autosaved available data must be restored automatically when the logged-in user revisits the Dental Health Check screen.
+2. An affirming notification (toast) saying 'Data restored', indicating that the autosaved data has been restored must be displayed after the assessment data is successfully loaded and must not appear if no saved data exists.
+3. The restored values for all available fields must be identical to the most recently autosaved data. 
+4. The restored data and affirming notification must be visible without requiring any additional action from the user.</t>
+  </si>
+  <si>
+    <t>have the data I enter in the available fields (cavities, fillings, etc), used the toggle switches (Use mouthwash regularly) and the dropdown options (Brushing frequency and flossing frequency) autosaved in the system if I tap the 'Back' button or close/remove the app from the background</t>
+  </si>
+  <si>
+    <t>I don't have to re-enter the data in the fields (cavities, fillings, etc), re-toggle the switches (Use mouthwash regularly) and the re-use dropdown options (Brushing frequency and flossing frequency)</t>
+  </si>
+  <si>
+    <t>1. All entered dental health field values (e.g., cavities, fillings, etc.) must be automatically saved whenever they are entered or updated.
+2. All toggle switch states (e.g., Use Mouthwash Regularly) must be automatically saved whenever they are changed.
+3. All selected dropdown options (e.g., Brushing Frequency and Flossing Frequency) must be automatically saved whenever they are changed.
+4. All autosaved dental health data must be restored when the user returns to the Dental Health Check screen after tapping the Back button.
+5. All autosaved dental health data must be restored when the user reopens the app after it has been closed or removed from the background.
+6. The most recent values entered in all fields, toggle switches, and dropdown selections must be displayed when the Dental Health Check is resumed, without requiring the user to re-enter or reselect the information.</t>
+  </si>
+  <si>
+    <t>see my previously entered data in the available fields (e.g., cavities, fillings, etc.), the status of the toggle switch (Use Mouthwash Regularly), and the selected dropdown options (Brushing Frequency and Flossing Frequency) restored along with an affirming notification (toast)</t>
   </si>
 </sst>
 </file>
@@ -977,7 +1084,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="9">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -989,43 +1096,6 @@
       <left style="thin">
         <color indexed="64"/>
       </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top/>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
       <right style="thin">
         <color indexed="64"/>
       </right>
@@ -1052,286 +1122,217 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top/>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="82">
+  <cellXfs count="70">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="5" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="7" borderId="5" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="8" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="8" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="8" borderId="5" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="9" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="9" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="8" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="10" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="10" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="10" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="10" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="11" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="13" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="13" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="11" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="13" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="13" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="14" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="14" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="14" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="14" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="8" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="9" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="10" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="10" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="13" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="14" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="15" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="15" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="11" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="11" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="11" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="11" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="11" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="11" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="15" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="15" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="15" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="15" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="15" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="15" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="15" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="15" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="5" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="16" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="16" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="16" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="16" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="16" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="9" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="8" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="15" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="15" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="13" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="5" fillId="12" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="12" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="12" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="14" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="13" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="14" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="12" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="12" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="12" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="12" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="15" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="10" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="10" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="10" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="10" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="10" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1617,1309 +1618,1437 @@
   <dimension ref="A1:L61"/>
   <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="5.88671875" style="2" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="32.88671875" style="2" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="11.109375" style="2" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="20.88671875" style="3" customWidth="1"/>
-    <col min="5" max="5" width="65" style="2" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="41" style="3" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="61.44140625" style="3" customWidth="1"/>
-    <col min="8" max="8" width="11.6640625" style="2" customWidth="1"/>
-    <col min="9" max="9" width="15.33203125" style="3" customWidth="1"/>
-    <col min="10" max="12" width="8.88671875" style="5" customWidth="1"/>
-    <col min="13" max="16384" width="8.88671875" style="5"/>
+    <col min="1" max="1" width="5.88671875" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="32.88671875" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="11.109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="20.88671875" style="2" customWidth="1"/>
+    <col min="5" max="5" width="64.88671875" style="1" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="41" style="2" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="61.44140625" style="2" customWidth="1"/>
+    <col min="8" max="8" width="11.6640625" style="1" customWidth="1"/>
+    <col min="9" max="9" width="15.33203125" style="2" customWidth="1"/>
+    <col min="10" max="12" width="8.88671875" style="3" customWidth="1"/>
+    <col min="13" max="16384" width="8.88671875" style="3"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="39.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="71" t="s">
+      <c r="A1" s="55" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="65" t="s">
+      <c r="B1" s="55" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="65" t="s">
+      <c r="C1" s="55" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="65" t="s">
+      <c r="D1" s="55" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="67"/>
-      <c r="F1" s="68"/>
-      <c r="G1" s="74" t="s">
+      <c r="E1" s="58"/>
+      <c r="F1" s="58"/>
+      <c r="G1" s="55" t="s">
         <v>4</v>
       </c>
-      <c r="H1" s="65" t="s">
+      <c r="H1" s="55" t="s">
         <v>5</v>
       </c>
-      <c r="I1" s="65" t="s">
+      <c r="I1" s="55" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A2" s="60"/>
-      <c r="B2" s="66"/>
-      <c r="C2" s="66"/>
-      <c r="D2" s="1" t="s">
+      <c r="A2" s="59"/>
+      <c r="B2" s="59"/>
+      <c r="C2" s="59"/>
+      <c r="D2" s="60" t="s">
         <v>7</v>
       </c>
-      <c r="E2" s="1" t="s">
+      <c r="E2" s="60" t="s">
         <v>8</v>
       </c>
-      <c r="F2" s="1" t="s">
+      <c r="F2" s="60" t="s">
         <v>9</v>
       </c>
-      <c r="G2" s="75"/>
-      <c r="H2" s="66"/>
-      <c r="I2" s="66"/>
-    </row>
-    <row r="3" spans="1:9" s="8" customFormat="1" ht="82.8" x14ac:dyDescent="0.3">
-      <c r="A3" s="36" t="s">
+      <c r="G2" s="55"/>
+      <c r="H2" s="59"/>
+      <c r="I2" s="59"/>
+    </row>
+    <row r="3" spans="1:9" s="4" customFormat="1" ht="82.8" x14ac:dyDescent="0.3">
+      <c r="A3" s="30" t="s">
         <v>141</v>
       </c>
-      <c r="B3" s="36" t="s">
+      <c r="B3" s="30" t="s">
         <v>125</v>
       </c>
-      <c r="C3" s="22">
+      <c r="C3" s="18">
         <v>13.2</v>
       </c>
-      <c r="D3" s="37" t="s">
+      <c r="D3" s="31" t="s">
         <v>126</v>
       </c>
-      <c r="E3" s="37" t="s">
+      <c r="E3" s="31" t="s">
         <v>127</v>
       </c>
-      <c r="F3" s="37" t="s">
+      <c r="F3" s="31" t="s">
         <v>128</v>
       </c>
-      <c r="G3" s="38" t="s">
+      <c r="G3" s="32" t="s">
         <v>131</v>
       </c>
-      <c r="H3" s="22" t="s">
+      <c r="H3" s="18" t="s">
         <v>60</v>
       </c>
-      <c r="I3" s="37" t="s">
+      <c r="I3" s="31" t="s">
         <v>132</v>
       </c>
     </row>
-    <row r="4" spans="1:9" s="8" customFormat="1" ht="55.2" x14ac:dyDescent="0.3">
-      <c r="A4" s="46">
+    <row r="4" spans="1:9" s="4" customFormat="1" ht="55.2" x14ac:dyDescent="0.3">
+      <c r="A4" s="61">
         <v>1</v>
       </c>
-      <c r="B4" s="46" t="s">
+      <c r="B4" s="61" t="s">
         <v>10</v>
       </c>
-      <c r="C4" s="47">
+      <c r="C4" s="39">
         <v>1.1000000000000001</v>
       </c>
-      <c r="D4" s="48" t="s">
+      <c r="D4" s="40" t="s">
         <v>11</v>
       </c>
-      <c r="E4" s="48" t="s">
+      <c r="E4" s="40" t="s">
         <v>103</v>
       </c>
-      <c r="F4" s="48" t="s">
+      <c r="F4" s="40" t="s">
         <v>104</v>
       </c>
-      <c r="G4" s="49" t="s">
+      <c r="G4" s="41" t="s">
         <v>105</v>
       </c>
-      <c r="H4" s="47" t="s">
+      <c r="H4" s="39" t="s">
         <v>12</v>
       </c>
-      <c r="I4" s="48" t="s">
+      <c r="I4" s="40" t="s">
         <v>129</v>
       </c>
     </row>
-    <row r="5" spans="1:9" s="35" customFormat="1" ht="82.8" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:9" s="29" customFormat="1" ht="69" x14ac:dyDescent="0.3">
       <c r="A5" s="62">
         <v>3</v>
       </c>
       <c r="B5" s="62" t="s">
         <v>13</v>
       </c>
-      <c r="C5" s="34">
+      <c r="C5" s="28">
         <v>3.1</v>
       </c>
-      <c r="D5" s="39" t="s">
+      <c r="D5" s="33" t="s">
         <v>11</v>
       </c>
-      <c r="E5" s="40" t="s">
+      <c r="E5" s="34" t="s">
         <v>106</v>
       </c>
-      <c r="F5" s="40" t="s">
+      <c r="F5" s="34" t="s">
         <v>107</v>
       </c>
-      <c r="G5" s="41" t="s">
+      <c r="G5" s="35" t="s">
         <v>110</v>
       </c>
-      <c r="H5" s="42" t="s">
+      <c r="H5" s="36" t="s">
         <v>97</v>
       </c>
-      <c r="I5" s="39" t="s">
+      <c r="I5" s="33" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="6" spans="1:9" s="8" customFormat="1" ht="82.8" x14ac:dyDescent="0.3">
-      <c r="A6" s="63"/>
-      <c r="B6" s="63"/>
-      <c r="C6" s="34">
+    <row r="6" spans="1:9" s="4" customFormat="1" ht="69" x14ac:dyDescent="0.3">
+      <c r="A6" s="62"/>
+      <c r="B6" s="62"/>
+      <c r="C6" s="28">
         <v>3.2</v>
       </c>
-      <c r="D6" s="39" t="s">
+      <c r="D6" s="33" t="s">
         <v>11</v>
       </c>
-      <c r="E6" s="40" t="s">
+      <c r="E6" s="34" t="s">
         <v>108</v>
       </c>
-      <c r="F6" s="40" t="s">
+      <c r="F6" s="34" t="s">
         <v>109</v>
       </c>
-      <c r="G6" s="41" t="s">
+      <c r="G6" s="35" t="s">
         <v>111</v>
       </c>
-      <c r="H6" s="34" t="s">
+      <c r="H6" s="28" t="s">
         <v>97</v>
       </c>
-      <c r="I6" s="39" t="s">
+      <c r="I6" s="33" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="7" spans="1:9" s="8" customFormat="1" ht="138" x14ac:dyDescent="0.3">
-      <c r="A7" s="45">
+    <row r="7" spans="1:9" s="4" customFormat="1" ht="124.2" x14ac:dyDescent="0.3">
+      <c r="A7" s="38">
         <v>5</v>
       </c>
-      <c r="B7" s="45" t="s">
+      <c r="B7" s="38" t="s">
         <v>16</v>
       </c>
-      <c r="C7" s="9">
+      <c r="C7" s="5">
         <v>5.2</v>
       </c>
-      <c r="D7" s="10" t="s">
+      <c r="D7" s="6" t="s">
         <v>133</v>
       </c>
-      <c r="E7" s="10" t="s">
+      <c r="E7" s="6" t="s">
         <v>135</v>
       </c>
-      <c r="F7" s="10" t="s">
+      <c r="F7" s="6" t="s">
         <v>134</v>
       </c>
-      <c r="G7" s="27" t="s">
+      <c r="G7" s="23" t="s">
         <v>136</v>
       </c>
-      <c r="H7" s="11" t="s">
+      <c r="H7" s="7" t="s">
         <v>98</v>
       </c>
-      <c r="I7" s="10" t="s">
+      <c r="I7" s="6" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="8" spans="1:9" s="8" customFormat="1" ht="27.6" x14ac:dyDescent="0.3">
-      <c r="A8" s="70">
+    <row r="8" spans="1:9" s="4" customFormat="1" ht="27.6" x14ac:dyDescent="0.3">
+      <c r="A8" s="49">
         <v>6</v>
       </c>
-      <c r="B8" s="70" t="s">
+      <c r="B8" s="49" t="s">
         <v>18</v>
       </c>
-      <c r="C8" s="12">
+      <c r="C8" s="8">
         <v>6.1</v>
       </c>
-      <c r="D8" s="13" t="s">
+      <c r="D8" s="9" t="s">
         <v>126</v>
       </c>
-      <c r="E8" s="50" t="s">
+      <c r="E8" s="42" t="s">
         <v>137</v>
       </c>
-      <c r="F8" s="50" t="s">
+      <c r="F8" s="42" t="s">
         <v>138</v>
       </c>
-      <c r="G8" s="51" t="s">
+      <c r="G8" s="43" t="s">
         <v>139</v>
       </c>
-      <c r="H8" s="14" t="s">
+      <c r="H8" s="10" t="s">
         <v>99</v>
       </c>
-      <c r="I8" s="13" t="s">
+      <c r="I8" s="9" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="9" spans="1:9" s="8" customFormat="1" ht="55.2" x14ac:dyDescent="0.3">
-      <c r="A9" s="60"/>
-      <c r="B9" s="60"/>
-      <c r="C9" s="12">
+    <row r="9" spans="1:9" s="4" customFormat="1" ht="55.2" x14ac:dyDescent="0.3">
+      <c r="A9" s="59"/>
+      <c r="B9" s="59"/>
+      <c r="C9" s="8">
         <v>6.3</v>
       </c>
-      <c r="D9" s="13" t="s">
+      <c r="D9" s="9" t="s">
         <v>126</v>
       </c>
-      <c r="E9" s="13" t="s">
+      <c r="E9" s="9" t="s">
         <v>20</v>
       </c>
-      <c r="F9" s="13" t="s">
+      <c r="F9" s="9" t="s">
         <v>21</v>
       </c>
-      <c r="G9" s="28" t="s">
+      <c r="G9" s="24" t="s">
         <v>140</v>
       </c>
-      <c r="H9" s="12" t="s">
+      <c r="H9" s="8" t="s">
         <v>99</v>
       </c>
-      <c r="I9" s="13"/>
-    </row>
-    <row r="10" spans="1:9" s="8" customFormat="1" ht="55.2" x14ac:dyDescent="0.3">
-      <c r="A10" s="61">
+      <c r="I9" s="9"/>
+    </row>
+    <row r="10" spans="1:9" s="4" customFormat="1" ht="55.2" x14ac:dyDescent="0.3">
+      <c r="A10" s="54">
         <v>7</v>
       </c>
-      <c r="B10" s="61" t="s">
+      <c r="B10" s="54" t="s">
         <v>22</v>
       </c>
-      <c r="C10" s="15">
+      <c r="C10" s="11">
         <v>7.1</v>
       </c>
-      <c r="D10" s="16" t="s">
+      <c r="D10" s="12" t="s">
         <v>126</v>
       </c>
-      <c r="E10" s="16" t="s">
+      <c r="E10" s="12" t="s">
         <v>23</v>
       </c>
-      <c r="F10" s="16" t="s">
+      <c r="F10" s="12" t="s">
         <v>24</v>
       </c>
-      <c r="G10" s="29" t="s">
+      <c r="G10" s="25" t="s">
         <v>25</v>
       </c>
-      <c r="H10" s="17" t="s">
+      <c r="H10" s="13" t="s">
         <v>100</v>
       </c>
-      <c r="I10" s="16" t="s">
+      <c r="I10" s="12" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="11" spans="1:9" s="8" customFormat="1" ht="55.2" x14ac:dyDescent="0.3">
-      <c r="A11" s="58"/>
-      <c r="B11" s="58"/>
-      <c r="C11" s="15">
+    <row r="11" spans="1:9" s="4" customFormat="1" ht="55.2" x14ac:dyDescent="0.3">
+      <c r="A11" s="59"/>
+      <c r="B11" s="59"/>
+      <c r="C11" s="11">
         <v>7.2</v>
       </c>
-      <c r="D11" s="16" t="s">
+      <c r="D11" s="12" t="s">
         <v>126</v>
       </c>
-      <c r="E11" s="16" t="s">
+      <c r="E11" s="12" t="s">
         <v>27</v>
       </c>
-      <c r="F11" s="16" t="s">
+      <c r="F11" s="12" t="s">
         <v>28</v>
       </c>
-      <c r="G11" s="29" t="s">
+      <c r="G11" s="25" t="s">
         <v>29</v>
       </c>
-      <c r="H11" s="15" t="s">
+      <c r="H11" s="11" t="s">
         <v>101</v>
       </c>
-      <c r="I11" s="16" t="s">
+      <c r="I11" s="12" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="12" spans="1:9" s="8" customFormat="1" ht="41.4" x14ac:dyDescent="0.3">
-      <c r="A12" s="60"/>
-      <c r="B12" s="60"/>
-      <c r="C12" s="15">
+    <row r="12" spans="1:9" s="4" customFormat="1" ht="41.4" x14ac:dyDescent="0.3">
+      <c r="A12" s="59"/>
+      <c r="B12" s="59"/>
+      <c r="C12" s="11">
         <v>7.3</v>
       </c>
-      <c r="D12" s="16" t="s">
+      <c r="D12" s="12" t="s">
         <v>126</v>
       </c>
-      <c r="E12" s="16" t="s">
+      <c r="E12" s="12" t="s">
         <v>30</v>
       </c>
-      <c r="F12" s="16" t="s">
+      <c r="F12" s="12" t="s">
         <v>31</v>
       </c>
-      <c r="G12" s="29" t="s">
+      <c r="G12" s="25" t="s">
         <v>32</v>
       </c>
-      <c r="H12" s="15" t="s">
+      <c r="H12" s="11" t="s">
         <v>100</v>
       </c>
-      <c r="I12" s="16"/>
-    </row>
-    <row r="13" spans="1:9" s="8" customFormat="1" ht="27.6" x14ac:dyDescent="0.3">
-      <c r="A13" s="59">
+      <c r="I12" s="12"/>
+    </row>
+    <row r="13" spans="1:9" s="4" customFormat="1" ht="27.6" x14ac:dyDescent="0.3">
+      <c r="A13" s="53">
         <v>9</v>
       </c>
-      <c r="B13" s="59" t="s">
+      <c r="B13" s="53" t="s">
         <v>33</v>
       </c>
-      <c r="C13" s="18">
+      <c r="C13" s="14">
         <v>9.1</v>
       </c>
-      <c r="D13" s="19" t="s">
+      <c r="D13" s="15" t="s">
         <v>15</v>
       </c>
-      <c r="E13" s="19" t="s">
+      <c r="E13" s="15" t="s">
         <v>34</v>
       </c>
-      <c r="F13" s="19" t="s">
+      <c r="F13" s="15" t="s">
         <v>35</v>
       </c>
-      <c r="G13" s="30" t="s">
+      <c r="G13" s="26" t="s">
         <v>36</v>
       </c>
-      <c r="H13" s="18"/>
-      <c r="I13" s="19"/>
-    </row>
-    <row r="14" spans="1:9" s="8" customFormat="1" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="58"/>
-      <c r="B14" s="58"/>
-      <c r="C14" s="18">
+      <c r="H13" s="14"/>
+      <c r="I13" s="15"/>
+    </row>
+    <row r="14" spans="1:9" s="4" customFormat="1" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A14" s="59"/>
+      <c r="B14" s="59"/>
+      <c r="C14" s="14">
         <v>9.1999999999999993</v>
       </c>
-      <c r="D14" s="19" t="s">
+      <c r="D14" s="15" t="s">
         <v>37</v>
       </c>
-      <c r="E14" s="19" t="s">
+      <c r="E14" s="15" t="s">
         <v>38</v>
       </c>
-      <c r="F14" s="19" t="s">
+      <c r="F14" s="15" t="s">
         <v>39</v>
       </c>
-      <c r="G14" s="30" t="s">
+      <c r="G14" s="26" t="s">
         <v>40</v>
       </c>
-      <c r="H14" s="18"/>
-      <c r="I14" s="19"/>
-    </row>
-    <row r="15" spans="1:9" s="8" customFormat="1" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="58"/>
-      <c r="B15" s="58"/>
-      <c r="C15" s="18">
+      <c r="H14" s="14"/>
+      <c r="I14" s="15"/>
+    </row>
+    <row r="15" spans="1:9" s="4" customFormat="1" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A15" s="59"/>
+      <c r="B15" s="59"/>
+      <c r="C15" s="14">
         <v>9.3000000000000007</v>
       </c>
-      <c r="D15" s="19" t="s">
+      <c r="D15" s="15" t="s">
         <v>41</v>
       </c>
-      <c r="E15" s="19" t="s">
+      <c r="E15" s="15" t="s">
         <v>42</v>
       </c>
-      <c r="F15" s="19" t="s">
+      <c r="F15" s="15" t="s">
         <v>43</v>
       </c>
-      <c r="G15" s="30" t="s">
+      <c r="G15" s="26" t="s">
         <v>44</v>
       </c>
-      <c r="H15" s="18"/>
-      <c r="I15" s="19" t="s">
+      <c r="H15" s="14"/>
+      <c r="I15" s="15" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="16" spans="1:9" s="8" customFormat="1" ht="55.2" x14ac:dyDescent="0.3">
-      <c r="A16" s="60"/>
-      <c r="B16" s="60"/>
-      <c r="C16" s="18">
+    <row r="16" spans="1:9" s="4" customFormat="1" ht="55.2" x14ac:dyDescent="0.3">
+      <c r="A16" s="59"/>
+      <c r="B16" s="59"/>
+      <c r="C16" s="14">
         <v>9.4</v>
       </c>
-      <c r="D16" s="19" t="s">
+      <c r="D16" s="15" t="s">
         <v>15</v>
       </c>
-      <c r="E16" s="19" t="s">
+      <c r="E16" s="15" t="s">
         <v>46</v>
       </c>
-      <c r="F16" s="19" t="s">
+      <c r="F16" s="15" t="s">
         <v>47</v>
       </c>
-      <c r="G16" s="30" t="s">
+      <c r="G16" s="26" t="s">
         <v>48</v>
       </c>
-      <c r="H16" s="18"/>
-      <c r="I16" s="19" t="s">
+      <c r="H16" s="14"/>
+      <c r="I16" s="15" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="17" spans="1:9" s="8" customFormat="1" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="78">
+    <row r="17" spans="1:9" s="4" customFormat="1" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A17" s="63">
         <v>12</v>
       </c>
-      <c r="B17" s="78" t="s">
+      <c r="B17" s="63" t="s">
         <v>183</v>
       </c>
-      <c r="C17" s="20">
+      <c r="C17" s="16">
         <v>12.1</v>
       </c>
-      <c r="D17" s="21" t="s">
-        <v>126</v>
-      </c>
-      <c r="E17" s="21" t="s">
+      <c r="D17" s="17" t="s">
+        <v>182</v>
+      </c>
+      <c r="E17" s="17" t="s">
         <v>49</v>
       </c>
-      <c r="F17" s="21" t="s">
+      <c r="F17" s="17" t="s">
         <v>50</v>
       </c>
-      <c r="G17" s="31" t="s">
+      <c r="G17" s="27" t="s">
         <v>51</v>
       </c>
-      <c r="H17" s="20" t="s">
+      <c r="H17" s="16" t="s">
         <v>52</v>
       </c>
-      <c r="I17" s="21" t="s">
+      <c r="I17" s="17" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="18" spans="1:9" s="8" customFormat="1" ht="55.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="79"/>
-      <c r="B18" s="79"/>
-      <c r="C18" s="20">
+    <row r="18" spans="1:9" s="4" customFormat="1" ht="55.2" x14ac:dyDescent="0.3">
+      <c r="A18" s="63"/>
+      <c r="B18" s="63"/>
+      <c r="C18" s="16">
         <v>12.2</v>
       </c>
-      <c r="D18" s="21" t="s">
-        <v>126</v>
-      </c>
-      <c r="E18" s="21" t="s">
+      <c r="D18" s="17" t="s">
+        <v>182</v>
+      </c>
+      <c r="E18" s="17" t="s">
         <v>54</v>
       </c>
-      <c r="F18" s="21" t="s">
+      <c r="F18" s="17" t="s">
         <v>55</v>
       </c>
-      <c r="G18" s="31" t="s">
+      <c r="G18" s="27" t="s">
         <v>56</v>
       </c>
-      <c r="H18" s="20" t="s">
+      <c r="H18" s="16" t="s">
         <v>52</v>
       </c>
-      <c r="I18" s="21" t="s">
+      <c r="I18" s="17" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="19" spans="1:9" s="8" customFormat="1" ht="55.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="79"/>
-      <c r="B19" s="79"/>
-      <c r="C19" s="20">
+    <row r="19" spans="1:9" s="4" customFormat="1" ht="41.4" x14ac:dyDescent="0.3">
+      <c r="A19" s="63"/>
+      <c r="B19" s="63"/>
+      <c r="C19" s="16">
         <v>12.3</v>
       </c>
-      <c r="D19" s="21" t="s">
-        <v>126</v>
-      </c>
-      <c r="E19" s="21" t="s">
+      <c r="D19" s="17" t="s">
+        <v>182</v>
+      </c>
+      <c r="E19" s="17" t="s">
         <v>57</v>
       </c>
-      <c r="F19" s="21" t="s">
+      <c r="F19" s="17" t="s">
         <v>58</v>
       </c>
-      <c r="G19" s="31" t="s">
+      <c r="G19" s="27" t="s">
         <v>59</v>
       </c>
-      <c r="H19" s="20" t="s">
+      <c r="H19" s="16" t="s">
         <v>52</v>
       </c>
-      <c r="I19" s="21"/>
-    </row>
-    <row r="20" spans="1:9" s="8" customFormat="1" ht="138" x14ac:dyDescent="0.3">
-      <c r="A20" s="80"/>
-      <c r="B20" s="80"/>
-      <c r="C20" s="20">
+      <c r="I19" s="17"/>
+    </row>
+    <row r="20" spans="1:9" s="4" customFormat="1" ht="138" x14ac:dyDescent="0.3">
+      <c r="A20" s="63"/>
+      <c r="B20" s="63"/>
+      <c r="C20" s="16">
         <v>12.4</v>
       </c>
-      <c r="D20" s="21" t="s">
+      <c r="D20" s="17" t="s">
         <v>182</v>
       </c>
-      <c r="E20" s="21" t="s">
+      <c r="E20" s="17" t="s">
         <v>184</v>
       </c>
-      <c r="F20" s="21" t="s">
+      <c r="F20" s="17" t="s">
         <v>185</v>
       </c>
-      <c r="G20" s="21" t="s">
+      <c r="G20" s="17" t="s">
         <v>186</v>
       </c>
-      <c r="H20" s="20"/>
-      <c r="I20" s="21"/>
-    </row>
-    <row r="21" spans="1:9" s="8" customFormat="1" ht="41.4" x14ac:dyDescent="0.3">
-      <c r="A21" s="81"/>
-      <c r="B21" s="81"/>
-      <c r="C21" s="20"/>
-      <c r="D21" s="21"/>
-      <c r="E21" s="21"/>
-      <c r="F21" s="21"/>
-      <c r="G21" s="31" t="s">
+      <c r="H20" s="16"/>
+      <c r="I20" s="17"/>
+    </row>
+    <row r="21" spans="1:9" s="4" customFormat="1" ht="124.2" x14ac:dyDescent="0.3">
+      <c r="A21" s="63"/>
+      <c r="B21" s="63"/>
+      <c r="C21" s="16">
+        <v>12.5</v>
+      </c>
+      <c r="D21" s="17" t="s">
         <v>187</v>
       </c>
-      <c r="H21" s="20"/>
-      <c r="I21" s="21"/>
-    </row>
-    <row r="22" spans="1:9" s="8" customFormat="1" ht="41.4" x14ac:dyDescent="0.3">
-      <c r="A22" s="72">
+      <c r="E21" s="17" t="s">
+        <v>189</v>
+      </c>
+      <c r="F21" s="17" t="s">
+        <v>188</v>
+      </c>
+      <c r="G21" s="27" t="s">
+        <v>190</v>
+      </c>
+      <c r="H21" s="16"/>
+      <c r="I21" s="17"/>
+    </row>
+    <row r="22" spans="1:9" s="4" customFormat="1" ht="41.4" x14ac:dyDescent="0.3">
+      <c r="A22" s="50">
         <v>14</v>
       </c>
-      <c r="B22" s="72" t="s">
+      <c r="B22" s="50" t="s">
         <v>61</v>
       </c>
-      <c r="C22" s="76">
+      <c r="C22" s="47">
         <v>14.1</v>
       </c>
-      <c r="D22" s="77" t="s">
+      <c r="D22" s="48" t="s">
         <v>15</v>
       </c>
-      <c r="E22" s="77" t="s">
+      <c r="E22" s="48" t="s">
         <v>146</v>
       </c>
-      <c r="F22" s="77" t="s">
+      <c r="F22" s="48" t="s">
         <v>147</v>
       </c>
-      <c r="G22" s="77" t="s">
+      <c r="G22" s="48" t="s">
         <v>171</v>
       </c>
-      <c r="H22" s="76" t="s">
+      <c r="H22" s="47" t="s">
         <v>102</v>
       </c>
-      <c r="I22" s="77" t="s">
+      <c r="I22" s="48" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="23" spans="1:9" s="8" customFormat="1" ht="55.2" x14ac:dyDescent="0.3">
-      <c r="A23" s="73"/>
-      <c r="B23" s="73"/>
-      <c r="C23" s="76">
+    <row r="23" spans="1:9" s="4" customFormat="1" ht="41.4" x14ac:dyDescent="0.3">
+      <c r="A23" s="50"/>
+      <c r="B23" s="50"/>
+      <c r="C23" s="47">
         <v>14.2</v>
       </c>
-      <c r="D23" s="77" t="s">
+      <c r="D23" s="48" t="s">
         <v>15</v>
       </c>
-      <c r="E23" s="77" t="s">
+      <c r="E23" s="48" t="s">
         <v>148</v>
       </c>
-      <c r="F23" s="77" t="s">
+      <c r="F23" s="48" t="s">
         <v>149</v>
       </c>
-      <c r="G23" s="77" t="s">
+      <c r="G23" s="48" t="s">
         <v>172</v>
       </c>
-      <c r="H23" s="76" t="s">
+      <c r="H23" s="47" t="s">
         <v>102</v>
       </c>
-      <c r="I23" s="77" t="s">
+      <c r="I23" s="48" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="24" spans="1:9" s="8" customFormat="1" ht="55.2" x14ac:dyDescent="0.3">
-      <c r="A24" s="73"/>
-      <c r="B24" s="73"/>
-      <c r="C24" s="76">
+    <row r="24" spans="1:9" s="4" customFormat="1" ht="41.4" x14ac:dyDescent="0.3">
+      <c r="A24" s="50"/>
+      <c r="B24" s="50"/>
+      <c r="C24" s="47">
         <v>14.3</v>
       </c>
-      <c r="D24" s="77" t="s">
+      <c r="D24" s="48" t="s">
         <v>150</v>
       </c>
-      <c r="E24" s="77" t="s">
+      <c r="E24" s="48" t="s">
         <v>151</v>
       </c>
-      <c r="F24" s="77" t="s">
+      <c r="F24" s="48" t="s">
         <v>152</v>
       </c>
-      <c r="G24" s="77" t="s">
+      <c r="G24" s="48" t="s">
         <v>173</v>
       </c>
-      <c r="H24" s="76" t="s">
+      <c r="H24" s="47" t="s">
         <v>102</v>
       </c>
-      <c r="I24" s="77" t="s">
+      <c r="I24" s="48" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="25" spans="1:9" s="8" customFormat="1" ht="55.2" x14ac:dyDescent="0.3">
-      <c r="A25" s="73"/>
-      <c r="B25" s="73"/>
-      <c r="C25" s="76">
+    <row r="25" spans="1:9" s="4" customFormat="1" ht="55.2" x14ac:dyDescent="0.3">
+      <c r="A25" s="50"/>
+      <c r="B25" s="50"/>
+      <c r="C25" s="47">
         <v>14.4</v>
       </c>
-      <c r="D25" s="77" t="s">
+      <c r="D25" s="48" t="s">
         <v>15</v>
       </c>
-      <c r="E25" s="77" t="s">
+      <c r="E25" s="48" t="s">
         <v>153</v>
       </c>
-      <c r="F25" s="77" t="s">
+      <c r="F25" s="48" t="s">
         <v>154</v>
       </c>
-      <c r="G25" s="77" t="s">
+      <c r="G25" s="48" t="s">
         <v>174</v>
       </c>
-      <c r="H25" s="76" t="s">
+      <c r="H25" s="47" t="s">
         <v>102</v>
       </c>
-      <c r="I25" s="77" t="s">
+      <c r="I25" s="48" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="26" spans="1:9" s="8" customFormat="1" ht="55.2" x14ac:dyDescent="0.3">
-      <c r="A26" s="73"/>
-      <c r="B26" s="73"/>
-      <c r="C26" s="76">
+    <row r="26" spans="1:9" s="4" customFormat="1" ht="41.4" x14ac:dyDescent="0.3">
+      <c r="A26" s="50"/>
+      <c r="B26" s="50"/>
+      <c r="C26" s="47">
         <v>14.5</v>
       </c>
-      <c r="D26" s="77" t="s">
+      <c r="D26" s="48" t="s">
         <v>15</v>
       </c>
-      <c r="E26" s="77" t="s">
+      <c r="E26" s="48" t="s">
         <v>155</v>
       </c>
-      <c r="F26" s="77" t="s">
+      <c r="F26" s="48" t="s">
         <v>156</v>
       </c>
-      <c r="G26" s="77" t="s">
+      <c r="G26" s="48" t="s">
         <v>175</v>
       </c>
-      <c r="H26" s="76" t="s">
+      <c r="H26" s="47" t="s">
         <v>102</v>
       </c>
-      <c r="I26" s="77" t="s">
+      <c r="I26" s="48" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="27" spans="1:9" s="8" customFormat="1" ht="41.4" x14ac:dyDescent="0.3">
-      <c r="A27" s="73"/>
-      <c r="B27" s="73"/>
-      <c r="C27" s="76">
+    <row r="27" spans="1:9" s="4" customFormat="1" ht="41.4" x14ac:dyDescent="0.3">
+      <c r="A27" s="50"/>
+      <c r="B27" s="50"/>
+      <c r="C27" s="47">
         <v>14.6</v>
       </c>
-      <c r="D27" s="77" t="s">
+      <c r="D27" s="48" t="s">
         <v>15</v>
       </c>
-      <c r="E27" s="77" t="s">
+      <c r="E27" s="48" t="s">
         <v>157</v>
       </c>
-      <c r="F27" s="77" t="s">
+      <c r="F27" s="48" t="s">
         <v>158</v>
       </c>
-      <c r="G27" s="77" t="s">
+      <c r="G27" s="48" t="s">
         <v>181</v>
       </c>
-      <c r="H27" s="76" t="s">
+      <c r="H27" s="47" t="s">
         <v>102</v>
       </c>
-      <c r="I27" s="77" t="s">
+      <c r="I27" s="48" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="28" spans="1:9" s="8" customFormat="1" ht="69" x14ac:dyDescent="0.3">
-      <c r="A28" s="73"/>
-      <c r="B28" s="73"/>
-      <c r="C28" s="76">
+    <row r="28" spans="1:9" s="4" customFormat="1" ht="41.4" x14ac:dyDescent="0.3">
+      <c r="A28" s="50"/>
+      <c r="B28" s="50"/>
+      <c r="C28" s="47">
         <v>14.7</v>
       </c>
-      <c r="D28" s="77" t="s">
+      <c r="D28" s="48" t="s">
         <v>15</v>
       </c>
-      <c r="E28" s="77" t="s">
+      <c r="E28" s="48" t="s">
         <v>159</v>
       </c>
-      <c r="F28" s="77" t="s">
+      <c r="F28" s="48" t="s">
         <v>160</v>
       </c>
-      <c r="G28" s="77" t="s">
+      <c r="G28" s="48" t="s">
         <v>176</v>
       </c>
-      <c r="H28" s="76" t="s">
+      <c r="H28" s="47" t="s">
         <v>102</v>
       </c>
-      <c r="I28" s="77" t="s">
+      <c r="I28" s="48" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="29" spans="1:9" s="8" customFormat="1" ht="55.2" x14ac:dyDescent="0.3">
-      <c r="A29" s="73"/>
-      <c r="B29" s="73"/>
-      <c r="C29" s="76">
+    <row r="29" spans="1:9" s="4" customFormat="1" ht="41.4" x14ac:dyDescent="0.3">
+      <c r="A29" s="50"/>
+      <c r="B29" s="50"/>
+      <c r="C29" s="47">
         <v>14.8</v>
       </c>
-      <c r="D29" s="77" t="s">
+      <c r="D29" s="48" t="s">
         <v>15</v>
       </c>
-      <c r="E29" s="77" t="s">
+      <c r="E29" s="48" t="s">
         <v>161</v>
       </c>
-      <c r="F29" s="77" t="s">
+      <c r="F29" s="48" t="s">
         <v>162</v>
       </c>
-      <c r="G29" s="77" t="s">
+      <c r="G29" s="48" t="s">
         <v>177</v>
       </c>
-      <c r="H29" s="76" t="s">
+      <c r="H29" s="47" t="s">
         <v>142</v>
       </c>
-      <c r="I29" s="77" t="s">
+      <c r="I29" s="48" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="30" spans="1:9" s="8" customFormat="1" ht="55.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A30" s="73"/>
-      <c r="B30" s="73"/>
-      <c r="C30" s="76">
+    <row r="30" spans="1:9" s="4" customFormat="1" ht="55.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A30" s="50"/>
+      <c r="B30" s="50"/>
+      <c r="C30" s="47">
         <v>14.9</v>
       </c>
-      <c r="D30" s="77" t="s">
+      <c r="D30" s="48" t="s">
         <v>15</v>
       </c>
-      <c r="E30" s="77" t="s">
+      <c r="E30" s="48" t="s">
         <v>163</v>
       </c>
-      <c r="F30" s="77" t="s">
+      <c r="F30" s="48" t="s">
         <v>164</v>
       </c>
-      <c r="G30" s="77" t="s">
+      <c r="G30" s="48" t="s">
         <v>178</v>
       </c>
-      <c r="H30" s="76" t="s">
+      <c r="H30" s="47" t="s">
         <v>142</v>
       </c>
-      <c r="I30" s="77" t="s">
+      <c r="I30" s="48" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="31" spans="1:9" s="8" customFormat="1" ht="69" x14ac:dyDescent="0.3">
-      <c r="A31" s="73"/>
-      <c r="B31" s="73"/>
-      <c r="C31" s="76">
+    <row r="31" spans="1:9" s="4" customFormat="1" ht="55.2" x14ac:dyDescent="0.3">
+      <c r="A31" s="50"/>
+      <c r="B31" s="50"/>
+      <c r="C31" s="47">
         <v>14.1</v>
       </c>
-      <c r="D31" s="77" t="s">
+      <c r="D31" s="48" t="s">
         <v>15</v>
       </c>
-      <c r="E31" s="77" t="s">
+      <c r="E31" s="48" t="s">
         <v>165</v>
       </c>
-      <c r="F31" s="77" t="s">
+      <c r="F31" s="48" t="s">
         <v>166</v>
       </c>
-      <c r="G31" s="77" t="s">
+      <c r="G31" s="48" t="s">
         <v>179</v>
       </c>
-      <c r="H31" s="76" t="s">
+      <c r="H31" s="47" t="s">
         <v>142</v>
       </c>
-      <c r="I31" s="77" t="s">
+      <c r="I31" s="48" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="32" spans="1:9" s="8" customFormat="1" ht="41.4" x14ac:dyDescent="0.3">
-      <c r="A32" s="73"/>
-      <c r="B32" s="73"/>
-      <c r="C32" s="76">
+    <row r="32" spans="1:9" s="4" customFormat="1" ht="41.4" x14ac:dyDescent="0.3">
+      <c r="A32" s="50"/>
+      <c r="B32" s="50"/>
+      <c r="C32" s="47">
         <v>14.11</v>
       </c>
-      <c r="D32" s="77" t="s">
+      <c r="D32" s="48" t="s">
         <v>15</v>
       </c>
-      <c r="E32" s="77" t="s">
+      <c r="E32" s="48" t="s">
         <v>167</v>
       </c>
-      <c r="F32" s="77" t="s">
+      <c r="F32" s="48" t="s">
         <v>168</v>
       </c>
-      <c r="G32" s="77" t="s">
+      <c r="G32" s="48" t="s">
         <v>180</v>
       </c>
-      <c r="H32" s="76" t="s">
+      <c r="H32" s="47" t="s">
         <v>142</v>
       </c>
-      <c r="I32" s="77" t="s">
+      <c r="I32" s="48" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="33" spans="1:9" s="8" customFormat="1" ht="27.6" x14ac:dyDescent="0.3">
-      <c r="A33" s="64">
+    <row r="33" spans="1:9" s="4" customFormat="1" ht="27.6" x14ac:dyDescent="0.3">
+      <c r="A33" s="52">
         <v>15</v>
       </c>
-      <c r="B33" s="64" t="s">
+      <c r="B33" s="52" t="s">
         <v>63</v>
       </c>
-      <c r="C33" s="23">
+      <c r="C33" s="19">
         <v>15.1</v>
       </c>
-      <c r="D33" s="24" t="s">
+      <c r="D33" s="20" t="s">
         <v>64</v>
       </c>
-      <c r="E33" s="24" t="s">
+      <c r="E33" s="20" t="s">
         <v>65</v>
       </c>
-      <c r="F33" s="24" t="s">
+      <c r="F33" s="20" t="s">
         <v>66</v>
       </c>
-      <c r="G33" s="32" t="s">
+      <c r="G33" s="20" t="s">
         <v>67</v>
       </c>
-      <c r="H33" s="23" t="s">
+      <c r="H33" s="19" t="s">
         <v>143</v>
       </c>
-      <c r="I33" s="24" t="s">
+      <c r="I33" s="20" t="s">
         <v>144</v>
       </c>
     </row>
-    <row r="34" spans="1:9" s="8" customFormat="1" ht="27.6" x14ac:dyDescent="0.3">
-      <c r="A34" s="58"/>
-      <c r="B34" s="58"/>
-      <c r="C34" s="23">
+    <row r="34" spans="1:9" s="4" customFormat="1" ht="27.6" x14ac:dyDescent="0.3">
+      <c r="A34" s="59"/>
+      <c r="B34" s="59"/>
+      <c r="C34" s="19">
         <v>15.2</v>
       </c>
-      <c r="D34" s="24" t="s">
+      <c r="D34" s="20" t="s">
         <v>64</v>
       </c>
-      <c r="E34" s="24" t="s">
+      <c r="E34" s="20" t="s">
         <v>68</v>
       </c>
-      <c r="F34" s="24" t="s">
+      <c r="F34" s="20" t="s">
         <v>69</v>
       </c>
-      <c r="G34" s="32" t="s">
+      <c r="G34" s="20" t="s">
         <v>70</v>
       </c>
-      <c r="H34" s="23" t="s">
+      <c r="H34" s="19" t="s">
         <v>143</v>
       </c>
-      <c r="I34" s="24" t="s">
+      <c r="I34" s="20" t="s">
         <v>144</v>
       </c>
     </row>
-    <row r="35" spans="1:9" s="8" customFormat="1" ht="27.6" x14ac:dyDescent="0.3">
-      <c r="A35" s="58"/>
-      <c r="B35" s="58"/>
-      <c r="C35" s="23">
+    <row r="35" spans="1:9" s="4" customFormat="1" ht="27.6" x14ac:dyDescent="0.3">
+      <c r="A35" s="59"/>
+      <c r="B35" s="59"/>
+      <c r="C35" s="19">
         <v>15.3</v>
       </c>
-      <c r="D35" s="24" t="s">
+      <c r="D35" s="20" t="s">
         <v>64</v>
       </c>
-      <c r="E35" s="24" t="s">
+      <c r="E35" s="20" t="s">
         <v>71</v>
       </c>
-      <c r="F35" s="24" t="s">
+      <c r="F35" s="20" t="s">
         <v>72</v>
       </c>
-      <c r="G35" s="32" t="s">
+      <c r="G35" s="20" t="s">
         <v>73</v>
       </c>
-      <c r="H35" s="23" t="s">
+      <c r="H35" s="19" t="s">
         <v>143</v>
       </c>
-      <c r="I35" s="24" t="s">
+      <c r="I35" s="20" t="s">
         <v>144</v>
       </c>
     </row>
-    <row r="36" spans="1:9" s="8" customFormat="1" ht="27.6" x14ac:dyDescent="0.3">
-      <c r="A36" s="58"/>
-      <c r="B36" s="58"/>
-      <c r="C36" s="23">
+    <row r="36" spans="1:9" s="4" customFormat="1" ht="27.6" x14ac:dyDescent="0.3">
+      <c r="A36" s="59"/>
+      <c r="B36" s="59"/>
+      <c r="C36" s="19">
         <v>15.4</v>
       </c>
-      <c r="D36" s="24" t="s">
+      <c r="D36" s="20" t="s">
         <v>64</v>
       </c>
-      <c r="E36" s="24" t="s">
+      <c r="E36" s="20" t="s">
         <v>74</v>
       </c>
-      <c r="F36" s="24" t="s">
+      <c r="F36" s="20" t="s">
         <v>75</v>
       </c>
-      <c r="G36" s="32" t="s">
+      <c r="G36" s="20" t="s">
         <v>76</v>
       </c>
-      <c r="H36" s="23" t="s">
+      <c r="H36" s="19" t="s">
         <v>145</v>
       </c>
-      <c r="I36" s="24" t="s">
+      <c r="I36" s="20" t="s">
         <v>144</v>
       </c>
     </row>
-    <row r="37" spans="1:9" s="8" customFormat="1" ht="27.6" x14ac:dyDescent="0.3">
-      <c r="A37" s="60"/>
-      <c r="B37" s="60"/>
-      <c r="C37" s="23">
+    <row r="37" spans="1:9" s="4" customFormat="1" ht="27.6" x14ac:dyDescent="0.3">
+      <c r="A37" s="59"/>
+      <c r="B37" s="59"/>
+      <c r="C37" s="19">
         <v>15.5</v>
       </c>
-      <c r="D37" s="24" t="s">
+      <c r="D37" s="20" t="s">
         <v>64</v>
       </c>
-      <c r="E37" s="24" t="s">
+      <c r="E37" s="20" t="s">
         <v>77</v>
       </c>
-      <c r="F37" s="24" t="s">
+      <c r="F37" s="20" t="s">
         <v>78</v>
       </c>
-      <c r="G37" s="32" t="s">
+      <c r="G37" s="20" t="s">
         <v>79</v>
       </c>
-      <c r="H37" s="23" t="s">
+      <c r="H37" s="19" t="s">
         <v>145</v>
       </c>
-      <c r="I37" s="24" t="s">
+      <c r="I37" s="20" t="s">
         <v>144</v>
       </c>
     </row>
-    <row r="38" spans="1:9" s="8" customFormat="1" ht="27.6" x14ac:dyDescent="0.3">
-      <c r="A38" s="69">
+    <row r="38" spans="1:9" s="4" customFormat="1" ht="27.6" x14ac:dyDescent="0.3">
+      <c r="A38" s="51">
         <v>16</v>
       </c>
-      <c r="B38" s="69" t="s">
+      <c r="B38" s="51" t="s">
         <v>80</v>
       </c>
-      <c r="C38" s="25">
+      <c r="C38" s="21">
         <v>16.100000000000001</v>
       </c>
-      <c r="D38" s="26" t="s">
+      <c r="D38" s="22" t="s">
         <v>81</v>
       </c>
-      <c r="E38" s="26" t="s">
+      <c r="E38" s="22" t="s">
         <v>82</v>
       </c>
-      <c r="F38" s="26" t="s">
+      <c r="F38" s="22" t="s">
         <v>83</v>
       </c>
-      <c r="G38" s="52" t="s">
+      <c r="G38" s="45" t="s">
         <v>84</v>
       </c>
-      <c r="H38" s="53" t="s">
+      <c r="H38" s="44" t="s">
         <v>145</v>
       </c>
-      <c r="I38" s="54" t="s">
+      <c r="I38" s="45" t="s">
         <v>144</v>
       </c>
     </row>
-    <row r="39" spans="1:9" s="8" customFormat="1" ht="27.6" x14ac:dyDescent="0.3">
-      <c r="A39" s="60"/>
-      <c r="B39" s="60"/>
-      <c r="C39" s="25">
+    <row r="39" spans="1:9" s="4" customFormat="1" ht="27.6" x14ac:dyDescent="0.3">
+      <c r="A39" s="59"/>
+      <c r="B39" s="59"/>
+      <c r="C39" s="21">
         <v>16.2</v>
       </c>
-      <c r="D39" s="26" t="s">
+      <c r="D39" s="22" t="s">
         <v>85</v>
       </c>
-      <c r="E39" s="26" t="s">
+      <c r="E39" s="22" t="s">
         <v>86</v>
       </c>
-      <c r="F39" s="26" t="s">
+      <c r="F39" s="22" t="s">
         <v>87</v>
       </c>
-      <c r="G39" s="33" t="s">
+      <c r="G39" s="22" t="s">
         <v>88</v>
       </c>
-      <c r="H39" s="53" t="s">
+      <c r="H39" s="44" t="s">
         <v>145</v>
       </c>
-      <c r="I39" s="54" t="s">
+      <c r="I39" s="45" t="s">
         <v>144</v>
       </c>
     </row>
-    <row r="40" spans="1:9" s="8" customFormat="1" ht="27.6" x14ac:dyDescent="0.3">
-      <c r="A40" s="57">
+    <row r="40" spans="1:9" s="4" customFormat="1" ht="27.6" x14ac:dyDescent="0.3">
+      <c r="A40" s="56">
         <v>17</v>
       </c>
-      <c r="B40" s="57" t="s">
+      <c r="B40" s="56" t="s">
         <v>89</v>
       </c>
-      <c r="C40" s="9">
+      <c r="C40" s="5">
         <v>17.100000000000001</v>
       </c>
-      <c r="D40" s="10" t="s">
+      <c r="D40" s="6" t="s">
         <v>90</v>
       </c>
-      <c r="E40" s="43" t="s">
+      <c r="E40" s="37" t="s">
         <v>169</v>
       </c>
-      <c r="F40" s="10" t="s">
+      <c r="F40" s="6" t="s">
         <v>91</v>
       </c>
-      <c r="G40" s="44" t="s">
+      <c r="G40" s="37" t="s">
         <v>170</v>
       </c>
-      <c r="H40" s="9" t="s">
+      <c r="H40" s="5" t="s">
         <v>102</v>
       </c>
-      <c r="I40" s="43" t="s">
+      <c r="I40" s="37" t="s">
         <v>124</v>
       </c>
     </row>
-    <row r="41" spans="1:9" s="8" customFormat="1" ht="27.6" x14ac:dyDescent="0.3">
-      <c r="A41" s="58"/>
-      <c r="B41" s="58"/>
-      <c r="C41" s="9">
+    <row r="41" spans="1:9" s="4" customFormat="1" ht="27.6" x14ac:dyDescent="0.3">
+      <c r="A41" s="59"/>
+      <c r="B41" s="59"/>
+      <c r="C41" s="5">
         <v>17.2</v>
       </c>
-      <c r="D41" s="10" t="s">
+      <c r="D41" s="6" t="s">
         <v>90</v>
       </c>
-      <c r="E41" s="43" t="s">
+      <c r="E41" s="37" t="s">
         <v>112</v>
       </c>
-      <c r="F41" s="10" t="s">
+      <c r="F41" s="6" t="s">
         <v>92</v>
       </c>
-      <c r="G41" s="44" t="s">
+      <c r="G41" s="37" t="s">
         <v>93</v>
       </c>
-      <c r="H41" s="9" t="s">
+      <c r="H41" s="5" t="s">
         <v>102</v>
       </c>
-      <c r="I41" s="43" t="s">
+      <c r="I41" s="37" t="s">
         <v>124</v>
       </c>
     </row>
-    <row r="42" spans="1:9" s="8" customFormat="1" ht="41.4" x14ac:dyDescent="0.3">
-      <c r="A42" s="58"/>
-      <c r="B42" s="58"/>
-      <c r="C42" s="9">
+    <row r="42" spans="1:9" s="4" customFormat="1" ht="27.6" x14ac:dyDescent="0.3">
+      <c r="A42" s="59"/>
+      <c r="B42" s="59"/>
+      <c r="C42" s="5">
         <v>17.3</v>
       </c>
-      <c r="D42" s="10" t="s">
+      <c r="D42" s="6" t="s">
         <v>90</v>
       </c>
-      <c r="E42" s="10" t="s">
+      <c r="E42" s="6" t="s">
         <v>94</v>
       </c>
-      <c r="F42" s="43" t="s">
+      <c r="F42" s="37" t="s">
         <v>113</v>
       </c>
-      <c r="G42" s="44" t="s">
+      <c r="G42" s="37" t="s">
         <v>116</v>
       </c>
-      <c r="H42" s="9" t="s">
+      <c r="H42" s="5" t="s">
         <v>102</v>
       </c>
-      <c r="I42" s="43" t="s">
+      <c r="I42" s="37" t="s">
         <v>124</v>
       </c>
     </row>
-    <row r="43" spans="1:9" s="8" customFormat="1" ht="27.6" x14ac:dyDescent="0.3">
-      <c r="A43" s="58"/>
-      <c r="B43" s="58"/>
-      <c r="C43" s="9">
+    <row r="43" spans="1:9" s="4" customFormat="1" ht="27.6" x14ac:dyDescent="0.3">
+      <c r="A43" s="59"/>
+      <c r="B43" s="59"/>
+      <c r="C43" s="5">
         <v>17.399999999999999</v>
       </c>
-      <c r="D43" s="10" t="s">
+      <c r="D43" s="6" t="s">
         <v>90</v>
       </c>
-      <c r="E43" s="43" t="s">
+      <c r="E43" s="37" t="s">
         <v>115</v>
       </c>
-      <c r="F43" s="43" t="s">
+      <c r="F43" s="37" t="s">
         <v>114</v>
       </c>
-      <c r="G43" s="44" t="s">
+      <c r="G43" s="37" t="s">
         <v>120</v>
       </c>
-      <c r="H43" s="9" t="s">
+      <c r="H43" s="5" t="s">
         <v>102</v>
       </c>
-      <c r="I43" s="43" t="s">
+      <c r="I43" s="37" t="s">
         <v>124</v>
       </c>
     </row>
-    <row r="44" spans="1:9" s="8" customFormat="1" ht="27.6" x14ac:dyDescent="0.3">
-      <c r="A44" s="58"/>
-      <c r="B44" s="58"/>
-      <c r="C44" s="9">
+    <row r="44" spans="1:9" s="4" customFormat="1" ht="27.6" x14ac:dyDescent="0.3">
+      <c r="A44" s="59"/>
+      <c r="B44" s="59"/>
+      <c r="C44" s="5">
         <v>17.5</v>
       </c>
-      <c r="D44" s="10" t="s">
+      <c r="D44" s="6" t="s">
         <v>90</v>
       </c>
-      <c r="E44" s="43" t="s">
+      <c r="E44" s="37" t="s">
         <v>117</v>
       </c>
-      <c r="F44" s="43" t="s">
+      <c r="F44" s="37" t="s">
         <v>118</v>
       </c>
-      <c r="G44" s="44" t="s">
+      <c r="G44" s="37" t="s">
         <v>119</v>
       </c>
-      <c r="H44" s="9" t="s">
+      <c r="H44" s="5" t="s">
         <v>102</v>
       </c>
-      <c r="I44" s="43" t="s">
+      <c r="I44" s="37" t="s">
         <v>124</v>
       </c>
     </row>
-    <row r="45" spans="1:9" s="8" customFormat="1" ht="27.6" x14ac:dyDescent="0.3">
-      <c r="A45" s="58"/>
-      <c r="B45" s="58"/>
-      <c r="C45" s="9">
+    <row r="45" spans="1:9" s="4" customFormat="1" ht="27.6" x14ac:dyDescent="0.3">
+      <c r="A45" s="59"/>
+      <c r="B45" s="59"/>
+      <c r="C45" s="5">
         <v>17.600000000000001</v>
       </c>
-      <c r="D45" s="10" t="s">
+      <c r="D45" s="6" t="s">
         <v>90</v>
       </c>
-      <c r="E45" s="10" t="s">
+      <c r="E45" s="6" t="s">
         <v>95</v>
       </c>
-      <c r="F45" s="43" t="s">
+      <c r="F45" s="37" t="s">
         <v>121</v>
       </c>
-      <c r="G45" s="44" t="s">
+      <c r="G45" s="37" t="s">
         <v>122</v>
       </c>
-      <c r="H45" s="9" t="s">
+      <c r="H45" s="5" t="s">
         <v>102</v>
       </c>
-      <c r="I45" s="43" t="s">
+      <c r="I45" s="37" t="s">
         <v>124</v>
       </c>
     </row>
-    <row r="46" spans="1:9" s="8" customFormat="1" ht="27.6" x14ac:dyDescent="0.3">
-      <c r="A46" s="58"/>
-      <c r="B46" s="58"/>
-      <c r="C46" s="9">
+    <row r="46" spans="1:9" s="4" customFormat="1" ht="27.6" x14ac:dyDescent="0.3">
+      <c r="A46" s="59"/>
+      <c r="B46" s="59"/>
+      <c r="C46" s="5">
         <v>17.7</v>
       </c>
-      <c r="D46" s="10" t="s">
+      <c r="D46" s="6" t="s">
         <v>90</v>
       </c>
-      <c r="E46" s="10" t="s">
+      <c r="E46" s="6" t="s">
         <v>96</v>
       </c>
-      <c r="F46" s="43" t="s">
+      <c r="F46" s="37" t="s">
         <v>123</v>
       </c>
-      <c r="G46" s="44" t="s">
+      <c r="G46" s="37" t="s">
         <v>130</v>
       </c>
-      <c r="H46" s="9" t="s">
+      <c r="H46" s="5" t="s">
         <v>102</v>
       </c>
-      <c r="I46" s="43" t="s">
+      <c r="I46" s="37" t="s">
         <v>124</v>
       </c>
     </row>
-    <row r="47" spans="1:9" s="8" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A47" s="2"/>
-      <c r="B47" s="3"/>
-      <c r="C47" s="3"/>
-      <c r="D47" s="3"/>
-      <c r="E47" s="3"/>
-      <c r="F47" s="3"/>
-      <c r="G47" s="4"/>
-      <c r="H47" s="6"/>
-      <c r="I47" s="3"/>
-    </row>
-    <row r="48" spans="1:9" s="8" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A48" s="7"/>
-      <c r="B48" s="2"/>
-      <c r="C48" s="2"/>
-      <c r="D48" s="3"/>
-      <c r="E48" s="2"/>
-      <c r="F48" s="3"/>
-      <c r="G48" s="4"/>
-      <c r="H48" s="2"/>
-      <c r="I48" s="3"/>
-    </row>
-    <row r="49" spans="1:12" s="8" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A49" s="7"/>
-      <c r="B49" s="2"/>
-      <c r="C49" s="2"/>
-      <c r="D49" s="3"/>
-      <c r="E49" s="2"/>
-      <c r="F49" s="3"/>
-      <c r="G49" s="3"/>
-      <c r="H49" s="2"/>
-      <c r="I49" s="3"/>
-    </row>
-    <row r="50" spans="1:12" s="8" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A50" s="7"/>
-      <c r="B50" s="55"/>
-      <c r="C50" s="56"/>
-      <c r="D50" s="56"/>
-      <c r="E50" s="56"/>
-      <c r="F50" s="56"/>
-      <c r="G50" s="56"/>
-      <c r="H50" s="56"/>
-      <c r="I50" s="56"/>
-      <c r="J50" s="5"/>
-      <c r="K50" s="5"/>
-      <c r="L50" s="5"/>
-    </row>
-    <row r="51" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A51" s="3"/>
-      <c r="B51" s="3"/>
-      <c r="C51" s="3"/>
-      <c r="E51" s="3"/>
-      <c r="H51" s="3"/>
-    </row>
-    <row r="52" spans="1:12" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="D52" s="2"/>
-      <c r="F52" s="2"/>
-      <c r="G52" s="2"/>
-      <c r="I52" s="2"/>
-    </row>
-    <row r="53" spans="1:12" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="D53" s="2"/>
-      <c r="F53" s="2"/>
-      <c r="G53" s="2"/>
-      <c r="I53" s="2"/>
-    </row>
-    <row r="54" spans="1:12" ht="36.450000000000003" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A54" s="55"/>
-      <c r="B54" s="55"/>
-      <c r="C54" s="55"/>
-      <c r="D54" s="55"/>
-      <c r="E54" s="55"/>
-      <c r="F54" s="55"/>
-      <c r="G54" s="55"/>
-      <c r="H54" s="55"/>
-      <c r="I54" s="55"/>
+    <row r="47" spans="1:9" s="4" customFormat="1" ht="82.8" x14ac:dyDescent="0.3">
+      <c r="A47" s="64">
+        <v>18</v>
+      </c>
+      <c r="B47" s="65" t="s">
+        <v>191</v>
+      </c>
+      <c r="C47" s="66">
+        <v>18.100000000000001</v>
+      </c>
+      <c r="D47" s="57" t="s">
+        <v>192</v>
+      </c>
+      <c r="E47" s="57" t="s">
+        <v>193</v>
+      </c>
+      <c r="F47" s="57" t="s">
+        <v>194</v>
+      </c>
+      <c r="G47" s="57" t="s">
+        <v>198</v>
+      </c>
+      <c r="H47" s="66"/>
+      <c r="I47" s="67"/>
+    </row>
+    <row r="48" spans="1:9" s="4" customFormat="1" ht="124.2" x14ac:dyDescent="0.3">
+      <c r="A48" s="64"/>
+      <c r="B48" s="65"/>
+      <c r="C48" s="68">
+        <v>18.2</v>
+      </c>
+      <c r="D48" s="57" t="s">
+        <v>195</v>
+      </c>
+      <c r="E48" s="57" t="s">
+        <v>196</v>
+      </c>
+      <c r="F48" s="57" t="s">
+        <v>188</v>
+      </c>
+      <c r="G48" s="57" t="s">
+        <v>197</v>
+      </c>
+      <c r="H48" s="66"/>
+      <c r="I48" s="67"/>
+    </row>
+    <row r="49" spans="1:12" s="4" customFormat="1" ht="82.8" x14ac:dyDescent="0.3">
+      <c r="A49" s="64">
+        <v>19</v>
+      </c>
+      <c r="B49" s="65" t="s">
+        <v>199</v>
+      </c>
+      <c r="C49" s="66">
+        <v>19.100000000000001</v>
+      </c>
+      <c r="D49" s="57" t="s">
+        <v>200</v>
+      </c>
+      <c r="E49" s="57" t="s">
+        <v>202</v>
+      </c>
+      <c r="F49" s="57" t="s">
+        <v>204</v>
+      </c>
+      <c r="G49" s="57" t="s">
+        <v>205</v>
+      </c>
+      <c r="H49" s="66"/>
+      <c r="I49" s="67"/>
+    </row>
+    <row r="50" spans="1:12" s="4" customFormat="1" ht="124.2" x14ac:dyDescent="0.3">
+      <c r="A50" s="64"/>
+      <c r="B50" s="65"/>
+      <c r="C50" s="68">
+        <v>19.2</v>
+      </c>
+      <c r="D50" s="57" t="s">
+        <v>201</v>
+      </c>
+      <c r="E50" s="57" t="s">
+        <v>203</v>
+      </c>
+      <c r="F50" s="57" t="s">
+        <v>188</v>
+      </c>
+      <c r="G50" s="57" t="s">
+        <v>206</v>
+      </c>
+      <c r="H50" s="66"/>
+      <c r="I50" s="67"/>
+      <c r="J50" s="3"/>
+      <c r="K50" s="3"/>
+      <c r="L50" s="3"/>
+    </row>
+    <row r="51" spans="1:12" ht="104.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A51" s="64">
+        <v>20</v>
+      </c>
+      <c r="B51" s="65" t="s">
+        <v>207</v>
+      </c>
+      <c r="C51" s="66">
+        <v>20.100000000000001</v>
+      </c>
+      <c r="D51" s="57" t="s">
+        <v>208</v>
+      </c>
+      <c r="E51" s="57" t="s">
+        <v>213</v>
+      </c>
+      <c r="F51" s="57" t="s">
+        <v>212</v>
+      </c>
+      <c r="G51" s="57" t="s">
+        <v>214</v>
+      </c>
+      <c r="H51" s="66"/>
+      <c r="I51" s="67"/>
+    </row>
+    <row r="52" spans="1:12" ht="135" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A52" s="64"/>
+      <c r="B52" s="65"/>
+      <c r="C52" s="68">
+        <v>20.2</v>
+      </c>
+      <c r="D52" s="57" t="s">
+        <v>209</v>
+      </c>
+      <c r="E52" s="57" t="s">
+        <v>211</v>
+      </c>
+      <c r="F52" s="57" t="s">
+        <v>188</v>
+      </c>
+      <c r="G52" s="57" t="s">
+        <v>210</v>
+      </c>
+      <c r="H52" s="66"/>
+      <c r="I52" s="67"/>
+    </row>
+    <row r="53" spans="1:12" ht="179.4" x14ac:dyDescent="0.3">
+      <c r="A53" s="64">
+        <v>21</v>
+      </c>
+      <c r="B53" s="65" t="s">
+        <v>215</v>
+      </c>
+      <c r="C53" s="66">
+        <v>21.1</v>
+      </c>
+      <c r="D53" s="57" t="s">
+        <v>216</v>
+      </c>
+      <c r="E53" s="57" t="s">
+        <v>219</v>
+      </c>
+      <c r="F53" s="57" t="s">
+        <v>220</v>
+      </c>
+      <c r="G53" s="57" t="s">
+        <v>221</v>
+      </c>
+      <c r="H53" s="66"/>
+      <c r="I53" s="67"/>
+    </row>
+    <row r="54" spans="1:12" ht="124.2" x14ac:dyDescent="0.3">
+      <c r="A54" s="64"/>
+      <c r="B54" s="65"/>
+      <c r="C54" s="68">
+        <v>21.2</v>
+      </c>
+      <c r="D54" s="57" t="s">
+        <v>217</v>
+      </c>
+      <c r="E54" s="69" t="s">
+        <v>222</v>
+      </c>
+      <c r="F54" s="57" t="s">
+        <v>188</v>
+      </c>
+      <c r="G54" s="57" t="s">
+        <v>218</v>
+      </c>
+      <c r="H54" s="66"/>
+      <c r="I54" s="67"/>
     </row>
     <row r="55" spans="1:12" ht="36" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A55" s="3"/>
-      <c r="B55" s="3"/>
-      <c r="C55" s="3"/>
-      <c r="E55" s="3"/>
-      <c r="H55" s="3"/>
+      <c r="A55" s="2"/>
+      <c r="B55" s="2"/>
+      <c r="C55" s="2"/>
+      <c r="E55" s="57"/>
+      <c r="H55" s="2"/>
     </row>
     <row r="56" spans="1:12" ht="31.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="D56" s="2"/>
-      <c r="F56" s="2"/>
-      <c r="G56" s="2"/>
-      <c r="I56" s="2"/>
+      <c r="D56" s="1"/>
+      <c r="F56" s="1"/>
+      <c r="G56" s="1"/>
+      <c r="I56" s="1"/>
     </row>
     <row r="57" spans="1:12" ht="34.950000000000003" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="D57" s="2"/>
-      <c r="F57" s="2"/>
-      <c r="G57" s="2"/>
-      <c r="I57" s="2"/>
+      <c r="D57" s="1"/>
+      <c r="F57" s="1"/>
+      <c r="G57" s="1"/>
+      <c r="I57" s="1"/>
     </row>
     <row r="58" spans="1:12" ht="31.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A58" s="55"/>
-      <c r="B58" s="55"/>
-      <c r="C58" s="55"/>
-      <c r="D58" s="55"/>
-      <c r="E58" s="55"/>
-      <c r="F58" s="55"/>
-      <c r="G58" s="55"/>
-      <c r="H58" s="55"/>
-      <c r="I58" s="55"/>
+      <c r="A58" s="46"/>
+      <c r="B58" s="46"/>
+      <c r="C58" s="46"/>
+      <c r="D58" s="46"/>
+      <c r="E58" s="46"/>
+      <c r="F58" s="46"/>
+      <c r="G58" s="46"/>
+      <c r="H58" s="46"/>
+      <c r="I58" s="46"/>
     </row>
     <row r="59" spans="1:12" ht="33.450000000000003" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A59" s="3"/>
-      <c r="B59" s="3"/>
-      <c r="C59" s="3"/>
-      <c r="E59" s="3"/>
-      <c r="H59" s="3"/>
+      <c r="A59" s="2"/>
+      <c r="B59" s="2"/>
+      <c r="C59" s="2"/>
+      <c r="E59" s="2"/>
+      <c r="H59" s="2"/>
     </row>
     <row r="60" spans="1:12" ht="31.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="D60" s="2"/>
-      <c r="F60" s="2"/>
-      <c r="G60" s="2"/>
-      <c r="I60" s="2"/>
+      <c r="D60" s="1"/>
+      <c r="F60" s="1"/>
+      <c r="G60" s="1"/>
+      <c r="I60" s="1"/>
     </row>
     <row r="61" spans="1:12" ht="27.45" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B61" s="3"/>
-      <c r="F61" s="2"/>
-      <c r="G61" s="2"/>
-      <c r="I61" s="2"/>
+      <c r="B61" s="2"/>
+      <c r="F61" s="1"/>
+      <c r="G61" s="1"/>
+      <c r="I61" s="1"/>
     </row>
   </sheetData>
   <autoFilter ref="I1:I19" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
-  <mergeCells count="25">
-    <mergeCell ref="B8:B9"/>
-    <mergeCell ref="B22:B32"/>
-    <mergeCell ref="B38:B39"/>
-    <mergeCell ref="B17:B20"/>
-    <mergeCell ref="A17:A20"/>
+  <mergeCells count="33">
+    <mergeCell ref="A53:A54"/>
+    <mergeCell ref="B53:B54"/>
+    <mergeCell ref="B47:B48"/>
+    <mergeCell ref="A47:A48"/>
+    <mergeCell ref="A49:A50"/>
+    <mergeCell ref="B49:B50"/>
+    <mergeCell ref="A51:A52"/>
+    <mergeCell ref="B51:B52"/>
+    <mergeCell ref="A40:A46"/>
+    <mergeCell ref="B13:B16"/>
+    <mergeCell ref="B40:B46"/>
+    <mergeCell ref="A10:A12"/>
+    <mergeCell ref="A38:A39"/>
+    <mergeCell ref="B17:B21"/>
+    <mergeCell ref="A17:A21"/>
     <mergeCell ref="B5:B6"/>
     <mergeCell ref="A5:A6"/>
     <mergeCell ref="A33:A37"/>
@@ -2935,11 +3064,9 @@
     <mergeCell ref="C1:C2"/>
     <mergeCell ref="G1:G2"/>
     <mergeCell ref="B1:B2"/>
-    <mergeCell ref="A40:A46"/>
-    <mergeCell ref="B13:B16"/>
-    <mergeCell ref="B40:B46"/>
-    <mergeCell ref="A10:A12"/>
-    <mergeCell ref="A38:A39"/>
+    <mergeCell ref="B8:B9"/>
+    <mergeCell ref="B22:B32"/>
+    <mergeCell ref="B38:B39"/>
   </mergeCells>
   <phoneticPr fontId="6" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Document wallet epic updated
</commit_message>
<xml_diff>
--- a/Soubhanik/checkupp_product_backlog_final.xlsx
+++ b/Soubhanik/checkupp_product_backlog_final.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Anodiam\2026\CheckUpp_Parent\CheckUpp\Soubhanik\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F541787C-31D8-4746-8E0E-39AE90D3A9A8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BA235ADE-84B4-42B6-8ADC-8CDC68A9616A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$I$1:$I$19</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$I$1:$I$21</definedName>
   </definedNames>
   <calcPr calcId="0"/>
 </workbook>
@@ -101,7 +101,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="B10" authorId="1" shapeId="0" xr:uid="{79DA11BF-BFE2-49FE-916B-7BBF40F206E7}">
+    <comment ref="B12" authorId="1" shapeId="0" xr:uid="{79DA11BF-BFE2-49FE-916B-7BBF40F206E7}">
       <text>
         <r>
           <rPr>
@@ -130,7 +130,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="310" uniqueCount="224">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="322" uniqueCount="231">
   <si>
     <t>Epic #</t>
   </si>
@@ -446,9 +446,6 @@
   </si>
   <si>
     <t>Slide 8-11</t>
-  </si>
-  <si>
-    <t>Slide 14</t>
   </si>
   <si>
     <t>Slide 15</t>
@@ -577,13 +574,6 @@
 d. Travel (age agnostic)</t>
   </si>
   <si>
-    <t>I can access them in app and in device's local file manager</t>
-  </si>
-  <si>
-    <t>1. Document wallet must list all the uploaded documents with name and date
-2. User must be able to interact with the options to download, view and delete the documents</t>
-  </si>
-  <si>
     <t xml:space="preserve"> </t>
   </si>
   <si>
@@ -882,14 +872,54 @@
     <t>see my previously entered data in the available fields (e.g., cavities, fillings, etc.), the status of the toggle switch (Use Mouthwash Regularly), and the selected dropdown options (Brushing Frequency and Flossing Frequency) restored along with an affirming notification (toast)</t>
   </si>
   <si>
-    <t>logged in user navigating the Document Wallet screen</t>
-  </si>
-  <si>
-    <t>store health documents(reports) in the app's cloud storage and my local device</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. Document captured/scanned must be visible in the Document Wallet
-2. User must be able to click on the download icon to save the document/image in their local device storage </t>
+    <t>upload health documents(reports) in the app's cloud storage from my local device</t>
+  </si>
+  <si>
+    <t>I can access them in app</t>
+  </si>
+  <si>
+    <t>1. The logged-in user must be able to select one or more health documents (e.g., reports) from their local device for upload to the Document Wallet.
+2. The selected health documents must be uploaded securely to the app's cloud storage and associated with the logged-in user's account.
+3. A confirmation message must be displayed to the user after each document has been successfully uploaded.
+4. If a document upload fails, an appropriate error message must be displayed, and the user must be able to retry the upload without affecting previously uploaded documents.</t>
+  </si>
+  <si>
+    <t>1. Document wallet must list all the uploaded documents with name and date
+2. User must be able to interact with the options to download, view and delete options for each document stored in the Document Wallet
+3. If a document cannot be opened, an appropriate error message must be displayed, and the user must be able to retry opening the document.
+4. The selected document must be displayed in a readable format within the app or using the device's supported document viewer.</t>
+  </si>
+  <si>
+    <t>logged in user navigating the 'Documents' section of the Document Wallet screen</t>
+  </si>
+  <si>
+    <t>logged in user navigating the 'Links' section of the Document Wallet screen</t>
+  </si>
+  <si>
+    <t>store my e-script links along with any associated text of my choice</t>
+  </si>
+  <si>
+    <t>I can view all my e-script links as a list along with a description of my choice for each link</t>
+  </si>
+  <si>
+    <t>1. User must be able to add an e-script link along with an associated text description of their choice in the Links section of the Document Wallet.
+2. The entered e-script link and its associated description must be securely saved
+3. All saved e-script links and their associated descriptions must be displayed as a list in the Links section of the Document Wallet.
+4. If an e-script link cannot be saved, an appropriate error message must be displayed, and the user must be able to retry the action without affecting previously saved links.</t>
+  </si>
+  <si>
+    <t>Slide 11</t>
+  </si>
+  <si>
+    <t>view a link stored in my wallet</t>
+  </si>
+  <si>
+    <t>I can review my e-script links at any time</t>
+  </si>
+  <si>
+    <t>1. Document wallet must list all the saved links with name and date
+2. User must be able to interact with the options to view and delete options for each link stored in the Document Wallet
+3. If the detailed view of a link cannot be opened, an appropriate error message must be displayed, and the user must be able to retry opening the detailed view of the link.</t>
   </si>
 </sst>
 </file>
@@ -1087,7 +1117,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -1125,12 +1155,49 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="70">
+  <cellXfs count="72">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1297,44 +1364,50 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="14" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="10" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="12" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="15" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="13" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="12" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="14" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="10" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1618,11 +1691,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:L61"/>
+  <dimension ref="A1:L63"/>
   <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="5.88671875" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="32.88671875" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="22.5546875" style="1" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="11.109375" style="1" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="20.88671875" style="2" customWidth="1"/>
     <col min="5" max="5" width="64.88671875" style="1" bestFit="1" customWidth="1"/>
@@ -1635,34 +1708,34 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="39.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="59" t="s">
+      <c r="A1" s="67" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="59" t="s">
+      <c r="B1" s="67" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="59" t="s">
+      <c r="C1" s="67" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="59" t="s">
+      <c r="D1" s="67" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="60"/>
-      <c r="F1" s="60"/>
-      <c r="G1" s="59" t="s">
+      <c r="E1" s="68"/>
+      <c r="F1" s="68"/>
+      <c r="G1" s="67" t="s">
         <v>4</v>
       </c>
-      <c r="H1" s="59" t="s">
+      <c r="H1" s="67" t="s">
         <v>5</v>
       </c>
-      <c r="I1" s="59" t="s">
+      <c r="I1" s="67" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A2" s="58"/>
-      <c r="B2" s="58"/>
-      <c r="C2" s="58"/>
+      <c r="A2" s="59"/>
+      <c r="B2" s="59"/>
+      <c r="C2" s="59"/>
       <c r="D2" s="50" t="s">
         <v>7</v>
       </c>
@@ -1672,37 +1745,37 @@
       <c r="F2" s="50" t="s">
         <v>9</v>
       </c>
-      <c r="G2" s="59"/>
-      <c r="H2" s="58"/>
-      <c r="I2" s="58"/>
+      <c r="G2" s="67"/>
+      <c r="H2" s="59"/>
+      <c r="I2" s="59"/>
     </row>
     <row r="3" spans="1:9" s="4" customFormat="1" ht="82.8" x14ac:dyDescent="0.3">
       <c r="A3" s="30" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
       <c r="B3" s="30" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="C3" s="18">
         <v>13.2</v>
       </c>
       <c r="D3" s="31" t="s">
+        <v>125</v>
+      </c>
+      <c r="E3" s="31" t="s">
         <v>126</v>
       </c>
-      <c r="E3" s="31" t="s">
+      <c r="F3" s="31" t="s">
         <v>127</v>
       </c>
-      <c r="F3" s="31" t="s">
-        <v>128</v>
-      </c>
       <c r="G3" s="32" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="H3" s="18" t="s">
         <v>60</v>
       </c>
       <c r="I3" s="31" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
     </row>
     <row r="4" spans="1:9" s="4" customFormat="1" ht="55.2" x14ac:dyDescent="0.3">
@@ -1719,26 +1792,26 @@
         <v>11</v>
       </c>
       <c r="E4" s="40" t="s">
+        <v>102</v>
+      </c>
+      <c r="F4" s="40" t="s">
         <v>103</v>
       </c>
-      <c r="F4" s="40" t="s">
+      <c r="G4" s="41" t="s">
         <v>104</v>
-      </c>
-      <c r="G4" s="41" t="s">
-        <v>105</v>
       </c>
       <c r="H4" s="39" t="s">
         <v>12</v>
       </c>
       <c r="I4" s="40" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="5" spans="1:9" s="29" customFormat="1" ht="69" x14ac:dyDescent="0.3">
-      <c r="A5" s="56">
+      <c r="A5" s="65">
         <v>3</v>
       </c>
-      <c r="B5" s="56" t="s">
+      <c r="B5" s="65" t="s">
         <v>13</v>
       </c>
       <c r="C5" s="28">
@@ -1748,13 +1821,13 @@
         <v>11</v>
       </c>
       <c r="E5" s="34" t="s">
+        <v>105</v>
+      </c>
+      <c r="F5" s="34" t="s">
         <v>106</v>
       </c>
-      <c r="F5" s="34" t="s">
-        <v>107</v>
-      </c>
       <c r="G5" s="35" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="H5" s="36" t="s">
         <v>97</v>
@@ -1764,8 +1837,8 @@
       </c>
     </row>
     <row r="6" spans="1:9" s="4" customFormat="1" ht="69" x14ac:dyDescent="0.3">
-      <c r="A6" s="56"/>
-      <c r="B6" s="56"/>
+      <c r="A6" s="65"/>
+      <c r="B6" s="65"/>
       <c r="C6" s="28">
         <v>3.2</v>
       </c>
@@ -1773,13 +1846,13 @@
         <v>11</v>
       </c>
       <c r="E6" s="34" t="s">
+        <v>107</v>
+      </c>
+      <c r="F6" s="34" t="s">
         <v>108</v>
       </c>
-      <c r="F6" s="34" t="s">
-        <v>109</v>
-      </c>
       <c r="G6" s="35" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="H6" s="28" t="s">
         <v>97</v>
@@ -1799,16 +1872,16 @@
         <v>5.2</v>
       </c>
       <c r="D7" s="6" t="s">
+        <v>132</v>
+      </c>
+      <c r="E7" s="6" t="s">
+        <v>134</v>
+      </c>
+      <c r="F7" s="6" t="s">
         <v>133</v>
       </c>
-      <c r="E7" s="6" t="s">
+      <c r="G7" s="23" t="s">
         <v>135</v>
-      </c>
-      <c r="F7" s="6" t="s">
-        <v>134</v>
-      </c>
-      <c r="G7" s="23" t="s">
-        <v>136</v>
       </c>
       <c r="H7" s="7" t="s">
         <v>98</v>
@@ -1817,43 +1890,43 @@
         <v>17</v>
       </c>
     </row>
-    <row r="8" spans="1:9" s="4" customFormat="1" ht="41.4" x14ac:dyDescent="0.3">
-      <c r="A8" s="62">
+    <row r="8" spans="1:9" s="4" customFormat="1" ht="124.2" x14ac:dyDescent="0.3">
+      <c r="A8" s="69">
         <v>6</v>
       </c>
-      <c r="B8" s="62" t="s">
+      <c r="B8" s="69" t="s">
         <v>18</v>
       </c>
       <c r="C8" s="8">
         <v>6.1</v>
       </c>
       <c r="D8" s="9" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="E8" s="42" t="s">
-        <v>222</v>
+        <v>218</v>
       </c>
       <c r="F8" s="42" t="s">
-        <v>137</v>
+        <v>219</v>
       </c>
       <c r="G8" s="43" t="s">
-        <v>223</v>
+        <v>220</v>
       </c>
       <c r="H8" s="10" t="s">
-        <v>99</v>
+        <v>227</v>
       </c>
       <c r="I8" s="9" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="9" spans="1:9" s="4" customFormat="1" ht="55.2" x14ac:dyDescent="0.3">
-      <c r="A9" s="58"/>
-      <c r="B9" s="58"/>
+    <row r="9" spans="1:9" s="4" customFormat="1" ht="110.4" x14ac:dyDescent="0.3">
+      <c r="A9" s="70"/>
+      <c r="B9" s="70"/>
       <c r="C9" s="8">
         <v>6.2</v>
       </c>
       <c r="D9" s="9" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="E9" s="9" t="s">
         <v>20</v>
@@ -1862,400 +1935,400 @@
         <v>21</v>
       </c>
       <c r="G9" s="24" t="s">
-        <v>138</v>
-      </c>
-      <c r="H9" s="8" t="s">
+        <v>221</v>
+      </c>
+      <c r="H9" s="10" t="s">
+        <v>227</v>
+      </c>
+      <c r="I9" s="9" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" s="4" customFormat="1" ht="124.2" x14ac:dyDescent="0.3">
+      <c r="A10" s="70"/>
+      <c r="B10" s="70"/>
+      <c r="C10" s="8">
+        <v>6.3</v>
+      </c>
+      <c r="D10" s="9" t="s">
+        <v>223</v>
+      </c>
+      <c r="E10" s="9" t="s">
+        <v>224</v>
+      </c>
+      <c r="F10" s="9" t="s">
+        <v>225</v>
+      </c>
+      <c r="G10" s="24" t="s">
+        <v>226</v>
+      </c>
+      <c r="H10" s="10" t="s">
+        <v>227</v>
+      </c>
+      <c r="I10" s="9" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" s="4" customFormat="1" ht="82.8" x14ac:dyDescent="0.3">
+      <c r="A11" s="71"/>
+      <c r="B11" s="71"/>
+      <c r="C11" s="8">
+        <v>6.4</v>
+      </c>
+      <c r="D11" s="9" t="s">
+        <v>223</v>
+      </c>
+      <c r="E11" s="9" t="s">
+        <v>228</v>
+      </c>
+      <c r="F11" s="9" t="s">
+        <v>229</v>
+      </c>
+      <c r="G11" s="24" t="s">
+        <v>230</v>
+      </c>
+      <c r="H11" s="10"/>
+      <c r="I11" s="9" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" s="4" customFormat="1" ht="55.2" x14ac:dyDescent="0.3">
+      <c r="A12" s="61">
+        <v>7</v>
+      </c>
+      <c r="B12" s="61" t="s">
+        <v>22</v>
+      </c>
+      <c r="C12" s="11">
+        <v>7.1</v>
+      </c>
+      <c r="D12" s="12" t="s">
+        <v>125</v>
+      </c>
+      <c r="E12" s="12" t="s">
+        <v>23</v>
+      </c>
+      <c r="F12" s="12" t="s">
+        <v>24</v>
+      </c>
+      <c r="G12" s="25" t="s">
+        <v>25</v>
+      </c>
+      <c r="H12" s="13" t="s">
         <v>99</v>
       </c>
-      <c r="I9" s="9"/>
-    </row>
-    <row r="10" spans="1:9" s="4" customFormat="1" ht="55.2" x14ac:dyDescent="0.3">
-      <c r="A10" s="63">
-        <v>7</v>
-      </c>
-      <c r="B10" s="63" t="s">
-        <v>22</v>
-      </c>
-      <c r="C10" s="11">
-        <v>7.1</v>
-      </c>
-      <c r="D10" s="12" t="s">
-        <v>126</v>
-      </c>
-      <c r="E10" s="12" t="s">
-        <v>23</v>
-      </c>
-      <c r="F10" s="12" t="s">
-        <v>24</v>
-      </c>
-      <c r="G10" s="25" t="s">
-        <v>25</v>
-      </c>
-      <c r="H10" s="13" t="s">
+      <c r="I12" s="12" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9" s="4" customFormat="1" ht="55.2" x14ac:dyDescent="0.3">
+      <c r="A13" s="59"/>
+      <c r="B13" s="59"/>
+      <c r="C13" s="11">
+        <v>7.2</v>
+      </c>
+      <c r="D13" s="12" t="s">
+        <v>125</v>
+      </c>
+      <c r="E13" s="12" t="s">
+        <v>27</v>
+      </c>
+      <c r="F13" s="12" t="s">
+        <v>28</v>
+      </c>
+      <c r="G13" s="25" t="s">
+        <v>29</v>
+      </c>
+      <c r="H13" s="11" t="s">
         <v>100</v>
       </c>
-      <c r="I10" s="12" t="s">
+      <c r="I13" s="12" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="11" spans="1:9" s="4" customFormat="1" ht="55.2" x14ac:dyDescent="0.3">
-      <c r="A11" s="58"/>
-      <c r="B11" s="58"/>
-      <c r="C11" s="11">
-        <v>7.2</v>
-      </c>
-      <c r="D11" s="12" t="s">
-        <v>126</v>
-      </c>
-      <c r="E11" s="12" t="s">
-        <v>27</v>
-      </c>
-      <c r="F11" s="12" t="s">
-        <v>28</v>
-      </c>
-      <c r="G11" s="25" t="s">
-        <v>29</v>
-      </c>
-      <c r="H11" s="11" t="s">
-        <v>101</v>
-      </c>
-      <c r="I11" s="12" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="12" spans="1:9" s="4" customFormat="1" ht="41.4" x14ac:dyDescent="0.3">
-      <c r="A12" s="58"/>
-      <c r="B12" s="58"/>
-      <c r="C12" s="11">
+    <row r="14" spans="1:9" s="4" customFormat="1" ht="41.4" x14ac:dyDescent="0.3">
+      <c r="A14" s="59"/>
+      <c r="B14" s="59"/>
+      <c r="C14" s="11">
         <v>7.3</v>
       </c>
-      <c r="D12" s="12" t="s">
-        <v>126</v>
-      </c>
-      <c r="E12" s="12" t="s">
+      <c r="D14" s="12" t="s">
+        <v>125</v>
+      </c>
+      <c r="E14" s="12" t="s">
         <v>30</v>
       </c>
-      <c r="F12" s="12" t="s">
+      <c r="F14" s="12" t="s">
         <v>31</v>
       </c>
-      <c r="G12" s="25" t="s">
+      <c r="G14" s="25" t="s">
         <v>32</v>
       </c>
-      <c r="H12" s="11" t="s">
-        <v>100</v>
-      </c>
-      <c r="I12" s="12"/>
-    </row>
-    <row r="13" spans="1:9" s="4" customFormat="1" ht="27.6" x14ac:dyDescent="0.3">
-      <c r="A13" s="61">
+      <c r="H14" s="11" t="s">
+        <v>99</v>
+      </c>
+      <c r="I14" s="12"/>
+    </row>
+    <row r="15" spans="1:9" s="4" customFormat="1" ht="27.6" x14ac:dyDescent="0.3">
+      <c r="A15" s="60">
         <v>9</v>
       </c>
-      <c r="B13" s="61" t="s">
+      <c r="B15" s="60" t="s">
         <v>33</v>
       </c>
-      <c r="C13" s="14">
+      <c r="C15" s="14">
         <v>9.1</v>
       </c>
-      <c r="D13" s="15" t="s">
+      <c r="D15" s="15" t="s">
         <v>15</v>
       </c>
-      <c r="E13" s="15" t="s">
+      <c r="E15" s="15" t="s">
         <v>34</v>
       </c>
-      <c r="F13" s="15" t="s">
+      <c r="F15" s="15" t="s">
         <v>35</v>
       </c>
-      <c r="G13" s="26" t="s">
+      <c r="G15" s="26" t="s">
         <v>36</v>
       </c>
-      <c r="H13" s="14"/>
-      <c r="I13" s="15"/>
-    </row>
-    <row r="14" spans="1:9" s="4" customFormat="1" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="58"/>
-      <c r="B14" s="58"/>
-      <c r="C14" s="14">
+      <c r="H15" s="14"/>
+      <c r="I15" s="15"/>
+    </row>
+    <row r="16" spans="1:9" s="4" customFormat="1" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A16" s="59"/>
+      <c r="B16" s="59"/>
+      <c r="C16" s="14">
         <v>9.1999999999999993</v>
       </c>
-      <c r="D14" s="15" t="s">
+      <c r="D16" s="15" t="s">
         <v>37</v>
       </c>
-      <c r="E14" s="15" t="s">
+      <c r="E16" s="15" t="s">
         <v>38</v>
       </c>
-      <c r="F14" s="15" t="s">
+      <c r="F16" s="15" t="s">
         <v>39</v>
       </c>
-      <c r="G14" s="26" t="s">
+      <c r="G16" s="26" t="s">
         <v>40</v>
       </c>
-      <c r="H14" s="14"/>
-      <c r="I14" s="15"/>
-    </row>
-    <row r="15" spans="1:9" s="4" customFormat="1" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="58"/>
-      <c r="B15" s="58"/>
-      <c r="C15" s="14">
+      <c r="H16" s="14"/>
+      <c r="I16" s="15"/>
+    </row>
+    <row r="17" spans="1:9" s="4" customFormat="1" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A17" s="59"/>
+      <c r="B17" s="59"/>
+      <c r="C17" s="14">
         <v>9.3000000000000007</v>
       </c>
-      <c r="D15" s="15" t="s">
+      <c r="D17" s="15" t="s">
         <v>41</v>
       </c>
-      <c r="E15" s="15" t="s">
+      <c r="E17" s="15" t="s">
         <v>42</v>
       </c>
-      <c r="F15" s="15" t="s">
+      <c r="F17" s="15" t="s">
         <v>43</v>
       </c>
-      <c r="G15" s="26" t="s">
+      <c r="G17" s="26" t="s">
         <v>44</v>
       </c>
-      <c r="H15" s="14"/>
-      <c r="I15" s="15" t="s">
+      <c r="H17" s="14"/>
+      <c r="I17" s="15" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="16" spans="1:9" s="4" customFormat="1" ht="55.2" x14ac:dyDescent="0.3">
-      <c r="A16" s="58"/>
-      <c r="B16" s="58"/>
-      <c r="C16" s="14">
+    <row r="18" spans="1:9" s="4" customFormat="1" ht="55.2" x14ac:dyDescent="0.3">
+      <c r="A18" s="59"/>
+      <c r="B18" s="59"/>
+      <c r="C18" s="14">
         <v>9.4</v>
       </c>
-      <c r="D16" s="15" t="s">
+      <c r="D18" s="15" t="s">
         <v>15</v>
       </c>
-      <c r="E16" s="15" t="s">
+      <c r="E18" s="15" t="s">
         <v>46</v>
       </c>
-      <c r="F16" s="15" t="s">
+      <c r="F18" s="15" t="s">
         <v>47</v>
       </c>
-      <c r="G16" s="26" t="s">
+      <c r="G18" s="26" t="s">
         <v>48</v>
       </c>
-      <c r="H16" s="14"/>
-      <c r="I16" s="15" t="s">
+      <c r="H18" s="14"/>
+      <c r="I18" s="15" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="17" spans="1:9" s="4" customFormat="1" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="67">
+    <row r="19" spans="1:9" s="4" customFormat="1" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A19" s="63">
         <v>12</v>
       </c>
-      <c r="B17" s="67" t="s">
-        <v>181</v>
-      </c>
-      <c r="C17" s="16">
+      <c r="B19" s="63" t="s">
+        <v>178</v>
+      </c>
+      <c r="C19" s="16">
         <v>12.1</v>
       </c>
-      <c r="D17" s="17" t="s">
-        <v>180</v>
-      </c>
-      <c r="E17" s="17" t="s">
+      <c r="D19" s="17" t="s">
+        <v>177</v>
+      </c>
+      <c r="E19" s="17" t="s">
         <v>49</v>
       </c>
-      <c r="F17" s="17" t="s">
+      <c r="F19" s="17" t="s">
         <v>50</v>
       </c>
-      <c r="G17" s="27" t="s">
+      <c r="G19" s="27" t="s">
         <v>51</v>
-      </c>
-      <c r="H17" s="16" t="s">
-        <v>52</v>
-      </c>
-      <c r="I17" s="17" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="18" spans="1:9" s="4" customFormat="1" ht="55.2" x14ac:dyDescent="0.3">
-      <c r="A18" s="67"/>
-      <c r="B18" s="67"/>
-      <c r="C18" s="16">
-        <v>12.2</v>
-      </c>
-      <c r="D18" s="17" t="s">
-        <v>180</v>
-      </c>
-      <c r="E18" s="17" t="s">
-        <v>54</v>
-      </c>
-      <c r="F18" s="17" t="s">
-        <v>55</v>
-      </c>
-      <c r="G18" s="27" t="s">
-        <v>56</v>
-      </c>
-      <c r="H18" s="16" t="s">
-        <v>52</v>
-      </c>
-      <c r="I18" s="17" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="19" spans="1:9" s="4" customFormat="1" ht="41.4" x14ac:dyDescent="0.3">
-      <c r="A19" s="67"/>
-      <c r="B19" s="67"/>
-      <c r="C19" s="16">
-        <v>12.3</v>
-      </c>
-      <c r="D19" s="17" t="s">
-        <v>180</v>
-      </c>
-      <c r="E19" s="17" t="s">
-        <v>57</v>
-      </c>
-      <c r="F19" s="17" t="s">
-        <v>58</v>
-      </c>
-      <c r="G19" s="27" t="s">
-        <v>59</v>
       </c>
       <c r="H19" s="16" t="s">
         <v>52</v>
       </c>
-      <c r="I19" s="17"/>
-    </row>
-    <row r="20" spans="1:9" s="4" customFormat="1" ht="138" x14ac:dyDescent="0.3">
-      <c r="A20" s="67"/>
-      <c r="B20" s="67"/>
+      <c r="I19" s="17" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="20" spans="1:9" s="4" customFormat="1" ht="55.2" x14ac:dyDescent="0.3">
+      <c r="A20" s="63"/>
+      <c r="B20" s="63"/>
       <c r="C20" s="16">
+        <v>12.2</v>
+      </c>
+      <c r="D20" s="17" t="s">
+        <v>177</v>
+      </c>
+      <c r="E20" s="17" t="s">
+        <v>54</v>
+      </c>
+      <c r="F20" s="17" t="s">
+        <v>55</v>
+      </c>
+      <c r="G20" s="27" t="s">
+        <v>56</v>
+      </c>
+      <c r="H20" s="16" t="s">
+        <v>52</v>
+      </c>
+      <c r="I20" s="17" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="21" spans="1:9" s="4" customFormat="1" ht="41.4" x14ac:dyDescent="0.3">
+      <c r="A21" s="63"/>
+      <c r="B21" s="63"/>
+      <c r="C21" s="16">
+        <v>12.3</v>
+      </c>
+      <c r="D21" s="17" t="s">
+        <v>177</v>
+      </c>
+      <c r="E21" s="17" t="s">
+        <v>57</v>
+      </c>
+      <c r="F21" s="17" t="s">
+        <v>58</v>
+      </c>
+      <c r="G21" s="27" t="s">
+        <v>59</v>
+      </c>
+      <c r="H21" s="16" t="s">
+        <v>52</v>
+      </c>
+      <c r="I21" s="17"/>
+    </row>
+    <row r="22" spans="1:9" s="4" customFormat="1" ht="138" x14ac:dyDescent="0.3">
+      <c r="A22" s="63"/>
+      <c r="B22" s="63"/>
+      <c r="C22" s="16">
         <v>12.4</v>
       </c>
-      <c r="D20" s="17" t="s">
+      <c r="D22" s="17" t="s">
+        <v>177</v>
+      </c>
+      <c r="E22" s="17" t="s">
+        <v>179</v>
+      </c>
+      <c r="F22" s="17" t="s">
         <v>180</v>
       </c>
-      <c r="E20" s="17" t="s">
+      <c r="G22" s="17" t="s">
+        <v>181</v>
+      </c>
+      <c r="H22" s="16"/>
+      <c r="I22" s="17"/>
+    </row>
+    <row r="23" spans="1:9" s="4" customFormat="1" ht="124.2" x14ac:dyDescent="0.3">
+      <c r="A23" s="63"/>
+      <c r="B23" s="63"/>
+      <c r="C23" s="16">
+        <v>12.5</v>
+      </c>
+      <c r="D23" s="17" t="s">
         <v>182</v>
       </c>
-      <c r="F20" s="17" t="s">
+      <c r="E23" s="17" t="s">
+        <v>184</v>
+      </c>
+      <c r="F23" s="17" t="s">
         <v>183</v>
       </c>
-      <c r="G20" s="17" t="s">
-        <v>184</v>
-      </c>
-      <c r="H20" s="16"/>
-      <c r="I20" s="17"/>
-    </row>
-    <row r="21" spans="1:9" s="4" customFormat="1" ht="124.2" x14ac:dyDescent="0.3">
-      <c r="A21" s="67"/>
-      <c r="B21" s="67"/>
-      <c r="C21" s="16">
-        <v>12.5</v>
-      </c>
-      <c r="D21" s="17" t="s">
+      <c r="G23" s="27" t="s">
         <v>185</v>
       </c>
-      <c r="E21" s="17" t="s">
-        <v>187</v>
-      </c>
-      <c r="F21" s="17" t="s">
-        <v>186</v>
-      </c>
-      <c r="G21" s="27" t="s">
-        <v>188</v>
-      </c>
-      <c r="H21" s="16"/>
-      <c r="I21" s="17"/>
-    </row>
-    <row r="22" spans="1:9" s="4" customFormat="1" ht="41.4" x14ac:dyDescent="0.3">
-      <c r="A22" s="64">
+      <c r="H23" s="16"/>
+      <c r="I23" s="17"/>
+    </row>
+    <row r="24" spans="1:9" s="4" customFormat="1" ht="41.4" x14ac:dyDescent="0.3">
+      <c r="A24" s="64">
         <v>14</v>
       </c>
-      <c r="B22" s="64" t="s">
+      <c r="B24" s="64" t="s">
         <v>61</v>
       </c>
-      <c r="C22" s="47">
+      <c r="C24" s="47">
         <v>14.1</v>
       </c>
-      <c r="D22" s="48" t="s">
+      <c r="D24" s="48" t="s">
         <v>15</v>
       </c>
-      <c r="E22" s="48" t="s">
-        <v>144</v>
-      </c>
-      <c r="F22" s="48" t="s">
-        <v>145</v>
-      </c>
-      <c r="G22" s="48" t="s">
-        <v>169</v>
-      </c>
-      <c r="H22" s="47" t="s">
-        <v>102</v>
-      </c>
-      <c r="I22" s="48" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="23" spans="1:9" s="4" customFormat="1" ht="41.4" x14ac:dyDescent="0.3">
-      <c r="A23" s="64"/>
-      <c r="B23" s="64"/>
-      <c r="C23" s="47">
-        <v>14.2</v>
-      </c>
-      <c r="D23" s="48" t="s">
-        <v>15</v>
-      </c>
-      <c r="E23" s="48" t="s">
-        <v>146</v>
-      </c>
-      <c r="F23" s="48" t="s">
-        <v>147</v>
-      </c>
-      <c r="G23" s="48" t="s">
-        <v>170</v>
-      </c>
-      <c r="H23" s="47" t="s">
-        <v>102</v>
-      </c>
-      <c r="I23" s="48" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="24" spans="1:9" s="4" customFormat="1" ht="41.4" x14ac:dyDescent="0.3">
-      <c r="A24" s="64"/>
-      <c r="B24" s="64"/>
-      <c r="C24" s="47">
-        <v>14.3</v>
-      </c>
-      <c r="D24" s="48" t="s">
-        <v>148</v>
-      </c>
       <c r="E24" s="48" t="s">
-        <v>149</v>
+        <v>141</v>
       </c>
       <c r="F24" s="48" t="s">
-        <v>150</v>
+        <v>142</v>
       </c>
       <c r="G24" s="48" t="s">
-        <v>171</v>
+        <v>166</v>
       </c>
       <c r="H24" s="47" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="I24" s="48" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="25" spans="1:9" s="4" customFormat="1" ht="55.2" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:9" s="4" customFormat="1" ht="41.4" x14ac:dyDescent="0.3">
       <c r="A25" s="64"/>
       <c r="B25" s="64"/>
       <c r="C25" s="47">
-        <v>14.4</v>
+        <v>14.2</v>
       </c>
       <c r="D25" s="48" t="s">
         <v>15</v>
       </c>
       <c r="E25" s="48" t="s">
-        <v>151</v>
+        <v>143</v>
       </c>
       <c r="F25" s="48" t="s">
-        <v>152</v>
+        <v>144</v>
       </c>
       <c r="G25" s="48" t="s">
-        <v>172</v>
+        <v>167</v>
       </c>
       <c r="H25" s="47" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="I25" s="48" t="s">
         <v>62</v>
@@ -2265,47 +2338,47 @@
       <c r="A26" s="64"/>
       <c r="B26" s="64"/>
       <c r="C26" s="47">
-        <v>14.5</v>
+        <v>14.3</v>
       </c>
       <c r="D26" s="48" t="s">
-        <v>15</v>
+        <v>145</v>
       </c>
       <c r="E26" s="48" t="s">
-        <v>153</v>
+        <v>146</v>
       </c>
       <c r="F26" s="48" t="s">
-        <v>154</v>
+        <v>147</v>
       </c>
       <c r="G26" s="48" t="s">
-        <v>173</v>
+        <v>168</v>
       </c>
       <c r="H26" s="47" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="I26" s="48" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="27" spans="1:9" s="4" customFormat="1" ht="41.4" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:9" s="4" customFormat="1" ht="55.2" x14ac:dyDescent="0.3">
       <c r="A27" s="64"/>
       <c r="B27" s="64"/>
       <c r="C27" s="47">
-        <v>14.6</v>
+        <v>14.4</v>
       </c>
       <c r="D27" s="48" t="s">
         <v>15</v>
       </c>
       <c r="E27" s="48" t="s">
-        <v>155</v>
+        <v>148</v>
       </c>
       <c r="F27" s="48" t="s">
-        <v>156</v>
+        <v>149</v>
       </c>
       <c r="G27" s="48" t="s">
-        <v>179</v>
+        <v>169</v>
       </c>
       <c r="H27" s="47" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="I27" s="48" t="s">
         <v>62</v>
@@ -2315,22 +2388,22 @@
       <c r="A28" s="64"/>
       <c r="B28" s="64"/>
       <c r="C28" s="47">
-        <v>14.7</v>
+        <v>14.5</v>
       </c>
       <c r="D28" s="48" t="s">
         <v>15</v>
       </c>
       <c r="E28" s="48" t="s">
-        <v>157</v>
+        <v>150</v>
       </c>
       <c r="F28" s="48" t="s">
-        <v>158</v>
+        <v>151</v>
       </c>
       <c r="G28" s="48" t="s">
-        <v>174</v>
+        <v>170</v>
       </c>
       <c r="H28" s="47" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="I28" s="48" t="s">
         <v>62</v>
@@ -2340,736 +2413,786 @@
       <c r="A29" s="64"/>
       <c r="B29" s="64"/>
       <c r="C29" s="47">
-        <v>14.8</v>
+        <v>14.6</v>
       </c>
       <c r="D29" s="48" t="s">
         <v>15</v>
       </c>
       <c r="E29" s="48" t="s">
-        <v>159</v>
+        <v>152</v>
       </c>
       <c r="F29" s="48" t="s">
-        <v>160</v>
+        <v>153</v>
       </c>
       <c r="G29" s="48" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="H29" s="47" t="s">
-        <v>140</v>
+        <v>101</v>
       </c>
       <c r="I29" s="48" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="30" spans="1:9" s="4" customFormat="1" ht="55.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:9" s="4" customFormat="1" ht="41.4" x14ac:dyDescent="0.3">
       <c r="A30" s="64"/>
       <c r="B30" s="64"/>
       <c r="C30" s="47">
-        <v>14.9</v>
+        <v>14.7</v>
       </c>
       <c r="D30" s="48" t="s">
         <v>15</v>
       </c>
       <c r="E30" s="48" t="s">
-        <v>161</v>
+        <v>154</v>
       </c>
       <c r="F30" s="48" t="s">
-        <v>162</v>
+        <v>155</v>
       </c>
       <c r="G30" s="48" t="s">
-        <v>176</v>
+        <v>171</v>
       </c>
       <c r="H30" s="47" t="s">
-        <v>140</v>
+        <v>101</v>
       </c>
       <c r="I30" s="48" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="31" spans="1:9" s="4" customFormat="1" ht="55.2" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:9" s="4" customFormat="1" ht="41.4" x14ac:dyDescent="0.3">
       <c r="A31" s="64"/>
       <c r="B31" s="64"/>
       <c r="C31" s="47">
-        <v>14.1</v>
+        <v>14.8</v>
       </c>
       <c r="D31" s="48" t="s">
         <v>15</v>
       </c>
       <c r="E31" s="48" t="s">
-        <v>163</v>
+        <v>156</v>
       </c>
       <c r="F31" s="48" t="s">
-        <v>164</v>
+        <v>157</v>
       </c>
       <c r="G31" s="48" t="s">
-        <v>177</v>
+        <v>172</v>
       </c>
       <c r="H31" s="47" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="I31" s="48" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="32" spans="1:9" s="4" customFormat="1" ht="41.4" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:9" s="4" customFormat="1" ht="55.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A32" s="64"/>
       <c r="B32" s="64"/>
       <c r="C32" s="47">
-        <v>14.11</v>
+        <v>14.9</v>
       </c>
       <c r="D32" s="48" t="s">
         <v>15</v>
       </c>
       <c r="E32" s="48" t="s">
-        <v>165</v>
+        <v>158</v>
       </c>
       <c r="F32" s="48" t="s">
-        <v>166</v>
+        <v>159</v>
       </c>
       <c r="G32" s="48" t="s">
-        <v>178</v>
+        <v>173</v>
       </c>
       <c r="H32" s="47" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="I32" s="48" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="33" spans="1:9" s="4" customFormat="1" ht="27.6" x14ac:dyDescent="0.3">
-      <c r="A33" s="57">
+    <row r="33" spans="1:9" s="4" customFormat="1" ht="55.2" x14ac:dyDescent="0.3">
+      <c r="A33" s="64"/>
+      <c r="B33" s="64"/>
+      <c r="C33" s="47">
+        <v>14.1</v>
+      </c>
+      <c r="D33" s="48" t="s">
         <v>15</v>
       </c>
-      <c r="B33" s="57" t="s">
+      <c r="E33" s="48" t="s">
+        <v>160</v>
+      </c>
+      <c r="F33" s="48" t="s">
+        <v>161</v>
+      </c>
+      <c r="G33" s="48" t="s">
+        <v>174</v>
+      </c>
+      <c r="H33" s="47" t="s">
+        <v>137</v>
+      </c>
+      <c r="I33" s="48" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="34" spans="1:9" s="4" customFormat="1" ht="41.4" x14ac:dyDescent="0.3">
+      <c r="A34" s="64"/>
+      <c r="B34" s="64"/>
+      <c r="C34" s="47">
+        <v>14.11</v>
+      </c>
+      <c r="D34" s="48" t="s">
+        <v>15</v>
+      </c>
+      <c r="E34" s="48" t="s">
+        <v>162</v>
+      </c>
+      <c r="F34" s="48" t="s">
+        <v>163</v>
+      </c>
+      <c r="G34" s="48" t="s">
+        <v>175</v>
+      </c>
+      <c r="H34" s="47" t="s">
+        <v>137</v>
+      </c>
+      <c r="I34" s="48" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="35" spans="1:9" s="4" customFormat="1" ht="27.6" x14ac:dyDescent="0.3">
+      <c r="A35" s="66">
+        <v>15</v>
+      </c>
+      <c r="B35" s="66" t="s">
         <v>63</v>
       </c>
-      <c r="C33" s="19">
+      <c r="C35" s="19">
         <v>15.1</v>
-      </c>
-      <c r="D33" s="20" t="s">
-        <v>64</v>
-      </c>
-      <c r="E33" s="20" t="s">
-        <v>65</v>
-      </c>
-      <c r="F33" s="20" t="s">
-        <v>66</v>
-      </c>
-      <c r="G33" s="20" t="s">
-        <v>67</v>
-      </c>
-      <c r="H33" s="19" t="s">
-        <v>141</v>
-      </c>
-      <c r="I33" s="20" t="s">
-        <v>142</v>
-      </c>
-    </row>
-    <row r="34" spans="1:9" s="4" customFormat="1" ht="27.6" x14ac:dyDescent="0.3">
-      <c r="A34" s="58"/>
-      <c r="B34" s="58"/>
-      <c r="C34" s="19">
-        <v>15.2</v>
-      </c>
-      <c r="D34" s="20" t="s">
-        <v>64</v>
-      </c>
-      <c r="E34" s="20" t="s">
-        <v>68</v>
-      </c>
-      <c r="F34" s="20" t="s">
-        <v>69</v>
-      </c>
-      <c r="G34" s="20" t="s">
-        <v>70</v>
-      </c>
-      <c r="H34" s="19" t="s">
-        <v>141</v>
-      </c>
-      <c r="I34" s="20" t="s">
-        <v>142</v>
-      </c>
-    </row>
-    <row r="35" spans="1:9" s="4" customFormat="1" ht="27.6" x14ac:dyDescent="0.3">
-      <c r="A35" s="58"/>
-      <c r="B35" s="58"/>
-      <c r="C35" s="19">
-        <v>15.3</v>
       </c>
       <c r="D35" s="20" t="s">
         <v>64</v>
       </c>
       <c r="E35" s="20" t="s">
-        <v>71</v>
+        <v>65</v>
       </c>
       <c r="F35" s="20" t="s">
-        <v>72</v>
+        <v>66</v>
       </c>
       <c r="G35" s="20" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="H35" s="19" t="s">
-        <v>141</v>
+        <v>138</v>
       </c>
       <c r="I35" s="20" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
     </row>
     <row r="36" spans="1:9" s="4" customFormat="1" ht="27.6" x14ac:dyDescent="0.3">
-      <c r="A36" s="58"/>
-      <c r="B36" s="58"/>
+      <c r="A36" s="59"/>
+      <c r="B36" s="59"/>
       <c r="C36" s="19">
-        <v>15.4</v>
+        <v>15.2</v>
       </c>
       <c r="D36" s="20" t="s">
         <v>64</v>
       </c>
       <c r="E36" s="20" t="s">
-        <v>74</v>
+        <v>68</v>
       </c>
       <c r="F36" s="20" t="s">
-        <v>75</v>
+        <v>69</v>
       </c>
       <c r="G36" s="20" t="s">
-        <v>76</v>
+        <v>70</v>
       </c>
       <c r="H36" s="19" t="s">
-        <v>143</v>
+        <v>138</v>
       </c>
       <c r="I36" s="20" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
     </row>
     <row r="37" spans="1:9" s="4" customFormat="1" ht="27.6" x14ac:dyDescent="0.3">
-      <c r="A37" s="58"/>
-      <c r="B37" s="58"/>
+      <c r="A37" s="59"/>
+      <c r="B37" s="59"/>
       <c r="C37" s="19">
-        <v>15.5</v>
+        <v>15.3</v>
       </c>
       <c r="D37" s="20" t="s">
         <v>64</v>
       </c>
       <c r="E37" s="20" t="s">
+        <v>71</v>
+      </c>
+      <c r="F37" s="20" t="s">
+        <v>72</v>
+      </c>
+      <c r="G37" s="20" t="s">
+        <v>73</v>
+      </c>
+      <c r="H37" s="19" t="s">
+        <v>138</v>
+      </c>
+      <c r="I37" s="20" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="38" spans="1:9" s="4" customFormat="1" ht="27.6" x14ac:dyDescent="0.3">
+      <c r="A38" s="59"/>
+      <c r="B38" s="59"/>
+      <c r="C38" s="19">
+        <v>15.4</v>
+      </c>
+      <c r="D38" s="20" t="s">
+        <v>64</v>
+      </c>
+      <c r="E38" s="20" t="s">
+        <v>74</v>
+      </c>
+      <c r="F38" s="20" t="s">
+        <v>75</v>
+      </c>
+      <c r="G38" s="20" t="s">
+        <v>76</v>
+      </c>
+      <c r="H38" s="19" t="s">
+        <v>140</v>
+      </c>
+      <c r="I38" s="20" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="39" spans="1:9" s="4" customFormat="1" ht="27.6" x14ac:dyDescent="0.3">
+      <c r="A39" s="59"/>
+      <c r="B39" s="59"/>
+      <c r="C39" s="19">
+        <v>15.5</v>
+      </c>
+      <c r="D39" s="20" t="s">
+        <v>64</v>
+      </c>
+      <c r="E39" s="20" t="s">
         <v>77</v>
       </c>
-      <c r="F37" s="20" t="s">
+      <c r="F39" s="20" t="s">
         <v>78</v>
       </c>
-      <c r="G37" s="20" t="s">
+      <c r="G39" s="20" t="s">
         <v>79</v>
       </c>
-      <c r="H37" s="19" t="s">
-        <v>143</v>
-      </c>
-      <c r="I37" s="20" t="s">
-        <v>142</v>
-      </c>
-    </row>
-    <row r="38" spans="1:9" s="4" customFormat="1" ht="27.6" x14ac:dyDescent="0.3">
-      <c r="A38" s="66">
+      <c r="H39" s="19" t="s">
+        <v>140</v>
+      </c>
+      <c r="I39" s="20" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="40" spans="1:9" s="4" customFormat="1" ht="27.6" x14ac:dyDescent="0.3">
+      <c r="A40" s="62">
         <v>16</v>
       </c>
-      <c r="B38" s="66" t="s">
+      <c r="B40" s="62" t="s">
         <v>80</v>
       </c>
-      <c r="C38" s="21">
+      <c r="C40" s="21">
         <v>16.100000000000001</v>
       </c>
-      <c r="D38" s="22" t="s">
+      <c r="D40" s="22" t="s">
         <v>81</v>
       </c>
-      <c r="E38" s="22" t="s">
+      <c r="E40" s="22" t="s">
         <v>82</v>
       </c>
-      <c r="F38" s="22" t="s">
+      <c r="F40" s="22" t="s">
         <v>83</v>
       </c>
-      <c r="G38" s="45" t="s">
+      <c r="G40" s="45" t="s">
         <v>84</v>
       </c>
-      <c r="H38" s="44" t="s">
-        <v>143</v>
-      </c>
-      <c r="I38" s="45" t="s">
-        <v>142</v>
-      </c>
-    </row>
-    <row r="39" spans="1:9" s="4" customFormat="1" ht="27.6" x14ac:dyDescent="0.3">
-      <c r="A39" s="58"/>
-      <c r="B39" s="58"/>
-      <c r="C39" s="21">
+      <c r="H40" s="44" t="s">
+        <v>140</v>
+      </c>
+      <c r="I40" s="45" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="41" spans="1:9" s="4" customFormat="1" ht="27.6" x14ac:dyDescent="0.3">
+      <c r="A41" s="59"/>
+      <c r="B41" s="59"/>
+      <c r="C41" s="21">
         <v>16.2</v>
       </c>
-      <c r="D39" s="22" t="s">
+      <c r="D41" s="22" t="s">
         <v>85</v>
       </c>
-      <c r="E39" s="22" t="s">
+      <c r="E41" s="22" t="s">
         <v>86</v>
       </c>
-      <c r="F39" s="22" t="s">
+      <c r="F41" s="22" t="s">
         <v>87</v>
       </c>
-      <c r="G39" s="22" t="s">
+      <c r="G41" s="22" t="s">
         <v>88</v>
       </c>
-      <c r="H39" s="44" t="s">
-        <v>143</v>
-      </c>
-      <c r="I39" s="45" t="s">
-        <v>142</v>
-      </c>
-    </row>
-    <row r="40" spans="1:9" s="4" customFormat="1" ht="27.6" x14ac:dyDescent="0.3">
-      <c r="A40" s="65">
+      <c r="H41" s="44" t="s">
+        <v>140</v>
+      </c>
+      <c r="I41" s="45" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="42" spans="1:9" s="4" customFormat="1" ht="27.6" x14ac:dyDescent="0.3">
+      <c r="A42" s="58">
         <v>17</v>
       </c>
-      <c r="B40" s="65" t="s">
+      <c r="B42" s="58" t="s">
         <v>89</v>
       </c>
-      <c r="C40" s="5">
+      <c r="C42" s="5">
         <v>17.100000000000001</v>
-      </c>
-      <c r="D40" s="6" t="s">
-        <v>90</v>
-      </c>
-      <c r="E40" s="37" t="s">
-        <v>167</v>
-      </c>
-      <c r="F40" s="6" t="s">
-        <v>91</v>
-      </c>
-      <c r="G40" s="37" t="s">
-        <v>168</v>
-      </c>
-      <c r="H40" s="5" t="s">
-        <v>102</v>
-      </c>
-      <c r="I40" s="37" t="s">
-        <v>124</v>
-      </c>
-    </row>
-    <row r="41" spans="1:9" s="4" customFormat="1" ht="27.6" x14ac:dyDescent="0.3">
-      <c r="A41" s="58"/>
-      <c r="B41" s="58"/>
-      <c r="C41" s="5">
-        <v>17.2</v>
-      </c>
-      <c r="D41" s="6" t="s">
-        <v>90</v>
-      </c>
-      <c r="E41" s="37" t="s">
-        <v>112</v>
-      </c>
-      <c r="F41" s="6" t="s">
-        <v>92</v>
-      </c>
-      <c r="G41" s="37" t="s">
-        <v>93</v>
-      </c>
-      <c r="H41" s="5" t="s">
-        <v>102</v>
-      </c>
-      <c r="I41" s="37" t="s">
-        <v>124</v>
-      </c>
-    </row>
-    <row r="42" spans="1:9" s="4" customFormat="1" ht="27.6" x14ac:dyDescent="0.3">
-      <c r="A42" s="58"/>
-      <c r="B42" s="58"/>
-      <c r="C42" s="5">
-        <v>17.3</v>
       </c>
       <c r="D42" s="6" t="s">
         <v>90</v>
       </c>
-      <c r="E42" s="6" t="s">
-        <v>94</v>
-      </c>
-      <c r="F42" s="37" t="s">
-        <v>113</v>
+      <c r="E42" s="37" t="s">
+        <v>164</v>
+      </c>
+      <c r="F42" s="6" t="s">
+        <v>91</v>
       </c>
       <c r="G42" s="37" t="s">
-        <v>116</v>
+        <v>165</v>
       </c>
       <c r="H42" s="5" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="I42" s="37" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
     </row>
     <row r="43" spans="1:9" s="4" customFormat="1" ht="27.6" x14ac:dyDescent="0.3">
-      <c r="A43" s="58"/>
-      <c r="B43" s="58"/>
+      <c r="A43" s="59"/>
+      <c r="B43" s="59"/>
       <c r="C43" s="5">
-        <v>17.399999999999999</v>
+        <v>17.2</v>
       </c>
       <c r="D43" s="6" t="s">
         <v>90</v>
       </c>
       <c r="E43" s="37" t="s">
-        <v>115</v>
-      </c>
-      <c r="F43" s="37" t="s">
-        <v>114</v>
+        <v>111</v>
+      </c>
+      <c r="F43" s="6" t="s">
+        <v>92</v>
       </c>
       <c r="G43" s="37" t="s">
-        <v>120</v>
+        <v>93</v>
       </c>
       <c r="H43" s="5" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="I43" s="37" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
     </row>
     <row r="44" spans="1:9" s="4" customFormat="1" ht="27.6" x14ac:dyDescent="0.3">
-      <c r="A44" s="58"/>
-      <c r="B44" s="58"/>
+      <c r="A44" s="59"/>
+      <c r="B44" s="59"/>
       <c r="C44" s="5">
-        <v>17.5</v>
+        <v>17.3</v>
       </c>
       <c r="D44" s="6" t="s">
         <v>90</v>
       </c>
-      <c r="E44" s="37" t="s">
-        <v>117</v>
+      <c r="E44" s="6" t="s">
+        <v>94</v>
       </c>
       <c r="F44" s="37" t="s">
-        <v>118</v>
+        <v>112</v>
       </c>
       <c r="G44" s="37" t="s">
-        <v>119</v>
+        <v>115</v>
       </c>
       <c r="H44" s="5" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="I44" s="37" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
     </row>
     <row r="45" spans="1:9" s="4" customFormat="1" ht="27.6" x14ac:dyDescent="0.3">
-      <c r="A45" s="58"/>
-      <c r="B45" s="58"/>
+      <c r="A45" s="59"/>
+      <c r="B45" s="59"/>
       <c r="C45" s="5">
-        <v>17.600000000000001</v>
+        <v>17.399999999999999</v>
       </c>
       <c r="D45" s="6" t="s">
         <v>90</v>
       </c>
-      <c r="E45" s="6" t="s">
-        <v>95</v>
+      <c r="E45" s="37" t="s">
+        <v>114</v>
       </c>
       <c r="F45" s="37" t="s">
-        <v>121</v>
+        <v>113</v>
       </c>
       <c r="G45" s="37" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="H45" s="5" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="I45" s="37" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
     </row>
     <row r="46" spans="1:9" s="4" customFormat="1" ht="27.6" x14ac:dyDescent="0.3">
-      <c r="A46" s="58"/>
-      <c r="B46" s="58"/>
+      <c r="A46" s="59"/>
+      <c r="B46" s="59"/>
       <c r="C46" s="5">
-        <v>17.7</v>
+        <v>17.5</v>
       </c>
       <c r="D46" s="6" t="s">
         <v>90</v>
       </c>
-      <c r="E46" s="6" t="s">
+      <c r="E46" s="37" t="s">
+        <v>116</v>
+      </c>
+      <c r="F46" s="37" t="s">
+        <v>117</v>
+      </c>
+      <c r="G46" s="37" t="s">
+        <v>118</v>
+      </c>
+      <c r="H46" s="5" t="s">
+        <v>101</v>
+      </c>
+      <c r="I46" s="37" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="47" spans="1:9" s="4" customFormat="1" ht="27.6" x14ac:dyDescent="0.3">
+      <c r="A47" s="59"/>
+      <c r="B47" s="59"/>
+      <c r="C47" s="5">
+        <v>17.600000000000001</v>
+      </c>
+      <c r="D47" s="6" t="s">
+        <v>90</v>
+      </c>
+      <c r="E47" s="6" t="s">
+        <v>95</v>
+      </c>
+      <c r="F47" s="37" t="s">
+        <v>120</v>
+      </c>
+      <c r="G47" s="37" t="s">
+        <v>121</v>
+      </c>
+      <c r="H47" s="5" t="s">
+        <v>101</v>
+      </c>
+      <c r="I47" s="37" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="48" spans="1:9" s="4" customFormat="1" ht="27.6" x14ac:dyDescent="0.3">
+      <c r="A48" s="59"/>
+      <c r="B48" s="59"/>
+      <c r="C48" s="5">
+        <v>17.7</v>
+      </c>
+      <c r="D48" s="6" t="s">
+        <v>90</v>
+      </c>
+      <c r="E48" s="6" t="s">
         <v>96</v>
       </c>
-      <c r="F46" s="37" t="s">
+      <c r="F48" s="37" t="s">
+        <v>122</v>
+      </c>
+      <c r="G48" s="37" t="s">
+        <v>129</v>
+      </c>
+      <c r="H48" s="5" t="s">
+        <v>101</v>
+      </c>
+      <c r="I48" s="37" t="s">
         <v>123</v>
       </c>
-      <c r="G46" s="37" t="s">
-        <v>130</v>
-      </c>
-      <c r="H46" s="5" t="s">
-        <v>102</v>
-      </c>
-      <c r="I46" s="37" t="s">
-        <v>124</v>
-      </c>
-    </row>
-    <row r="47" spans="1:9" s="4" customFormat="1" ht="82.8" x14ac:dyDescent="0.3">
-      <c r="A47" s="68">
+    </row>
+    <row r="49" spans="1:12" s="4" customFormat="1" ht="82.8" x14ac:dyDescent="0.3">
+      <c r="A49" s="56">
         <v>18</v>
       </c>
-      <c r="B47" s="69" t="s">
+      <c r="B49" s="57" t="s">
+        <v>186</v>
+      </c>
+      <c r="C49" s="53">
+        <v>18.100000000000001</v>
+      </c>
+      <c r="D49" s="49" t="s">
+        <v>187</v>
+      </c>
+      <c r="E49" s="49" t="s">
+        <v>188</v>
+      </c>
+      <c r="F49" s="49" t="s">
         <v>189</v>
       </c>
-      <c r="C47" s="53">
-        <v>18.100000000000001</v>
-      </c>
-      <c r="D47" s="49" t="s">
-        <v>190</v>
-      </c>
-      <c r="E47" s="49" t="s">
-        <v>191</v>
-      </c>
-      <c r="F47" s="49" t="s">
-        <v>192</v>
-      </c>
-      <c r="G47" s="49" t="s">
-        <v>196</v>
-      </c>
-      <c r="H47" s="53"/>
-      <c r="I47" s="54"/>
-    </row>
-    <row r="48" spans="1:9" s="4" customFormat="1" ht="124.2" x14ac:dyDescent="0.3">
-      <c r="A48" s="68"/>
-      <c r="B48" s="69"/>
-      <c r="C48" s="52">
-        <v>18.2</v>
-      </c>
-      <c r="D48" s="49" t="s">
+      <c r="G49" s="49" t="s">
         <v>193</v>
-      </c>
-      <c r="E48" s="49" t="s">
-        <v>194</v>
-      </c>
-      <c r="F48" s="49" t="s">
-        <v>186</v>
-      </c>
-      <c r="G48" s="49" t="s">
-        <v>195</v>
-      </c>
-      <c r="H48" s="53"/>
-      <c r="I48" s="54"/>
-    </row>
-    <row r="49" spans="1:12" s="4" customFormat="1" ht="82.8" x14ac:dyDescent="0.3">
-      <c r="A49" s="68">
-        <v>19</v>
-      </c>
-      <c r="B49" s="69" t="s">
-        <v>197</v>
-      </c>
-      <c r="C49" s="53">
-        <v>19.100000000000001</v>
-      </c>
-      <c r="D49" s="49" t="s">
-        <v>198</v>
-      </c>
-      <c r="E49" s="49" t="s">
-        <v>200</v>
-      </c>
-      <c r="F49" s="49" t="s">
-        <v>202</v>
-      </c>
-      <c r="G49" s="49" t="s">
-        <v>203</v>
       </c>
       <c r="H49" s="53"/>
       <c r="I49" s="54"/>
     </row>
     <row r="50" spans="1:12" s="4" customFormat="1" ht="124.2" x14ac:dyDescent="0.3">
-      <c r="A50" s="68"/>
-      <c r="B50" s="69"/>
+      <c r="A50" s="56"/>
+      <c r="B50" s="57"/>
       <c r="C50" s="52">
-        <v>19.2</v>
+        <v>18.2</v>
       </c>
       <c r="D50" s="49" t="s">
-        <v>199</v>
+        <v>190</v>
       </c>
       <c r="E50" s="49" t="s">
-        <v>201</v>
+        <v>191</v>
       </c>
       <c r="F50" s="49" t="s">
-        <v>186</v>
+        <v>183</v>
       </c>
       <c r="G50" s="49" t="s">
-        <v>204</v>
+        <v>192</v>
       </c>
       <c r="H50" s="53"/>
       <c r="I50" s="54"/>
-      <c r="J50" s="3"/>
-      <c r="K50" s="3"/>
-      <c r="L50" s="3"/>
-    </row>
-    <row r="51" spans="1:12" ht="104.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A51" s="68">
-        <v>20</v>
-      </c>
-      <c r="B51" s="69" t="s">
-        <v>205</v>
+    </row>
+    <row r="51" spans="1:12" s="4" customFormat="1" ht="82.8" x14ac:dyDescent="0.3">
+      <c r="A51" s="56">
+        <v>19</v>
+      </c>
+      <c r="B51" s="57" t="s">
+        <v>194</v>
       </c>
       <c r="C51" s="53">
-        <v>20.100000000000001</v>
+        <v>19.100000000000001</v>
       </c>
       <c r="D51" s="49" t="s">
-        <v>206</v>
+        <v>195</v>
       </c>
       <c r="E51" s="49" t="s">
-        <v>211</v>
+        <v>197</v>
       </c>
       <c r="F51" s="49" t="s">
-        <v>210</v>
+        <v>199</v>
       </c>
       <c r="G51" s="49" t="s">
-        <v>212</v>
+        <v>200</v>
       </c>
       <c r="H51" s="53"/>
       <c r="I51" s="54"/>
     </row>
-    <row r="52" spans="1:12" ht="135" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A52" s="68"/>
-      <c r="B52" s="69"/>
+    <row r="52" spans="1:12" s="4" customFormat="1" ht="124.2" x14ac:dyDescent="0.3">
+      <c r="A52" s="56"/>
+      <c r="B52" s="57"/>
       <c r="C52" s="52">
-        <v>20.2</v>
+        <v>19.2</v>
       </c>
       <c r="D52" s="49" t="s">
-        <v>207</v>
+        <v>196</v>
       </c>
       <c r="E52" s="49" t="s">
-        <v>209</v>
+        <v>198</v>
       </c>
       <c r="F52" s="49" t="s">
-        <v>186</v>
+        <v>183</v>
       </c>
       <c r="G52" s="49" t="s">
-        <v>208</v>
+        <v>201</v>
       </c>
       <c r="H52" s="53"/>
       <c r="I52" s="54"/>
-    </row>
-    <row r="53" spans="1:12" ht="179.4" x14ac:dyDescent="0.3">
-      <c r="A53" s="68">
-        <v>21</v>
-      </c>
-      <c r="B53" s="69" t="s">
-        <v>213</v>
+      <c r="J52" s="3"/>
+      <c r="K52" s="3"/>
+      <c r="L52" s="3"/>
+    </row>
+    <row r="53" spans="1:12" ht="104.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A53" s="56">
+        <v>20</v>
+      </c>
+      <c r="B53" s="57" t="s">
+        <v>202</v>
       </c>
       <c r="C53" s="53">
-        <v>21.1</v>
+        <v>20.100000000000001</v>
       </c>
       <c r="D53" s="49" t="s">
-        <v>214</v>
+        <v>203</v>
       </c>
       <c r="E53" s="49" t="s">
-        <v>217</v>
+        <v>208</v>
       </c>
       <c r="F53" s="49" t="s">
-        <v>218</v>
+        <v>207</v>
       </c>
       <c r="G53" s="49" t="s">
-        <v>219</v>
+        <v>209</v>
       </c>
       <c r="H53" s="53"/>
       <c r="I53" s="54"/>
     </row>
-    <row r="54" spans="1:12" ht="124.2" x14ac:dyDescent="0.3">
-      <c r="A54" s="68"/>
-      <c r="B54" s="69"/>
+    <row r="54" spans="1:12" ht="135" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A54" s="56"/>
+      <c r="B54" s="57"/>
       <c r="C54" s="52">
-        <v>21.2</v>
+        <v>20.2</v>
       </c>
       <c r="D54" s="49" t="s">
-        <v>215</v>
-      </c>
-      <c r="E54" s="55" t="s">
-        <v>220</v>
+        <v>204</v>
+      </c>
+      <c r="E54" s="49" t="s">
+        <v>206</v>
       </c>
       <c r="F54" s="49" t="s">
-        <v>186</v>
+        <v>183</v>
       </c>
       <c r="G54" s="49" t="s">
-        <v>216</v>
+        <v>205</v>
       </c>
       <c r="H54" s="53"/>
       <c r="I54" s="54"/>
     </row>
-    <row r="55" spans="1:12" ht="36" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A55" s="2"/>
-      <c r="B55" s="2"/>
-      <c r="C55" s="2"/>
-      <c r="E55" s="49"/>
-      <c r="H55" s="2"/>
-    </row>
-    <row r="56" spans="1:12" ht="31.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="D56" s="1"/>
-      <c r="F56" s="1"/>
-      <c r="G56" s="1"/>
-      <c r="I56" s="1"/>
-    </row>
-    <row r="57" spans="1:12" ht="34.950000000000003" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="D57" s="1"/>
-      <c r="F57" s="1"/>
-      <c r="G57" s="1"/>
-      <c r="I57" s="1"/>
-    </row>
-    <row r="58" spans="1:12" ht="31.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A58" s="46"/>
-      <c r="B58" s="46"/>
-      <c r="C58" s="46"/>
-      <c r="D58" s="46"/>
-      <c r="E58" s="46"/>
-      <c r="F58" s="46"/>
-      <c r="G58" s="46"/>
-      <c r="H58" s="46"/>
-      <c r="I58" s="46"/>
-    </row>
-    <row r="59" spans="1:12" ht="33.450000000000003" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A59" s="2"/>
-      <c r="B59" s="2"/>
-      <c r="C59" s="2"/>
-      <c r="E59" s="2"/>
-      <c r="H59" s="2"/>
-    </row>
-    <row r="60" spans="1:12" ht="31.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="D60" s="1"/>
-      <c r="F60" s="1"/>
-      <c r="G60" s="1"/>
-      <c r="I60" s="1"/>
-    </row>
-    <row r="61" spans="1:12" ht="27.45" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:12" ht="179.4" x14ac:dyDescent="0.3">
+      <c r="A55" s="56">
+        <v>21</v>
+      </c>
+      <c r="B55" s="57" t="s">
+        <v>210</v>
+      </c>
+      <c r="C55" s="53">
+        <v>21.1</v>
+      </c>
+      <c r="D55" s="49" t="s">
+        <v>211</v>
+      </c>
+      <c r="E55" s="49" t="s">
+        <v>214</v>
+      </c>
+      <c r="F55" s="49" t="s">
+        <v>215</v>
+      </c>
+      <c r="G55" s="49" t="s">
+        <v>216</v>
+      </c>
+      <c r="H55" s="53"/>
+      <c r="I55" s="54"/>
+    </row>
+    <row r="56" spans="1:12" ht="124.2" x14ac:dyDescent="0.3">
+      <c r="A56" s="56"/>
+      <c r="B56" s="57"/>
+      <c r="C56" s="52">
+        <v>21.2</v>
+      </c>
+      <c r="D56" s="49" t="s">
+        <v>212</v>
+      </c>
+      <c r="E56" s="55" t="s">
+        <v>217</v>
+      </c>
+      <c r="F56" s="49" t="s">
+        <v>183</v>
+      </c>
+      <c r="G56" s="49" t="s">
+        <v>213</v>
+      </c>
+      <c r="H56" s="53"/>
+      <c r="I56" s="54"/>
+    </row>
+    <row r="57" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A57" s="2"/>
+      <c r="B57" s="2"/>
+      <c r="C57" s="2"/>
+      <c r="E57" s="49"/>
+      <c r="H57" s="2"/>
+    </row>
+    <row r="58" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="D58" s="1"/>
+      <c r="F58" s="1"/>
+      <c r="G58" s="1"/>
+      <c r="I58" s="1"/>
+    </row>
+    <row r="59" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="D59" s="1"/>
+      <c r="F59" s="1"/>
+      <c r="G59" s="1"/>
+      <c r="I59" s="1"/>
+    </row>
+    <row r="60" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A60" s="46"/>
+      <c r="B60" s="46"/>
+      <c r="C60" s="46"/>
+      <c r="D60" s="46"/>
+      <c r="E60" s="46"/>
+      <c r="F60" s="46"/>
+      <c r="G60" s="46"/>
+      <c r="H60" s="46"/>
+      <c r="I60" s="46"/>
+    </row>
+    <row r="61" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A61" s="2"/>
       <c r="B61" s="2"/>
-      <c r="F61" s="1"/>
-      <c r="G61" s="1"/>
-      <c r="I61" s="1"/>
+      <c r="C61" s="2"/>
+      <c r="E61" s="2"/>
+      <c r="H61" s="2"/>
+    </row>
+    <row r="62" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="D62" s="1"/>
+      <c r="F62" s="1"/>
+      <c r="G62" s="1"/>
+      <c r="I62" s="1"/>
+    </row>
+    <row r="63" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="B63" s="2"/>
+      <c r="F63" s="1"/>
+      <c r="G63" s="1"/>
+      <c r="I63" s="1"/>
     </row>
   </sheetData>
-  <autoFilter ref="I1:I19" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
+  <autoFilter ref="I1:I21" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
   <mergeCells count="33">
-    <mergeCell ref="A53:A54"/>
-    <mergeCell ref="B53:B54"/>
-    <mergeCell ref="B47:B48"/>
-    <mergeCell ref="A47:A48"/>
-    <mergeCell ref="A49:A50"/>
-    <mergeCell ref="B49:B50"/>
-    <mergeCell ref="A51:A52"/>
-    <mergeCell ref="B51:B52"/>
-    <mergeCell ref="A40:A46"/>
-    <mergeCell ref="B13:B16"/>
-    <mergeCell ref="B40:B46"/>
-    <mergeCell ref="A10:A12"/>
-    <mergeCell ref="A38:A39"/>
-    <mergeCell ref="B17:B21"/>
-    <mergeCell ref="A17:A21"/>
-    <mergeCell ref="B22:B32"/>
-    <mergeCell ref="B38:B39"/>
+    <mergeCell ref="B8:B11"/>
+    <mergeCell ref="A8:A11"/>
     <mergeCell ref="B5:B6"/>
     <mergeCell ref="A5:A6"/>
-    <mergeCell ref="A33:A37"/>
+    <mergeCell ref="A35:A39"/>
     <mergeCell ref="I1:I2"/>
     <mergeCell ref="D1:F1"/>
-    <mergeCell ref="A13:A16"/>
-    <mergeCell ref="A8:A9"/>
-    <mergeCell ref="B10:B12"/>
+    <mergeCell ref="A15:A18"/>
+    <mergeCell ref="B12:B14"/>
     <mergeCell ref="H1:H2"/>
-    <mergeCell ref="B33:B37"/>
+    <mergeCell ref="B35:B39"/>
     <mergeCell ref="A1:A2"/>
-    <mergeCell ref="A22:A32"/>
+    <mergeCell ref="A24:A34"/>
     <mergeCell ref="C1:C2"/>
     <mergeCell ref="G1:G2"/>
     <mergeCell ref="B1:B2"/>
-    <mergeCell ref="B8:B9"/>
+    <mergeCell ref="A42:A48"/>
+    <mergeCell ref="B15:B18"/>
+    <mergeCell ref="B42:B48"/>
+    <mergeCell ref="A12:A14"/>
+    <mergeCell ref="A40:A41"/>
+    <mergeCell ref="B19:B23"/>
+    <mergeCell ref="A19:A23"/>
+    <mergeCell ref="B24:B34"/>
+    <mergeCell ref="B40:B41"/>
+    <mergeCell ref="A55:A56"/>
+    <mergeCell ref="B55:B56"/>
+    <mergeCell ref="B49:B50"/>
+    <mergeCell ref="A49:A50"/>
+    <mergeCell ref="A51:A52"/>
+    <mergeCell ref="B51:B52"/>
+    <mergeCell ref="A53:A54"/>
+    <mergeCell ref="B53:B54"/>
   </mergeCells>
   <phoneticPr fontId="6" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Ambiguities added, product backlog updated
</commit_message>
<xml_diff>
--- a/Soubhanik/checkupp_product_backlog_final.xlsx
+++ b/Soubhanik/checkupp_product_backlog_final.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Anodiam\2026\CheckUpp_Parent\CheckUpp\Soubhanik\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GitHub\CheckUpp\Soubhanik\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{43CB0B16-3146-438B-94C7-AFE204B96F65}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F7E4E8CF-3396-47EF-8A96-4CC709A97038}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -3241,11 +3241,18 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="15" x14ac:knownFonts="1">
+  <fonts count="16" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -3532,7 +3539,7 @@
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="80">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
@@ -3545,10 +3552,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
@@ -3566,211 +3573,211 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="15" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="14" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="15" fillId="14" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="15" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="5" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="16" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="16" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="16" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="6" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="14" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="14" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="14" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="15" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="17" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="17" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="13" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="13" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="15" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="15" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="15" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="6" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="6" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="14" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="14" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="14" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="13" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="13" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="13" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="13" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="5" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="16" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="16" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="16" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="6" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="6" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="6" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="7" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="14" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="14" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="14" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="14" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="17" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="14" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="17" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="14" fillId="7" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="13" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="13" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="13" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="13" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="13" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="13" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="15" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="15" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="15" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="14" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -4006,34 +4013,34 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A1" s="15" t="s">
+      <c r="A1" s="55" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="15" t="s">
+      <c r="B1" s="55" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="15" t="s">
+      <c r="C1" s="55" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="15" t="s">
+      <c r="D1" s="55" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="17"/>
-      <c r="F1" s="17"/>
-      <c r="G1" s="16" t="s">
+      <c r="E1" s="56"/>
+      <c r="F1" s="56"/>
+      <c r="G1" s="60" t="s">
         <v>4</v>
       </c>
-      <c r="H1" s="15" t="s">
+      <c r="H1" s="55" t="s">
         <v>5</v>
       </c>
-      <c r="I1" s="15" t="s">
+      <c r="I1" s="55" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A2" s="17"/>
-      <c r="B2" s="17"/>
-      <c r="C2" s="17"/>
+      <c r="A2" s="56"/>
+      <c r="B2" s="56"/>
+      <c r="C2" s="56"/>
       <c r="D2" s="4" t="s">
         <v>7</v>
       </c>
@@ -4043,1899 +4050,1899 @@
       <c r="F2" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="G2" s="16"/>
-      <c r="H2" s="17"/>
-      <c r="I2" s="17"/>
+      <c r="G2" s="60"/>
+      <c r="H2" s="56"/>
+      <c r="I2" s="56"/>
     </row>
     <row r="3" spans="1:9" s="5" customFormat="1" ht="156" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="18">
+      <c r="A3" s="61">
         <v>1</v>
       </c>
-      <c r="B3" s="18" t="s">
+      <c r="B3" s="61" t="s">
         <v>10</v>
       </c>
-      <c r="C3" s="19">
+      <c r="C3" s="16">
         <v>1.1000000000000001</v>
       </c>
-      <c r="D3" s="19" t="s">
+      <c r="D3" s="16" t="s">
         <v>166</v>
       </c>
-      <c r="E3" s="19" t="s">
+      <c r="E3" s="16" t="s">
         <v>165</v>
       </c>
-      <c r="F3" s="19" t="s">
+      <c r="F3" s="16" t="s">
         <v>174</v>
       </c>
-      <c r="G3" s="20" t="s">
+      <c r="G3" s="17" t="s">
         <v>177</v>
       </c>
-      <c r="H3" s="19" t="s">
+      <c r="H3" s="16" t="s">
         <v>11</v>
       </c>
-      <c r="I3" s="19" t="s">
+      <c r="I3" s="16" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="4" spans="1:9" s="6" customFormat="1" ht="130.05000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="18"/>
-      <c r="B4" s="18"/>
-      <c r="C4" s="19">
+    <row r="4" spans="1:9" s="6" customFormat="1" ht="144" x14ac:dyDescent="0.3">
+      <c r="A4" s="61"/>
+      <c r="B4" s="61"/>
+      <c r="C4" s="16">
         <v>1.2</v>
       </c>
-      <c r="D4" s="19" t="s">
+      <c r="D4" s="16" t="s">
         <v>176</v>
       </c>
-      <c r="E4" s="19" t="s">
+      <c r="E4" s="16" t="s">
         <v>170</v>
       </c>
-      <c r="F4" s="19" t="s">
+      <c r="F4" s="16" t="s">
         <v>159</v>
       </c>
-      <c r="G4" s="20" t="s">
+      <c r="G4" s="17" t="s">
         <v>168</v>
       </c>
-      <c r="H4" s="19"/>
-      <c r="I4" s="19"/>
+      <c r="H4" s="16"/>
+      <c r="I4" s="16"/>
     </row>
     <row r="5" spans="1:9" s="6" customFormat="1" ht="144" x14ac:dyDescent="0.3">
-      <c r="A5" s="18"/>
-      <c r="B5" s="18"/>
-      <c r="C5" s="19">
+      <c r="A5" s="61"/>
+      <c r="B5" s="61"/>
+      <c r="C5" s="16">
         <v>1.3</v>
       </c>
-      <c r="D5" s="19" t="s">
+      <c r="D5" s="16" t="s">
         <v>176</v>
       </c>
-      <c r="E5" s="19" t="s">
+      <c r="E5" s="16" t="s">
         <v>171</v>
       </c>
-      <c r="F5" s="19" t="s">
+      <c r="F5" s="16" t="s">
         <v>160</v>
       </c>
-      <c r="G5" s="20" t="s">
+      <c r="G5" s="17" t="s">
         <v>169</v>
       </c>
-      <c r="H5" s="19"/>
-      <c r="I5" s="19"/>
+      <c r="H5" s="16"/>
+      <c r="I5" s="16"/>
     </row>
     <row r="6" spans="1:9" s="6" customFormat="1" ht="144" x14ac:dyDescent="0.3">
-      <c r="A6" s="18"/>
-      <c r="B6" s="18"/>
-      <c r="C6" s="19">
+      <c r="A6" s="61"/>
+      <c r="B6" s="61"/>
+      <c r="C6" s="16">
         <v>1.4</v>
       </c>
-      <c r="D6" s="19" t="s">
+      <c r="D6" s="16" t="s">
         <v>176</v>
       </c>
-      <c r="E6" s="19" t="s">
+      <c r="E6" s="16" t="s">
         <v>172</v>
       </c>
-      <c r="F6" s="19" t="s">
+      <c r="F6" s="16" t="s">
         <v>161</v>
       </c>
-      <c r="G6" s="20" t="s">
+      <c r="G6" s="17" t="s">
         <v>167</v>
       </c>
-      <c r="H6" s="19"/>
-      <c r="I6" s="19"/>
+      <c r="H6" s="16"/>
+      <c r="I6" s="16"/>
     </row>
     <row r="7" spans="1:9" s="6" customFormat="1" ht="172.8" x14ac:dyDescent="0.3">
-      <c r="A7" s="18"/>
-      <c r="B7" s="18"/>
-      <c r="C7" s="19">
+      <c r="A7" s="61"/>
+      <c r="B7" s="61"/>
+      <c r="C7" s="16">
         <v>1.5</v>
       </c>
-      <c r="D7" s="19" t="s">
+      <c r="D7" s="16" t="s">
         <v>176</v>
       </c>
-      <c r="E7" s="19" t="s">
+      <c r="E7" s="16" t="s">
         <v>173</v>
       </c>
-      <c r="F7" s="19" t="s">
+      <c r="F7" s="16" t="s">
         <v>162</v>
       </c>
-      <c r="G7" s="20" t="s">
+      <c r="G7" s="17" t="s">
         <v>175</v>
       </c>
-      <c r="H7" s="19"/>
-      <c r="I7" s="19"/>
+      <c r="H7" s="16"/>
+      <c r="I7" s="16"/>
     </row>
     <row r="8" spans="1:9" s="6" customFormat="1" ht="129.6" x14ac:dyDescent="0.3">
-      <c r="A8" s="21">
+      <c r="A8" s="57">
         <v>5</v>
       </c>
-      <c r="B8" s="21" t="s">
+      <c r="B8" s="57" t="s">
         <v>13</v>
       </c>
-      <c r="C8" s="22">
+      <c r="C8" s="18">
         <v>5.0999999999999996</v>
       </c>
-      <c r="D8" s="22" t="s">
+      <c r="D8" s="18" t="s">
         <v>14</v>
       </c>
-      <c r="E8" s="22" t="s">
+      <c r="E8" s="18" t="s">
         <v>15</v>
       </c>
-      <c r="F8" s="22" t="s">
+      <c r="F8" s="18" t="s">
         <v>16</v>
       </c>
-      <c r="G8" s="23" t="s">
+      <c r="G8" s="19" t="s">
         <v>17</v>
       </c>
-      <c r="H8" s="24" t="s">
+      <c r="H8" s="20" t="s">
         <v>18</v>
       </c>
-      <c r="I8" s="22" t="s">
+      <c r="I8" s="18" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="9" spans="1:9" s="6" customFormat="1" ht="129.6" x14ac:dyDescent="0.3">
-      <c r="A9" s="25"/>
-      <c r="B9" s="25"/>
-      <c r="C9" s="22">
+      <c r="A9" s="58"/>
+      <c r="B9" s="58"/>
+      <c r="C9" s="18">
         <v>5.2</v>
       </c>
-      <c r="D9" s="22" t="s">
+      <c r="D9" s="18" t="s">
         <v>20</v>
       </c>
-      <c r="E9" s="22" t="s">
+      <c r="E9" s="18" t="s">
         <v>15</v>
       </c>
-      <c r="F9" s="22" t="s">
+      <c r="F9" s="18" t="s">
         <v>16</v>
       </c>
-      <c r="G9" s="23" t="s">
+      <c r="G9" s="19" t="s">
         <v>17</v>
       </c>
-      <c r="H9" s="24"/>
-      <c r="I9" s="22"/>
+      <c r="H9" s="20"/>
+      <c r="I9" s="18"/>
     </row>
     <row r="10" spans="1:9" s="6" customFormat="1" ht="172.8" x14ac:dyDescent="0.3">
-      <c r="A10" s="25"/>
-      <c r="B10" s="25"/>
-      <c r="C10" s="22">
+      <c r="A10" s="58"/>
+      <c r="B10" s="58"/>
+      <c r="C10" s="18">
         <v>5.3</v>
       </c>
-      <c r="D10" s="22" t="s">
+      <c r="D10" s="18" t="s">
         <v>21</v>
       </c>
-      <c r="E10" s="22" t="s">
+      <c r="E10" s="18" t="s">
         <v>22</v>
       </c>
-      <c r="F10" s="22" t="s">
+      <c r="F10" s="18" t="s">
         <v>23</v>
       </c>
-      <c r="G10" s="23" t="s">
+      <c r="G10" s="19" t="s">
         <v>24</v>
       </c>
-      <c r="H10" s="24"/>
-      <c r="I10" s="22"/>
+      <c r="H10" s="20"/>
+      <c r="I10" s="18"/>
     </row>
     <row r="11" spans="1:9" s="14" customFormat="1" ht="230.4" x14ac:dyDescent="0.3">
-      <c r="A11" s="25"/>
-      <c r="B11" s="25"/>
-      <c r="C11" s="26">
+      <c r="A11" s="58"/>
+      <c r="B11" s="58"/>
+      <c r="C11" s="21">
         <v>5.4</v>
       </c>
-      <c r="D11" s="26" t="s">
+      <c r="D11" s="21" t="s">
         <v>181</v>
       </c>
-      <c r="E11" s="26" t="s">
+      <c r="E11" s="21" t="s">
         <v>184</v>
       </c>
-      <c r="F11" s="26" t="s">
+      <c r="F11" s="21" t="s">
         <v>183</v>
       </c>
-      <c r="G11" s="27" t="s">
+      <c r="G11" s="22" t="s">
         <v>185</v>
       </c>
-      <c r="H11" s="28"/>
-      <c r="I11" s="26"/>
+      <c r="H11" s="23"/>
+      <c r="I11" s="21"/>
     </row>
     <row r="12" spans="1:9" s="14" customFormat="1" ht="158.4" x14ac:dyDescent="0.3">
-      <c r="A12" s="29"/>
-      <c r="B12" s="29"/>
-      <c r="C12" s="26">
+      <c r="A12" s="59"/>
+      <c r="B12" s="59"/>
+      <c r="C12" s="21">
         <v>5.5</v>
       </c>
-      <c r="D12" s="26" t="s">
+      <c r="D12" s="21" t="s">
         <v>178</v>
       </c>
-      <c r="E12" s="26" t="s">
+      <c r="E12" s="21" t="s">
         <v>182</v>
       </c>
-      <c r="F12" s="26" t="s">
+      <c r="F12" s="21" t="s">
         <v>180</v>
       </c>
-      <c r="G12" s="27" t="s">
+      <c r="G12" s="22" t="s">
         <v>179</v>
       </c>
-      <c r="H12" s="28"/>
-      <c r="I12" s="26"/>
+      <c r="H12" s="23"/>
+      <c r="I12" s="21"/>
     </row>
     <row r="13" spans="1:9" s="14" customFormat="1" ht="172.8" x14ac:dyDescent="0.3">
-      <c r="A13" s="30">
+      <c r="A13" s="49">
         <v>6</v>
       </c>
-      <c r="B13" s="30" t="s">
+      <c r="B13" s="49" t="s">
         <v>25</v>
       </c>
-      <c r="C13" s="26">
+      <c r="C13" s="21">
         <v>6.1</v>
       </c>
-      <c r="D13" s="26" t="s">
+      <c r="D13" s="21" t="s">
         <v>26</v>
       </c>
-      <c r="E13" s="26" t="s">
+      <c r="E13" s="21" t="s">
         <v>27</v>
       </c>
-      <c r="F13" s="26" t="s">
+      <c r="F13" s="21" t="s">
         <v>28</v>
       </c>
-      <c r="G13" s="27" t="s">
+      <c r="G13" s="22" t="s">
         <v>29</v>
       </c>
-      <c r="H13" s="28" t="s">
+      <c r="H13" s="23" t="s">
         <v>30</v>
       </c>
-      <c r="I13" s="26" t="s">
+      <c r="I13" s="21" t="s">
         <v>31</v>
       </c>
     </row>
     <row r="14" spans="1:9" s="6" customFormat="1" ht="144" x14ac:dyDescent="0.3">
-      <c r="A14" s="31"/>
-      <c r="B14" s="31"/>
-      <c r="C14" s="32">
+      <c r="A14" s="50"/>
+      <c r="B14" s="50"/>
+      <c r="C14" s="24">
         <v>6.2</v>
       </c>
-      <c r="D14" s="32" t="s">
+      <c r="D14" s="24" t="s">
         <v>26</v>
       </c>
-      <c r="E14" s="32" t="s">
+      <c r="E14" s="24" t="s">
         <v>187</v>
       </c>
-      <c r="F14" s="32" t="s">
+      <c r="F14" s="24" t="s">
         <v>186</v>
       </c>
-      <c r="G14" s="33" t="s">
+      <c r="G14" s="25" t="s">
         <v>188</v>
       </c>
-      <c r="H14" s="34"/>
-      <c r="I14" s="32"/>
-    </row>
-    <row r="15" spans="1:9" s="6" customFormat="1" ht="158.4" x14ac:dyDescent="0.3">
-      <c r="A15" s="31"/>
-      <c r="B15" s="31"/>
-      <c r="C15" s="32">
+      <c r="H14" s="26"/>
+      <c r="I14" s="24"/>
+    </row>
+    <row r="15" spans="1:9" s="6" customFormat="1" ht="172.8" x14ac:dyDescent="0.3">
+      <c r="A15" s="50"/>
+      <c r="B15" s="50"/>
+      <c r="C15" s="24">
         <v>6.3</v>
       </c>
-      <c r="D15" s="32" t="s">
+      <c r="D15" s="24" t="s">
         <v>26</v>
       </c>
-      <c r="E15" s="32" t="s">
+      <c r="E15" s="24" t="s">
         <v>32</v>
       </c>
-      <c r="F15" s="32" t="s">
+      <c r="F15" s="24" t="s">
         <v>33</v>
       </c>
-      <c r="G15" s="33" t="s">
+      <c r="G15" s="25" t="s">
         <v>34</v>
       </c>
-      <c r="H15" s="34"/>
-      <c r="I15" s="32"/>
+      <c r="H15" s="26"/>
+      <c r="I15" s="24"/>
     </row>
     <row r="16" spans="1:9" s="6" customFormat="1" ht="72" x14ac:dyDescent="0.3">
-      <c r="A16" s="31"/>
-      <c r="B16" s="35"/>
-      <c r="C16" s="36">
+      <c r="A16" s="50"/>
+      <c r="B16" s="51"/>
+      <c r="C16" s="27">
         <v>6.4</v>
       </c>
-      <c r="D16" s="32" t="s">
+      <c r="D16" s="24" t="s">
         <v>26</v>
       </c>
-      <c r="E16" s="32" t="s">
+      <c r="E16" s="24" t="s">
         <v>35</v>
       </c>
-      <c r="F16" s="32" t="s">
+      <c r="F16" s="24" t="s">
         <v>36</v>
       </c>
-      <c r="G16" s="33" t="s">
+      <c r="G16" s="25" t="s">
         <v>37</v>
       </c>
-      <c r="H16" s="34" t="s">
+      <c r="H16" s="26" t="s">
         <v>30</v>
       </c>
-      <c r="I16" s="32" t="s">
+      <c r="I16" s="24" t="s">
         <v>31</v>
       </c>
     </row>
     <row r="17" spans="1:9" s="6" customFormat="1" ht="144" x14ac:dyDescent="0.3">
-      <c r="A17" s="37">
+      <c r="A17" s="52">
         <v>7</v>
       </c>
-      <c r="B17" s="30" t="s">
+      <c r="B17" s="49" t="s">
         <v>38</v>
       </c>
-      <c r="C17" s="32">
+      <c r="C17" s="24">
         <v>7.1</v>
       </c>
-      <c r="D17" s="32" t="s">
+      <c r="D17" s="24" t="s">
         <v>39</v>
       </c>
-      <c r="E17" s="32" t="s">
+      <c r="E17" s="24" t="s">
         <v>40</v>
       </c>
-      <c r="F17" s="32" t="s">
+      <c r="F17" s="24" t="s">
         <v>41</v>
       </c>
-      <c r="G17" s="33" t="s">
+      <c r="G17" s="25" t="s">
         <v>42</v>
       </c>
-      <c r="H17" s="34" t="s">
+      <c r="H17" s="26" t="s">
         <v>30</v>
       </c>
-      <c r="I17" s="32" t="s">
+      <c r="I17" s="24" t="s">
         <v>31</v>
       </c>
     </row>
     <row r="18" spans="1:9" s="6" customFormat="1" ht="72" x14ac:dyDescent="0.3">
-      <c r="A18" s="38"/>
-      <c r="B18" s="31"/>
-      <c r="C18" s="32">
+      <c r="A18" s="53"/>
+      <c r="B18" s="50"/>
+      <c r="C18" s="24">
         <v>7.2</v>
       </c>
-      <c r="D18" s="32" t="s">
+      <c r="D18" s="24" t="s">
         <v>39</v>
       </c>
-      <c r="E18" s="32" t="s">
+      <c r="E18" s="24" t="s">
         <v>43</v>
       </c>
-      <c r="F18" s="32" t="s">
+      <c r="F18" s="24" t="s">
         <v>44</v>
       </c>
-      <c r="G18" s="33" t="s">
+      <c r="G18" s="25" t="s">
         <v>45</v>
       </c>
-      <c r="H18" s="34"/>
-      <c r="I18" s="32" t="s">
+      <c r="H18" s="26"/>
+      <c r="I18" s="24" t="s">
         <v>31</v>
       </c>
     </row>
     <row r="19" spans="1:9" s="6" customFormat="1" ht="187.2" x14ac:dyDescent="0.3">
-      <c r="A19" s="38"/>
-      <c r="B19" s="31"/>
-      <c r="C19" s="32">
+      <c r="A19" s="53"/>
+      <c r="B19" s="50"/>
+      <c r="C19" s="24">
         <v>7.3</v>
       </c>
-      <c r="D19" s="32" t="s">
+      <c r="D19" s="24" t="s">
         <v>39</v>
       </c>
-      <c r="E19" s="32" t="s">
+      <c r="E19" s="24" t="s">
         <v>163</v>
       </c>
-      <c r="F19" s="32" t="s">
+      <c r="F19" s="24" t="s">
         <v>46</v>
       </c>
-      <c r="G19" s="33" t="s">
+      <c r="G19" s="25" t="s">
         <v>47</v>
       </c>
-      <c r="H19" s="34"/>
-      <c r="I19" s="32"/>
+      <c r="H19" s="26"/>
+      <c r="I19" s="24"/>
     </row>
     <row r="20" spans="1:9" s="6" customFormat="1" ht="172.8" x14ac:dyDescent="0.3">
-      <c r="A20" s="39"/>
-      <c r="B20" s="35"/>
-      <c r="C20" s="32">
+      <c r="A20" s="54"/>
+      <c r="B20" s="51"/>
+      <c r="C20" s="24">
         <v>7.4</v>
       </c>
-      <c r="D20" s="32" t="s">
+      <c r="D20" s="24" t="s">
         <v>39</v>
       </c>
-      <c r="E20" s="32" t="s">
+      <c r="E20" s="24" t="s">
         <v>164</v>
       </c>
-      <c r="F20" s="32" t="s">
+      <c r="F20" s="24" t="s">
         <v>48</v>
       </c>
-      <c r="G20" s="33" t="s">
+      <c r="G20" s="25" t="s">
         <v>49</v>
       </c>
-      <c r="H20" s="34"/>
-      <c r="I20" s="32"/>
+      <c r="H20" s="26"/>
+      <c r="I20" s="24"/>
     </row>
     <row r="21" spans="1:9" s="6" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A21" s="40">
+      <c r="A21" s="77">
         <v>8</v>
       </c>
-      <c r="B21" s="40" t="s">
+      <c r="B21" s="77" t="s">
         <v>50</v>
       </c>
-      <c r="C21" s="41">
+      <c r="C21" s="28">
         <v>9.1999999999999993</v>
       </c>
-      <c r="D21" s="41" t="s">
+      <c r="D21" s="28" t="s">
         <v>51</v>
       </c>
-      <c r="E21" s="41" t="s">
+      <c r="E21" s="28" t="s">
         <v>52</v>
       </c>
-      <c r="F21" s="41" t="s">
+      <c r="F21" s="28" t="s">
         <v>53</v>
       </c>
-      <c r="G21" s="42" t="s">
+      <c r="G21" s="29" t="s">
         <v>54</v>
       </c>
-      <c r="H21" s="41"/>
-      <c r="I21" s="41" t="s">
+      <c r="H21" s="28"/>
+      <c r="I21" s="28" t="s">
         <v>55</v>
       </c>
     </row>
     <row r="22" spans="1:9" s="6" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A22" s="43"/>
-      <c r="B22" s="43"/>
-      <c r="C22" s="41">
+      <c r="A22" s="78"/>
+      <c r="B22" s="78"/>
+      <c r="C22" s="28">
         <v>9.3000000000000007</v>
       </c>
-      <c r="D22" s="41" t="s">
+      <c r="D22" s="28" t="s">
         <v>56</v>
       </c>
-      <c r="E22" s="41" t="s">
+      <c r="E22" s="28" t="s">
         <v>57</v>
       </c>
-      <c r="F22" s="41" t="s">
+      <c r="F22" s="28" t="s">
         <v>58</v>
       </c>
-      <c r="G22" s="42" t="s">
+      <c r="G22" s="29" t="s">
         <v>59</v>
       </c>
-      <c r="H22" s="41"/>
-      <c r="I22" s="41" t="s">
+      <c r="H22" s="28"/>
+      <c r="I22" s="28" t="s">
         <v>55</v>
       </c>
     </row>
     <row r="23" spans="1:9" s="6" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A23" s="44"/>
-      <c r="B23" s="44"/>
-      <c r="C23" s="41">
+      <c r="A23" s="79"/>
+      <c r="B23" s="79"/>
+      <c r="C23" s="28">
         <v>9.4</v>
       </c>
-      <c r="D23" s="41" t="s">
+      <c r="D23" s="28" t="s">
         <v>60</v>
       </c>
-      <c r="E23" s="41" t="s">
+      <c r="E23" s="28" t="s">
         <v>61</v>
       </c>
-      <c r="F23" s="41" t="s">
+      <c r="F23" s="28" t="s">
         <v>62</v>
       </c>
-      <c r="G23" s="42" t="s">
+      <c r="G23" s="29" t="s">
         <v>63</v>
       </c>
-      <c r="H23" s="41"/>
-      <c r="I23" s="41" t="s">
+      <c r="H23" s="28"/>
+      <c r="I23" s="28" t="s">
         <v>55</v>
       </c>
     </row>
     <row r="24" spans="1:9" s="6" customFormat="1" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A24" s="45">
+      <c r="A24" s="75">
         <v>12</v>
       </c>
-      <c r="B24" s="45" t="s">
+      <c r="B24" s="75" t="s">
         <v>64</v>
       </c>
-      <c r="C24" s="46">
+      <c r="C24" s="31">
         <v>12.1</v>
       </c>
-      <c r="D24" s="46" t="s">
+      <c r="D24" s="31" t="s">
         <v>65</v>
       </c>
-      <c r="E24" s="46" t="s">
+      <c r="E24" s="31" t="s">
         <v>66</v>
       </c>
-      <c r="F24" s="46" t="s">
+      <c r="F24" s="31" t="s">
         <v>67</v>
       </c>
-      <c r="G24" s="47" t="s">
+      <c r="G24" s="32" t="s">
         <v>68</v>
       </c>
-      <c r="H24" s="46" t="s">
+      <c r="H24" s="31" t="s">
         <v>69</v>
       </c>
-      <c r="I24" s="46" t="s">
+      <c r="I24" s="31" t="s">
         <v>70</v>
       </c>
     </row>
     <row r="25" spans="1:9" s="6" customFormat="1" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A25" s="45"/>
-      <c r="B25" s="45"/>
-      <c r="C25" s="46">
+      <c r="A25" s="75"/>
+      <c r="B25" s="75"/>
+      <c r="C25" s="31">
         <v>12.2</v>
       </c>
-      <c r="D25" s="46" t="s">
+      <c r="D25" s="31" t="s">
         <v>65</v>
       </c>
-      <c r="E25" s="46" t="s">
+      <c r="E25" s="31" t="s">
         <v>71</v>
       </c>
-      <c r="F25" s="46" t="s">
+      <c r="F25" s="31" t="s">
         <v>72</v>
       </c>
-      <c r="G25" s="47" t="s">
+      <c r="G25" s="32" t="s">
         <v>73</v>
       </c>
-      <c r="H25" s="46" t="s">
+      <c r="H25" s="31" t="s">
         <v>69</v>
       </c>
-      <c r="I25" s="46" t="s">
+      <c r="I25" s="31" t="s">
         <v>70</v>
       </c>
     </row>
     <row r="26" spans="1:9" s="6" customFormat="1" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A26" s="45"/>
-      <c r="B26" s="45"/>
-      <c r="C26" s="46">
+      <c r="A26" s="75"/>
+      <c r="B26" s="75"/>
+      <c r="C26" s="31">
         <v>12.3</v>
       </c>
-      <c r="D26" s="46" t="s">
+      <c r="D26" s="31" t="s">
         <v>65</v>
       </c>
-      <c r="E26" s="46" t="s">
+      <c r="E26" s="31" t="s">
         <v>74</v>
       </c>
-      <c r="F26" s="46" t="s">
+      <c r="F26" s="31" t="s">
         <v>75</v>
       </c>
-      <c r="G26" s="47" t="s">
+      <c r="G26" s="32" t="s">
         <v>76</v>
       </c>
-      <c r="H26" s="46" t="s">
+      <c r="H26" s="31" t="s">
         <v>69</v>
       </c>
-      <c r="I26" s="46" t="s">
+      <c r="I26" s="31" t="s">
         <v>70</v>
       </c>
     </row>
     <row r="27" spans="1:9" s="6" customFormat="1" ht="123.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A27" s="45"/>
-      <c r="B27" s="45"/>
-      <c r="C27" s="46">
+      <c r="A27" s="75"/>
+      <c r="B27" s="75"/>
+      <c r="C27" s="31">
         <v>12.4</v>
       </c>
-      <c r="D27" s="46" t="s">
+      <c r="D27" s="31" t="s">
         <v>65</v>
       </c>
-      <c r="E27" s="46" t="s">
+      <c r="E27" s="31" t="s">
         <v>283</v>
       </c>
-      <c r="F27" s="46" t="s">
+      <c r="F27" s="31" t="s">
         <v>284</v>
       </c>
-      <c r="G27" s="47" t="s">
+      <c r="G27" s="32" t="s">
         <v>285</v>
       </c>
-      <c r="H27" s="46" t="s">
+      <c r="H27" s="31" t="s">
         <v>69</v>
       </c>
-      <c r="I27" s="46" t="s">
+      <c r="I27" s="31" t="s">
         <v>70</v>
       </c>
     </row>
     <row r="28" spans="1:9" s="6" customFormat="1" ht="129.6" x14ac:dyDescent="0.3">
-      <c r="A28" s="45"/>
-      <c r="B28" s="45"/>
-      <c r="C28" s="46">
+      <c r="A28" s="75"/>
+      <c r="B28" s="75"/>
+      <c r="C28" s="31">
         <v>12.5</v>
       </c>
-      <c r="D28" s="46" t="s">
+      <c r="D28" s="31" t="s">
         <v>77</v>
       </c>
-      <c r="E28" s="46" t="s">
+      <c r="E28" s="31" t="s">
         <v>78</v>
       </c>
-      <c r="F28" s="46" t="s">
+      <c r="F28" s="31" t="s">
         <v>282</v>
       </c>
-      <c r="G28" s="47" t="s">
+      <c r="G28" s="32" t="s">
         <v>79</v>
       </c>
-      <c r="H28" s="46" t="s">
+      <c r="H28" s="31" t="s">
         <v>69</v>
       </c>
-      <c r="I28" s="46" t="s">
+      <c r="I28" s="31" t="s">
         <v>70</v>
       </c>
     </row>
     <row r="29" spans="1:9" s="6" customFormat="1" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A29" s="48"/>
-      <c r="B29" s="48"/>
-      <c r="C29" s="19">
+      <c r="A29" s="30"/>
+      <c r="B29" s="30"/>
+      <c r="C29" s="16">
         <v>12.6</v>
       </c>
-      <c r="D29" s="19" t="s">
+      <c r="D29" s="16" t="s">
         <v>144</v>
       </c>
-      <c r="E29" s="19" t="s">
+      <c r="E29" s="16" t="s">
         <v>148</v>
       </c>
-      <c r="F29" s="19"/>
-      <c r="G29" s="20"/>
-      <c r="H29" s="49"/>
-      <c r="I29" s="50"/>
+      <c r="F29" s="16"/>
+      <c r="G29" s="17"/>
+      <c r="H29" s="33"/>
+      <c r="I29" s="34"/>
     </row>
     <row r="30" spans="1:9" s="6" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A30" s="51">
+      <c r="A30" s="76">
         <v>14</v>
       </c>
-      <c r="B30" s="51" t="s">
+      <c r="B30" s="76" t="s">
         <v>80</v>
       </c>
-      <c r="C30" s="52">
+      <c r="C30" s="35">
         <v>14.1</v>
       </c>
-      <c r="D30" s="53" t="s">
+      <c r="D30" s="36" t="s">
         <v>133</v>
       </c>
-      <c r="E30" s="53" t="s">
+      <c r="E30" s="36" t="s">
         <v>253</v>
       </c>
-      <c r="F30" s="53" t="s">
+      <c r="F30" s="36" t="s">
         <v>219</v>
       </c>
-      <c r="G30" s="54" t="s">
+      <c r="G30" s="37" t="s">
         <v>269</v>
       </c>
-      <c r="H30" s="52" t="s">
+      <c r="H30" s="35" t="s">
         <v>82</v>
       </c>
-      <c r="I30" s="52" t="s">
+      <c r="I30" s="35" t="s">
         <v>83</v>
       </c>
     </row>
     <row r="31" spans="1:9" s="6" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A31" s="51"/>
-      <c r="B31" s="51"/>
-      <c r="C31" s="52">
+      <c r="A31" s="76"/>
+      <c r="B31" s="76"/>
+      <c r="C31" s="35">
         <v>14.2</v>
       </c>
-      <c r="D31" s="53" t="s">
+      <c r="D31" s="36" t="s">
         <v>133</v>
       </c>
-      <c r="E31" s="53" t="s">
+      <c r="E31" s="36" t="s">
         <v>254</v>
       </c>
-      <c r="F31" s="53" t="s">
+      <c r="F31" s="36" t="s">
         <v>255</v>
       </c>
-      <c r="G31" s="54" t="s">
+      <c r="G31" s="37" t="s">
         <v>270</v>
       </c>
-      <c r="H31" s="52" t="s">
+      <c r="H31" s="35" t="s">
         <v>82</v>
       </c>
-      <c r="I31" s="52" t="s">
+      <c r="I31" s="35" t="s">
         <v>83</v>
       </c>
     </row>
     <row r="32" spans="1:9" s="6" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A32" s="51"/>
-      <c r="B32" s="51"/>
-      <c r="C32" s="52">
+      <c r="A32" s="76"/>
+      <c r="B32" s="76"/>
+      <c r="C32" s="35">
         <v>14.3</v>
       </c>
-      <c r="D32" s="53" t="s">
+      <c r="D32" s="36" t="s">
         <v>224</v>
       </c>
-      <c r="E32" s="53" t="s">
+      <c r="E32" s="36" t="s">
         <v>256</v>
       </c>
-      <c r="F32" s="53" t="s">
+      <c r="F32" s="36" t="s">
         <v>257</v>
       </c>
-      <c r="G32" s="54" t="s">
+      <c r="G32" s="37" t="s">
         <v>271</v>
       </c>
-      <c r="H32" s="52" t="s">
+      <c r="H32" s="35" t="s">
         <v>82</v>
       </c>
-      <c r="I32" s="52" t="s">
+      <c r="I32" s="35" t="s">
         <v>83</v>
       </c>
     </row>
     <row r="33" spans="1:9" s="6" customFormat="1" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A33" s="51"/>
-      <c r="B33" s="51"/>
-      <c r="C33" s="52">
+      <c r="A33" s="76"/>
+      <c r="B33" s="76"/>
+      <c r="C33" s="35">
         <v>14.4</v>
       </c>
-      <c r="D33" s="53" t="s">
+      <c r="D33" s="36" t="s">
         <v>133</v>
       </c>
-      <c r="E33" s="53" t="s">
+      <c r="E33" s="36" t="s">
         <v>258</v>
       </c>
-      <c r="F33" s="53" t="s">
+      <c r="F33" s="36" t="s">
         <v>229</v>
       </c>
-      <c r="G33" s="54" t="s">
+      <c r="G33" s="37" t="s">
         <v>272</v>
       </c>
-      <c r="H33" s="52" t="s">
+      <c r="H33" s="35" t="s">
         <v>82</v>
       </c>
-      <c r="I33" s="52" t="s">
+      <c r="I33" s="35" t="s">
         <v>83</v>
       </c>
     </row>
     <row r="34" spans="1:9" s="6" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A34" s="51"/>
-      <c r="B34" s="51"/>
-      <c r="C34" s="52">
+      <c r="A34" s="76"/>
+      <c r="B34" s="76"/>
+      <c r="C34" s="35">
         <v>14.5</v>
       </c>
-      <c r="D34" s="53" t="s">
+      <c r="D34" s="36" t="s">
         <v>133</v>
       </c>
-      <c r="E34" s="53" t="s">
+      <c r="E34" s="36" t="s">
         <v>259</v>
       </c>
-      <c r="F34" s="53" t="s">
+      <c r="F34" s="36" t="s">
         <v>232</v>
       </c>
-      <c r="G34" s="54" t="s">
+      <c r="G34" s="37" t="s">
         <v>273</v>
       </c>
-      <c r="H34" s="52" t="s">
+      <c r="H34" s="35" t="s">
         <v>82</v>
       </c>
-      <c r="I34" s="52" t="s">
+      <c r="I34" s="35" t="s">
         <v>83</v>
       </c>
     </row>
     <row r="35" spans="1:9" s="6" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A35" s="51"/>
-      <c r="B35" s="51"/>
-      <c r="C35" s="52">
+      <c r="A35" s="76"/>
+      <c r="B35" s="76"/>
+      <c r="C35" s="35">
         <v>14.6</v>
       </c>
-      <c r="D35" s="53" t="s">
+      <c r="D35" s="36" t="s">
         <v>133</v>
       </c>
-      <c r="E35" s="53" t="s">
+      <c r="E35" s="36" t="s">
         <v>260</v>
       </c>
-      <c r="F35" s="53" t="s">
+      <c r="F35" s="36" t="s">
         <v>261</v>
       </c>
-      <c r="G35" s="54" t="s">
+      <c r="G35" s="37" t="s">
         <v>274</v>
       </c>
-      <c r="H35" s="52" t="s">
+      <c r="H35" s="35" t="s">
         <v>82</v>
       </c>
-      <c r="I35" s="52" t="s">
+      <c r="I35" s="35" t="s">
         <v>83</v>
       </c>
     </row>
     <row r="36" spans="1:9" s="6" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A36" s="51"/>
-      <c r="B36" s="51"/>
-      <c r="C36" s="52">
+      <c r="A36" s="76"/>
+      <c r="B36" s="76"/>
+      <c r="C36" s="35">
         <v>14.7</v>
       </c>
-      <c r="D36" s="53" t="s">
+      <c r="D36" s="36" t="s">
         <v>133</v>
       </c>
-      <c r="E36" s="53" t="s">
+      <c r="E36" s="36" t="s">
         <v>262</v>
       </c>
-      <c r="F36" s="53" t="s">
+      <c r="F36" s="36" t="s">
         <v>263</v>
       </c>
-      <c r="G36" s="54" t="s">
+      <c r="G36" s="37" t="s">
         <v>275</v>
       </c>
-      <c r="H36" s="52" t="s">
+      <c r="H36" s="35" t="s">
         <v>82</v>
       </c>
-      <c r="I36" s="52" t="s">
+      <c r="I36" s="35" t="s">
         <v>83</v>
       </c>
     </row>
     <row r="37" spans="1:9" s="6" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A37" s="51"/>
-      <c r="B37" s="51"/>
-      <c r="C37" s="52">
+      <c r="A37" s="76"/>
+      <c r="B37" s="76"/>
+      <c r="C37" s="35">
         <v>14.8</v>
       </c>
-      <c r="D37" s="53" t="s">
+      <c r="D37" s="36" t="s">
         <v>133</v>
       </c>
-      <c r="E37" s="53" t="s">
+      <c r="E37" s="36" t="s">
         <v>264</v>
       </c>
-      <c r="F37" s="53" t="s">
+      <c r="F37" s="36" t="s">
         <v>265</v>
       </c>
-      <c r="G37" s="54" t="s">
+      <c r="G37" s="37" t="s">
         <v>276</v>
       </c>
-      <c r="H37" s="52" t="s">
+      <c r="H37" s="35" t="s">
         <v>84</v>
       </c>
-      <c r="I37" s="52" t="s">
+      <c r="I37" s="35" t="s">
         <v>83</v>
       </c>
     </row>
     <row r="38" spans="1:9" s="6" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A38" s="51"/>
-      <c r="B38" s="51"/>
-      <c r="C38" s="52">
+      <c r="A38" s="76"/>
+      <c r="B38" s="76"/>
+      <c r="C38" s="35">
         <v>14.9</v>
       </c>
-      <c r="D38" s="53" t="s">
+      <c r="D38" s="36" t="s">
         <v>133</v>
       </c>
-      <c r="E38" s="53" t="s">
+      <c r="E38" s="36" t="s">
         <v>266</v>
       </c>
-      <c r="F38" s="53" t="s">
+      <c r="F38" s="36" t="s">
         <v>244</v>
       </c>
-      <c r="G38" s="54" t="s">
+      <c r="G38" s="37" t="s">
         <v>277</v>
       </c>
-      <c r="H38" s="52" t="s">
+      <c r="H38" s="35" t="s">
         <v>84</v>
       </c>
-      <c r="I38" s="52" t="s">
+      <c r="I38" s="35" t="s">
         <v>83</v>
       </c>
     </row>
     <row r="39" spans="1:9" s="6" customFormat="1" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A39" s="51"/>
-      <c r="B39" s="51"/>
-      <c r="C39" s="52">
+      <c r="A39" s="76"/>
+      <c r="B39" s="76"/>
+      <c r="C39" s="35">
         <v>14.1</v>
       </c>
-      <c r="D39" s="53" t="s">
+      <c r="D39" s="36" t="s">
         <v>133</v>
       </c>
-      <c r="E39" s="53" t="s">
+      <c r="E39" s="36" t="s">
         <v>267</v>
       </c>
-      <c r="F39" s="53" t="s">
+      <c r="F39" s="36" t="s">
         <v>248</v>
       </c>
-      <c r="G39" s="54" t="s">
+      <c r="G39" s="37" t="s">
         <v>278</v>
       </c>
-      <c r="H39" s="52" t="s">
+      <c r="H39" s="35" t="s">
         <v>84</v>
       </c>
-      <c r="I39" s="52" t="s">
+      <c r="I39" s="35" t="s">
         <v>83</v>
       </c>
     </row>
     <row r="40" spans="1:9" s="6" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A40" s="51"/>
-      <c r="B40" s="51"/>
-      <c r="C40" s="52">
+      <c r="A40" s="76"/>
+      <c r="B40" s="76"/>
+      <c r="C40" s="35">
         <v>14.11</v>
       </c>
-      <c r="D40" s="53" t="s">
+      <c r="D40" s="36" t="s">
         <v>133</v>
       </c>
-      <c r="E40" s="53" t="s">
+      <c r="E40" s="36" t="s">
         <v>268</v>
       </c>
-      <c r="F40" s="53" t="s">
+      <c r="F40" s="36" t="s">
         <v>251</v>
       </c>
-      <c r="G40" s="54" t="s">
+      <c r="G40" s="37" t="s">
         <v>279</v>
       </c>
-      <c r="H40" s="52" t="s">
+      <c r="H40" s="35" t="s">
         <v>84</v>
       </c>
-      <c r="I40" s="52" t="s">
+      <c r="I40" s="35" t="s">
         <v>83</v>
       </c>
     </row>
     <row r="41" spans="1:9" s="6" customFormat="1" ht="86.4" x14ac:dyDescent="0.3">
-      <c r="A41" s="55">
+      <c r="A41" s="62">
         <v>15</v>
       </c>
-      <c r="B41" s="55" t="s">
+      <c r="B41" s="62" t="s">
         <v>85</v>
       </c>
-      <c r="C41" s="56">
+      <c r="C41" s="38">
         <v>15.1</v>
       </c>
-      <c r="D41" s="56" t="s">
+      <c r="D41" s="38" t="s">
         <v>86</v>
       </c>
-      <c r="E41" s="56" t="s">
+      <c r="E41" s="38" t="s">
         <v>87</v>
       </c>
-      <c r="F41" s="56" t="s">
+      <c r="F41" s="38" t="s">
         <v>88</v>
       </c>
-      <c r="G41" s="57" t="s">
+      <c r="G41" s="39" t="s">
         <v>189</v>
       </c>
-      <c r="H41" s="56" t="s">
+      <c r="H41" s="38" t="s">
         <v>123</v>
       </c>
-      <c r="I41" s="56" t="s">
+      <c r="I41" s="38" t="s">
         <v>108</v>
       </c>
     </row>
     <row r="42" spans="1:9" s="6" customFormat="1" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A42" s="17"/>
-      <c r="B42" s="17"/>
-      <c r="C42" s="56">
+      <c r="A42" s="56"/>
+      <c r="B42" s="56"/>
+      <c r="C42" s="38">
         <v>15.2</v>
       </c>
-      <c r="D42" s="56" t="s">
+      <c r="D42" s="38" t="s">
         <v>86</v>
       </c>
-      <c r="E42" s="56" t="s">
+      <c r="E42" s="38" t="s">
         <v>89</v>
       </c>
-      <c r="F42" s="56" t="s">
+      <c r="F42" s="38" t="s">
         <v>90</v>
       </c>
-      <c r="G42" s="57" t="s">
+      <c r="G42" s="39" t="s">
         <v>190</v>
       </c>
-      <c r="H42" s="56" t="s">
+      <c r="H42" s="38" t="s">
         <v>107</v>
       </c>
-      <c r="I42" s="56" t="s">
+      <c r="I42" s="38" t="s">
         <v>108</v>
       </c>
     </row>
     <row r="43" spans="1:9" s="6" customFormat="1" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A43" s="17"/>
-      <c r="B43" s="17"/>
-      <c r="C43" s="56">
+      <c r="A43" s="56"/>
+      <c r="B43" s="56"/>
+      <c r="C43" s="38">
         <v>15.3</v>
       </c>
-      <c r="D43" s="56" t="s">
+      <c r="D43" s="38" t="s">
         <v>86</v>
       </c>
-      <c r="E43" s="56" t="s">
+      <c r="E43" s="38" t="s">
         <v>91</v>
       </c>
-      <c r="F43" s="56" t="s">
+      <c r="F43" s="38" t="s">
         <v>92</v>
       </c>
-      <c r="G43" s="57" t="s">
+      <c r="G43" s="39" t="s">
         <v>191</v>
       </c>
-      <c r="H43" s="56" t="s">
+      <c r="H43" s="38" t="s">
         <v>107</v>
       </c>
-      <c r="I43" s="56" t="s">
+      <c r="I43" s="38" t="s">
         <v>108</v>
       </c>
     </row>
     <row r="44" spans="1:9" s="6" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A44" s="17"/>
-      <c r="B44" s="17"/>
-      <c r="C44" s="56">
+      <c r="A44" s="56"/>
+      <c r="B44" s="56"/>
+      <c r="C44" s="38">
         <v>15.4</v>
       </c>
-      <c r="D44" s="56" t="s">
+      <c r="D44" s="38" t="s">
         <v>86</v>
       </c>
-      <c r="E44" s="56" t="s">
+      <c r="E44" s="38" t="s">
         <v>93</v>
       </c>
-      <c r="F44" s="56" t="s">
+      <c r="F44" s="38" t="s">
         <v>94</v>
       </c>
-      <c r="G44" s="57" t="s">
+      <c r="G44" s="39" t="s">
         <v>192</v>
       </c>
-      <c r="H44" s="56" t="s">
+      <c r="H44" s="38" t="s">
         <v>107</v>
       </c>
-      <c r="I44" s="56" t="s">
+      <c r="I44" s="38" t="s">
         <v>108</v>
       </c>
     </row>
     <row r="45" spans="1:9" s="6" customFormat="1" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A45" s="17"/>
-      <c r="B45" s="17"/>
-      <c r="C45" s="56">
+      <c r="A45" s="56"/>
+      <c r="B45" s="56"/>
+      <c r="C45" s="38">
         <v>15.5</v>
       </c>
-      <c r="D45" s="56" t="s">
+      <c r="D45" s="38" t="s">
         <v>86</v>
       </c>
-      <c r="E45" s="56" t="s">
+      <c r="E45" s="38" t="s">
         <v>95</v>
       </c>
-      <c r="F45" s="56" t="s">
+      <c r="F45" s="38" t="s">
         <v>96</v>
       </c>
-      <c r="G45" s="57" t="s">
+      <c r="G45" s="39" t="s">
         <v>193</v>
       </c>
-      <c r="H45" s="56" t="s">
+      <c r="H45" s="38" t="s">
         <v>107</v>
       </c>
-      <c r="I45" s="56" t="s">
+      <c r="I45" s="38" t="s">
         <v>108</v>
       </c>
     </row>
     <row r="46" spans="1:9" s="6" customFormat="1" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A46" s="17"/>
-      <c r="B46" s="17"/>
-      <c r="C46" s="56">
+      <c r="A46" s="56"/>
+      <c r="B46" s="56"/>
+      <c r="C46" s="38">
         <v>15.6</v>
       </c>
-      <c r="D46" s="56" t="s">
+      <c r="D46" s="38" t="s">
         <v>86</v>
       </c>
-      <c r="E46" s="56" t="s">
+      <c r="E46" s="38" t="s">
         <v>97</v>
       </c>
-      <c r="F46" s="56" t="s">
+      <c r="F46" s="38" t="s">
         <v>98</v>
       </c>
-      <c r="G46" s="57" t="s">
+      <c r="G46" s="39" t="s">
         <v>194</v>
       </c>
-      <c r="H46" s="56" t="s">
+      <c r="H46" s="38" t="s">
         <v>107</v>
       </c>
-      <c r="I46" s="56" t="s">
+      <c r="I46" s="38" t="s">
         <v>108</v>
       </c>
     </row>
     <row r="47" spans="1:9" s="6" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A47" s="17"/>
-      <c r="B47" s="17"/>
-      <c r="C47" s="56">
+      <c r="A47" s="56"/>
+      <c r="B47" s="56"/>
+      <c r="C47" s="38">
         <v>15.7</v>
       </c>
-      <c r="D47" s="56" t="s">
+      <c r="D47" s="38" t="s">
         <v>86</v>
       </c>
-      <c r="E47" s="56" t="s">
+      <c r="E47" s="38" t="s">
         <v>99</v>
       </c>
-      <c r="F47" s="56" t="s">
+      <c r="F47" s="38" t="s">
         <v>100</v>
       </c>
-      <c r="G47" s="57" t="s">
+      <c r="G47" s="39" t="s">
         <v>195</v>
       </c>
-      <c r="H47" s="56" t="s">
+      <c r="H47" s="38" t="s">
         <v>107</v>
       </c>
-      <c r="I47" s="56" t="s">
+      <c r="I47" s="38" t="s">
         <v>108</v>
       </c>
     </row>
     <row r="48" spans="1:9" s="6" customFormat="1" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A48" s="17"/>
-      <c r="B48" s="17"/>
-      <c r="C48" s="56">
+      <c r="A48" s="56"/>
+      <c r="B48" s="56"/>
+      <c r="C48" s="38">
         <v>15.8</v>
       </c>
-      <c r="D48" s="56" t="s">
+      <c r="D48" s="38" t="s">
         <v>86</v>
       </c>
-      <c r="E48" s="56" t="s">
+      <c r="E48" s="38" t="s">
         <v>101</v>
       </c>
-      <c r="F48" s="56" t="s">
+      <c r="F48" s="38" t="s">
         <v>102</v>
       </c>
-      <c r="G48" s="57" t="s">
+      <c r="G48" s="39" t="s">
         <v>196</v>
       </c>
-      <c r="H48" s="56" t="s">
+      <c r="H48" s="38" t="s">
         <v>107</v>
       </c>
-      <c r="I48" s="56" t="s">
+      <c r="I48" s="38" t="s">
         <v>108</v>
       </c>
     </row>
     <row r="49" spans="1:9" s="6" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A49" s="58">
+      <c r="A49" s="69">
         <v>16</v>
       </c>
-      <c r="B49" s="58" t="s">
+      <c r="B49" s="69" t="s">
         <v>103</v>
       </c>
-      <c r="C49" s="59">
+      <c r="C49" s="40">
         <v>16.100000000000001</v>
       </c>
-      <c r="D49" s="60" t="s">
+      <c r="D49" s="41" t="s">
         <v>104</v>
       </c>
-      <c r="E49" s="60" t="s">
+      <c r="E49" s="41" t="s">
         <v>105</v>
       </c>
-      <c r="F49" s="60" t="s">
+      <c r="F49" s="41" t="s">
         <v>106</v>
       </c>
-      <c r="G49" s="61" t="s">
+      <c r="G49" s="42" t="s">
         <v>197</v>
       </c>
-      <c r="H49" s="60" t="s">
+      <c r="H49" s="41" t="s">
         <v>107</v>
       </c>
-      <c r="I49" s="60" t="s">
+      <c r="I49" s="41" t="s">
         <v>108</v>
       </c>
     </row>
     <row r="50" spans="1:9" s="6" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A50" s="58"/>
-      <c r="B50" s="58"/>
-      <c r="C50" s="59">
+      <c r="A50" s="69"/>
+      <c r="B50" s="69"/>
+      <c r="C50" s="40">
         <v>16.2</v>
       </c>
-      <c r="D50" s="60" t="s">
+      <c r="D50" s="41" t="s">
         <v>104</v>
       </c>
-      <c r="E50" s="60" t="s">
+      <c r="E50" s="41" t="s">
         <v>109</v>
       </c>
-      <c r="F50" s="60" t="s">
+      <c r="F50" s="41" t="s">
         <v>110</v>
       </c>
-      <c r="G50" s="61" t="s">
+      <c r="G50" s="42" t="s">
         <v>198</v>
       </c>
-      <c r="H50" s="60" t="s">
+      <c r="H50" s="41" t="s">
         <v>107</v>
       </c>
-      <c r="I50" s="60" t="s">
+      <c r="I50" s="41" t="s">
         <v>108</v>
       </c>
     </row>
     <row r="51" spans="1:9" s="6" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A51" s="58"/>
-      <c r="B51" s="58"/>
-      <c r="C51" s="59">
+      <c r="A51" s="69"/>
+      <c r="B51" s="69"/>
+      <c r="C51" s="40">
         <v>16.3</v>
       </c>
-      <c r="D51" s="60" t="s">
+      <c r="D51" s="41" t="s">
         <v>104</v>
       </c>
-      <c r="E51" s="60" t="s">
+      <c r="E51" s="41" t="s">
         <v>111</v>
       </c>
-      <c r="F51" s="60" t="s">
+      <c r="F51" s="41" t="s">
         <v>112</v>
       </c>
-      <c r="G51" s="61" t="s">
+      <c r="G51" s="42" t="s">
         <v>199</v>
       </c>
-      <c r="H51" s="60" t="s">
+      <c r="H51" s="41" t="s">
         <v>107</v>
       </c>
-      <c r="I51" s="60" t="s">
+      <c r="I51" s="41" t="s">
         <v>108</v>
       </c>
     </row>
     <row r="52" spans="1:9" s="6" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A52" s="58"/>
-      <c r="B52" s="58"/>
-      <c r="C52" s="59">
+      <c r="A52" s="69"/>
+      <c r="B52" s="69"/>
+      <c r="C52" s="40">
         <v>16.399999999999999</v>
       </c>
-      <c r="D52" s="60" t="s">
+      <c r="D52" s="41" t="s">
         <v>104</v>
       </c>
-      <c r="E52" s="60" t="s">
+      <c r="E52" s="41" t="s">
         <v>113</v>
       </c>
-      <c r="F52" s="60" t="s">
+      <c r="F52" s="41" t="s">
         <v>114</v>
       </c>
-      <c r="G52" s="61" t="s">
+      <c r="G52" s="42" t="s">
         <v>200</v>
       </c>
-      <c r="H52" s="60" t="s">
+      <c r="H52" s="41" t="s">
         <v>107</v>
       </c>
-      <c r="I52" s="60" t="s">
+      <c r="I52" s="41" t="s">
         <v>108</v>
       </c>
     </row>
     <row r="53" spans="1:9" s="6" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A53" s="58"/>
-      <c r="B53" s="58"/>
-      <c r="C53" s="59">
+      <c r="A53" s="69"/>
+      <c r="B53" s="69"/>
+      <c r="C53" s="40">
         <v>16.5</v>
       </c>
-      <c r="D53" s="60" t="s">
+      <c r="D53" s="41" t="s">
         <v>104</v>
       </c>
-      <c r="E53" s="60" t="s">
+      <c r="E53" s="41" t="s">
         <v>115</v>
       </c>
-      <c r="F53" s="60" t="s">
+      <c r="F53" s="41" t="s">
         <v>116</v>
       </c>
-      <c r="G53" s="61" t="s">
+      <c r="G53" s="42" t="s">
         <v>201</v>
       </c>
-      <c r="H53" s="60" t="s">
+      <c r="H53" s="41" t="s">
         <v>107</v>
       </c>
-      <c r="I53" s="60" t="s">
+      <c r="I53" s="41" t="s">
         <v>108</v>
       </c>
     </row>
     <row r="54" spans="1:9" s="6" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A54" s="17"/>
-      <c r="B54" s="17"/>
-      <c r="C54" s="59">
+      <c r="A54" s="56"/>
+      <c r="B54" s="56"/>
+      <c r="C54" s="40">
         <v>16.600000000000001</v>
       </c>
-      <c r="D54" s="60" t="s">
+      <c r="D54" s="41" t="s">
         <v>104</v>
       </c>
-      <c r="E54" s="60" t="s">
+      <c r="E54" s="41" t="s">
         <v>117</v>
       </c>
-      <c r="F54" s="60" t="s">
+      <c r="F54" s="41" t="s">
         <v>118</v>
       </c>
-      <c r="G54" s="61" t="s">
+      <c r="G54" s="42" t="s">
         <v>202</v>
       </c>
-      <c r="H54" s="60" t="s">
+      <c r="H54" s="41" t="s">
         <v>107</v>
       </c>
-      <c r="I54" s="60" t="s">
+      <c r="I54" s="41" t="s">
         <v>108</v>
       </c>
     </row>
     <row r="55" spans="1:9" s="6" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A55" s="62">
+      <c r="A55" s="70">
         <v>17</v>
       </c>
-      <c r="B55" s="63" t="s">
+      <c r="B55" s="73" t="s">
         <v>119</v>
       </c>
-      <c r="C55" s="64">
+      <c r="C55" s="43">
         <v>17.100000000000001</v>
       </c>
-      <c r="D55" s="64" t="s">
+      <c r="D55" s="43" t="s">
         <v>120</v>
       </c>
-      <c r="E55" s="64" t="s">
+      <c r="E55" s="43" t="s">
         <v>121</v>
       </c>
-      <c r="F55" s="64" t="s">
+      <c r="F55" s="43" t="s">
         <v>122</v>
       </c>
-      <c r="G55" s="65" t="s">
+      <c r="G55" s="44" t="s">
         <v>203</v>
       </c>
-      <c r="H55" s="64" t="s">
+      <c r="H55" s="43" t="s">
         <v>123</v>
       </c>
-      <c r="I55" s="64" t="s">
+      <c r="I55" s="43" t="s">
         <v>108</v>
       </c>
     </row>
     <row r="56" spans="1:9" s="6" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A56" s="66"/>
-      <c r="B56" s="63"/>
-      <c r="C56" s="64">
+      <c r="A56" s="71"/>
+      <c r="B56" s="73"/>
+      <c r="C56" s="43">
         <v>17.2</v>
       </c>
-      <c r="D56" s="64" t="s">
+      <c r="D56" s="43" t="s">
         <v>120</v>
       </c>
-      <c r="E56" s="64" t="s">
+      <c r="E56" s="43" t="s">
         <v>124</v>
       </c>
-      <c r="F56" s="64" t="s">
+      <c r="F56" s="43" t="s">
         <v>125</v>
       </c>
-      <c r="G56" s="65" t="s">
+      <c r="G56" s="44" t="s">
         <v>204</v>
       </c>
-      <c r="H56" s="64" t="s">
+      <c r="H56" s="43" t="s">
         <v>123</v>
       </c>
-      <c r="I56" s="64" t="s">
+      <c r="I56" s="43" t="s">
         <v>108</v>
       </c>
     </row>
     <row r="57" spans="1:9" s="6" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A57" s="66"/>
-      <c r="B57" s="63"/>
-      <c r="C57" s="64">
+      <c r="A57" s="71"/>
+      <c r="B57" s="73"/>
+      <c r="C57" s="43">
         <v>17.3</v>
       </c>
-      <c r="D57" s="64" t="s">
+      <c r="D57" s="43" t="s">
         <v>120</v>
       </c>
-      <c r="E57" s="64" t="s">
+      <c r="E57" s="43" t="s">
         <v>126</v>
       </c>
-      <c r="F57" s="64" t="s">
+      <c r="F57" s="43" t="s">
         <v>127</v>
       </c>
-      <c r="G57" s="65" t="s">
+      <c r="G57" s="44" t="s">
         <v>205</v>
       </c>
-      <c r="H57" s="64" t="s">
+      <c r="H57" s="43" t="s">
         <v>107</v>
       </c>
-      <c r="I57" s="64" t="s">
+      <c r="I57" s="43" t="s">
         <v>108</v>
       </c>
     </row>
     <row r="58" spans="1:9" s="6" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A58" s="66"/>
-      <c r="B58" s="63"/>
-      <c r="C58" s="64">
+      <c r="A58" s="71"/>
+      <c r="B58" s="73"/>
+      <c r="C58" s="43">
         <v>17.399999999999999</v>
       </c>
-      <c r="D58" s="64" t="s">
+      <c r="D58" s="43" t="s">
         <v>120</v>
       </c>
-      <c r="E58" s="64" t="s">
+      <c r="E58" s="43" t="s">
         <v>128</v>
       </c>
-      <c r="F58" s="64" t="s">
+      <c r="F58" s="43" t="s">
         <v>129</v>
       </c>
-      <c r="G58" s="65" t="s">
+      <c r="G58" s="44" t="s">
         <v>206</v>
       </c>
-      <c r="H58" s="64" t="s">
+      <c r="H58" s="43" t="s">
         <v>123</v>
       </c>
-      <c r="I58" s="64" t="s">
+      <c r="I58" s="43" t="s">
         <v>108</v>
       </c>
     </row>
     <row r="59" spans="1:9" s="6" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A59" s="67"/>
-      <c r="B59" s="63"/>
-      <c r="C59" s="64">
+      <c r="A59" s="72"/>
+      <c r="B59" s="73"/>
+      <c r="C59" s="43">
         <v>17.5</v>
       </c>
-      <c r="D59" s="64" t="s">
+      <c r="D59" s="43" t="s">
         <v>120</v>
       </c>
-      <c r="E59" s="64" t="s">
+      <c r="E59" s="43" t="s">
         <v>130</v>
       </c>
-      <c r="F59" s="64" t="s">
+      <c r="F59" s="43" t="s">
         <v>131</v>
       </c>
-      <c r="G59" s="65" t="s">
+      <c r="G59" s="44" t="s">
         <v>207</v>
       </c>
-      <c r="H59" s="64" t="s">
+      <c r="H59" s="43" t="s">
         <v>123</v>
       </c>
-      <c r="I59" s="64" t="s">
+      <c r="I59" s="43" t="s">
         <v>108</v>
       </c>
     </row>
     <row r="60" spans="1:9" s="6" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A60" s="68">
+      <c r="A60" s="74">
         <v>18</v>
       </c>
-      <c r="B60" s="68" t="s">
+      <c r="B60" s="74" t="s">
         <v>132</v>
       </c>
-      <c r="C60" s="22">
+      <c r="C60" s="18">
         <v>17.100000000000001</v>
       </c>
-      <c r="D60" s="22" t="s">
+      <c r="D60" s="18" t="s">
         <v>133</v>
       </c>
-      <c r="E60" s="22" t="s">
+      <c r="E60" s="18" t="s">
         <v>291</v>
       </c>
-      <c r="F60" s="22" t="s">
+      <c r="F60" s="18" t="s">
         <v>134</v>
       </c>
-      <c r="G60" s="23" t="s">
+      <c r="G60" s="19" t="s">
         <v>208</v>
       </c>
-      <c r="H60" s="22" t="s">
+      <c r="H60" s="18" t="s">
         <v>82</v>
       </c>
-      <c r="I60" s="22" t="s">
+      <c r="I60" s="18" t="s">
         <v>135</v>
       </c>
     </row>
     <row r="61" spans="1:9" s="6" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A61" s="17"/>
-      <c r="B61" s="17"/>
-      <c r="C61" s="22">
+      <c r="A61" s="56"/>
+      <c r="B61" s="56"/>
+      <c r="C61" s="18">
         <v>17.2</v>
       </c>
-      <c r="D61" s="22" t="s">
+      <c r="D61" s="18" t="s">
         <v>133</v>
       </c>
-      <c r="E61" s="22" t="s">
+      <c r="E61" s="18" t="s">
         <v>292</v>
       </c>
-      <c r="F61" s="22" t="s">
+      <c r="F61" s="18" t="s">
         <v>136</v>
       </c>
-      <c r="G61" s="23" t="s">
+      <c r="G61" s="19" t="s">
         <v>209</v>
       </c>
-      <c r="H61" s="22" t="s">
+      <c r="H61" s="18" t="s">
         <v>82</v>
       </c>
-      <c r="I61" s="22" t="s">
+      <c r="I61" s="18" t="s">
         <v>135</v>
       </c>
     </row>
     <row r="62" spans="1:9" s="6" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A62" s="17"/>
-      <c r="B62" s="17"/>
-      <c r="C62" s="22">
+      <c r="A62" s="56"/>
+      <c r="B62" s="56"/>
+      <c r="C62" s="18">
         <v>17.3</v>
       </c>
-      <c r="D62" s="22" t="s">
+      <c r="D62" s="18" t="s">
         <v>133</v>
       </c>
-      <c r="E62" s="22" t="s">
+      <c r="E62" s="18" t="s">
         <v>293</v>
       </c>
-      <c r="F62" s="22" t="s">
+      <c r="F62" s="18" t="s">
         <v>137</v>
       </c>
-      <c r="G62" s="23" t="s">
+      <c r="G62" s="19" t="s">
         <v>210</v>
       </c>
-      <c r="H62" s="22" t="s">
+      <c r="H62" s="18" t="s">
         <v>82</v>
       </c>
-      <c r="I62" s="22" t="s">
+      <c r="I62" s="18" t="s">
         <v>135</v>
       </c>
     </row>
     <row r="63" spans="1:9" s="6" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A63" s="17"/>
-      <c r="B63" s="17"/>
-      <c r="C63" s="22">
+      <c r="A63" s="56"/>
+      <c r="B63" s="56"/>
+      <c r="C63" s="18">
         <v>17.399999999999999</v>
       </c>
-      <c r="D63" s="22" t="s">
+      <c r="D63" s="18" t="s">
         <v>133</v>
       </c>
-      <c r="E63" s="22" t="s">
+      <c r="E63" s="18" t="s">
         <v>294</v>
       </c>
-      <c r="F63" s="22" t="s">
+      <c r="F63" s="18" t="s">
         <v>81</v>
       </c>
-      <c r="G63" s="23" t="s">
+      <c r="G63" s="19" t="s">
         <v>211</v>
       </c>
-      <c r="H63" s="22" t="s">
+      <c r="H63" s="18" t="s">
         <v>82</v>
       </c>
-      <c r="I63" s="22" t="s">
+      <c r="I63" s="18" t="s">
         <v>135</v>
       </c>
     </row>
     <row r="64" spans="1:9" s="6" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A64" s="17"/>
-      <c r="B64" s="17"/>
-      <c r="C64" s="22">
+      <c r="A64" s="56"/>
+      <c r="B64" s="56"/>
+      <c r="C64" s="18">
         <v>17.5</v>
       </c>
-      <c r="D64" s="22" t="s">
+      <c r="D64" s="18" t="s">
         <v>133</v>
       </c>
-      <c r="E64" s="22" t="s">
+      <c r="E64" s="18" t="s">
         <v>295</v>
       </c>
-      <c r="F64" s="22" t="s">
+      <c r="F64" s="18" t="s">
         <v>138</v>
       </c>
-      <c r="G64" s="23" t="s">
+      <c r="G64" s="19" t="s">
         <v>212</v>
       </c>
-      <c r="H64" s="22" t="s">
+      <c r="H64" s="18" t="s">
         <v>82</v>
       </c>
-      <c r="I64" s="22" t="s">
+      <c r="I64" s="18" t="s">
         <v>135</v>
       </c>
     </row>
     <row r="65" spans="1:12" s="6" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A65" s="17"/>
-      <c r="B65" s="17"/>
-      <c r="C65" s="22">
+      <c r="A65" s="56"/>
+      <c r="B65" s="56"/>
+      <c r="C65" s="18">
         <v>17.600000000000001</v>
       </c>
-      <c r="D65" s="22" t="s">
+      <c r="D65" s="18" t="s">
         <v>133</v>
       </c>
-      <c r="E65" s="22" t="s">
+      <c r="E65" s="18" t="s">
         <v>296</v>
       </c>
-      <c r="F65" s="22" t="s">
+      <c r="F65" s="18" t="s">
         <v>139</v>
       </c>
-      <c r="G65" s="23" t="s">
+      <c r="G65" s="19" t="s">
         <v>213</v>
       </c>
-      <c r="H65" s="22" t="s">
+      <c r="H65" s="18" t="s">
         <v>82</v>
       </c>
-      <c r="I65" s="22" t="s">
+      <c r="I65" s="18" t="s">
         <v>135</v>
       </c>
     </row>
     <row r="66" spans="1:12" s="6" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A66" s="17"/>
-      <c r="B66" s="17"/>
-      <c r="C66" s="22">
+      <c r="A66" s="56"/>
+      <c r="B66" s="56"/>
+      <c r="C66" s="18">
         <v>17.7</v>
       </c>
-      <c r="D66" s="22" t="s">
+      <c r="D66" s="18" t="s">
         <v>133</v>
       </c>
-      <c r="E66" s="22" t="s">
+      <c r="E66" s="18" t="s">
         <v>297</v>
       </c>
-      <c r="F66" s="22" t="s">
+      <c r="F66" s="18" t="s">
         <v>140</v>
       </c>
-      <c r="G66" s="23" t="s">
+      <c r="G66" s="19" t="s">
         <v>214</v>
       </c>
-      <c r="H66" s="22" t="s">
+      <c r="H66" s="18" t="s">
         <v>82</v>
       </c>
-      <c r="I66" s="22" t="s">
+      <c r="I66" s="18" t="s">
         <v>135</v>
       </c>
     </row>
     <row r="67" spans="1:12" s="6" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A67" s="17"/>
-      <c r="B67" s="17"/>
-      <c r="C67" s="22">
+      <c r="A67" s="56"/>
+      <c r="B67" s="56"/>
+      <c r="C67" s="18">
         <v>17.8</v>
       </c>
-      <c r="D67" s="22" t="s">
+      <c r="D67" s="18" t="s">
         <v>133</v>
       </c>
-      <c r="E67" s="22" t="s">
+      <c r="E67" s="18" t="s">
         <v>298</v>
       </c>
-      <c r="F67" s="22" t="s">
+      <c r="F67" s="18" t="s">
         <v>141</v>
       </c>
-      <c r="G67" s="23" t="s">
+      <c r="G67" s="19" t="s">
         <v>215</v>
       </c>
-      <c r="H67" s="22" t="s">
+      <c r="H67" s="18" t="s">
         <v>82</v>
       </c>
-      <c r="I67" s="22" t="s">
+      <c r="I67" s="18" t="s">
         <v>135</v>
       </c>
     </row>
     <row r="68" spans="1:12" s="6" customFormat="1" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A68" s="17"/>
-      <c r="B68" s="17"/>
-      <c r="C68" s="22">
+      <c r="A68" s="56"/>
+      <c r="B68" s="56"/>
+      <c r="C68" s="18">
         <v>17.899999999999999</v>
       </c>
-      <c r="D68" s="22" t="s">
+      <c r="D68" s="18" t="s">
         <v>133</v>
       </c>
-      <c r="E68" s="22" t="s">
+      <c r="E68" s="18" t="s">
         <v>299</v>
       </c>
-      <c r="F68" s="22" t="s">
+      <c r="F68" s="18" t="s">
         <v>142</v>
       </c>
-      <c r="G68" s="23" t="s">
+      <c r="G68" s="19" t="s">
         <v>216</v>
       </c>
-      <c r="H68" s="22" t="s">
+      <c r="H68" s="18" t="s">
         <v>82</v>
       </c>
-      <c r="I68" s="22" t="s">
+      <c r="I68" s="18" t="s">
         <v>135</v>
       </c>
     </row>
     <row r="69" spans="1:12" s="6" customFormat="1" ht="86.4" x14ac:dyDescent="0.3">
-      <c r="A69" s="69">
+      <c r="A69" s="63">
         <v>19</v>
       </c>
-      <c r="B69" s="70" t="s">
+      <c r="B69" s="66" t="s">
         <v>143</v>
       </c>
-      <c r="C69" s="71">
+      <c r="C69" s="45">
         <v>19.100000000000001</v>
       </c>
-      <c r="D69" s="72" t="s">
+      <c r="D69" s="46" t="s">
         <v>144</v>
       </c>
-      <c r="E69" s="72" t="s">
+      <c r="E69" s="46" t="s">
         <v>287</v>
       </c>
-      <c r="F69" s="72" t="s">
+      <c r="F69" s="46" t="s">
         <v>286</v>
       </c>
-      <c r="G69" s="73" t="s">
+      <c r="G69" s="47" t="s">
         <v>288</v>
       </c>
-      <c r="H69" s="71"/>
-      <c r="I69" s="74"/>
+      <c r="H69" s="45"/>
+      <c r="I69" s="48"/>
     </row>
     <row r="70" spans="1:12" s="6" customFormat="1" ht="129.6" x14ac:dyDescent="0.3">
-      <c r="A70" s="75"/>
-      <c r="B70" s="76"/>
-      <c r="C70" s="77">
+      <c r="A70" s="64"/>
+      <c r="B70" s="67"/>
+      <c r="C70" s="15">
         <v>19.2</v>
       </c>
-      <c r="D70" s="72" t="s">
+      <c r="D70" s="46" t="s">
         <v>145</v>
       </c>
-      <c r="E70" s="72" t="s">
+      <c r="E70" s="46" t="s">
         <v>146</v>
       </c>
-      <c r="F70" s="72" t="s">
+      <c r="F70" s="46" t="s">
         <v>282</v>
       </c>
-      <c r="G70" s="73" t="s">
+      <c r="G70" s="47" t="s">
         <v>147</v>
       </c>
-      <c r="H70" s="71"/>
-      <c r="I70" s="74"/>
+      <c r="H70" s="45"/>
+      <c r="I70" s="48"/>
     </row>
     <row r="71" spans="1:12" s="6" customFormat="1" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A71" s="78"/>
-      <c r="B71" s="79"/>
-      <c r="C71" s="50">
+      <c r="A71" s="65"/>
+      <c r="B71" s="68"/>
+      <c r="C71" s="34">
         <v>19.3</v>
       </c>
-      <c r="D71" s="19" t="s">
+      <c r="D71" s="16" t="s">
         <v>144</v>
       </c>
-      <c r="E71" s="19" t="s">
+      <c r="E71" s="16" t="s">
         <v>148</v>
       </c>
-      <c r="F71" s="19" t="s">
+      <c r="F71" s="16" t="s">
         <v>149</v>
       </c>
-      <c r="G71" s="20"/>
-      <c r="H71" s="49"/>
-      <c r="I71" s="50"/>
+      <c r="G71" s="17"/>
+      <c r="H71" s="33"/>
+      <c r="I71" s="34"/>
     </row>
     <row r="72" spans="1:12" s="6" customFormat="1" ht="201.6" x14ac:dyDescent="0.3">
-      <c r="A72" s="69">
+      <c r="A72" s="63">
         <v>20</v>
       </c>
-      <c r="B72" s="70" t="s">
+      <c r="B72" s="66" t="s">
         <v>150</v>
       </c>
-      <c r="C72" s="71">
+      <c r="C72" s="45">
         <v>20.100000000000001</v>
       </c>
-      <c r="D72" s="72" t="s">
+      <c r="D72" s="46" t="s">
         <v>151</v>
       </c>
-      <c r="E72" s="72" t="s">
+      <c r="E72" s="46" t="s">
         <v>308</v>
       </c>
-      <c r="F72" s="72" t="s">
+      <c r="F72" s="46" t="s">
         <v>309</v>
       </c>
-      <c r="G72" s="73" t="s">
+      <c r="G72" s="47" t="s">
         <v>310</v>
       </c>
-      <c r="H72" s="71"/>
-      <c r="I72" s="74"/>
+      <c r="H72" s="45"/>
+      <c r="I72" s="48"/>
     </row>
     <row r="73" spans="1:12" s="6" customFormat="1" ht="158.4" x14ac:dyDescent="0.3">
-      <c r="A73" s="75"/>
-      <c r="B73" s="76"/>
-      <c r="C73" s="77">
+      <c r="A73" s="64"/>
+      <c r="B73" s="67"/>
+      <c r="C73" s="15">
         <v>20.2</v>
       </c>
-      <c r="D73" s="72" t="s">
+      <c r="D73" s="46" t="s">
         <v>152</v>
       </c>
-      <c r="E73" s="72" t="s">
+      <c r="E73" s="46" t="s">
         <v>289</v>
       </c>
-      <c r="F73" s="72" t="s">
+      <c r="F73" s="46" t="s">
         <v>282</v>
       </c>
-      <c r="G73" s="73" t="s">
+      <c r="G73" s="47" t="s">
         <v>290</v>
       </c>
-      <c r="H73" s="71"/>
-      <c r="I73" s="74"/>
+      <c r="H73" s="45"/>
+      <c r="I73" s="48"/>
       <c r="J73" s="1"/>
       <c r="K73" s="1"/>
       <c r="L73" s="1"/>
     </row>
     <row r="74" spans="1:12" s="6" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A74" s="78"/>
-      <c r="B74" s="79"/>
-      <c r="C74" s="49">
+      <c r="A74" s="65"/>
+      <c r="B74" s="68"/>
+      <c r="C74" s="33">
         <v>20.3</v>
       </c>
-      <c r="D74" s="19" t="s">
+      <c r="D74" s="16" t="s">
         <v>151</v>
       </c>
-      <c r="E74" s="19" t="s">
+      <c r="E74" s="16" t="s">
         <v>148</v>
       </c>
-      <c r="F74" s="19"/>
-      <c r="G74" s="20"/>
-      <c r="H74" s="49"/>
-      <c r="I74" s="50"/>
+      <c r="F74" s="16"/>
+      <c r="G74" s="17"/>
+      <c r="H74" s="33"/>
+      <c r="I74" s="34"/>
       <c r="J74" s="1"/>
       <c r="K74" s="1"/>
       <c r="L74" s="1"/>
     </row>
     <row r="75" spans="1:12" ht="187.2" x14ac:dyDescent="0.3">
-      <c r="A75" s="69">
+      <c r="A75" s="63">
         <v>21</v>
       </c>
-      <c r="B75" s="70" t="s">
+      <c r="B75" s="66" t="s">
         <v>153</v>
       </c>
-      <c r="C75" s="71">
+      <c r="C75" s="45">
         <v>21.1</v>
       </c>
-      <c r="D75" s="72" t="s">
+      <c r="D75" s="46" t="s">
         <v>154</v>
       </c>
-      <c r="E75" s="72" t="s">
+      <c r="E75" s="46" t="s">
         <v>300</v>
       </c>
-      <c r="F75" s="72" t="s">
+      <c r="F75" s="46" t="s">
         <v>301</v>
       </c>
-      <c r="G75" s="73" t="s">
+      <c r="G75" s="47" t="s">
         <v>302</v>
       </c>
-      <c r="H75" s="71"/>
-      <c r="I75" s="74"/>
+      <c r="H75" s="45"/>
+      <c r="I75" s="48"/>
     </row>
     <row r="76" spans="1:12" ht="129.6" x14ac:dyDescent="0.3">
-      <c r="A76" s="75"/>
-      <c r="B76" s="76"/>
-      <c r="C76" s="77">
+      <c r="A76" s="64"/>
+      <c r="B76" s="67"/>
+      <c r="C76" s="15">
         <v>21.2</v>
       </c>
-      <c r="D76" s="72" t="s">
+      <c r="D76" s="46" t="s">
         <v>155</v>
       </c>
-      <c r="E76" s="72" t="s">
+      <c r="E76" s="46" t="s">
         <v>281</v>
       </c>
-      <c r="F76" s="72" t="s">
+      <c r="F76" s="46" t="s">
         <v>282</v>
       </c>
-      <c r="G76" s="73" t="s">
+      <c r="G76" s="47" t="s">
         <v>156</v>
       </c>
-      <c r="H76" s="71"/>
-      <c r="I76" s="74"/>
+      <c r="H76" s="45"/>
+      <c r="I76" s="48"/>
     </row>
     <row r="77" spans="1:12" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A77" s="78"/>
-      <c r="B77" s="79"/>
-      <c r="C77" s="49">
+      <c r="A77" s="65"/>
+      <c r="B77" s="68"/>
+      <c r="C77" s="33">
         <v>21.3</v>
       </c>
-      <c r="D77" s="19" t="s">
+      <c r="D77" s="16" t="s">
         <v>154</v>
       </c>
-      <c r="E77" s="19" t="s">
+      <c r="E77" s="16" t="s">
         <v>148</v>
       </c>
-      <c r="F77" s="19"/>
-      <c r="G77" s="20"/>
-      <c r="H77" s="49"/>
-      <c r="I77" s="50"/>
+      <c r="F77" s="16"/>
+      <c r="G77" s="17"/>
+      <c r="H77" s="33"/>
+      <c r="I77" s="34"/>
     </row>
     <row r="78" spans="1:12" ht="259.2" x14ac:dyDescent="0.3">
-      <c r="A78" s="69">
+      <c r="A78" s="63">
         <v>22</v>
       </c>
-      <c r="B78" s="70" t="s">
+      <c r="B78" s="66" t="s">
         <v>157</v>
       </c>
-      <c r="C78" s="71">
+      <c r="C78" s="45">
         <v>22.1</v>
       </c>
-      <c r="D78" s="72" t="s">
+      <c r="D78" s="46" t="s">
         <v>158</v>
       </c>
-      <c r="E78" s="72" t="s">
+      <c r="E78" s="46" t="s">
         <v>305</v>
       </c>
-      <c r="F78" s="72" t="s">
+      <c r="F78" s="46" t="s">
         <v>306</v>
       </c>
-      <c r="G78" s="73" t="s">
+      <c r="G78" s="47" t="s">
         <v>307</v>
       </c>
-      <c r="H78" s="71"/>
-      <c r="I78" s="74"/>
+      <c r="H78" s="45"/>
+      <c r="I78" s="48"/>
     </row>
     <row r="79" spans="1:12" ht="244.8" x14ac:dyDescent="0.3">
-      <c r="A79" s="75"/>
-      <c r="B79" s="76"/>
-      <c r="C79" s="77">
+      <c r="A79" s="64"/>
+      <c r="B79" s="67"/>
+      <c r="C79" s="15">
         <v>22.2</v>
       </c>
-      <c r="D79" s="72" t="s">
+      <c r="D79" s="46" t="s">
         <v>280</v>
       </c>
-      <c r="E79" s="71" t="s">
+      <c r="E79" s="45" t="s">
         <v>303</v>
       </c>
-      <c r="F79" s="72" t="s">
+      <c r="F79" s="46" t="s">
         <v>282</v>
       </c>
-      <c r="G79" s="73" t="s">
+      <c r="G79" s="47" t="s">
         <v>304</v>
       </c>
-      <c r="H79" s="71"/>
-      <c r="I79" s="74"/>
+      <c r="H79" s="45"/>
+      <c r="I79" s="48"/>
     </row>
     <row r="80" spans="1:12" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A80" s="78"/>
-      <c r="B80" s="79"/>
-      <c r="C80" s="49">
+      <c r="A80" s="65"/>
+      <c r="B80" s="68"/>
+      <c r="C80" s="33">
         <v>22.3</v>
       </c>
-      <c r="D80" s="19" t="s">
+      <c r="D80" s="16" t="s">
         <v>158</v>
       </c>
-      <c r="E80" s="49" t="s">
+      <c r="E80" s="33" t="s">
         <v>148</v>
       </c>
-      <c r="F80" s="19"/>
-      <c r="G80" s="20"/>
-      <c r="H80" s="49"/>
-      <c r="I80" s="50"/>
+      <c r="F80" s="16"/>
+      <c r="G80" s="17"/>
+      <c r="H80" s="33"/>
+      <c r="I80" s="34"/>
     </row>
     <row r="81" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A81" s="3"/>
@@ -6038,21 +6045,12 @@
   </sheetData>
   <autoFilter ref="I1:I26" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
   <mergeCells count="37">
-    <mergeCell ref="A13:A16"/>
-    <mergeCell ref="B13:B16"/>
-    <mergeCell ref="A17:A20"/>
-    <mergeCell ref="H1:H2"/>
-    <mergeCell ref="I1:I2"/>
-    <mergeCell ref="A8:A12"/>
-    <mergeCell ref="B8:B12"/>
-    <mergeCell ref="A1:A2"/>
-    <mergeCell ref="B1:B2"/>
-    <mergeCell ref="C1:C2"/>
-    <mergeCell ref="D1:F1"/>
-    <mergeCell ref="G1:G2"/>
-    <mergeCell ref="A3:A7"/>
-    <mergeCell ref="B3:B7"/>
-    <mergeCell ref="B17:B20"/>
+    <mergeCell ref="A24:A28"/>
+    <mergeCell ref="B24:B28"/>
+    <mergeCell ref="A30:A40"/>
+    <mergeCell ref="B30:B40"/>
+    <mergeCell ref="A21:A23"/>
+    <mergeCell ref="B21:B23"/>
     <mergeCell ref="A41:A48"/>
     <mergeCell ref="B41:B48"/>
     <mergeCell ref="A75:A77"/>
@@ -6069,14 +6067,23 @@
     <mergeCell ref="B69:B71"/>
     <mergeCell ref="A72:A74"/>
     <mergeCell ref="B72:B74"/>
-    <mergeCell ref="A24:A28"/>
-    <mergeCell ref="B24:B28"/>
-    <mergeCell ref="A30:A40"/>
-    <mergeCell ref="B30:B40"/>
-    <mergeCell ref="A21:A23"/>
-    <mergeCell ref="B21:B23"/>
+    <mergeCell ref="A13:A16"/>
+    <mergeCell ref="B13:B16"/>
+    <mergeCell ref="A17:A20"/>
+    <mergeCell ref="H1:H2"/>
+    <mergeCell ref="I1:I2"/>
+    <mergeCell ref="A8:A12"/>
+    <mergeCell ref="B8:B12"/>
+    <mergeCell ref="A1:A2"/>
+    <mergeCell ref="B1:B2"/>
+    <mergeCell ref="C1:C2"/>
+    <mergeCell ref="D1:F1"/>
+    <mergeCell ref="G1:G2"/>
+    <mergeCell ref="A3:A7"/>
+    <mergeCell ref="B3:B7"/>
+    <mergeCell ref="B17:B20"/>
   </mergeCells>
-  <phoneticPr fontId="10" type="noConversion"/>
+  <phoneticPr fontId="11" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait"/>
   <legacyDrawing r:id="rId1"/>

</xml_diff>

<commit_message>
Copied checkupp repos for backend and web
</commit_message>
<xml_diff>
--- a/Soubhanik/checkupp_product_backlog_final.xlsx
+++ b/Soubhanik/checkupp_product_backlog_final.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GitHub\CheckUpp\Soubhanik\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{303B43DF-6A2A-4839-9905-224C3A45929B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CC212EFE-3A18-44FF-AB50-E204DB1FF9D3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1071,27 +1071,6 @@
     <t>logged-in user</t>
   </si>
   <si>
-    <t>1. All appointments with a Completed status must be displayed under the Completed tab.
-2. Each completed appointment must display its appointment name, completed appointment date, and completed appointment time.
-3. The logged-in user must be able to tap any Completed appointment from the list to view its details.
-4. Only appointments associated with the logged-in user's account must be displayed under the Completed tab.
-5. If no Completed appointments exist, an appropriate message (e.g.- No completed appointments).</t>
-  </si>
-  <si>
-    <t>1. All appointments with an Upcoming status must be displayed under the Upcoming tab.
-2. Each upcoming appointment must display its appointment name, scheduled date, and scheduled time.
-3. The logged-in user must be able to tap any Upcoming appointment from the list to view its details.
-4. Only appointments associated with the logged-in user's account must be displayed under the Upcoming tab.
-5. If no Upcoming appointments exist, an appropriate message (e.g.- No upcoming appointments) must be displayed.</t>
-  </si>
-  <si>
-    <t>1. All appointments with a Rescheduled status must be displayed under the Rescheduled tab.
-2. Each rescheduled appointment must display its appointment name, updated date, and updated time.
-3. The logged-in user must be able to tap any Rescheduled appointment from the list to see details.
-4. Only appointments associated with the logged-in user's account must be displayed under the Rescheduled tab.
-5. If no Rescheduled appointments exist, an appropriate message (e.g.- No Rescheduled appointments) must be displayed.</t>
-  </si>
-  <si>
     <t>Logged-in user</t>
   </si>
   <si>
@@ -3215,13 +3194,6 @@
     <t>I can view my Upcoming, Due and Completed appointments in Your Appointments section</t>
   </si>
   <si>
-    <t>1. The User must be able to access the Your Appointments section by tapping the Your Health Overview section on the Home Screen.
-2. The user's Upcoming, Due, and Completed appointment categories filter (top tabs) must be displayed in the Your Appointments section.
-3. The total number of appointments in each category must be displayed in the Upccoming, Due and Completed top tabs.
-4. Only appointments associated with the logged-in user's account must be displayed.
-5. If no appointments are available in a category (upcoming/due/completed), an appropriate message (e.g.- "You don't have any upcoming/due/completed appointments right now") must be displayed indicating that no appointments are available, in the Your Appointments section.</t>
-  </si>
-  <si>
     <r>
       <t xml:space="preserve">View my </t>
     </r>
@@ -3701,6 +3673,245 @@
         <family val="2"/>
       </rPr>
       <t xml:space="preserve"> bottom sheet must send the user back to the previous screen (where they opened the bottom sheet).</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">1. The User must be able to access the </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>Your Appointments</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> screen by tapping the </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>Your Health Overview</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> section on the Home Screen.
+2. The user's </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>Upcoming</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>Due</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">, and </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>Completed</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> appointment categories filter (top tabs) must be displayed in the </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>Your Appointments</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> screen.
+3. The total number of appointments in each category must be displayed in the </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>Upccoming</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>Due</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> and </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>Completed</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> top tabs.
+4. Only appointments associated with the logged-in user's account must be displayed.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">1. All appointments with an Upcoming status must be displayed under the </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>Upcoming</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> tab.
+2. Each upcoming appointment must display its appointment name, scheduled date, and scheduled time.
+3. The logged-in user must be able to tap any Upcoming appointment from the list to view its details.
+4. Only appointments associated with the logged-in user's account must be displayed under the Upcoming tab.
+5. If no Upcoming appointments exist, an appropriate message: "You don't have any upcoming appointments" must be displayed.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">1. All appointments with a Due status must be displayed under the </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>Due</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> tab.
+2. Each due appointment must display its appointment name, updated date, and updated time.
+3. The logged-in user must be able to tap any due appointment from the list to see details.
+4. Only appointments associated with the logged-in user's account must be displayed under the Rescheduled tab.
+5. If no due appointments exist, an appropriate message: "You don't have any upcoming appointments" must be displayed.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">1. All appointments with a Completed status must be displayed under the </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>Completed</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> tab.
+2. Each completed appointment must display its appointment name, completed appointment date, and completed appointment time.
+3. The logged-in user must be able to tap any Completed appointment from the list to view its details.
+4. Only appointments associated with the logged-in user's account must be displayed under the Completed tab.
+5. If no Completed appointments exist, an appropriate message: "You don't have any upcoming appointments" must be displayed.</t>
     </r>
   </si>
 </sst>
@@ -4154,6 +4365,63 @@
     <xf numFmtId="0" fontId="2" fillId="15" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="14" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="7" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="13" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="13" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="13" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="13" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="14" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -4175,9 +4443,6 @@
     <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="14" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -4191,60 +4456,6 @@
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="14" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="13" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="13" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="13" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="13" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="7" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -4480,34 +4691,34 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A1" s="55" t="s">
+      <c r="A1" s="74" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="55" t="s">
+      <c r="B1" s="74" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="55" t="s">
+      <c r="C1" s="74" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="55" t="s">
+      <c r="D1" s="74" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="56"/>
-      <c r="F1" s="56"/>
-      <c r="G1" s="60" t="s">
+      <c r="E1" s="55"/>
+      <c r="F1" s="55"/>
+      <c r="G1" s="78" t="s">
         <v>4</v>
       </c>
-      <c r="H1" s="55" t="s">
+      <c r="H1" s="74" t="s">
         <v>5</v>
       </c>
-      <c r="I1" s="55" t="s">
+      <c r="I1" s="74" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A2" s="56"/>
-      <c r="B2" s="56"/>
-      <c r="C2" s="56"/>
+      <c r="A2" s="55"/>
+      <c r="B2" s="55"/>
+      <c r="C2" s="55"/>
       <c r="D2" s="4" t="s">
         <v>7</v>
       </c>
@@ -4517,15 +4728,15 @@
       <c r="F2" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="G2" s="60"/>
-      <c r="H2" s="56"/>
-      <c r="I2" s="56"/>
-    </row>
-    <row r="3" spans="1:9" s="5" customFormat="1" ht="158.4" x14ac:dyDescent="0.3">
-      <c r="A3" s="61">
+      <c r="G2" s="78"/>
+      <c r="H2" s="55"/>
+      <c r="I2" s="55"/>
+    </row>
+    <row r="3" spans="1:9" s="5" customFormat="1" ht="100.8" x14ac:dyDescent="0.3">
+      <c r="A3" s="79">
         <v>1</v>
       </c>
-      <c r="B3" s="61" t="s">
+      <c r="B3" s="79" t="s">
         <v>10</v>
       </c>
       <c r="C3" s="16">
@@ -4538,10 +4749,10 @@
         <v>163</v>
       </c>
       <c r="F3" s="16" t="s">
-        <v>302</v>
+        <v>299</v>
       </c>
       <c r="G3" s="17" t="s">
-        <v>303</v>
+        <v>307</v>
       </c>
       <c r="H3" s="16" t="s">
         <v>11</v>
@@ -4551,94 +4762,94 @@
       </c>
     </row>
     <row r="4" spans="1:9" s="6" customFormat="1" ht="144" x14ac:dyDescent="0.3">
-      <c r="A4" s="61"/>
-      <c r="B4" s="61"/>
+      <c r="A4" s="79"/>
+      <c r="B4" s="79"/>
       <c r="C4" s="16">
         <v>1.2</v>
       </c>
       <c r="D4" s="16" t="s">
-        <v>168</v>
+        <v>165</v>
       </c>
       <c r="E4" s="16" t="s">
-        <v>305</v>
+        <v>301</v>
       </c>
       <c r="F4" s="16" t="s">
         <v>159</v>
       </c>
       <c r="G4" s="17" t="s">
-        <v>166</v>
+        <v>308</v>
       </c>
       <c r="H4" s="16"/>
       <c r="I4" s="16"/>
     </row>
-    <row r="5" spans="1:9" s="6" customFormat="1" ht="144" x14ac:dyDescent="0.3">
-      <c r="A5" s="61"/>
-      <c r="B5" s="61"/>
+    <row r="5" spans="1:9" s="6" customFormat="1" ht="129.6" x14ac:dyDescent="0.3">
+      <c r="A5" s="79"/>
+      <c r="B5" s="79"/>
       <c r="C5" s="16">
         <v>1.3</v>
       </c>
       <c r="D5" s="16" t="s">
-        <v>168</v>
+        <v>165</v>
       </c>
       <c r="E5" s="16" t="s">
-        <v>304</v>
+        <v>300</v>
       </c>
       <c r="F5" s="16" t="s">
         <v>160</v>
       </c>
       <c r="G5" s="17" t="s">
-        <v>167</v>
+        <v>309</v>
       </c>
       <c r="H5" s="16"/>
       <c r="I5" s="16"/>
     </row>
     <row r="6" spans="1:9" s="6" customFormat="1" ht="144" x14ac:dyDescent="0.3">
-      <c r="A6" s="61"/>
-      <c r="B6" s="61"/>
+      <c r="A6" s="79"/>
+      <c r="B6" s="79"/>
       <c r="C6" s="16">
         <v>1.4</v>
       </c>
       <c r="D6" s="16" t="s">
-        <v>168</v>
+        <v>165</v>
       </c>
       <c r="E6" s="16" t="s">
-        <v>306</v>
+        <v>302</v>
       </c>
       <c r="F6" s="16" t="s">
-        <v>307</v>
+        <v>303</v>
       </c>
       <c r="G6" s="17" t="s">
-        <v>165</v>
+        <v>310</v>
       </c>
       <c r="H6" s="16"/>
       <c r="I6" s="16"/>
     </row>
     <row r="7" spans="1:9" s="6" customFormat="1" ht="282" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="61"/>
-      <c r="B7" s="61"/>
+      <c r="A7" s="79"/>
+      <c r="B7" s="79"/>
       <c r="C7" s="16">
         <v>1.5</v>
       </c>
       <c r="D7" s="16" t="s">
-        <v>168</v>
+        <v>165</v>
       </c>
       <c r="E7" s="16" t="s">
-        <v>309</v>
+        <v>305</v>
       </c>
       <c r="F7" s="16" t="s">
-        <v>308</v>
+        <v>304</v>
       </c>
       <c r="G7" s="17" t="s">
-        <v>310</v>
+        <v>306</v>
       </c>
       <c r="H7" s="16"/>
       <c r="I7" s="16"/>
     </row>
     <row r="8" spans="1:9" s="6" customFormat="1" ht="129.6" x14ac:dyDescent="0.3">
-      <c r="A8" s="57">
+      <c r="A8" s="75">
         <v>5</v>
       </c>
-      <c r="B8" s="57" t="s">
+      <c r="B8" s="75" t="s">
         <v>13</v>
       </c>
       <c r="C8" s="18">
@@ -4664,8 +4875,8 @@
       </c>
     </row>
     <row r="9" spans="1:9" s="6" customFormat="1" ht="129.6" x14ac:dyDescent="0.3">
-      <c r="A9" s="58"/>
-      <c r="B9" s="58"/>
+      <c r="A9" s="76"/>
+      <c r="B9" s="76"/>
       <c r="C9" s="18">
         <v>5.2</v>
       </c>
@@ -4685,8 +4896,8 @@
       <c r="I9" s="18"/>
     </row>
     <row r="10" spans="1:9" s="6" customFormat="1" ht="172.8" x14ac:dyDescent="0.3">
-      <c r="A10" s="58"/>
-      <c r="B10" s="58"/>
+      <c r="A10" s="76"/>
+      <c r="B10" s="76"/>
       <c r="C10" s="18">
         <v>5.3</v>
       </c>
@@ -4706,52 +4917,52 @@
       <c r="I10" s="18"/>
     </row>
     <row r="11" spans="1:9" s="14" customFormat="1" ht="230.4" x14ac:dyDescent="0.3">
-      <c r="A11" s="58"/>
-      <c r="B11" s="58"/>
+      <c r="A11" s="76"/>
+      <c r="B11" s="76"/>
       <c r="C11" s="21">
         <v>5.4</v>
       </c>
       <c r="D11" s="21" t="s">
+        <v>169</v>
+      </c>
+      <c r="E11" s="21" t="s">
         <v>172</v>
       </c>
-      <c r="E11" s="21" t="s">
-        <v>175</v>
-      </c>
       <c r="F11" s="21" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
       <c r="G11" s="22" t="s">
-        <v>176</v>
+        <v>173</v>
       </c>
       <c r="H11" s="23"/>
       <c r="I11" s="21"/>
     </row>
     <row r="12" spans="1:9" s="14" customFormat="1" ht="158.4" x14ac:dyDescent="0.3">
-      <c r="A12" s="59"/>
-      <c r="B12" s="59"/>
+      <c r="A12" s="77"/>
+      <c r="B12" s="77"/>
       <c r="C12" s="21">
         <v>5.5</v>
       </c>
       <c r="D12" s="21" t="s">
-        <v>169</v>
+        <v>166</v>
       </c>
       <c r="E12" s="21" t="s">
-        <v>173</v>
+        <v>170</v>
       </c>
       <c r="F12" s="21" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
       <c r="G12" s="22" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="H12" s="23"/>
       <c r="I12" s="21"/>
     </row>
     <row r="13" spans="1:9" s="14" customFormat="1" ht="172.8" x14ac:dyDescent="0.3">
-      <c r="A13" s="49">
+      <c r="A13" s="68">
         <v>6</v>
       </c>
-      <c r="B13" s="49" t="s">
+      <c r="B13" s="68" t="s">
         <v>25</v>
       </c>
       <c r="C13" s="21">
@@ -4777,8 +4988,8 @@
       </c>
     </row>
     <row r="14" spans="1:9" s="6" customFormat="1" ht="144" x14ac:dyDescent="0.3">
-      <c r="A14" s="50"/>
-      <c r="B14" s="50"/>
+      <c r="A14" s="69"/>
+      <c r="B14" s="69"/>
       <c r="C14" s="24">
         <v>6.2</v>
       </c>
@@ -4786,20 +4997,20 @@
         <v>26</v>
       </c>
       <c r="E14" s="24" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
       <c r="F14" s="24" t="s">
-        <v>177</v>
+        <v>174</v>
       </c>
       <c r="G14" s="25" t="s">
-        <v>179</v>
+        <v>176</v>
       </c>
       <c r="H14" s="26"/>
       <c r="I14" s="24"/>
     </row>
     <row r="15" spans="1:9" s="6" customFormat="1" ht="172.8" x14ac:dyDescent="0.3">
-      <c r="A15" s="50"/>
-      <c r="B15" s="50"/>
+      <c r="A15" s="69"/>
+      <c r="B15" s="69"/>
       <c r="C15" s="24">
         <v>6.3</v>
       </c>
@@ -4819,8 +5030,8 @@
       <c r="I15" s="24"/>
     </row>
     <row r="16" spans="1:9" s="6" customFormat="1" ht="72" x14ac:dyDescent="0.3">
-      <c r="A16" s="50"/>
-      <c r="B16" s="51"/>
+      <c r="A16" s="69"/>
+      <c r="B16" s="70"/>
       <c r="C16" s="27">
         <v>6.4</v>
       </c>
@@ -4844,10 +5055,10 @@
       </c>
     </row>
     <row r="17" spans="1:9" s="6" customFormat="1" ht="144" x14ac:dyDescent="0.3">
-      <c r="A17" s="52">
+      <c r="A17" s="71">
         <v>7</v>
       </c>
-      <c r="B17" s="49" t="s">
+      <c r="B17" s="68" t="s">
         <v>38</v>
       </c>
       <c r="C17" s="24">
@@ -4873,8 +5084,8 @@
       </c>
     </row>
     <row r="18" spans="1:9" s="6" customFormat="1" ht="72" x14ac:dyDescent="0.3">
-      <c r="A18" s="53"/>
-      <c r="B18" s="50"/>
+      <c r="A18" s="72"/>
+      <c r="B18" s="69"/>
       <c r="C18" s="24">
         <v>7.2</v>
       </c>
@@ -4896,8 +5107,8 @@
       </c>
     </row>
     <row r="19" spans="1:9" s="6" customFormat="1" ht="187.2" x14ac:dyDescent="0.3">
-      <c r="A19" s="53"/>
-      <c r="B19" s="50"/>
+      <c r="A19" s="72"/>
+      <c r="B19" s="69"/>
       <c r="C19" s="24">
         <v>7.3</v>
       </c>
@@ -4917,8 +5128,8 @@
       <c r="I19" s="24"/>
     </row>
     <row r="20" spans="1:9" s="6" customFormat="1" ht="172.8" x14ac:dyDescent="0.3">
-      <c r="A20" s="54"/>
-      <c r="B20" s="51"/>
+      <c r="A20" s="73"/>
+      <c r="B20" s="70"/>
       <c r="C20" s="24">
         <v>7.4</v>
       </c>
@@ -4938,10 +5149,10 @@
       <c r="I20" s="24"/>
     </row>
     <row r="21" spans="1:9" s="6" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A21" s="77">
+      <c r="A21" s="51">
         <v>8</v>
       </c>
-      <c r="B21" s="77" t="s">
+      <c r="B21" s="51" t="s">
         <v>50</v>
       </c>
       <c r="C21" s="28">
@@ -4965,8 +5176,8 @@
       </c>
     </row>
     <row r="22" spans="1:9" s="6" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A22" s="78"/>
-      <c r="B22" s="78"/>
+      <c r="A22" s="52"/>
+      <c r="B22" s="52"/>
       <c r="C22" s="28">
         <v>9.3000000000000007</v>
       </c>
@@ -4988,8 +5199,8 @@
       </c>
     </row>
     <row r="23" spans="1:9" s="6" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A23" s="79"/>
-      <c r="B23" s="79"/>
+      <c r="A23" s="53"/>
+      <c r="B23" s="53"/>
       <c r="C23" s="28">
         <v>9.4</v>
       </c>
@@ -5011,10 +5222,10 @@
       </c>
     </row>
     <row r="24" spans="1:9" s="6" customFormat="1" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A24" s="75">
+      <c r="A24" s="49">
         <v>12</v>
       </c>
-      <c r="B24" s="75" t="s">
+      <c r="B24" s="49" t="s">
         <v>64</v>
       </c>
       <c r="C24" s="31">
@@ -5040,8 +5251,8 @@
       </c>
     </row>
     <row r="25" spans="1:9" s="6" customFormat="1" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A25" s="75"/>
-      <c r="B25" s="75"/>
+      <c r="A25" s="49"/>
+      <c r="B25" s="49"/>
       <c r="C25" s="31">
         <v>12.2</v>
       </c>
@@ -5065,8 +5276,8 @@
       </c>
     </row>
     <row r="26" spans="1:9" s="6" customFormat="1" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A26" s="75"/>
-      <c r="B26" s="75"/>
+      <c r="A26" s="49"/>
+      <c r="B26" s="49"/>
       <c r="C26" s="31">
         <v>12.3</v>
       </c>
@@ -5090,8 +5301,8 @@
       </c>
     </row>
     <row r="27" spans="1:9" s="6" customFormat="1" ht="123.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A27" s="75"/>
-      <c r="B27" s="75"/>
+      <c r="A27" s="49"/>
+      <c r="B27" s="49"/>
       <c r="C27" s="31">
         <v>12.4</v>
       </c>
@@ -5099,13 +5310,13 @@
         <v>65</v>
       </c>
       <c r="E27" s="31" t="s">
-        <v>274</v>
+        <v>271</v>
       </c>
       <c r="F27" s="31" t="s">
-        <v>275</v>
+        <v>272</v>
       </c>
       <c r="G27" s="32" t="s">
-        <v>276</v>
+        <v>273</v>
       </c>
       <c r="H27" s="31" t="s">
         <v>69</v>
@@ -5115,8 +5326,8 @@
       </c>
     </row>
     <row r="28" spans="1:9" s="6" customFormat="1" ht="129.6" x14ac:dyDescent="0.3">
-      <c r="A28" s="75"/>
-      <c r="B28" s="75"/>
+      <c r="A28" s="49"/>
+      <c r="B28" s="49"/>
       <c r="C28" s="31">
         <v>12.5</v>
       </c>
@@ -5127,7 +5338,7 @@
         <v>78</v>
       </c>
       <c r="F28" s="31" t="s">
-        <v>273</v>
+        <v>270</v>
       </c>
       <c r="G28" s="32" t="s">
         <v>79</v>
@@ -5157,10 +5368,10 @@
       <c r="I29" s="34"/>
     </row>
     <row r="30" spans="1:9" s="6" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A30" s="76">
+      <c r="A30" s="50">
         <v>14</v>
       </c>
-      <c r="B30" s="76" t="s">
+      <c r="B30" s="50" t="s">
         <v>80</v>
       </c>
       <c r="C30" s="35">
@@ -5170,13 +5381,13 @@
         <v>133</v>
       </c>
       <c r="E30" s="36" t="s">
-        <v>244</v>
+        <v>241</v>
       </c>
       <c r="F30" s="36" t="s">
-        <v>210</v>
+        <v>207</v>
       </c>
       <c r="G30" s="37" t="s">
-        <v>260</v>
+        <v>257</v>
       </c>
       <c r="H30" s="35" t="s">
         <v>82</v>
@@ -5186,8 +5397,8 @@
       </c>
     </row>
     <row r="31" spans="1:9" s="6" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A31" s="76"/>
-      <c r="B31" s="76"/>
+      <c r="A31" s="50"/>
+      <c r="B31" s="50"/>
       <c r="C31" s="35">
         <v>14.2</v>
       </c>
@@ -5195,13 +5406,13 @@
         <v>133</v>
       </c>
       <c r="E31" s="36" t="s">
-        <v>245</v>
+        <v>242</v>
       </c>
       <c r="F31" s="36" t="s">
-        <v>246</v>
+        <v>243</v>
       </c>
       <c r="G31" s="37" t="s">
-        <v>261</v>
+        <v>258</v>
       </c>
       <c r="H31" s="35" t="s">
         <v>82</v>
@@ -5211,22 +5422,22 @@
       </c>
     </row>
     <row r="32" spans="1:9" s="6" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A32" s="76"/>
-      <c r="B32" s="76"/>
+      <c r="A32" s="50"/>
+      <c r="B32" s="50"/>
       <c r="C32" s="35">
         <v>14.3</v>
       </c>
       <c r="D32" s="36" t="s">
-        <v>215</v>
+        <v>212</v>
       </c>
       <c r="E32" s="36" t="s">
-        <v>247</v>
+        <v>244</v>
       </c>
       <c r="F32" s="36" t="s">
-        <v>248</v>
+        <v>245</v>
       </c>
       <c r="G32" s="37" t="s">
-        <v>262</v>
+        <v>259</v>
       </c>
       <c r="H32" s="35" t="s">
         <v>82</v>
@@ -5236,8 +5447,8 @@
       </c>
     </row>
     <row r="33" spans="1:9" s="6" customFormat="1" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A33" s="76"/>
-      <c r="B33" s="76"/>
+      <c r="A33" s="50"/>
+      <c r="B33" s="50"/>
       <c r="C33" s="35">
         <v>14.4</v>
       </c>
@@ -5245,13 +5456,13 @@
         <v>133</v>
       </c>
       <c r="E33" s="36" t="s">
-        <v>249</v>
+        <v>246</v>
       </c>
       <c r="F33" s="36" t="s">
-        <v>220</v>
+        <v>217</v>
       </c>
       <c r="G33" s="37" t="s">
-        <v>263</v>
+        <v>260</v>
       </c>
       <c r="H33" s="35" t="s">
         <v>82</v>
@@ -5261,8 +5472,8 @@
       </c>
     </row>
     <row r="34" spans="1:9" s="6" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A34" s="76"/>
-      <c r="B34" s="76"/>
+      <c r="A34" s="50"/>
+      <c r="B34" s="50"/>
       <c r="C34" s="35">
         <v>14.5</v>
       </c>
@@ -5270,13 +5481,13 @@
         <v>133</v>
       </c>
       <c r="E34" s="36" t="s">
-        <v>250</v>
+        <v>247</v>
       </c>
       <c r="F34" s="36" t="s">
-        <v>223</v>
+        <v>220</v>
       </c>
       <c r="G34" s="37" t="s">
-        <v>264</v>
+        <v>261</v>
       </c>
       <c r="H34" s="35" t="s">
         <v>82</v>
@@ -5286,8 +5497,8 @@
       </c>
     </row>
     <row r="35" spans="1:9" s="6" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A35" s="76"/>
-      <c r="B35" s="76"/>
+      <c r="A35" s="50"/>
+      <c r="B35" s="50"/>
       <c r="C35" s="35">
         <v>14.6</v>
       </c>
@@ -5295,13 +5506,13 @@
         <v>133</v>
       </c>
       <c r="E35" s="36" t="s">
-        <v>251</v>
+        <v>248</v>
       </c>
       <c r="F35" s="36" t="s">
-        <v>252</v>
+        <v>249</v>
       </c>
       <c r="G35" s="37" t="s">
-        <v>265</v>
+        <v>262</v>
       </c>
       <c r="H35" s="35" t="s">
         <v>82</v>
@@ -5311,8 +5522,8 @@
       </c>
     </row>
     <row r="36" spans="1:9" s="6" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A36" s="76"/>
-      <c r="B36" s="76"/>
+      <c r="A36" s="50"/>
+      <c r="B36" s="50"/>
       <c r="C36" s="35">
         <v>14.7</v>
       </c>
@@ -5320,13 +5531,13 @@
         <v>133</v>
       </c>
       <c r="E36" s="36" t="s">
-        <v>253</v>
+        <v>250</v>
       </c>
       <c r="F36" s="36" t="s">
-        <v>254</v>
+        <v>251</v>
       </c>
       <c r="G36" s="37" t="s">
-        <v>266</v>
+        <v>263</v>
       </c>
       <c r="H36" s="35" t="s">
         <v>82</v>
@@ -5336,8 +5547,8 @@
       </c>
     </row>
     <row r="37" spans="1:9" s="6" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A37" s="76"/>
-      <c r="B37" s="76"/>
+      <c r="A37" s="50"/>
+      <c r="B37" s="50"/>
       <c r="C37" s="35">
         <v>14.8</v>
       </c>
@@ -5345,13 +5556,13 @@
         <v>133</v>
       </c>
       <c r="E37" s="36" t="s">
-        <v>255</v>
+        <v>252</v>
       </c>
       <c r="F37" s="36" t="s">
-        <v>256</v>
+        <v>253</v>
       </c>
       <c r="G37" s="37" t="s">
-        <v>267</v>
+        <v>264</v>
       </c>
       <c r="H37" s="35" t="s">
         <v>84</v>
@@ -5361,8 +5572,8 @@
       </c>
     </row>
     <row r="38" spans="1:9" s="6" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A38" s="76"/>
-      <c r="B38" s="76"/>
+      <c r="A38" s="50"/>
+      <c r="B38" s="50"/>
       <c r="C38" s="35">
         <v>14.9</v>
       </c>
@@ -5370,13 +5581,13 @@
         <v>133</v>
       </c>
       <c r="E38" s="36" t="s">
-        <v>257</v>
+        <v>254</v>
       </c>
       <c r="F38" s="36" t="s">
-        <v>235</v>
+        <v>232</v>
       </c>
       <c r="G38" s="37" t="s">
-        <v>268</v>
+        <v>265</v>
       </c>
       <c r="H38" s="35" t="s">
         <v>84</v>
@@ -5386,8 +5597,8 @@
       </c>
     </row>
     <row r="39" spans="1:9" s="6" customFormat="1" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A39" s="76"/>
-      <c r="B39" s="76"/>
+      <c r="A39" s="50"/>
+      <c r="B39" s="50"/>
       <c r="C39" s="35">
         <v>14.1</v>
       </c>
@@ -5395,13 +5606,13 @@
         <v>133</v>
       </c>
       <c r="E39" s="36" t="s">
-        <v>258</v>
+        <v>255</v>
       </c>
       <c r="F39" s="36" t="s">
-        <v>239</v>
+        <v>236</v>
       </c>
       <c r="G39" s="37" t="s">
-        <v>269</v>
+        <v>266</v>
       </c>
       <c r="H39" s="35" t="s">
         <v>84</v>
@@ -5411,8 +5622,8 @@
       </c>
     </row>
     <row r="40" spans="1:9" s="6" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A40" s="76"/>
-      <c r="B40" s="76"/>
+      <c r="A40" s="50"/>
+      <c r="B40" s="50"/>
       <c r="C40" s="35">
         <v>14.11</v>
       </c>
@@ -5420,13 +5631,13 @@
         <v>133</v>
       </c>
       <c r="E40" s="36" t="s">
-        <v>259</v>
+        <v>256</v>
       </c>
       <c r="F40" s="36" t="s">
-        <v>242</v>
+        <v>239</v>
       </c>
       <c r="G40" s="37" t="s">
-        <v>270</v>
+        <v>267</v>
       </c>
       <c r="H40" s="35" t="s">
         <v>84</v>
@@ -5436,10 +5647,10 @@
       </c>
     </row>
     <row r="41" spans="1:9" s="6" customFormat="1" ht="86.4" x14ac:dyDescent="0.3">
-      <c r="A41" s="62">
+      <c r="A41" s="54">
         <v>15</v>
       </c>
-      <c r="B41" s="62" t="s">
+      <c r="B41" s="54" t="s">
         <v>85</v>
       </c>
       <c r="C41" s="38">
@@ -5455,7 +5666,7 @@
         <v>88</v>
       </c>
       <c r="G41" s="39" t="s">
-        <v>180</v>
+        <v>177</v>
       </c>
       <c r="H41" s="38" t="s">
         <v>123</v>
@@ -5465,8 +5676,8 @@
       </c>
     </row>
     <row r="42" spans="1:9" s="6" customFormat="1" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A42" s="56"/>
-      <c r="B42" s="56"/>
+      <c r="A42" s="55"/>
+      <c r="B42" s="55"/>
       <c r="C42" s="38">
         <v>15.2</v>
       </c>
@@ -5480,7 +5691,7 @@
         <v>90</v>
       </c>
       <c r="G42" s="39" t="s">
-        <v>181</v>
+        <v>178</v>
       </c>
       <c r="H42" s="38" t="s">
         <v>107</v>
@@ -5490,8 +5701,8 @@
       </c>
     </row>
     <row r="43" spans="1:9" s="6" customFormat="1" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A43" s="56"/>
-      <c r="B43" s="56"/>
+      <c r="A43" s="55"/>
+      <c r="B43" s="55"/>
       <c r="C43" s="38">
         <v>15.3</v>
       </c>
@@ -5505,7 +5716,7 @@
         <v>92</v>
       </c>
       <c r="G43" s="39" t="s">
-        <v>182</v>
+        <v>179</v>
       </c>
       <c r="H43" s="38" t="s">
         <v>107</v>
@@ -5515,8 +5726,8 @@
       </c>
     </row>
     <row r="44" spans="1:9" s="6" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A44" s="56"/>
-      <c r="B44" s="56"/>
+      <c r="A44" s="55"/>
+      <c r="B44" s="55"/>
       <c r="C44" s="38">
         <v>15.4</v>
       </c>
@@ -5530,7 +5741,7 @@
         <v>94</v>
       </c>
       <c r="G44" s="39" t="s">
-        <v>183</v>
+        <v>180</v>
       </c>
       <c r="H44" s="38" t="s">
         <v>107</v>
@@ -5540,8 +5751,8 @@
       </c>
     </row>
     <row r="45" spans="1:9" s="6" customFormat="1" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A45" s="56"/>
-      <c r="B45" s="56"/>
+      <c r="A45" s="55"/>
+      <c r="B45" s="55"/>
       <c r="C45" s="38">
         <v>15.5</v>
       </c>
@@ -5555,7 +5766,7 @@
         <v>96</v>
       </c>
       <c r="G45" s="39" t="s">
-        <v>184</v>
+        <v>181</v>
       </c>
       <c r="H45" s="38" t="s">
         <v>107</v>
@@ -5565,8 +5776,8 @@
       </c>
     </row>
     <row r="46" spans="1:9" s="6" customFormat="1" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A46" s="56"/>
-      <c r="B46" s="56"/>
+      <c r="A46" s="55"/>
+      <c r="B46" s="55"/>
       <c r="C46" s="38">
         <v>15.6</v>
       </c>
@@ -5580,7 +5791,7 @@
         <v>98</v>
       </c>
       <c r="G46" s="39" t="s">
-        <v>185</v>
+        <v>182</v>
       </c>
       <c r="H46" s="38" t="s">
         <v>107</v>
@@ -5590,8 +5801,8 @@
       </c>
     </row>
     <row r="47" spans="1:9" s="6" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A47" s="56"/>
-      <c r="B47" s="56"/>
+      <c r="A47" s="55"/>
+      <c r="B47" s="55"/>
       <c r="C47" s="38">
         <v>15.7</v>
       </c>
@@ -5605,7 +5816,7 @@
         <v>100</v>
       </c>
       <c r="G47" s="39" t="s">
-        <v>186</v>
+        <v>183</v>
       </c>
       <c r="H47" s="38" t="s">
         <v>107</v>
@@ -5615,8 +5826,8 @@
       </c>
     </row>
     <row r="48" spans="1:9" s="6" customFormat="1" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A48" s="56"/>
-      <c r="B48" s="56"/>
+      <c r="A48" s="55"/>
+      <c r="B48" s="55"/>
       <c r="C48" s="38">
         <v>15.8</v>
       </c>
@@ -5630,7 +5841,7 @@
         <v>102</v>
       </c>
       <c r="G48" s="39" t="s">
-        <v>187</v>
+        <v>184</v>
       </c>
       <c r="H48" s="38" t="s">
         <v>107</v>
@@ -5640,10 +5851,10 @@
       </c>
     </row>
     <row r="49" spans="1:9" s="6" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A49" s="69">
+      <c r="A49" s="62">
         <v>16</v>
       </c>
-      <c r="B49" s="69" t="s">
+      <c r="B49" s="62" t="s">
         <v>103</v>
       </c>
       <c r="C49" s="40">
@@ -5659,7 +5870,7 @@
         <v>106</v>
       </c>
       <c r="G49" s="42" t="s">
-        <v>188</v>
+        <v>185</v>
       </c>
       <c r="H49" s="41" t="s">
         <v>107</v>
@@ -5669,8 +5880,8 @@
       </c>
     </row>
     <row r="50" spans="1:9" s="6" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A50" s="69"/>
-      <c r="B50" s="69"/>
+      <c r="A50" s="62"/>
+      <c r="B50" s="62"/>
       <c r="C50" s="40">
         <v>16.2</v>
       </c>
@@ -5684,7 +5895,7 @@
         <v>110</v>
       </c>
       <c r="G50" s="42" t="s">
-        <v>189</v>
+        <v>186</v>
       </c>
       <c r="H50" s="41" t="s">
         <v>107</v>
@@ -5694,8 +5905,8 @@
       </c>
     </row>
     <row r="51" spans="1:9" s="6" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A51" s="69"/>
-      <c r="B51" s="69"/>
+      <c r="A51" s="62"/>
+      <c r="B51" s="62"/>
       <c r="C51" s="40">
         <v>16.3</v>
       </c>
@@ -5709,7 +5920,7 @@
         <v>112</v>
       </c>
       <c r="G51" s="42" t="s">
-        <v>190</v>
+        <v>187</v>
       </c>
       <c r="H51" s="41" t="s">
         <v>107</v>
@@ -5719,8 +5930,8 @@
       </c>
     </row>
     <row r="52" spans="1:9" s="6" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A52" s="69"/>
-      <c r="B52" s="69"/>
+      <c r="A52" s="62"/>
+      <c r="B52" s="62"/>
       <c r="C52" s="40">
         <v>16.399999999999999</v>
       </c>
@@ -5734,7 +5945,7 @@
         <v>114</v>
       </c>
       <c r="G52" s="42" t="s">
-        <v>191</v>
+        <v>188</v>
       </c>
       <c r="H52" s="41" t="s">
         <v>107</v>
@@ -5744,8 +5955,8 @@
       </c>
     </row>
     <row r="53" spans="1:9" s="6" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A53" s="69"/>
-      <c r="B53" s="69"/>
+      <c r="A53" s="62"/>
+      <c r="B53" s="62"/>
       <c r="C53" s="40">
         <v>16.5</v>
       </c>
@@ -5759,7 +5970,7 @@
         <v>116</v>
       </c>
       <c r="G53" s="42" t="s">
-        <v>192</v>
+        <v>189</v>
       </c>
       <c r="H53" s="41" t="s">
         <v>107</v>
@@ -5769,8 +5980,8 @@
       </c>
     </row>
     <row r="54" spans="1:9" s="6" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A54" s="56"/>
-      <c r="B54" s="56"/>
+      <c r="A54" s="55"/>
+      <c r="B54" s="55"/>
       <c r="C54" s="40">
         <v>16.600000000000001</v>
       </c>
@@ -5784,7 +5995,7 @@
         <v>118</v>
       </c>
       <c r="G54" s="42" t="s">
-        <v>193</v>
+        <v>190</v>
       </c>
       <c r="H54" s="41" t="s">
         <v>107</v>
@@ -5794,10 +6005,10 @@
       </c>
     </row>
     <row r="55" spans="1:9" s="6" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A55" s="70">
+      <c r="A55" s="63">
         <v>17</v>
       </c>
-      <c r="B55" s="73" t="s">
+      <c r="B55" s="66" t="s">
         <v>119</v>
       </c>
       <c r="C55" s="43">
@@ -5813,7 +6024,7 @@
         <v>122</v>
       </c>
       <c r="G55" s="44" t="s">
-        <v>194</v>
+        <v>191</v>
       </c>
       <c r="H55" s="43" t="s">
         <v>123</v>
@@ -5823,8 +6034,8 @@
       </c>
     </row>
     <row r="56" spans="1:9" s="6" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A56" s="71"/>
-      <c r="B56" s="73"/>
+      <c r="A56" s="64"/>
+      <c r="B56" s="66"/>
       <c r="C56" s="43">
         <v>17.2</v>
       </c>
@@ -5838,7 +6049,7 @@
         <v>125</v>
       </c>
       <c r="G56" s="44" t="s">
-        <v>195</v>
+        <v>192</v>
       </c>
       <c r="H56" s="43" t="s">
         <v>123</v>
@@ -5848,8 +6059,8 @@
       </c>
     </row>
     <row r="57" spans="1:9" s="6" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A57" s="71"/>
-      <c r="B57" s="73"/>
+      <c r="A57" s="64"/>
+      <c r="B57" s="66"/>
       <c r="C57" s="43">
         <v>17.3</v>
       </c>
@@ -5863,7 +6074,7 @@
         <v>127</v>
       </c>
       <c r="G57" s="44" t="s">
-        <v>196</v>
+        <v>193</v>
       </c>
       <c r="H57" s="43" t="s">
         <v>107</v>
@@ -5873,8 +6084,8 @@
       </c>
     </row>
     <row r="58" spans="1:9" s="6" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A58" s="71"/>
-      <c r="B58" s="73"/>
+      <c r="A58" s="64"/>
+      <c r="B58" s="66"/>
       <c r="C58" s="43">
         <v>17.399999999999999</v>
       </c>
@@ -5888,7 +6099,7 @@
         <v>129</v>
       </c>
       <c r="G58" s="44" t="s">
-        <v>197</v>
+        <v>194</v>
       </c>
       <c r="H58" s="43" t="s">
         <v>123</v>
@@ -5898,8 +6109,8 @@
       </c>
     </row>
     <row r="59" spans="1:9" s="6" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A59" s="72"/>
-      <c r="B59" s="73"/>
+      <c r="A59" s="65"/>
+      <c r="B59" s="66"/>
       <c r="C59" s="43">
         <v>17.5</v>
       </c>
@@ -5913,7 +6124,7 @@
         <v>131</v>
       </c>
       <c r="G59" s="44" t="s">
-        <v>198</v>
+        <v>195</v>
       </c>
       <c r="H59" s="43" t="s">
         <v>123</v>
@@ -5923,10 +6134,10 @@
       </c>
     </row>
     <row r="60" spans="1:9" s="6" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A60" s="74">
+      <c r="A60" s="67">
         <v>18</v>
       </c>
-      <c r="B60" s="74" t="s">
+      <c r="B60" s="67" t="s">
         <v>132</v>
       </c>
       <c r="C60" s="18">
@@ -5936,13 +6147,13 @@
         <v>133</v>
       </c>
       <c r="E60" s="18" t="s">
-        <v>282</v>
+        <v>279</v>
       </c>
       <c r="F60" s="18" t="s">
         <v>134</v>
       </c>
       <c r="G60" s="19" t="s">
-        <v>199</v>
+        <v>196</v>
       </c>
       <c r="H60" s="18" t="s">
         <v>82</v>
@@ -5952,8 +6163,8 @@
       </c>
     </row>
     <row r="61" spans="1:9" s="6" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A61" s="56"/>
-      <c r="B61" s="56"/>
+      <c r="A61" s="55"/>
+      <c r="B61" s="55"/>
       <c r="C61" s="18">
         <v>18.2</v>
       </c>
@@ -5961,13 +6172,13 @@
         <v>133</v>
       </c>
       <c r="E61" s="18" t="s">
-        <v>283</v>
+        <v>280</v>
       </c>
       <c r="F61" s="18" t="s">
         <v>136</v>
       </c>
       <c r="G61" s="19" t="s">
-        <v>200</v>
+        <v>197</v>
       </c>
       <c r="H61" s="18" t="s">
         <v>82</v>
@@ -5977,8 +6188,8 @@
       </c>
     </row>
     <row r="62" spans="1:9" s="6" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A62" s="56"/>
-      <c r="B62" s="56"/>
+      <c r="A62" s="55"/>
+      <c r="B62" s="55"/>
       <c r="C62" s="18">
         <v>18.3</v>
       </c>
@@ -5986,13 +6197,13 @@
         <v>133</v>
       </c>
       <c r="E62" s="18" t="s">
-        <v>284</v>
+        <v>281</v>
       </c>
       <c r="F62" s="18" t="s">
         <v>137</v>
       </c>
       <c r="G62" s="19" t="s">
-        <v>201</v>
+        <v>198</v>
       </c>
       <c r="H62" s="18" t="s">
         <v>82</v>
@@ -6002,8 +6213,8 @@
       </c>
     </row>
     <row r="63" spans="1:9" s="6" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A63" s="56"/>
-      <c r="B63" s="56"/>
+      <c r="A63" s="55"/>
+      <c r="B63" s="55"/>
       <c r="C63" s="18">
         <v>18.399999999999999</v>
       </c>
@@ -6011,13 +6222,13 @@
         <v>133</v>
       </c>
       <c r="E63" s="18" t="s">
-        <v>285</v>
+        <v>282</v>
       </c>
       <c r="F63" s="18" t="s">
         <v>81</v>
       </c>
       <c r="G63" s="19" t="s">
-        <v>202</v>
+        <v>199</v>
       </c>
       <c r="H63" s="18" t="s">
         <v>82</v>
@@ -6027,8 +6238,8 @@
       </c>
     </row>
     <row r="64" spans="1:9" s="6" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A64" s="56"/>
-      <c r="B64" s="56"/>
+      <c r="A64" s="55"/>
+      <c r="B64" s="55"/>
       <c r="C64" s="18">
         <v>18.5</v>
       </c>
@@ -6036,13 +6247,13 @@
         <v>133</v>
       </c>
       <c r="E64" s="18" t="s">
-        <v>286</v>
+        <v>283</v>
       </c>
       <c r="F64" s="18" t="s">
         <v>138</v>
       </c>
       <c r="G64" s="19" t="s">
-        <v>203</v>
+        <v>200</v>
       </c>
       <c r="H64" s="18" t="s">
         <v>82</v>
@@ -6052,8 +6263,8 @@
       </c>
     </row>
     <row r="65" spans="1:12" s="6" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A65" s="56"/>
-      <c r="B65" s="56"/>
+      <c r="A65" s="55"/>
+      <c r="B65" s="55"/>
       <c r="C65" s="18">
         <v>18.600000000000001</v>
       </c>
@@ -6061,13 +6272,13 @@
         <v>133</v>
       </c>
       <c r="E65" s="18" t="s">
-        <v>287</v>
+        <v>284</v>
       </c>
       <c r="F65" s="18" t="s">
         <v>139</v>
       </c>
       <c r="G65" s="19" t="s">
-        <v>204</v>
+        <v>201</v>
       </c>
       <c r="H65" s="18" t="s">
         <v>82</v>
@@ -6077,8 +6288,8 @@
       </c>
     </row>
     <row r="66" spans="1:12" s="6" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A66" s="56"/>
-      <c r="B66" s="56"/>
+      <c r="A66" s="55"/>
+      <c r="B66" s="55"/>
       <c r="C66" s="18">
         <v>18.7</v>
       </c>
@@ -6086,13 +6297,13 @@
         <v>133</v>
       </c>
       <c r="E66" s="18" t="s">
-        <v>288</v>
+        <v>285</v>
       </c>
       <c r="F66" s="18" t="s">
         <v>140</v>
       </c>
       <c r="G66" s="19" t="s">
-        <v>205</v>
+        <v>202</v>
       </c>
       <c r="H66" s="18" t="s">
         <v>82</v>
@@ -6102,8 +6313,8 @@
       </c>
     </row>
     <row r="67" spans="1:12" s="6" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A67" s="56"/>
-      <c r="B67" s="56"/>
+      <c r="A67" s="55"/>
+      <c r="B67" s="55"/>
       <c r="C67" s="18">
         <v>18.8</v>
       </c>
@@ -6111,13 +6322,13 @@
         <v>133</v>
       </c>
       <c r="E67" s="18" t="s">
-        <v>289</v>
+        <v>286</v>
       </c>
       <c r="F67" s="18" t="s">
         <v>141</v>
       </c>
       <c r="G67" s="19" t="s">
-        <v>206</v>
+        <v>203</v>
       </c>
       <c r="H67" s="18" t="s">
         <v>82</v>
@@ -6127,8 +6338,8 @@
       </c>
     </row>
     <row r="68" spans="1:12" s="6" customFormat="1" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A68" s="56"/>
-      <c r="B68" s="56"/>
+      <c r="A68" s="55"/>
+      <c r="B68" s="55"/>
       <c r="C68" s="18">
         <v>18.899999999999999</v>
       </c>
@@ -6136,13 +6347,13 @@
         <v>133</v>
       </c>
       <c r="E68" s="18" t="s">
-        <v>290</v>
+        <v>287</v>
       </c>
       <c r="F68" s="18" t="s">
         <v>142</v>
       </c>
       <c r="G68" s="19" t="s">
-        <v>207</v>
+        <v>204</v>
       </c>
       <c r="H68" s="18" t="s">
         <v>82</v>
@@ -6152,10 +6363,10 @@
       </c>
     </row>
     <row r="69" spans="1:12" s="6" customFormat="1" ht="86.4" x14ac:dyDescent="0.3">
-      <c r="A69" s="63">
+      <c r="A69" s="56">
         <v>19</v>
       </c>
-      <c r="B69" s="66" t="s">
+      <c r="B69" s="59" t="s">
         <v>143</v>
       </c>
       <c r="C69" s="45">
@@ -6165,20 +6376,20 @@
         <v>144</v>
       </c>
       <c r="E69" s="46" t="s">
-        <v>278</v>
+        <v>275</v>
       </c>
       <c r="F69" s="46" t="s">
-        <v>277</v>
+        <v>274</v>
       </c>
       <c r="G69" s="47" t="s">
-        <v>279</v>
+        <v>276</v>
       </c>
       <c r="H69" s="45"/>
       <c r="I69" s="48"/>
     </row>
     <row r="70" spans="1:12" s="6" customFormat="1" ht="129.6" x14ac:dyDescent="0.3">
-      <c r="A70" s="64"/>
-      <c r="B70" s="67"/>
+      <c r="A70" s="57"/>
+      <c r="B70" s="60"/>
       <c r="C70" s="15">
         <v>19.2</v>
       </c>
@@ -6189,7 +6400,7 @@
         <v>146</v>
       </c>
       <c r="F70" s="46" t="s">
-        <v>273</v>
+        <v>270</v>
       </c>
       <c r="G70" s="47" t="s">
         <v>147</v>
@@ -6198,8 +6409,8 @@
       <c r="I70" s="48"/>
     </row>
     <row r="71" spans="1:12" s="6" customFormat="1" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A71" s="65"/>
-      <c r="B71" s="68"/>
+      <c r="A71" s="58"/>
+      <c r="B71" s="61"/>
       <c r="C71" s="34">
         <v>19.3</v>
       </c>
@@ -6217,10 +6428,10 @@
       <c r="I71" s="34"/>
     </row>
     <row r="72" spans="1:12" s="6" customFormat="1" ht="201.6" x14ac:dyDescent="0.3">
-      <c r="A72" s="63">
+      <c r="A72" s="56">
         <v>20</v>
       </c>
-      <c r="B72" s="66" t="s">
+      <c r="B72" s="59" t="s">
         <v>150</v>
       </c>
       <c r="C72" s="45">
@@ -6230,20 +6441,20 @@
         <v>151</v>
       </c>
       <c r="E72" s="46" t="s">
-        <v>299</v>
+        <v>296</v>
       </c>
       <c r="F72" s="46" t="s">
-        <v>300</v>
+        <v>297</v>
       </c>
       <c r="G72" s="47" t="s">
-        <v>301</v>
+        <v>298</v>
       </c>
       <c r="H72" s="45"/>
       <c r="I72" s="48"/>
     </row>
     <row r="73" spans="1:12" s="6" customFormat="1" ht="158.4" x14ac:dyDescent="0.3">
-      <c r="A73" s="64"/>
-      <c r="B73" s="67"/>
+      <c r="A73" s="57"/>
+      <c r="B73" s="60"/>
       <c r="C73" s="15">
         <v>20.2</v>
       </c>
@@ -6251,13 +6462,13 @@
         <v>152</v>
       </c>
       <c r="E73" s="46" t="s">
-        <v>280</v>
+        <v>277</v>
       </c>
       <c r="F73" s="46" t="s">
-        <v>273</v>
+        <v>270</v>
       </c>
       <c r="G73" s="47" t="s">
-        <v>281</v>
+        <v>278</v>
       </c>
       <c r="H73" s="45"/>
       <c r="I73" s="48"/>
@@ -6266,8 +6477,8 @@
       <c r="L73" s="1"/>
     </row>
     <row r="74" spans="1:12" s="6" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A74" s="65"/>
-      <c r="B74" s="68"/>
+      <c r="A74" s="58"/>
+      <c r="B74" s="61"/>
       <c r="C74" s="33">
         <v>20.3</v>
       </c>
@@ -6286,10 +6497,10 @@
       <c r="L74" s="1"/>
     </row>
     <row r="75" spans="1:12" ht="187.2" x14ac:dyDescent="0.3">
-      <c r="A75" s="63">
+      <c r="A75" s="56">
         <v>21</v>
       </c>
-      <c r="B75" s="66" t="s">
+      <c r="B75" s="59" t="s">
         <v>153</v>
       </c>
       <c r="C75" s="45">
@@ -6299,20 +6510,20 @@
         <v>154</v>
       </c>
       <c r="E75" s="46" t="s">
-        <v>291</v>
+        <v>288</v>
       </c>
       <c r="F75" s="46" t="s">
-        <v>292</v>
+        <v>289</v>
       </c>
       <c r="G75" s="47" t="s">
-        <v>293</v>
+        <v>290</v>
       </c>
       <c r="H75" s="45"/>
       <c r="I75" s="48"/>
     </row>
     <row r="76" spans="1:12" ht="129.6" x14ac:dyDescent="0.3">
-      <c r="A76" s="64"/>
-      <c r="B76" s="67"/>
+      <c r="A76" s="57"/>
+      <c r="B76" s="60"/>
       <c r="C76" s="15">
         <v>21.2</v>
       </c>
@@ -6320,10 +6531,10 @@
         <v>155</v>
       </c>
       <c r="E76" s="46" t="s">
-        <v>272</v>
+        <v>269</v>
       </c>
       <c r="F76" s="46" t="s">
-        <v>273</v>
+        <v>270</v>
       </c>
       <c r="G76" s="47" t="s">
         <v>156</v>
@@ -6332,8 +6543,8 @@
       <c r="I76" s="48"/>
     </row>
     <row r="77" spans="1:12" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A77" s="65"/>
-      <c r="B77" s="68"/>
+      <c r="A77" s="58"/>
+      <c r="B77" s="61"/>
       <c r="C77" s="33">
         <v>21.3</v>
       </c>
@@ -6349,10 +6560,10 @@
       <c r="I77" s="34"/>
     </row>
     <row r="78" spans="1:12" ht="259.2" x14ac:dyDescent="0.3">
-      <c r="A78" s="63">
+      <c r="A78" s="56">
         <v>22</v>
       </c>
-      <c r="B78" s="66" t="s">
+      <c r="B78" s="59" t="s">
         <v>157</v>
       </c>
       <c r="C78" s="45">
@@ -6362,41 +6573,41 @@
         <v>158</v>
       </c>
       <c r="E78" s="46" t="s">
-        <v>296</v>
+        <v>293</v>
       </c>
       <c r="F78" s="46" t="s">
-        <v>297</v>
+        <v>294</v>
       </c>
       <c r="G78" s="47" t="s">
-        <v>298</v>
+        <v>295</v>
       </c>
       <c r="H78" s="45"/>
       <c r="I78" s="48"/>
     </row>
     <row r="79" spans="1:12" ht="259.2" x14ac:dyDescent="0.3">
-      <c r="A79" s="64"/>
-      <c r="B79" s="67"/>
+      <c r="A79" s="57"/>
+      <c r="B79" s="60"/>
       <c r="C79" s="15">
         <v>22.2</v>
       </c>
       <c r="D79" s="46" t="s">
-        <v>271</v>
+        <v>268</v>
       </c>
       <c r="E79" s="45" t="s">
-        <v>294</v>
+        <v>291</v>
       </c>
       <c r="F79" s="46" t="s">
-        <v>273</v>
+        <v>270</v>
       </c>
       <c r="G79" s="47" t="s">
-        <v>295</v>
+        <v>292</v>
       </c>
       <c r="H79" s="45"/>
       <c r="I79" s="48"/>
     </row>
     <row r="80" spans="1:12" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A80" s="65"/>
-      <c r="B80" s="68"/>
+      <c r="A80" s="58"/>
+      <c r="B80" s="61"/>
       <c r="C80" s="33">
         <v>22.3</v>
       </c>
@@ -6512,12 +6723,21 @@
   </sheetData>
   <autoFilter ref="I1:I26" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
   <mergeCells count="37">
-    <mergeCell ref="A24:A28"/>
-    <mergeCell ref="B24:B28"/>
-    <mergeCell ref="A30:A40"/>
-    <mergeCell ref="B30:B40"/>
-    <mergeCell ref="A21:A23"/>
-    <mergeCell ref="B21:B23"/>
+    <mergeCell ref="A13:A16"/>
+    <mergeCell ref="B13:B16"/>
+    <mergeCell ref="A17:A20"/>
+    <mergeCell ref="H1:H2"/>
+    <mergeCell ref="I1:I2"/>
+    <mergeCell ref="A8:A12"/>
+    <mergeCell ref="B8:B12"/>
+    <mergeCell ref="A1:A2"/>
+    <mergeCell ref="B1:B2"/>
+    <mergeCell ref="C1:C2"/>
+    <mergeCell ref="D1:F1"/>
+    <mergeCell ref="G1:G2"/>
+    <mergeCell ref="A3:A7"/>
+    <mergeCell ref="B3:B7"/>
+    <mergeCell ref="B17:B20"/>
     <mergeCell ref="A41:A48"/>
     <mergeCell ref="B41:B48"/>
     <mergeCell ref="A75:A77"/>
@@ -6534,21 +6754,12 @@
     <mergeCell ref="B69:B71"/>
     <mergeCell ref="A72:A74"/>
     <mergeCell ref="B72:B74"/>
-    <mergeCell ref="A13:A16"/>
-    <mergeCell ref="B13:B16"/>
-    <mergeCell ref="A17:A20"/>
-    <mergeCell ref="H1:H2"/>
-    <mergeCell ref="I1:I2"/>
-    <mergeCell ref="A8:A12"/>
-    <mergeCell ref="B8:B12"/>
-    <mergeCell ref="A1:A2"/>
-    <mergeCell ref="B1:B2"/>
-    <mergeCell ref="C1:C2"/>
-    <mergeCell ref="D1:F1"/>
-    <mergeCell ref="G1:G2"/>
-    <mergeCell ref="A3:A7"/>
-    <mergeCell ref="B3:B7"/>
-    <mergeCell ref="B17:B20"/>
+    <mergeCell ref="A24:A28"/>
+    <mergeCell ref="B24:B28"/>
+    <mergeCell ref="A30:A40"/>
+    <mergeCell ref="B30:B40"/>
+    <mergeCell ref="A21:A23"/>
+    <mergeCell ref="B21:B23"/>
   </mergeCells>
   <phoneticPr fontId="11" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -6609,7 +6820,7 @@
         <v>8</v>
       </c>
       <c r="H3" s="12" t="s">
-        <v>208</v>
+        <v>205</v>
       </c>
       <c r="I3" s="12" t="s">
         <v>4</v>
@@ -6630,13 +6841,13 @@
         <v>133</v>
       </c>
       <c r="G4" s="8" t="s">
-        <v>209</v>
+        <v>206</v>
       </c>
       <c r="H4" s="8" t="s">
-        <v>210</v>
+        <v>207</v>
       </c>
       <c r="I4" s="13" t="s">
-        <v>211</v>
+        <v>208</v>
       </c>
       <c r="J4" s="9"/>
     </row>
@@ -6654,13 +6865,13 @@
         <v>133</v>
       </c>
       <c r="G5" s="8" t="s">
-        <v>212</v>
+        <v>209</v>
       </c>
       <c r="H5" s="8" t="s">
-        <v>213</v>
+        <v>210</v>
       </c>
       <c r="I5" s="13" t="s">
-        <v>214</v>
+        <v>211</v>
       </c>
       <c r="J5" s="9"/>
     </row>
@@ -6675,16 +6886,16 @@
         <v>14.3</v>
       </c>
       <c r="F6" s="8" t="s">
+        <v>212</v>
+      </c>
+      <c r="G6" s="8" t="s">
+        <v>213</v>
+      </c>
+      <c r="H6" s="8" t="s">
+        <v>214</v>
+      </c>
+      <c r="I6" s="13" t="s">
         <v>215</v>
-      </c>
-      <c r="G6" s="8" t="s">
-        <v>216</v>
-      </c>
-      <c r="H6" s="8" t="s">
-        <v>217</v>
-      </c>
-      <c r="I6" s="13" t="s">
-        <v>218</v>
       </c>
       <c r="J6" s="9"/>
     </row>
@@ -6702,13 +6913,13 @@
         <v>133</v>
       </c>
       <c r="G7" s="8" t="s">
-        <v>219</v>
+        <v>216</v>
       </c>
       <c r="H7" s="8" t="s">
-        <v>220</v>
+        <v>217</v>
       </c>
       <c r="I7" s="13" t="s">
-        <v>221</v>
+        <v>218</v>
       </c>
       <c r="J7" s="9"/>
     </row>
@@ -6726,13 +6937,13 @@
         <v>133</v>
       </c>
       <c r="G8" s="8" t="s">
-        <v>222</v>
+        <v>219</v>
       </c>
       <c r="H8" s="8" t="s">
-        <v>223</v>
+        <v>220</v>
       </c>
       <c r="I8" s="13" t="s">
-        <v>224</v>
+        <v>221</v>
       </c>
       <c r="J8" s="9"/>
     </row>
@@ -6750,13 +6961,13 @@
         <v>133</v>
       </c>
       <c r="G9" s="8" t="s">
-        <v>225</v>
+        <v>222</v>
       </c>
       <c r="H9" s="8" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="I9" s="13" t="s">
-        <v>227</v>
+        <v>224</v>
       </c>
       <c r="J9" s="9"/>
     </row>
@@ -6774,13 +6985,13 @@
         <v>133</v>
       </c>
       <c r="G10" s="8" t="s">
-        <v>228</v>
+        <v>225</v>
       </c>
       <c r="H10" s="8" t="s">
-        <v>229</v>
+        <v>226</v>
       </c>
       <c r="I10" s="13" t="s">
-        <v>230</v>
+        <v>227</v>
       </c>
       <c r="J10" s="9"/>
     </row>
@@ -6798,13 +7009,13 @@
         <v>133</v>
       </c>
       <c r="G11" s="8" t="s">
-        <v>231</v>
+        <v>228</v>
       </c>
       <c r="H11" s="8" t="s">
-        <v>232</v>
+        <v>229</v>
       </c>
       <c r="I11" s="13" t="s">
-        <v>233</v>
+        <v>230</v>
       </c>
       <c r="J11" s="9"/>
     </row>
@@ -6822,13 +7033,13 @@
         <v>133</v>
       </c>
       <c r="G12" s="8" t="s">
-        <v>234</v>
+        <v>231</v>
       </c>
       <c r="H12" s="8" t="s">
-        <v>235</v>
+        <v>232</v>
       </c>
       <c r="I12" s="13" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
       <c r="J12" s="9"/>
     </row>
@@ -6840,19 +7051,19 @@
         <v>80</v>
       </c>
       <c r="E13" s="13" t="s">
-        <v>237</v>
+        <v>234</v>
       </c>
       <c r="F13" s="8" t="s">
         <v>133</v>
       </c>
       <c r="G13" s="8" t="s">
-        <v>238</v>
+        <v>235</v>
       </c>
       <c r="H13" s="8" t="s">
-        <v>239</v>
+        <v>236</v>
       </c>
       <c r="I13" s="13" t="s">
-        <v>240</v>
+        <v>237</v>
       </c>
       <c r="J13" s="9"/>
     </row>
@@ -6870,13 +7081,13 @@
         <v>133</v>
       </c>
       <c r="G14" s="8" t="s">
-        <v>241</v>
+        <v>238</v>
       </c>
       <c r="H14" s="8" t="s">
-        <v>242</v>
+        <v>239</v>
       </c>
       <c r="I14" s="13" t="s">
-        <v>243</v>
+        <v>240</v>
       </c>
       <c r="J14" s="9"/>
     </row>

</xml_diff>